<commit_message>
Revert Game 14 to set up a real end-to-end pipeline test
Restores deck-strength.xlsx to the exact pre-Game-14 state (copied
straight from the untouched Downloads original -- verified zero
unexpected diffs beyond the Game 14 rows and the Player Adjusted Ranks
fix before doing this) and regenerates player-win-rates.json to match.

Games to Update should now show Game 14 as missing again, so it can be
re-added for real through the deployed Cloudflare Worker -> GitHub
Actions pipeline instead of the manual edit used the first time.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deck-strength.xlsx
+++ b/deck-strength.xlsx
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Game Log Season 3'!$A$2:$X$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Player Adjusted Ranks'!$A$1:$L$9</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
   <pivotCaches>
     <pivotCache cacheId="5" r:id="rId7"/>
   </pivotCaches>
@@ -26624,253 +26624,22 @@
       </c>
     </row>
     <row r="51" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A51" s="1">
-        <v>46236</v>
-      </c>
-      <c r="B51" s="7">
-        <v>14</v>
-      </c>
-      <c r="C51" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="D51" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="E51" s="3">
-        <v>2.3</v>
-      </c>
-      <c r="F51" s="7">
-        <v>1</v>
-      </c>
-      <c r="G51" s="7">
-        <v>1</v>
-      </c>
-      <c r="H51" s="7">
-        <v>3</v>
-      </c>
-      <c r="I51" s="7">
-        <v>2</v>
-      </c>
-      <c r="J51" s="7">
-        <f>F51-(1/H51)</f>
-        <v>0.6666666666666667</v>
-      </c>
-      <c r="K51" s="7">
-        <f>((I51-((H51-1)/H51))-(-5/6))/((5-(5/6))-(-5/6))</f>
-        <v>0.4333333333333334</v>
-      </c>
-      <c r="L51" s="7">
-        <f>E51-((E52+E53)/2)</f>
-        <v>-0.75</v>
-      </c>
-      <c r="M51" s="48">
-        <f>0.5+(L51*0.09)</f>
-        <v>0.4325</v>
-      </c>
-      <c r="N51" s="7">
-        <f>((H51-(G51-1))/H51)*(IF(I51&lt;&gt;0,(I51+H51)/H51,1))</f>
-        <v>1.6666666666666667</v>
-      </c>
-      <c r="O51" s="8">
-        <f>(N51-(1/6))/(10/6)</f>
-        <v>0.8999999999999999</v>
-      </c>
-      <c r="P51" s="7">
-        <v>8</v>
-      </c>
-      <c r="Q51" s="8">
-        <f>IF(F51=1,(((1-((P51-3)/15))*0.5)+0.5),((P51/18)*0.5))</f>
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="R51" s="7">
-        <v>1</v>
-      </c>
-      <c r="S51" s="7">
-        <v>0</v>
-      </c>
-      <c r="T51" s="7">
-        <v>0</v>
-      </c>
-      <c r="U51" s="8">
-        <f>IFERROR(T51/S51, 1)</f>
-        <v>1</v>
-      </c>
-      <c r="V51" s="10">
-        <v>0</v>
-      </c>
-      <c r="W51" s="14">
-        <v>2</v>
-      </c>
-      <c r="X51" s="3">
-        <f>((O51*0.3)+(Q51*0.175)+(R51*0.175)+(U51*0.175)+((1-V51)*0.175))+W51</f>
-        <v>2.9408333333333334</v>
-      </c>
+      <c r="A51" s="1"/>
+      <c r="E51" s="3"/>
+      <c r="M51" s="48"/>
+      <c r="X51" s="3"/>
     </row>
     <row r="52" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A52" s="1">
-        <v>46236</v>
-      </c>
-      <c r="B52" s="7">
-        <v>14</v>
-      </c>
-      <c r="C52" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D52" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="E52" s="3">
-        <v>2.5</v>
-      </c>
-      <c r="F52" s="7">
-        <v>0</v>
-      </c>
-      <c r="G52" s="7">
-        <v>2</v>
-      </c>
-      <c r="H52" s="7">
-        <v>3</v>
-      </c>
-      <c r="I52" s="7">
-        <v>0</v>
-      </c>
-      <c r="J52" s="7">
-        <f>F52-(1/H52)</f>
-        <v>-0.3333333333333333</v>
-      </c>
-      <c r="K52" s="7">
-        <f>((I52-((H52-1)/H52))-(-5/6))/((5-(5/6))-(-5/6))</f>
-        <v>0.03333333333333335</v>
-      </c>
-      <c r="L52" s="7">
-        <f>E52-((E51+E53)/2)</f>
-        <v>-0.4500000000000002</v>
-      </c>
-      <c r="M52" s="48">
-        <f>0.5+(L52*0.09)</f>
-        <v>0.45949999999999996</v>
-      </c>
-      <c r="N52" s="7">
-        <f>((H52-(G52-1))/H52)*(IF(I52&lt;&gt;0,(I52+H52)/H52,1))</f>
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="O52" s="8">
-        <f>(N52-(1/6))/(10/6)</f>
-        <v>0.3</v>
-      </c>
-      <c r="P52" s="7">
-        <v>8</v>
-      </c>
-      <c r="Q52" s="8">
-        <f>IF(F52=1,(((1-((P52-3)/15))*0.5)+0.5),((P52/18)*0.5))</f>
-        <v>0.2222222222222222</v>
-      </c>
-      <c r="R52" s="7">
-        <v>0</v>
-      </c>
-      <c r="S52" s="7">
-        <v>1</v>
-      </c>
-      <c r="T52" s="7">
-        <v>0</v>
-      </c>
-      <c r="U52" s="8">
-        <f>IFERROR(T52/S52, 1)</f>
-        <v>0.0</v>
-      </c>
-      <c r="V52" s="10">
-        <v>0</v>
-      </c>
-      <c r="W52" s="14">
-        <v>2</v>
-      </c>
-      <c r="X52" s="3">
-        <f>((O52*0.3)+(Q52*0.175)+(R52*0.175)+(U52*0.175)+((1-V52)*0.175))+W52</f>
-        <v>2.303888888888889</v>
-      </c>
+      <c r="A52" s="1"/>
+      <c r="E52" s="3"/>
+      <c r="M52" s="48"/>
+      <c r="X52" s="3"/>
     </row>
     <row r="53" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A53" s="1">
-        <v>46236</v>
-      </c>
-      <c r="B53" s="7">
-        <v>14</v>
-      </c>
-      <c r="C53" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="D53" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="E53" s="3">
-        <v>3.6</v>
-      </c>
-      <c r="F53" s="7">
-        <v>0</v>
-      </c>
-      <c r="G53" s="7">
-        <v>3</v>
-      </c>
-      <c r="H53" s="7">
-        <v>3</v>
-      </c>
-      <c r="I53" s="7">
-        <v>0</v>
-      </c>
-      <c r="J53" s="7">
-        <f>F53-(1/H53)</f>
-        <v>-0.3333333333333333</v>
-      </c>
-      <c r="K53" s="7">
-        <f>((I53-((H53-1)/H53))-(-5/6))/((5-(5/6))-(-5/6))</f>
-        <v>0.03333333333333335</v>
-      </c>
-      <c r="L53" s="7">
-        <f>E53-((E51+E52)/2)</f>
-        <v>1.2000000000000002</v>
-      </c>
-      <c r="M53" s="48">
-        <f>0.5+(L53*0.09)</f>
-        <v>0.608</v>
-      </c>
-      <c r="N53" s="7">
-        <f>((H53-(G53-1))/H53)*(IF(I53&lt;&gt;0,(I53+H53)/H53,1))</f>
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="O53" s="8">
-        <f>(N53-(1/6))/(10/6)</f>
-        <v>0.09999999999999999</v>
-      </c>
-      <c r="P53" s="7">
-        <v>7</v>
-      </c>
-      <c r="Q53" s="8">
-        <f>IF(F53=1,(((1-((P53-3)/15))*0.5)+0.5),((P53/18)*0.5))</f>
-        <v>0.19444444444444445</v>
-      </c>
-      <c r="R53" s="7">
-        <v>0</v>
-      </c>
-      <c r="S53" s="7">
-        <v>1</v>
-      </c>
-      <c r="T53" s="7">
-        <v>0</v>
-      </c>
-      <c r="U53" s="8">
-        <f>IFERROR(T53/S53, 1)</f>
-        <v>0.0</v>
-      </c>
-      <c r="V53" s="10">
-        <v>0</v>
-      </c>
-      <c r="W53" s="14">
-        <v>3</v>
-      </c>
-      <c r="X53" s="3">
-        <f>((O53*0.3)+(Q53*0.175)+(R53*0.175)+(U53*0.175)+((1-V53)*0.175))+W53</f>
-        <v>3.239027777777778</v>
-      </c>
+      <c r="A53" s="1"/>
+      <c r="E53" s="3"/>
+      <c r="M53" s="48"/>
+      <c r="X53" s="3"/>
     </row>
     <row r="54" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
@@ -28602,7 +28371,7 @@
       </c>
       <c r="B3" s="36">
         <f t="shared" si="0"/>
-        <v>0.24978876904265432</v>
+        <v>0.27472520353960433</v>
       </c>
       <c r="C3">
         <f>COUNTIFS('Game Log Season 3'!$C$3:$C$126, "Ryan", 'Game Log Season 3'!$F$3:$F$126, 1)</f>
@@ -28610,11 +28379,11 @@
       </c>
       <c r="D3">
         <f>COUNTIFS('Game Log Season 3'!$C$3:$C$126, "Ryan", 'Game Log Season 3'!$F$3:$F$126, 0)</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E3" s="36">
         <f t="shared" si="1"/>
-        <v>0.2727272727272727</v>
+        <v>0.3</v>
       </c>
       <c r="F3">
         <f>SUMIFS('Game Log Season 3'!$J$3:$J$126, 'Game Log Season 3'!$C$3:$C$126, "Ryan", 'Game Log Season 3'!$F$3:$F$126, 1)</f>
@@ -28622,15 +28391,15 @@
       </c>
       <c r="G3">
         <f>IFERROR((1-(AVERAGEIFS('Game Log Season 3'!$J$3:$J$126, 'Game Log Season 3'!$C$3:$C$126, "Ryan", 'Game Log Season 3'!$F$3:$F$126, 0)*-1))*D3,0)</f>
-        <v>5.716666666666667</v>
+        <v>5.0500000000000007</v>
       </c>
       <c r="H3" s="36">
         <f t="shared" si="2"/>
-        <v>0.2717622080679406</v>
+        <v>0.29698375870069604</v>
       </c>
       <c r="I3" s="36">
         <f>IF(C3&lt;&gt;0,AVERAGEIF('Game Log Season 3'!$C$3:$C$126, "Ryan", 'Game Log Season 3'!$K$3:$K$126),0)</f>
-        <v>0.1875757575757576</v>
+        <v>0.20300000000000007</v>
       </c>
       <c r="J3">
         <f>IFERROR((1-(AVERAGEIFS('Game Log Season 3'!$M$3:$M$126, 'Game Log Season 3'!$C$3:$C$126, "Ryan", 'Game Log Season 3'!$F$3:$F$126, 1)-0.5))*C3, 0)</f>
@@ -28638,11 +28407,11 @@
       </c>
       <c r="K3">
         <f>IFERROR((1+(AVERAGEIFS('Game Log Season 3'!$M$3:$M$126, 'Game Log Season 3'!$C$3:$C$126, "Ryan", 'Game Log Season 3'!$F$3:$F$126, 0)-0.5))*D3, 0)</f>
-        <v>8.307500000000001</v>
+        <v>7.1994999999999996</v>
       </c>
       <c r="L3" s="36">
         <f t="shared" si="3"/>
-        <v>0.26148991021424123</v>
+        <v>0.29006015185879103</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
@@ -28700,11 +28469,11 @@
       </c>
       <c r="B5" s="36">
         <f t="shared" si="0"/>
-        <v>0.2596530147667175</v>
+        <v>0.20924751206541659</v>
       </c>
       <c r="C5">
         <f>COUNTIFS('Game Log Season 3'!$C$3:$C$126, "Manny", 'Game Log Season 3'!$F$3:$F$126, 1)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D5">
         <f>COUNTIFS('Game Log Season 3'!$C$3:$C$126, "Manny", 'Game Log Season 3'!$F$3:$F$126, 0)</f>
@@ -28712,35 +28481,35 @@
       </c>
       <c r="E5" s="36">
         <f t="shared" si="1"/>
-        <v>0.2857142857142857</v>
+        <v>0.23076923076923078</v>
       </c>
       <c r="F5">
         <f>SUMIFS('Game Log Season 3'!$J$3:$J$126, 'Game Log Season 3'!$C$3:$C$126, "Manny", 'Game Log Season 3'!$F$3:$F$126, 1)</f>
-        <v>2.8333333333333335</v>
+        <v>2.166666666666667</v>
       </c>
       <c r="G5">
         <f>IFERROR((1-(AVERAGEIFS('Game Log Season 3'!$J$3:$J$126, 'Game Log Season 3'!$C$3:$C$126, "Manny", 'Game Log Season 3'!$F$3:$F$126, 0)*-1))*D5,0)</f>
-        <v>7.183333333333334</v>
+        <v>7.1833333333333327</v>
       </c>
       <c r="H5" s="36">
         <f t="shared" si="2"/>
-        <v>0.2828618968386023</v>
+        <v>0.23172905525846707</v>
       </c>
       <c r="I5" s="36">
         <f>IF(C5&lt;&gt;0,AVERAGEIF('Game Log Season 3'!$C$3:$C$126, "Manny", 'Game Log Season 3'!$K$3:$K$126),0)</f>
-        <v>0.16642857142857145</v>
+        <v>0.14589743589743592</v>
       </c>
       <c r="J5">
         <f>IFERROR((1-(AVERAGEIFS('Game Log Season 3'!$M$3:$M$126, 'Game Log Season 3'!$C$3:$C$126, "Manny", 'Game Log Season 3'!$F$3:$F$126, 1)-0.5))*C5, 0)</f>
-        <v>3.8005</v>
+        <v>2.7330000000000001</v>
       </c>
       <c r="K5">
         <f>IFERROR((1+(AVERAGEIFS('Game Log Season 3'!$M$3:$M$126, 'Game Log Season 3'!$C$3:$C$126, "Manny", 'Game Log Season 3'!$F$3:$F$126, 0)-0.5))*D5, 0)</f>
-        <v>9.628</v>
+        <v>9.6280000000000001</v>
       </c>
       <c r="L5" s="36">
         <f t="shared" si="3"/>
-        <v>0.283017462858845</v>
+        <v>0.22109861661677857</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Replace the fragile Deck Win Rates pivot table with plain formulas
Confirmed via a real LibreOffice refresh that this pivot's rendering is
incompatible with Excel's -- refreshing it via automation re-lays the
table out with an extra header row, permanently misaligning the
hand-placed Win Rate formulas beside it. Its cache was also hardcoded to
only the first 48 rows, so it was never going to reflect current data
regardless.

Rebuilt using the exact same player/deck row layout as Current Deck
Strength (COUNTIFS/SUMIFS against Game Log Season 3 instead of a pivot
cache), so both tabs describe the same roster in the same order and can
be maintained by the same future add_player.py/add_deck.py scripts. This
also means it recalculates correctly under the existing headless
LibreOffice pipeline with no special handling needed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deck-strength.xlsx
+++ b/deck-strength.xlsx
@@ -27,9 +27,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Player Adjusted Ranks'!$A$1:$L$9</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
-  <pivotCaches>
-    <pivotCache cacheId="5" r:id="rId7"/>
-  </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -924,1591 +921,6 @@
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
-<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Ryan Munden" refreshedDate="46229.755866898151" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="48" xr:uid="{8056E9D3-2684-4CF2-9B4C-2A704DDBBC90}">
-  <cacheSource type="worksheet">
-    <worksheetSource ref="A2:X50" sheet="Game Log Season 3"/>
-  </cacheSource>
-  <cacheFields count="24">
-    <cacheField name="Game Date" numFmtId="14">
-      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-07-01T00:00:00" maxDate="2026-07-26T00:00:00"/>
-    </cacheField>
-    <cacheField name="Game #" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="13"/>
-    </cacheField>
-    <cacheField name="Player Name" numFmtId="0">
-      <sharedItems count="7">
-        <s v="Becca"/>
-        <s v="Mateo"/>
-        <s v="Manny"/>
-        <s v="Ryan"/>
-        <s v="Kristy"/>
-        <s v="Michelle"/>
-        <s v="Joseph"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Commander" numFmtId="0">
-      <sharedItems count="27">
-        <s v="Ms. Bumbleflower"/>
-        <s v="Captain America, Team Leader"/>
-        <s v="Kruphix, God of Horizons"/>
-        <s v="Fire Lord Zuko"/>
-        <s v="Auntie Ool, Cursewretch"/>
-        <s v="Teval, the Balanced Scale"/>
-        <s v="The Wise Mothman"/>
-        <s v="Killian, Decisive Mentor"/>
-        <s v="Galadriel, Light of Valinor"/>
-        <s v="Zurgo Stormrender"/>
-        <s v="Ureni of the Unwritten"/>
-        <s v="Zada, Hedron Grinder"/>
-        <s v="Rootha, Mastering the Moment"/>
-        <s v="Kratos, God of War"/>
-        <s v="Ultima, Origin of Oblivion"/>
-        <s v="Ashling, The Limitless"/>
-        <s v="Doctor Doom, King of Latveria"/>
-        <s v="Aragorn, the Uniter"/>
-        <s v="Arna Kennerud, Skycaptain"/>
-        <s v="Eshki, Temur's Roar (Manny's)"/>
-        <s v="Witherbloom, The Balancer"/>
-        <s v="Preston Garvey, Minuteman"/>
-        <s v="Lucy MacLean, Positively Armed"/>
-        <s v="Chatterfang, Squirrel General"/>
-        <s v="Namor the Sub-Mariner"/>
-        <s v="Avatar Aang"/>
-        <s v="Yuna, Grand Summoner"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Commander Strength" numFmtId="164">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="2" maxValue="3.9"/>
-    </cacheField>
-    <cacheField name="Game Result" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="1"/>
-    </cacheField>
-    <cacheField name="Place" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="5"/>
-    </cacheField>
-    <cacheField name="Pod Size" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="3" maxValue="5"/>
-    </cacheField>
-    <cacheField name="Knockouts" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="4"/>
-    </cacheField>
-    <cacheField name="Adjusted Pod Size Win/Loss Score" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="-0.33333333333333331" maxValue="0.8"/>
-    </cacheField>
-    <cacheField name="Knockout Score" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="6.6666666666666654E-3" maxValue="0.80666666666666664"/>
-    </cacheField>
-    <cacheField name="Deck Strength Comparison Differential" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="-1.4750000000000001" maxValue="1.2000000000000002"/>
-    </cacheField>
-    <cacheField name="Win Probability based on Deck Strength" numFmtId="9">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0.36724999999999997" maxValue="0.60799999999999998"/>
-    </cacheField>
-    <cacheField name="Player Score" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0.2" maxValue="1.8"/>
-    </cacheField>
-    <cacheField name="Normalized Player Score" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="2.0000000000000011E-2" maxValue="0.98"/>
-    </cacheField>
-    <cacheField name="TOV" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="6" maxValue="14"/>
-    </cacheField>
-    <cacheField name="Normalized TOV" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0.16666666666666666" maxValue="0.8666666666666667"/>
-    </cacheField>
-    <cacheField name="Pop-Off" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="1"/>
-    </cacheField>
-    <cacheField name="Disruptions" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="5"/>
-    </cacheField>
-    <cacheField name="Successful Recoveries" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="3"/>
-    </cacheField>
-    <cacheField name="Deck Resilience Score" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0" maxValue="1"/>
-    </cacheField>
-    <cacheField name="Games Clearly Behind" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="1"/>
-    </cacheField>
-    <cacheField name="Current Deck Bracket" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="2" maxValue="3"/>
-    </cacheField>
-    <cacheField name="Game Calculated Deck Strength" numFmtId="164">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="2.2848611111111112" maxValue="3.9558333333333335"/>
-    </cacheField>
-  </cacheFields>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="48">
-  <r>
-    <d v="2026-07-01T00:00:00"/>
-    <n v="1"/>
-    <x v="0"/>
-    <x v="0"/>
-    <n v="2.9"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="5"/>
-    <n v="0"/>
-    <n v="-0.2"/>
-    <n v="6.6666666666666654E-3"/>
-    <n v="-0.35000000000000009"/>
-    <n v="0.46849999999999997"/>
-    <n v="0.8"/>
-    <n v="0.38"/>
-    <n v="10"/>
-    <n v="0.27777777777777779"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.5126111111111111"/>
-  </r>
-  <r>
-    <d v="2026-07-01T00:00:00"/>
-    <n v="1"/>
-    <x v="1"/>
-    <x v="1"/>
-    <n v="3.7"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="5"/>
-    <n v="0"/>
-    <n v="-0.2"/>
-    <n v="6.6666666666666654E-3"/>
-    <n v="0.64999999999999991"/>
-    <n v="0.5585"/>
-    <n v="0.8"/>
-    <n v="0.38"/>
-    <n v="10"/>
-    <n v="0.27777777777777779"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.687611111111111"/>
-  </r>
-  <r>
-    <d v="2026-07-01T00:00:00"/>
-    <n v="1"/>
-    <x v="2"/>
-    <x v="2"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="5"/>
-    <n v="0"/>
-    <n v="-0.2"/>
-    <n v="6.6666666666666654E-3"/>
-    <n v="-1.4750000000000001"/>
-    <n v="0.36724999999999997"/>
-    <n v="0.8"/>
-    <n v="0.38"/>
-    <n v="10"/>
-    <n v="0.27777777777777779"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.687611111111111"/>
-  </r>
-  <r>
-    <d v="2026-07-01T00:00:00"/>
-    <n v="1"/>
-    <x v="3"/>
-    <x v="3"/>
-    <n v="3.9"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="5"/>
-    <n v="4"/>
-    <n v="0.8"/>
-    <n v="0.80666666666666664"/>
-    <n v="0.89999999999999991"/>
-    <n v="0.58099999999999996"/>
-    <n v="1.8"/>
-    <n v="0.98"/>
-    <n v="10"/>
-    <n v="0.76666666666666661"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.7781666666666665"/>
-  </r>
-  <r>
-    <d v="2026-07-01T00:00:00"/>
-    <n v="1"/>
-    <x v="4"/>
-    <x v="4"/>
-    <n v="3.4"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="5"/>
-    <n v="0"/>
-    <n v="-0.2"/>
-    <n v="6.6666666666666654E-3"/>
-    <n v="0.27499999999999991"/>
-    <n v="0.52474999999999994"/>
-    <n v="0.8"/>
-    <n v="0.38"/>
-    <n v="10"/>
-    <n v="0.27777777777777779"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.3376111111111113"/>
-  </r>
-  <r>
-    <d v="2026-07-03T00:00:00"/>
-    <n v="2"/>
-    <x v="1"/>
-    <x v="5"/>
-    <n v="3"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="4"/>
-    <n v="3"/>
-    <n v="0.75"/>
-    <n v="0.6166666666666667"/>
-    <n v="0"/>
-    <n v="0.5"/>
-    <n v="1.75"/>
-    <n v="0.95"/>
-    <n v="8"/>
-    <n v="0.83333333333333337"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.9558333333333335"/>
-  </r>
-  <r>
-    <d v="2026-07-03T00:00:00"/>
-    <n v="2"/>
-    <x v="5"/>
-    <x v="6"/>
-    <n v="2.7"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="4"/>
-    <n v="0"/>
-    <n v="-0.25"/>
-    <n v="1.6666666666666673E-2"/>
-    <n v="-0.39999999999999991"/>
-    <n v="0.46400000000000002"/>
-    <n v="0.75"/>
-    <n v="0.35000000000000003"/>
-    <n v="8"/>
-    <n v="0.22222222222222221"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.6688888888888886"/>
-  </r>
-  <r>
-    <d v="2026-07-03T00:00:00"/>
-    <n v="2"/>
-    <x v="0"/>
-    <x v="7"/>
-    <n v="2.7"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="4"/>
-    <n v="0"/>
-    <n v="-0.25"/>
-    <n v="1.6666666666666673E-2"/>
-    <n v="-0.39999999999999991"/>
-    <n v="0.46400000000000002"/>
-    <n v="0.75"/>
-    <n v="0.35000000000000003"/>
-    <n v="8"/>
-    <n v="0.22222222222222221"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.4938888888888888"/>
-  </r>
-  <r>
-    <d v="2026-07-03T00:00:00"/>
-    <n v="2"/>
-    <x v="2"/>
-    <x v="8"/>
-    <n v="3.6"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="4"/>
-    <n v="0"/>
-    <n v="-0.25"/>
-    <n v="1.6666666666666673E-2"/>
-    <n v="0.79999999999999982"/>
-    <n v="0.57199999999999995"/>
-    <n v="0.75"/>
-    <n v="0.35000000000000003"/>
-    <n v="8"/>
-    <n v="0.22222222222222221"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="3.318888888888889"/>
-  </r>
-  <r>
-    <d v="2026-07-03T00:00:00"/>
-    <n v="3"/>
-    <x v="0"/>
-    <x v="7"/>
-    <n v="2.5"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="4"/>
-    <n v="1"/>
-    <n v="0.75"/>
-    <n v="0.2166666666666667"/>
-    <n v="-0.80000000000000027"/>
-    <n v="0.42799999999999999"/>
-    <n v="1.25"/>
-    <n v="0.64999999999999991"/>
-    <n v="9"/>
-    <n v="0.8"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.8600000000000003"/>
-  </r>
-  <r>
-    <d v="2026-07-03T00:00:00"/>
-    <n v="3"/>
-    <x v="2"/>
-    <x v="8"/>
-    <n v="3.3"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="4"/>
-    <n v="1"/>
-    <n v="-0.25"/>
-    <n v="0.2166666666666667"/>
-    <n v="0.26666666666666661"/>
-    <n v="0.52400000000000002"/>
-    <n v="0.9375"/>
-    <n v="0.46250000000000002"/>
-    <n v="9"/>
-    <n v="0.25"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="3.3574999999999999"/>
-  </r>
-  <r>
-    <d v="2026-07-03T00:00:00"/>
-    <n v="3"/>
-    <x v="5"/>
-    <x v="6"/>
-    <n v="2.7"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="4"/>
-    <n v="1"/>
-    <n v="-0.25"/>
-    <n v="0.2166666666666667"/>
-    <n v="-0.53333333333333277"/>
-    <n v="0.45200000000000007"/>
-    <n v="0.625"/>
-    <n v="0.27500000000000002"/>
-    <n v="8"/>
-    <n v="0.22222222222222221"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.4713888888888889"/>
-  </r>
-  <r>
-    <d v="2026-07-03T00:00:00"/>
-    <n v="3"/>
-    <x v="1"/>
-    <x v="9"/>
-    <n v="3.9"/>
-    <n v="0"/>
-    <n v="4"/>
-    <n v="4"/>
-    <n v="0"/>
-    <n v="-0.25"/>
-    <n v="1.6666666666666673E-2"/>
-    <n v="1.0666666666666664"/>
-    <n v="0.59599999999999997"/>
-    <n v="0.25"/>
-    <n v="0.05"/>
-    <n v="7"/>
-    <n v="0.19444444444444445"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.5740277777777778"/>
-  </r>
-  <r>
-    <d v="2026-07-03T00:00:00"/>
-    <n v="4"/>
-    <x v="1"/>
-    <x v="10"/>
-    <n v="3.8"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="2"/>
-    <n v="0.66666666666666674"/>
-    <n v="0.4333333333333334"/>
-    <n v="1.0999999999999996"/>
-    <n v="0.59899999999999998"/>
-    <n v="1.6666666666666667"/>
-    <n v="0.89999999999999991"/>
-    <n v="8"/>
-    <n v="0.83333333333333337"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.9408333333333334"/>
-  </r>
-  <r>
-    <d v="2026-07-03T00:00:00"/>
-    <n v="4"/>
-    <x v="0"/>
-    <x v="7"/>
-    <n v="2.9"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="-0.33333333333333331"/>
-    <n v="3.3333333333333347E-2"/>
-    <n v="-0.25"/>
-    <n v="0.47749999999999998"/>
-    <n v="0.66666666666666663"/>
-    <n v="0.3"/>
-    <n v="8"/>
-    <n v="0.22222222222222221"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.3038888888888889"/>
-  </r>
-  <r>
-    <d v="2026-07-03T00:00:00"/>
-    <n v="4"/>
-    <x v="2"/>
-    <x v="11"/>
-    <n v="2.5"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="-0.33333333333333331"/>
-    <n v="3.3333333333333347E-2"/>
-    <n v="-0.84999999999999964"/>
-    <n v="0.42350000000000004"/>
-    <n v="0.66666666666666663"/>
-    <n v="0.3"/>
-    <n v="8"/>
-    <n v="0.22222222222222221"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.3038888888888889"/>
-  </r>
-  <r>
-    <d v="2026-07-08T00:00:00"/>
-    <n v="5"/>
-    <x v="0"/>
-    <x v="0"/>
-    <n v="2.5"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="4"/>
-    <n v="1"/>
-    <n v="0.75"/>
-    <n v="0.2166666666666667"/>
-    <n v="-0.86666666666666714"/>
-    <n v="0.42199999999999993"/>
-    <n v="1.25"/>
-    <n v="0.64999999999999991"/>
-    <n v="14"/>
-    <n v="0.6333333333333333"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="2"/>
-    <n v="0.66666666666666663"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.7725"/>
-  </r>
-  <r>
-    <d v="2026-07-08T00:00:00"/>
-    <n v="5"/>
-    <x v="1"/>
-    <x v="1"/>
-    <n v="3.7"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="4"/>
-    <n v="2"/>
-    <n v="-0.25"/>
-    <n v="0.41666666666666669"/>
-    <n v="0.73333333333333339"/>
-    <n v="0.56600000000000006"/>
-    <n v="1.125"/>
-    <n v="0.57499999999999996"/>
-    <n v="14"/>
-    <n v="0.3888888888888889"/>
-    <n v="1"/>
-    <n v="5"/>
-    <n v="2"/>
-    <n v="0.4"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.6605555555555558"/>
-  </r>
-  <r>
-    <d v="2026-07-08T00:00:00"/>
-    <n v="5"/>
-    <x v="3"/>
-    <x v="12"/>
-    <n v="3.7"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="4"/>
-    <n v="0"/>
-    <n v="-0.25"/>
-    <n v="1.6666666666666673E-2"/>
-    <n v="0.73333333333333339"/>
-    <n v="0.56600000000000006"/>
-    <n v="0.5"/>
-    <n v="0.2"/>
-    <n v="14"/>
-    <n v="0.3888888888888889"/>
-    <n v="1"/>
-    <n v="5"/>
-    <n v="3"/>
-    <n v="0.6"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.5830555555555552"/>
-  </r>
-  <r>
-    <d v="2026-07-08T00:00:00"/>
-    <n v="5"/>
-    <x v="2"/>
-    <x v="2"/>
-    <n v="2.7"/>
-    <n v="0"/>
-    <n v="4"/>
-    <n v="4"/>
-    <n v="0"/>
-    <n v="-0.25"/>
-    <n v="1.6666666666666673E-2"/>
-    <n v="-0.60000000000000009"/>
-    <n v="0.44600000000000001"/>
-    <n v="0.25"/>
-    <n v="0.05"/>
-    <n v="12"/>
-    <n v="0.33333333333333331"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.5983333333333336"/>
-  </r>
-  <r>
-    <d v="2026-07-17T00:00:00"/>
-    <n v="6"/>
-    <x v="1"/>
-    <x v="13"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="5"/>
-    <n v="2"/>
-    <n v="0.8"/>
-    <n v="0.40666666666666662"/>
-    <n v="-0.77499999999999991"/>
-    <n v="0.43025000000000002"/>
-    <n v="1.4"/>
-    <n v="0.73999999999999988"/>
-    <n v="9"/>
-    <n v="0.8"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.887"/>
-  </r>
-  <r>
-    <d v="2026-07-17T00:00:00"/>
-    <n v="6"/>
-    <x v="6"/>
-    <x v="14"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="5"/>
-    <n v="2"/>
-    <n v="-0.2"/>
-    <n v="0.40666666666666662"/>
-    <n v="0.47500000000000009"/>
-    <n v="0.54274999999999995"/>
-    <n v="1.1199999999999999"/>
-    <n v="0.57199999999999995"/>
-    <n v="9"/>
-    <n v="0.25"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.7403500000000003"/>
-  </r>
-  <r>
-    <d v="2026-07-17T00:00:00"/>
-    <n v="6"/>
-    <x v="2"/>
-    <x v="2"/>
-    <n v="2.6"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="5"/>
-    <n v="0"/>
-    <n v="-0.2"/>
-    <n v="6.6666666666666654E-3"/>
-    <n v="-2.4999999999999911E-2"/>
-    <n v="0.49775000000000003"/>
-    <n v="0.6"/>
-    <n v="0.26"/>
-    <n v="8"/>
-    <n v="0.22222222222222221"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.4668888888888887"/>
-  </r>
-  <r>
-    <d v="2026-07-17T00:00:00"/>
-    <n v="6"/>
-    <x v="3"/>
-    <x v="15"/>
-    <n v="3.5"/>
-    <n v="0"/>
-    <n v="4"/>
-    <n v="5"/>
-    <n v="0"/>
-    <n v="-0.2"/>
-    <n v="6.6666666666666654E-3"/>
-    <n v="1.1000000000000001"/>
-    <n v="0.59899999999999998"/>
-    <n v="0.4"/>
-    <n v="0.14000000000000001"/>
-    <n v="8"/>
-    <n v="0.22222222222222221"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.4308888888888891"/>
-  </r>
-  <r>
-    <d v="2026-07-17T00:00:00"/>
-    <n v="6"/>
-    <x v="4"/>
-    <x v="16"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="5"/>
-    <n v="5"/>
-    <n v="0"/>
-    <n v="-0.2"/>
-    <n v="6.6666666666666654E-3"/>
-    <n v="-0.77499999999999991"/>
-    <n v="0.43025000000000002"/>
-    <n v="0.2"/>
-    <n v="2.0000000000000011E-2"/>
-    <n v="8"/>
-    <n v="0.22222222222222221"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.3948888888888886"/>
-  </r>
-  <r>
-    <d v="2026-07-17T00:00:00"/>
-    <n v="7"/>
-    <x v="2"/>
-    <x v="17"/>
-    <n v="3.5"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="4"/>
-    <n v="2"/>
-    <n v="0.75"/>
-    <n v="0.41666666666666669"/>
-    <n v="0.66666666666666652"/>
-    <n v="0.55999999999999994"/>
-    <n v="1.5"/>
-    <n v="0.79999999999999993"/>
-    <n v="8"/>
-    <n v="0.83333333333333337"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.9108333333333336"/>
-  </r>
-  <r>
-    <d v="2026-07-17T00:00:00"/>
-    <n v="7"/>
-    <x v="3"/>
-    <x v="18"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="4"/>
-    <n v="1"/>
-    <n v="-0.25"/>
-    <n v="0.2166666666666667"/>
-    <n v="-1.3333333333333335"/>
-    <n v="0.38"/>
-    <n v="0.9375"/>
-    <n v="0.46250000000000002"/>
-    <n v="8"/>
-    <n v="0.22222222222222221"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.702638888888889"/>
-  </r>
-  <r>
-    <d v="2026-07-17T00:00:00"/>
-    <n v="7"/>
-    <x v="1"/>
-    <x v="1"/>
-    <n v="3.7"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="4"/>
-    <n v="0"/>
-    <n v="-0.25"/>
-    <n v="1.6666666666666673E-2"/>
-    <n v="0.93333333333333313"/>
-    <n v="0.58399999999999996"/>
-    <n v="0.75"/>
-    <n v="0.35000000000000003"/>
-    <n v="8"/>
-    <n v="0.22222222222222221"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.4938888888888888"/>
-  </r>
-  <r>
-    <d v="2026-07-17T00:00:00"/>
-    <n v="7"/>
-    <x v="0"/>
-    <x v="0"/>
-    <n v="2.8"/>
-    <n v="0"/>
-    <n v="4"/>
-    <n v="4"/>
-    <n v="0"/>
-    <n v="-0.25"/>
-    <n v="1.6666666666666673E-2"/>
-    <n v="-0.26666666666666661"/>
-    <n v="0.47599999999999998"/>
-    <n v="0.25"/>
-    <n v="0.05"/>
-    <n v="8"/>
-    <n v="0.22222222222222221"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.403888888888889"/>
-  </r>
-  <r>
-    <d v="2026-07-22T00:00:00"/>
-    <n v="8"/>
-    <x v="2"/>
-    <x v="8"/>
-    <n v="3.4"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="2"/>
-    <n v="0.66666666666666674"/>
-    <n v="0.4333333333333334"/>
-    <n v="1.1999999999999997"/>
-    <n v="0.60799999999999998"/>
-    <n v="1.6666666666666667"/>
-    <n v="0.89999999999999991"/>
-    <n v="9"/>
-    <n v="0.8"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.9350000000000001"/>
-  </r>
-  <r>
-    <d v="2026-07-22T00:00:00"/>
-    <n v="8"/>
-    <x v="0"/>
-    <x v="19"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="-0.33333333333333331"/>
-    <n v="3.3333333333333347E-2"/>
-    <n v="-0.89999999999999991"/>
-    <n v="0.41900000000000004"/>
-    <n v="0.66666666666666663"/>
-    <n v="0.3"/>
-    <n v="9"/>
-    <n v="0.25"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.4837500000000001"/>
-  </r>
-  <r>
-    <d v="2026-07-22T00:00:00"/>
-    <n v="8"/>
-    <x v="3"/>
-    <x v="20"/>
-    <n v="2.4"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="-0.33333333333333331"/>
-    <n v="3.3333333333333347E-2"/>
-    <n v="-0.30000000000000027"/>
-    <n v="0.47299999999999998"/>
-    <n v="0.33333333333333331"/>
-    <n v="9.9999999999999992E-2"/>
-    <n v="8"/>
-    <n v="0.22222222222222221"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.5938888888888889"/>
-  </r>
-  <r>
-    <d v="2026-07-24T00:00:00"/>
-    <n v="9"/>
-    <x v="2"/>
-    <x v="8"/>
-    <n v="3.9"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="4"/>
-    <n v="3"/>
-    <n v="0.75"/>
-    <n v="0.6166666666666667"/>
-    <n v="1.0999999999999996"/>
-    <n v="0.59899999999999998"/>
-    <n v="1.75"/>
-    <n v="0.95"/>
-    <n v="13"/>
-    <n v="0.66666666666666674"/>
-    <n v="1"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="0.5"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.8391666666666664"/>
-  </r>
-  <r>
-    <d v="2026-07-24T00:00:00"/>
-    <n v="9"/>
-    <x v="3"/>
-    <x v="21"/>
-    <n v="3.5"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="4"/>
-    <n v="0"/>
-    <n v="-0.25"/>
-    <n v="1.6666666666666673E-2"/>
-    <n v="0.56666666666666643"/>
-    <n v="0.55099999999999993"/>
-    <n v="0.75"/>
-    <n v="0.35000000000000003"/>
-    <n v="13"/>
-    <n v="0.3611111111111111"/>
-    <n v="1"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="0.5"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.6056944444444445"/>
-  </r>
-  <r>
-    <d v="2026-07-24T00:00:00"/>
-    <n v="9"/>
-    <x v="1"/>
-    <x v="13"/>
-    <n v="2.9"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="4"/>
-    <n v="0"/>
-    <n v="-0.25"/>
-    <n v="1.6666666666666673E-2"/>
-    <n v="-0.23333333333333339"/>
-    <n v="0.47899999999999998"/>
-    <n v="0.75"/>
-    <n v="0.35000000000000003"/>
-    <n v="13"/>
-    <n v="0.3611111111111111"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="2"/>
-    <n v="0.66666666666666663"/>
-    <n v="1"/>
-    <n v="2"/>
-    <n v="2.2848611111111112"/>
-  </r>
-  <r>
-    <d v="2026-07-24T00:00:00"/>
-    <n v="9"/>
-    <x v="5"/>
-    <x v="22"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="4"/>
-    <n v="0"/>
-    <n v="-0.25"/>
-    <n v="1.6666666666666673E-2"/>
-    <n v="-1.4333333333333336"/>
-    <n v="0.371"/>
-    <n v="0.75"/>
-    <n v="0.35000000000000003"/>
-    <n v="13"/>
-    <n v="0.3611111111111111"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="0.5"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.4306944444444443"/>
-  </r>
-  <r>
-    <d v="2026-07-24T00:00:00"/>
-    <n v="10"/>
-    <x v="1"/>
-    <x v="23"/>
-    <n v="3"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="2"/>
-    <n v="0.66666666666666674"/>
-    <n v="0.4333333333333334"/>
-    <n v="0.25"/>
-    <n v="0.52249999999999996"/>
-    <n v="1.6666666666666667"/>
-    <n v="0.89999999999999991"/>
-    <n v="9"/>
-    <n v="0.8"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.9350000000000001"/>
-  </r>
-  <r>
-    <d v="2026-07-24T00:00:00"/>
-    <n v="10"/>
-    <x v="2"/>
-    <x v="2"/>
-    <n v="2.5"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="-0.33333333333333331"/>
-    <n v="3.3333333333333347E-2"/>
-    <n v="-0.5"/>
-    <n v="0.45500000000000002"/>
-    <n v="0.66666666666666663"/>
-    <n v="0.3"/>
-    <n v="9"/>
-    <n v="0.25"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.4837500000000001"/>
-  </r>
-  <r>
-    <d v="2026-07-24T00:00:00"/>
-    <n v="10"/>
-    <x v="3"/>
-    <x v="24"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="-0.33333333333333331"/>
-    <n v="3.3333333333333347E-2"/>
-    <n v="0.25"/>
-    <n v="0.52249999999999996"/>
-    <n v="0.66666666666666663"/>
-    <n v="0.3"/>
-    <n v="9"/>
-    <n v="0.25"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="3.3087499999999999"/>
-  </r>
-  <r>
-    <d v="2026-07-25T00:00:00"/>
-    <n v="11"/>
-    <x v="3"/>
-    <x v="18"/>
-    <n v="2.7"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="2"/>
-    <n v="0.66666666666666674"/>
-    <n v="0.4333333333333334"/>
-    <n v="-0.19999999999999973"/>
-    <n v="0.48200000000000004"/>
-    <n v="1.6666666666666667"/>
-    <n v="0.89999999999999991"/>
-    <n v="8"/>
-    <n v="0.83333333333333337"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.9408333333333334"/>
-  </r>
-  <r>
-    <d v="2026-07-25T00:00:00"/>
-    <n v="11"/>
-    <x v="2"/>
-    <x v="11"/>
-    <n v="2.2999999999999998"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="-0.33333333333333331"/>
-    <n v="3.3333333333333347E-2"/>
-    <n v="-0.80000000000000027"/>
-    <n v="0.42799999999999999"/>
-    <n v="0.66666666666666663"/>
-    <n v="0.3"/>
-    <n v="8"/>
-    <n v="0.22222222222222221"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.653888888888889"/>
-  </r>
-  <r>
-    <d v="2026-07-25T00:00:00"/>
-    <n v="11"/>
-    <x v="1"/>
-    <x v="1"/>
-    <n v="3.5"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="-0.33333333333333331"/>
-    <n v="3.3333333333333347E-2"/>
-    <n v="1"/>
-    <n v="0.59"/>
-    <n v="0.66666666666666663"/>
-    <n v="0.3"/>
-    <n v="8"/>
-    <n v="0.22222222222222221"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.653888888888889"/>
-  </r>
-  <r>
-    <d v="2026-07-25T00:00:00"/>
-    <n v="12"/>
-    <x v="1"/>
-    <x v="13"/>
-    <n v="2.2999999999999998"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="2"/>
-    <n v="0.66666666666666674"/>
-    <n v="0.4333333333333334"/>
-    <n v="-0.75"/>
-    <n v="0.4325"/>
-    <n v="1.6666666666666667"/>
-    <n v="0.89999999999999991"/>
-    <n v="7"/>
-    <n v="0.8666666666666667"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2.9466666666666668"/>
-  </r>
-  <r>
-    <d v="2026-07-25T00:00:00"/>
-    <n v="12"/>
-    <x v="2"/>
-    <x v="2"/>
-    <n v="2.5"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="-0.33333333333333331"/>
-    <n v="3.3333333333333347E-2"/>
-    <n v="-0.45000000000000018"/>
-    <n v="0.45949999999999996"/>
-    <n v="0.66666666666666663"/>
-    <n v="0.3"/>
-    <n v="7"/>
-    <n v="0.19444444444444445"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="2"/>
-    <n v="2.2990277777777779"/>
-  </r>
-  <r>
-    <d v="2026-07-25T00:00:00"/>
-    <n v="12"/>
-    <x v="3"/>
-    <x v="12"/>
-    <n v="3.6"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="-0.33333333333333331"/>
-    <n v="3.3333333333333347E-2"/>
-    <n v="1.2000000000000002"/>
-    <n v="0.60799999999999998"/>
-    <n v="0.33333333333333331"/>
-    <n v="9.9999999999999992E-2"/>
-    <n v="6"/>
-    <n v="0.16666666666666666"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.5841666666666665"/>
-  </r>
-  <r>
-    <d v="2026-07-25T00:00:00"/>
-    <n v="13"/>
-    <x v="3"/>
-    <x v="24"/>
-    <n v="3.3"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="2"/>
-    <n v="0.66666666666666674"/>
-    <n v="0.4333333333333334"/>
-    <n v="-5.0000000000000266E-2"/>
-    <n v="0.4955"/>
-    <n v="1.6666666666666667"/>
-    <n v="0.89999999999999991"/>
-    <n v="11"/>
-    <n v="0.73333333333333339"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.9233333333333333"/>
-  </r>
-  <r>
-    <d v="2026-07-25T00:00:00"/>
-    <n v="13"/>
-    <x v="2"/>
-    <x v="25"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="-0.33333333333333331"/>
-    <n v="3.3333333333333347E-2"/>
-    <n v="-0.5"/>
-    <n v="0.45500000000000002"/>
-    <n v="0.66666666666666663"/>
-    <n v="0.3"/>
-    <n v="11"/>
-    <n v="0.30555555555555558"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.4934722222222221"/>
-  </r>
-  <r>
-    <d v="2026-07-25T00:00:00"/>
-    <n v="13"/>
-    <x v="1"/>
-    <x v="26"/>
-    <n v="3.7"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="-0.33333333333333331"/>
-    <n v="3.3333333333333347E-2"/>
-    <n v="0.55000000000000027"/>
-    <n v="0.54949999999999999"/>
-    <n v="0.33333333333333331"/>
-    <n v="9.9999999999999992E-2"/>
-    <n v="9"/>
-    <n v="0.25"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="3.5987499999999999"/>
-  </r>
-</pivotCacheRecords>
-</file>
-
-<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5EA05A64-BCF0-4340-B4AC-DDB207BCA579}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A1:C36" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="24">
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="8">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="28">
-        <item x="0"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item x="15"/>
-        <item x="16"/>
-        <item x="17"/>
-        <item x="18"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item x="21"/>
-        <item x="22"/>
-        <item x="23"/>
-        <item x="24"/>
-        <item x="25"/>
-        <item x="26"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="9" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="164" showAll="0"/>
-  </pivotFields>
-  <rowFields count="2">
-    <field x="2"/>
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="35">
-    <i>
-      <x/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i r="1">
-      <x v="7"/>
-    </i>
-    <i r="1">
-      <x v="19"/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="8"/>
-    </i>
-    <i r="1">
-      <x v="11"/>
-    </i>
-    <i r="1">
-      <x v="17"/>
-    </i>
-    <i r="1">
-      <x v="25"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i r="1">
-      <x v="9"/>
-    </i>
-    <i r="1">
-      <x v="10"/>
-    </i>
-    <i r="1">
-      <x v="13"/>
-    </i>
-    <i r="1">
-      <x v="23"/>
-    </i>
-    <i r="1">
-      <x v="26"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="12"/>
-    </i>
-    <i r="1">
-      <x v="15"/>
-    </i>
-    <i r="1">
-      <x v="18"/>
-    </i>
-    <i r="1">
-      <x v="20"/>
-    </i>
-    <i r="1">
-      <x v="21"/>
-    </i>
-    <i r="1">
-      <x v="24"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="16"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i r="1">
-      <x v="6"/>
-    </i>
-    <i r="1">
-      <x v="22"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i r="1">
-      <x v="14"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-  </colItems>
-  <dataFields count="2">
-    <dataField name="Count of Game Result" fld="5" subtotal="count" baseField="2" baseItem="0"/>
-    <dataField name="Sum of Game Result" fld="5" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -28109,7 +26521,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78721C01-74C8-4B39-8A98-A9995A31B797}">
-  <dimension ref="A1:D54"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.88671875" bestFit="1" customWidth="1"/>
@@ -28118,598 +26530,1224 @@
     <col min="4" max="4" width="23.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D1" s="58" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="43" t="s">
+    <row r="1" spans="1:4">
+      <c r="A1" s="51" t="inlineStr">
+        <is>
+          <t>Player / Deck</t>
+        </is>
+      </c>
+      <c r="B1" s="51" t="inlineStr">
+        <is>
+          <t>Games Played</t>
+        </is>
+      </c>
+      <c r="C1" s="51" t="inlineStr">
+        <is>
+          <t>Wins</t>
+        </is>
+      </c>
+      <c r="D1" s="51" t="inlineStr">
+        <is>
+          <t>Win Rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="50" t="inlineStr">
+        <is>
+          <t>Becca</t>
+        </is>
+      </c>
+      <c r="B2" s="52">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A2)</f>
+        <v>7</v>
+      </c>
+      <c r="C2" s="52">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A2,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>2</v>
+      </c>
+      <c r="D2" s="52">
+        <f>IFERROR(C2/B2,0)</f>
+        <v>0.2857142857142857</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="41" t="inlineStr">
+        <is>
+          <t>Ms. Bumbleflower</t>
+        </is>
+      </c>
+      <c r="B3" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A3)</f>
+        <v>3</v>
+      </c>
+      <c r="C3" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A3,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>1</v>
+      </c>
+      <c r="D3" s="41">
+        <f>IFERROR(C3/B3,0)</f>
+        <v>0.3333333333333333</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="41" t="inlineStr">
+        <is>
+          <t>Aminatou, Veil Piercer</t>
+        </is>
+      </c>
+      <c r="B4" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A4)</f>
+        <v>0</v>
+      </c>
+      <c r="C4" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A4,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D4" s="41">
+        <f>IFERROR(C4/B4,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="41" t="inlineStr">
+        <is>
+          <t>Killian, Decisive Mentor</t>
+        </is>
+      </c>
+      <c r="B5" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A5)</f>
+        <v>3</v>
+      </c>
+      <c r="C5" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A5,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>1</v>
+      </c>
+      <c r="D5" s="41">
+        <f>IFERROR(C5/B5,0)</f>
+        <v>0.3333333333333333</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="41" t="inlineStr">
+        <is>
+          <t>Eshki, Temur's Roar (Manny's)</t>
+        </is>
+      </c>
+      <c r="B6" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A6)</f>
+        <v>1</v>
+      </c>
+      <c r="C6" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A6,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="41">
+        <f>IFERROR(C6/B6,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="50" t="inlineStr">
+        <is>
+          <t>Manny</t>
+        </is>
+      </c>
+      <c r="B7" s="52">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A7)</f>
+        <v>14</v>
+      </c>
+      <c r="C7" s="52">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A7,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>4</v>
+      </c>
+      <c r="D7" s="52">
+        <f>IFERROR(C7/B7,0)</f>
+        <v>0.2857142857142857</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="41" t="inlineStr">
+        <is>
+          <t>Galadriel, Light of Valinor</t>
+        </is>
+      </c>
+      <c r="B8" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A8)</f>
+        <v>4</v>
+      </c>
+      <c r="C8" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A8,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>2</v>
+      </c>
+      <c r="D8" s="41">
+        <f>IFERROR(C8/B8,0)</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="41" t="inlineStr">
+        <is>
+          <t>Atraxa, Praetor's Voice</t>
+        </is>
+      </c>
+      <c r="B9" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A9)</f>
+        <v>0</v>
+      </c>
+      <c r="C9" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A9,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D9" s="41">
+        <f>IFERROR(C9/B9,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="41" t="inlineStr">
+        <is>
+          <t>Athreos, God of Passage</t>
+        </is>
+      </c>
+      <c r="B10" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A10)</f>
+        <v>0</v>
+      </c>
+      <c r="C10" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A10,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D10" s="41">
+        <f>IFERROR(C10/B10,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="41" t="inlineStr">
+        <is>
+          <t>Fynn, the Fangbearer</t>
+        </is>
+      </c>
+      <c r="B11" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A11)</f>
+        <v>0</v>
+      </c>
+      <c r="C11" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A11,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D11" s="41">
+        <f>IFERROR(C11/B11,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="41" t="inlineStr">
+        <is>
+          <t>Frodo, Adventurous Hobbit/Sam, Loyal Attendant</t>
+        </is>
+      </c>
+      <c r="B12" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A12)</f>
+        <v>0</v>
+      </c>
+      <c r="C12" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A12,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D12" s="41">
+        <f>IFERROR(C12/B12,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="41" t="inlineStr">
+        <is>
+          <t>Zada, Hedron Grinder</t>
+        </is>
+      </c>
+      <c r="B13" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A13)</f>
+        <v>2</v>
+      </c>
+      <c r="C13" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A13,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D13" s="41">
+        <f>IFERROR(C13/B13,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="41" t="inlineStr">
+        <is>
+          <t>Ureni of the Unwritten</t>
+        </is>
+      </c>
+      <c r="B14" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A14)</f>
+        <v>0</v>
+      </c>
+      <c r="C14" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A14,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D14" s="41">
+        <f>IFERROR(C14/B14,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="41" t="inlineStr">
+        <is>
+          <t>Aragorn, the Uniter</t>
+        </is>
+      </c>
+      <c r="B15" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A15)</f>
+        <v>1</v>
+      </c>
+      <c r="C15" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A15,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>1</v>
+      </c>
+      <c r="D15" s="41">
+        <f>IFERROR(C15/B15,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="41" t="inlineStr">
+        <is>
+          <t>Kruphix, God of Horizons</t>
+        </is>
+      </c>
+      <c r="B16" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A16)</f>
+        <v>6</v>
+      </c>
+      <c r="C16" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A16,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>1</v>
+      </c>
+      <c r="D16" s="41">
+        <f>IFERROR(C16/B16,0)</f>
+        <v>0.16666666666666666</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="41" t="inlineStr">
+        <is>
+          <t>Avatar Aang</t>
+        </is>
+      </c>
+      <c r="B17" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A17)</f>
+        <v>1</v>
+      </c>
+      <c r="C17" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A17,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D17" s="41">
+        <f>IFERROR(C17/B17,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="50" t="inlineStr">
+        <is>
+          <t>Mateo</t>
+        </is>
+      </c>
+      <c r="B18" s="52">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A18)</f>
+        <v>12</v>
+      </c>
+      <c r="C18" s="52">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A18,'Game Log Season 3'!$F$3:$F$1000,1)</f>
         <v>5</v>
       </c>
-      <c r="B2">
-        <v>7</v>
-      </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2" s="45">
-        <f t="shared" ref="D2:D36" si="0">C2/B2</f>
-        <v>0.2857142857142857</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="44" t="s">
+      <c r="D18" s="52">
+        <f>IFERROR(C18/B18,0)</f>
+        <v>0.4166666666666667</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="41" t="inlineStr">
+        <is>
+          <t>High Perfect Morcant</t>
+        </is>
+      </c>
+      <c r="B19" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A19)</f>
+        <v>0</v>
+      </c>
+      <c r="C19" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A19,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D19" s="41">
+        <f>IFERROR(C19/B19,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="41" t="inlineStr">
+        <is>
+          <t>Leonardo, the Balance/Michelangelo, the Heart</t>
+        </is>
+      </c>
+      <c r="B20" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A20)</f>
+        <v>0</v>
+      </c>
+      <c r="C20" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A20,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D20" s="41">
+        <f>IFERROR(C20/B20,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="41" t="inlineStr">
+        <is>
+          <t>Zurgo Stormrender</t>
+        </is>
+      </c>
+      <c r="B21" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A21)</f>
+        <v>1</v>
+      </c>
+      <c r="C21" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A21,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D21" s="41">
+        <f>IFERROR(C21/B21,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>Fire Lord Azula</t>
+        </is>
+      </c>
+      <c r="B22" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A22)</f>
+        <v>0</v>
+      </c>
+      <c r="C22" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A22,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D22" s="41">
+        <f>IFERROR(C22/B22,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="41" t="inlineStr">
+        <is>
+          <t>Quintorius, History Chaser</t>
+        </is>
+      </c>
+      <c r="B23" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A23)</f>
+        <v>0</v>
+      </c>
+      <c r="C23" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A23,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D23" s="41">
+        <f>IFERROR(C23/B23,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" s="41" t="inlineStr">
+        <is>
+          <t>Auntie Ool, Cursewretch</t>
+        </is>
+      </c>
+      <c r="B24" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A24)</f>
+        <v>0</v>
+      </c>
+      <c r="C24" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A24,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D24" s="41">
+        <f>IFERROR(C24/B24,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="41" t="inlineStr">
+        <is>
+          <t>Killian, Decisive Mentor (Becca's)</t>
+        </is>
+      </c>
+      <c r="B25" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A25)</f>
+        <v>0</v>
+      </c>
+      <c r="C25" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A25,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D25" s="41">
+        <f>IFERROR(C25/B25,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="41" t="inlineStr">
+        <is>
+          <t>Noctis, Heir Apparent</t>
+        </is>
+      </c>
+      <c r="B26" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A26)</f>
+        <v>0</v>
+      </c>
+      <c r="C26" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A26,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D26" s="41">
+        <f>IFERROR(C26/B26,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="41" t="inlineStr">
+        <is>
+          <t>Yuna, Grand Summoner</t>
+        </is>
+      </c>
+      <c r="B27" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A27)</f>
+        <v>1</v>
+      </c>
+      <c r="C27" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A27,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D27" s="41">
+        <f>IFERROR(C27/B27,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="41" t="inlineStr">
+        <is>
+          <t>Ureni of the Unwritten</t>
+        </is>
+      </c>
+      <c r="B28" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A28)</f>
+        <v>1</v>
+      </c>
+      <c r="C28" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A28,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>1</v>
+      </c>
+      <c r="D28" s="41">
+        <f>IFERROR(C28/B28,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" s="41" t="inlineStr">
+        <is>
+          <t>Captain America, Team Leader</t>
+        </is>
+      </c>
+      <c r="B29" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A29)</f>
+        <v>4</v>
+      </c>
+      <c r="C29" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A29,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D29" s="41">
+        <f>IFERROR(C29/B29,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" s="41" t="inlineStr">
+        <is>
+          <t>Teval, the Balanced Scale</t>
+        </is>
+      </c>
+      <c r="B30" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A30)</f>
+        <v>1</v>
+      </c>
+      <c r="C30" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A30,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>1</v>
+      </c>
+      <c r="D30" s="41">
+        <f>IFERROR(C30/B30,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="41" t="inlineStr">
+        <is>
+          <t>Kratos, God of War</t>
+        </is>
+      </c>
+      <c r="B31" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A31)</f>
+        <v>3</v>
+      </c>
+      <c r="C31" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A31,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>2</v>
+      </c>
+      <c r="D31" s="41">
+        <f>IFERROR(C31/B31,0)</f>
+        <v>0.6666666666666666</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" s="41" t="inlineStr">
+        <is>
+          <t>Chatterfang, Squirrel General</t>
+        </is>
+      </c>
+      <c r="B32" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A32)</f>
+        <v>1</v>
+      </c>
+      <c r="C32" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A32,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>1</v>
+      </c>
+      <c r="D32" s="41">
+        <f>IFERROR(C32/B32,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="50" t="inlineStr">
+        <is>
+          <t>Ryan</t>
+        </is>
+      </c>
+      <c r="B33" s="52">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A33)</f>
         <v>11</v>
       </c>
-      <c r="B3">
-        <v>3</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3" s="36">
-        <f t="shared" si="0"/>
-        <v>0.33333333333333331</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="44" t="s">
-        <v>90</v>
-      </c>
-      <c r="B4">
-        <v>3</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4" s="36">
-        <f t="shared" si="0"/>
-        <v>0.33333333333333331</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="44" t="s">
-        <v>117</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5" s="36">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6">
-        <v>13</v>
-      </c>
-      <c r="C6">
-        <v>3</v>
-      </c>
-      <c r="D6" s="45">
-        <f t="shared" si="0"/>
-        <v>0.23076923076923078</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="44" t="s">
-        <v>113</v>
-      </c>
-      <c r="B7">
-        <v>5</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7" s="36">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="44" t="s">
-        <v>86</v>
-      </c>
-      <c r="B8">
+      <c r="C33" s="52">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A33,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>3</v>
+      </c>
+      <c r="D33" s="52">
+        <f>IFERROR(C33/B33,0)</f>
+        <v>0.2727272727272727</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" s="41" t="inlineStr">
+        <is>
+          <t>Eowyn, Shieldmaiden</t>
+        </is>
+      </c>
+      <c r="B34" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A34)</f>
+        <v>0</v>
+      </c>
+      <c r="C34" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A34,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D34" s="41">
+        <f>IFERROR(C34/B34,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35" s="41" t="inlineStr">
+        <is>
+          <t>Ashling, The Limitless</t>
+        </is>
+      </c>
+      <c r="B35" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A35)</f>
+        <v>1</v>
+      </c>
+      <c r="C35" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A35,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D35" s="41">
+        <f>IFERROR(C35/B35,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" s="41" t="inlineStr">
+        <is>
+          <t>Cloud, Ex-SOLDIER</t>
+        </is>
+      </c>
+      <c r="B36" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A36)</f>
+        <v>0</v>
+      </c>
+      <c r="C36" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A36,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D36" s="41">
+        <f>IFERROR(C36/B36,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" s="41" t="inlineStr">
+        <is>
+          <t>Kratos, Stoic Father/Atreus, Impulsive Son</t>
+        </is>
+      </c>
+      <c r="B37" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A37)</f>
+        <v>0</v>
+      </c>
+      <c r="C37" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A37,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D37" s="41">
+        <f>IFERROR(C37/B37,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38" s="41" t="inlineStr">
+        <is>
+          <t>Fire Lord Zuko</t>
+        </is>
+      </c>
+      <c r="B38" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A38)</f>
+        <v>1</v>
+      </c>
+      <c r="C38" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A38,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>1</v>
+      </c>
+      <c r="D38" s="41">
+        <f>IFERROR(C38/B38,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" s="41" t="inlineStr">
+        <is>
+          <t>Witherbloom, The Balancer</t>
+        </is>
+      </c>
+      <c r="B39" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A39)</f>
+        <v>1</v>
+      </c>
+      <c r="C39" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A39,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D39" s="41">
+        <f>IFERROR(C39/B39,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" s="41" t="inlineStr">
+        <is>
+          <t>Preston Garvey, Minuteman</t>
+        </is>
+      </c>
+      <c r="B40" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A40)</f>
+        <v>2</v>
+      </c>
+      <c r="C40" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A40,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D40" s="41">
+        <f>IFERROR(C40/B40,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" s="41" t="inlineStr">
+        <is>
+          <t>Giada, Font of Hope</t>
+        </is>
+      </c>
+      <c r="B41" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A41)</f>
+        <v>0</v>
+      </c>
+      <c r="C41" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A41,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D41" s="41">
+        <f>IFERROR(C41/B41,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" s="41" t="inlineStr">
+        <is>
+          <t>Rootha, Mastering the Moment</t>
+        </is>
+      </c>
+      <c r="B42" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A42)</f>
+        <v>2</v>
+      </c>
+      <c r="C42" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A42,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D42" s="41">
+        <f>IFERROR(C42/B42,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" s="41" t="inlineStr">
+        <is>
+          <t>Arna Kennerud, Skycaptain</t>
+        </is>
+      </c>
+      <c r="B43" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A43)</f>
+        <v>2</v>
+      </c>
+      <c r="C43" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A43,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>1</v>
+      </c>
+      <c r="D43" s="41">
+        <f>IFERROR(C43/B43,0)</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" s="41" t="inlineStr">
+        <is>
+          <t>Namor the Sub-Mariner</t>
+        </is>
+      </c>
+      <c r="B44" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A44)</f>
+        <v>2</v>
+      </c>
+      <c r="C44" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A44,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>1</v>
+      </c>
+      <c r="D44" s="41">
+        <f>IFERROR(C44/B44,0)</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45" s="50" t="inlineStr">
+        <is>
+          <t>Kristy</t>
+        </is>
+      </c>
+      <c r="B45" s="52">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A45)</f>
+        <v>2</v>
+      </c>
+      <c r="C45" s="52">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A45,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D45" s="52">
+        <f>IFERROR(C45/B45,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" s="41" t="inlineStr">
+        <is>
+          <t>Edgar Markov</t>
+        </is>
+      </c>
+      <c r="B46" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A46)</f>
+        <v>0</v>
+      </c>
+      <c r="C46" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A46,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D46" s="41">
+        <f>IFERROR(C46/B46,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" s="41" t="inlineStr">
+        <is>
+          <t>Auntie Ool, Cursewretch</t>
+        </is>
+      </c>
+      <c r="B47" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A47)</f>
+        <v>1</v>
+      </c>
+      <c r="C47" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A47,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D47" s="41">
+        <f>IFERROR(C47/B47,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
+      <c r="A48" s="41" t="inlineStr">
+        <is>
+          <t>Dina, Essence Brewer</t>
+        </is>
+      </c>
+      <c r="B48" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A48)</f>
+        <v>0</v>
+      </c>
+      <c r="C48" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A48,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D48" s="41">
+        <f>IFERROR(C48/B48,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
+      <c r="A49" s="41" t="inlineStr">
+        <is>
+          <t>Niv-Mizzet, Parun</t>
+        </is>
+      </c>
+      <c r="B49" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A49)</f>
+        <v>0</v>
+      </c>
+      <c r="C49" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A49,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D49" s="41">
+        <f>IFERROR(C49/B49,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
+      <c r="A50" s="41" t="inlineStr">
+        <is>
+          <t>Doctor Doom, King of Latveria</t>
+        </is>
+      </c>
+      <c r="B50" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A50)</f>
+        <v>1</v>
+      </c>
+      <c r="C50" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A50,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D50" s="41">
+        <f>IFERROR(C50/B50,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
+      <c r="A51" s="50" t="inlineStr">
+        <is>
+          <t>Joseph</t>
+        </is>
+      </c>
+      <c r="B51" s="52">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A51)</f>
+        <v>1</v>
+      </c>
+      <c r="C51" s="52">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A51,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D51" s="52">
+        <f>IFERROR(C51/B51,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
+      <c r="A52" s="41" t="inlineStr">
+        <is>
+          <t>Valgavoth, Harrower of Souls</t>
+        </is>
+      </c>
+      <c r="B52" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A52)</f>
+        <v>0</v>
+      </c>
+      <c r="C52" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A52,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D52" s="41">
+        <f>IFERROR(C52/B52,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="A53" s="41" t="inlineStr">
+        <is>
+          <t>Zimone, Infinite Analyst</t>
+        </is>
+      </c>
+      <c r="B53" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A53)</f>
+        <v>0</v>
+      </c>
+      <c r="C53" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A53,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D53" s="41">
+        <f>IFERROR(C53/B53,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="A54" s="41" t="inlineStr">
+        <is>
+          <t>Super Shredder</t>
+        </is>
+      </c>
+      <c r="B54" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A54)</f>
+        <v>0</v>
+      </c>
+      <c r="C54" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A54,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D54" s="41">
+        <f>IFERROR(C54/B54,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
+      <c r="A55" s="41" t="inlineStr">
+        <is>
+          <t>Hei Bai, Forest Guardian</t>
+        </is>
+      </c>
+      <c r="B55" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A55)</f>
+        <v>0</v>
+      </c>
+      <c r="C55" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A55,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D55" s="41">
+        <f>IFERROR(C55/B55,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="A56" s="41" t="inlineStr">
+        <is>
+          <t>Ultima, Origin of Oblivion</t>
+        </is>
+      </c>
+      <c r="B56" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A56)</f>
+        <v>1</v>
+      </c>
+      <c r="C56" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A56,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D56" s="41">
+        <f>IFERROR(C56/B56,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
+      <c r="A57" s="50" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="B57" s="52">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A57)</f>
+        <v>0</v>
+      </c>
+      <c r="C57" s="52">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A57,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D57" s="52">
+        <f>IFERROR(C57/B57,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
+      <c r="A58" s="41" t="inlineStr">
+        <is>
+          <t>Cloud, Ex-SOLDIER</t>
+        </is>
+      </c>
+      <c r="B58" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A58)</f>
+        <v>0</v>
+      </c>
+      <c r="C58" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A58,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D58" s="41">
+        <f>IFERROR(C58/B58,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
+      <c r="A59" s="41" t="inlineStr">
+        <is>
+          <t>Squall, SeeD Mercenary</t>
+        </is>
+      </c>
+      <c r="B59" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A59)</f>
+        <v>0</v>
+      </c>
+      <c r="C59" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A59,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D59" s="41">
+        <f>IFERROR(C59/B59,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="A60" s="41" t="inlineStr">
+        <is>
+          <t>Sanar, Innovative First-Year</t>
+        </is>
+      </c>
+      <c r="B60" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A60)</f>
+        <v>0</v>
+      </c>
+      <c r="C60" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A60,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D60" s="41">
+        <f>IFERROR(C60/B60,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" s="50" t="inlineStr">
+        <is>
+          <t>Michelle</t>
+        </is>
+      </c>
+      <c r="B61" s="52">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A61)</f>
         <v>4</v>
       </c>
-      <c r="C8">
-        <v>2</v>
-      </c>
-      <c r="D8" s="36">
-        <f t="shared" si="0"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="44" t="s">
-        <v>109</v>
-      </c>
-      <c r="B9">
-        <v>2</v>
-      </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="D9" s="36">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="44" t="s">
-        <v>39</v>
-      </c>
-      <c r="B10">
-        <v>1</v>
-      </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-      <c r="D10" s="36">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="44" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11">
-        <v>1</v>
-      </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-      <c r="D11" s="36">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="43" t="s">
-        <v>6</v>
-      </c>
-      <c r="B12">
-        <v>12</v>
-      </c>
-      <c r="C12">
-        <v>5</v>
-      </c>
-      <c r="D12" s="45">
-        <f t="shared" si="0"/>
-        <v>0.41666666666666669</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="44" t="s">
-        <v>111</v>
-      </c>
-      <c r="B13">
-        <v>4</v>
-      </c>
-      <c r="C13">
-        <v>0</v>
-      </c>
-      <c r="D13" s="36">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="44" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14">
-        <v>1</v>
-      </c>
-      <c r="C14">
-        <v>1</v>
-      </c>
-      <c r="D14" s="36">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="44" t="s">
-        <v>23</v>
-      </c>
-      <c r="B15">
-        <v>1</v>
-      </c>
-      <c r="C15">
-        <v>0</v>
-      </c>
-      <c r="D15" s="36">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="44" t="s">
-        <v>46</v>
-      </c>
-      <c r="B16">
-        <v>1</v>
-      </c>
-      <c r="C16">
-        <v>1</v>
-      </c>
-      <c r="D16" s="36">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="44" t="s">
-        <v>114</v>
-      </c>
-      <c r="B17">
-        <v>3</v>
-      </c>
-      <c r="C17">
-        <v>2</v>
-      </c>
-      <c r="D17" s="36">
-        <f t="shared" si="0"/>
-        <v>0.66666666666666663</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="44" t="s">
-        <v>38</v>
-      </c>
-      <c r="B18">
-        <v>1</v>
-      </c>
-      <c r="C18">
-        <v>1</v>
-      </c>
-      <c r="D18" s="36">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="44" t="s">
-        <v>103</v>
-      </c>
-      <c r="B19">
-        <v>1</v>
-      </c>
-      <c r="C19">
-        <v>0</v>
-      </c>
-      <c r="D19" s="36">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="43" t="s">
-        <v>2</v>
-      </c>
-      <c r="B20">
-        <v>10</v>
-      </c>
-      <c r="C20">
-        <v>3</v>
-      </c>
-      <c r="D20" s="45">
-        <f t="shared" si="0"/>
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="44" t="s">
-        <v>37</v>
-      </c>
-      <c r="B21">
-        <v>1</v>
-      </c>
-      <c r="C21">
-        <v>1</v>
-      </c>
-      <c r="D21" s="36">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="44" t="s">
-        <v>110</v>
-      </c>
-      <c r="B22">
-        <v>2</v>
-      </c>
-      <c r="C22">
-        <v>0</v>
-      </c>
-      <c r="D22" s="36">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="44" t="s">
-        <v>76</v>
-      </c>
-      <c r="B23">
-        <v>1</v>
-      </c>
-      <c r="C23">
-        <v>0</v>
-      </c>
-      <c r="D23" s="36">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="44" t="s">
-        <v>116</v>
-      </c>
-      <c r="B24">
-        <v>2</v>
-      </c>
-      <c r="C24">
-        <v>1</v>
-      </c>
-      <c r="D24" s="36">
-        <f t="shared" si="0"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="44" t="s">
-        <v>97</v>
-      </c>
-      <c r="B25">
-        <v>1</v>
-      </c>
-      <c r="C25">
-        <v>0</v>
-      </c>
-      <c r="D25" s="36">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="44" t="s">
-        <v>52</v>
-      </c>
-      <c r="B26">
-        <v>1</v>
-      </c>
-      <c r="C26">
-        <v>0</v>
-      </c>
-      <c r="D26" s="36">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="44" t="s">
-        <v>119</v>
-      </c>
-      <c r="B27">
-        <v>2</v>
-      </c>
-      <c r="C27">
-        <v>1</v>
-      </c>
-      <c r="D27" s="36">
-        <f t="shared" si="0"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="43" t="s">
-        <v>87</v>
-      </c>
-      <c r="B28">
-        <v>2</v>
-      </c>
-      <c r="C28">
-        <v>0</v>
-      </c>
-      <c r="D28" s="45">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="44" t="s">
-        <v>71</v>
-      </c>
-      <c r="B29">
-        <v>1</v>
-      </c>
-      <c r="C29">
-        <v>0</v>
-      </c>
-      <c r="D29" s="36">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="44" t="s">
-        <v>115</v>
-      </c>
-      <c r="B30">
-        <v>1</v>
-      </c>
-      <c r="C30">
-        <v>0</v>
-      </c>
-      <c r="D30" s="36">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="43" t="s">
-        <v>49</v>
-      </c>
-      <c r="B31">
-        <v>3</v>
-      </c>
-      <c r="C31">
-        <v>0</v>
-      </c>
-      <c r="D31" s="45">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="44" t="s">
-        <v>50</v>
-      </c>
-      <c r="B32">
-        <v>2</v>
-      </c>
-      <c r="C32">
-        <v>0</v>
-      </c>
-      <c r="D32" s="36">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="B33">
-        <v>1</v>
-      </c>
-      <c r="C33">
-        <v>0</v>
-      </c>
-      <c r="D33" s="36">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="43" t="s">
-        <v>4</v>
-      </c>
-      <c r="B34">
-        <v>1</v>
-      </c>
-      <c r="C34">
-        <v>0</v>
-      </c>
-      <c r="D34" s="45">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="44" t="s">
-        <v>79</v>
-      </c>
-      <c r="B35">
-        <v>1</v>
-      </c>
-      <c r="C35">
-        <v>0</v>
-      </c>
-      <c r="D35" s="36">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A36" s="43" t="s">
-        <v>19</v>
-      </c>
-      <c r="B36">
-        <v>48</v>
-      </c>
-      <c r="C36">
-        <v>13</v>
-      </c>
-      <c r="D36" s="46">
-        <f t="shared" si="0"/>
-        <v>0.27083333333333331</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="D37" s="54"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="D38" s="48"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="D39" s="48"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="D40" s="48"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="D41" s="48"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="D42" s="54"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="D43" s="48"/>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="D44" s="48"/>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="D45" s="48"/>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="D46" s="48"/>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="D47" s="54"/>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="D48" s="48"/>
-    </row>
-    <row r="49" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D49" s="48"/>
-    </row>
-    <row r="50" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D50" s="48"/>
-    </row>
-    <row r="51" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D51" s="54"/>
-    </row>
-    <row r="52" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D52" s="48"/>
-    </row>
-    <row r="53" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D53" s="48"/>
-    </row>
-    <row r="54" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D54" s="55"/>
+      <c r="C61" s="52">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A61,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D61" s="52">
+        <f>IFERROR(C61/B61,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" s="41" t="inlineStr">
+        <is>
+          <t>The Wise Mothman</t>
+        </is>
+      </c>
+      <c r="B62" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A62)</f>
+        <v>3</v>
+      </c>
+      <c r="C62" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A62,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D62" s="41">
+        <f>IFERROR(C62/B62,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
+      <c r="A63" s="41" t="inlineStr">
+        <is>
+          <t>Szarel, Genesis Shepard</t>
+        </is>
+      </c>
+      <c r="B63" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A63)</f>
+        <v>0</v>
+      </c>
+      <c r="C63" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A63,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D63" s="41">
+        <f>IFERROR(C63/B63,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4">
+      <c r="A64" s="41" t="inlineStr">
+        <is>
+          <t>Lucy MacLean, Positively Armed</t>
+        </is>
+      </c>
+      <c r="B64" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A64)</f>
+        <v>1</v>
+      </c>
+      <c r="C64" s="41">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A64,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D64" s="41">
+        <f>IFERROR(C64/B64,0)</f>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
test: add_player.py dry run with ZZTestPlayer (to be reverted)
</commit_message>
<xml_diff>
--- a/deck-strength.xlsx
+++ b/deck-strength.xlsx
@@ -25670,7 +25670,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D67"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.33"/>
@@ -26501,6 +26501,48 @@
       </c>
       <c r="D64" s="48" t="n">
         <v>2.4</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
+      <c r="A65" s="46" t="inlineStr">
+        <is>
+          <t>ZZTestPlayer</t>
+        </is>
+      </c>
+      <c r="B65" s="47">
+        <f>AVERAGE(B66:B67)</f>
+        <v>2.8</v>
+      </c>
+      <c r="C65" s="45"/>
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66" s="48" t="inlineStr">
+        <is>
+          <t>Test Commander One</t>
+        </is>
+      </c>
+      <c r="B66" s="48">
+        <f>IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="ZZTestPlayer")*('Game Log Season 3'!$D$3:$D$1000=A66)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D66)</f>
+        <v>3.1</v>
+      </c>
+      <c r="C66" s="45"/>
+      <c r="D66" s="48">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
+      <c r="A67" s="48" t="inlineStr">
+        <is>
+          <t>Test Commander Two</t>
+        </is>
+      </c>
+      <c r="B67" s="48">
+        <f>IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="ZZTestPlayer")*('Game Log Season 3'!$D$3:$D$1000=A67)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D67)</f>
+        <v>2.5</v>
+      </c>
+      <c r="C67" s="45"/>
+      <c r="D67" s="48">
+        <v>2.5</v>
       </c>
     </row>
   </sheetData>
@@ -26519,7 +26561,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D67"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="29.89"/>
@@ -27610,6 +27652,63 @@
       </c>
       <c r="D64" s="48" t="n">
         <f aca="false">IFERROR(C64/B64,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
+      <c r="A65" s="46" t="inlineStr">
+        <is>
+          <t>ZZTestPlayer</t>
+        </is>
+      </c>
+      <c r="B65" s="47">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A65)</f>
+        <v>0</v>
+      </c>
+      <c r="C65" s="47">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A65,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D65" s="47">
+        <f>IFERROR(C65/B65,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66" s="48" t="inlineStr">
+        <is>
+          <t>Test Commander One</t>
+        </is>
+      </c>
+      <c r="B66" s="48">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"ZZTestPlayer",'Game Log Season 3'!$D$3:$D$1000,A66)</f>
+        <v>0</v>
+      </c>
+      <c r="C66" s="48">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"ZZTestPlayer",'Game Log Season 3'!$D$3:$D$1000,A66,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D66" s="48">
+        <f>IFERROR(C66/B66,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
+      <c r="A67" s="48" t="inlineStr">
+        <is>
+          <t>Test Commander Two</t>
+        </is>
+      </c>
+      <c r="B67" s="48">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"ZZTestPlayer",'Game Log Season 3'!$D$3:$D$1000,A67)</f>
+        <v>0</v>
+      </c>
+      <c r="C67" s="48">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"ZZTestPlayer",'Game Log Season 3'!$D$3:$D$1000,A67,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D67" s="48">
+        <f>IFERROR(C67/B67,0)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
test: add_deck.py dry run adding a deck to Becca's block (to be reverted)
</commit_message>
<xml_diff>
--- a/deck-strength.xlsx
+++ b/deck-strength.xlsx
@@ -25670,7 +25670,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D65"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.33"/>
@@ -25696,7 +25696,7 @@
         <v>26</v>
       </c>
       <c r="B2" s="47" t="n">
-        <f aca="false">AVERAGE(B3:B6)</f>
+        <f aca="false">AVERAGE(B3:B7)</f>
         <v>2.72288194444444</v>
       </c>
       <c r="C2" s="45"/>
@@ -25755,206 +25755,208 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="46" t="s">
+    <row r="7" spans="1:4">
+      <c r="A7" s="48" t="inlineStr">
+        <is>
+          <t>ZZ Test New Deck</t>
+        </is>
+      </c>
+      <c r="B7" s="48">
+        <f>IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Becca")*('Game Log Season 3'!$D$3:$D$1000=A7)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D7)</f>
+        <v>2.9</v>
+      </c>
+      <c r="C7" s="45"/>
+      <c r="D7" s="48">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="47" t="n">
-        <f aca="false">AVERAGE(B8:B17)</f>
+      <c r="B8" s="47" t="n">
+        <f aca="false">AVERAGE(B9:B18)</f>
         <v>3.28381944444444</v>
       </c>
-      <c r="C7" s="45"/>
-    </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="48" t="s">
-        <v>68</v>
-      </c>
-      <c r="B8" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A8)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D8)</f>
-        <v>3.83916666666667</v>
-      </c>
       <c r="C8" s="45"/>
-      <c r="D8" s="48" t="n">
-        <v>3.8</v>
-      </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="48" t="s">
-        <v>42</v>
+        <v>68</v>
       </c>
       <c r="B9" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A9)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D9)</f>
-        <v>3.9</v>
+        <v>3.83916666666667</v>
       </c>
       <c r="C9" s="45"/>
       <c r="D9" s="48" t="n">
-        <v>3.9</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="48" t="s">
-        <v>67</v>
+        <v>42</v>
       </c>
       <c r="B10" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A10)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D10)</f>
-        <v>3.4</v>
-      </c>
-      <c r="C10" s="45" t="s">
-        <v>102</v>
-      </c>
+        <v>3.9</v>
+      </c>
+      <c r="C10" s="45"/>
       <c r="D10" s="48" t="n">
-        <v>3.4</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="48" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="B11" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A11)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D11)</f>
-        <v>2.6</v>
-      </c>
-      <c r="C11" s="45"/>
+        <v>3.4</v>
+      </c>
+      <c r="C11" s="45" t="s">
+        <v>102</v>
+      </c>
       <c r="D11" s="48" t="n">
-        <v>2.6</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="48" t="s">
-        <v>44</v>
+        <v>82</v>
       </c>
       <c r="B12" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A12)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D12)</f>
-        <v>3.5</v>
-      </c>
-      <c r="C12" s="45" t="s">
-        <v>101</v>
-      </c>
+        <v>2.6</v>
+      </c>
+      <c r="C12" s="45"/>
       <c r="D12" s="48" t="n">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="48" t="s">
-        <v>88</v>
+        <v>44</v>
       </c>
       <c r="B13" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A13)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D13)</f>
-        <v>2.65388888888889</v>
-      </c>
-      <c r="C13" s="45"/>
+        <v>3.5</v>
+      </c>
+      <c r="C13" s="45" t="s">
+        <v>101</v>
+      </c>
       <c r="D13" s="48" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="48" t="s">
-        <v>48</v>
+        <v>88</v>
       </c>
       <c r="B14" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A14)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D14)</f>
-        <v>2.6</v>
+        <v>2.65388888888889</v>
       </c>
       <c r="C14" s="45"/>
       <c r="D14" s="48" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="48" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="B15" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A15)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D15)</f>
-        <v>3.91083333333333</v>
+        <v>2.6</v>
       </c>
       <c r="C15" s="45"/>
       <c r="D15" s="48" t="n">
-        <v>3.9</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="48" t="s">
-        <v>91</v>
+        <v>37</v>
       </c>
       <c r="B16" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A16)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D16)</f>
-        <v>2.94083333333333</v>
+        <v>3.91083333333333</v>
       </c>
       <c r="C16" s="45"/>
       <c r="D16" s="48" t="n">
-        <v>2.3</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="48" t="s">
-        <v>47</v>
+        <v>91</v>
       </c>
       <c r="B17" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A17)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D17)</f>
-        <v>3.49347222222222</v>
+        <v>2.94083333333333</v>
       </c>
       <c r="C17" s="45"/>
       <c r="D17" s="48" t="n">
+        <v>2.3</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="48" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A18)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D18)</f>
+        <v>3.49347222222222</v>
+      </c>
+      <c r="C18" s="45"/>
+      <c r="D18" s="48" t="n">
         <v>3.5</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="46" t="s">
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="47" t="n">
-        <f aca="false">AVERAGE(B19:B32)</f>
+      <c r="B19" s="47" t="n">
+        <f aca="false">AVERAGE(B20:B33)</f>
         <v>3.31464285714286</v>
       </c>
-      <c r="C18" s="45"/>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="48" t="s">
-        <v>73</v>
-      </c>
-      <c r="B19" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A19)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D19)</f>
-        <v>2.4</v>
-      </c>
       <c r="C19" s="45"/>
-      <c r="D19" s="48" t="n">
-        <v>2.4</v>
-      </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="48" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B20" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A20)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D20)</f>
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="C20" s="45"/>
       <c r="D20" s="48" t="n">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="48" t="s">
-        <v>31</v>
+        <v>66</v>
       </c>
       <c r="B21" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A21)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D21)</f>
-        <v>3.57402777777778</v>
+        <v>2.6</v>
       </c>
       <c r="C21" s="45"/>
       <c r="D21" s="48" t="n">
-        <v>3.6</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="48" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B22" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A22)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D22)</f>
-        <v>3.6</v>
+        <v>3.57402777777778</v>
       </c>
       <c r="C22" s="45"/>
       <c r="D22" s="48" t="n">
@@ -25963,543 +25965,556 @@
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="48" t="s">
-        <v>74</v>
+        <v>34</v>
       </c>
       <c r="B23" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A23)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D23)</f>
-        <v>2.9</v>
+        <v>3.6</v>
       </c>
       <c r="C23" s="45"/>
       <c r="D23" s="48" t="n">
-        <v>2.9</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="48" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="B24" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A24)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D24)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C24" s="45" t="s">
-        <v>101</v>
-      </c>
+        <v>2.9</v>
+      </c>
+      <c r="C24" s="45"/>
       <c r="D24" s="48" t="n">
-        <v>3.9</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="48" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
       <c r="B25" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A25)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D25)</f>
-        <v>2.8</v>
-      </c>
-      <c r="C25" s="45"/>
+        <v>3.9</v>
+      </c>
+      <c r="C25" s="45" t="s">
+        <v>101</v>
+      </c>
       <c r="D25" s="48" t="n">
-        <v>2.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="48" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B26" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A26)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D26)</f>
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="C26" s="45"/>
       <c r="D26" s="48" t="n">
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="48" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B27" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A27)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D27)</f>
-        <v>3.59875</v>
-      </c>
-      <c r="C27" s="45" t="s">
-        <v>103</v>
-      </c>
+        <v>2.6</v>
+      </c>
+      <c r="C27" s="45"/>
       <c r="D27" s="48" t="n">
-        <v>3.6</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="48" t="s">
-        <v>48</v>
+        <v>83</v>
       </c>
       <c r="B28" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A28)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D28)</f>
-        <v>3.94083333333333</v>
-      </c>
-      <c r="C28" s="45"/>
+        <v>3.59875</v>
+      </c>
+      <c r="C28" s="45" t="s">
+        <v>103</v>
+      </c>
       <c r="D28" s="48" t="n">
-        <v>3.9</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="48" t="s">
-        <v>90</v>
+        <v>48</v>
       </c>
       <c r="B29" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A29)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D29)</f>
-        <v>3.65388888888889</v>
+        <v>3.94083333333333</v>
       </c>
       <c r="C29" s="45"/>
       <c r="D29" s="48" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="48" t="s">
-        <v>46</v>
-      </c>
-      <c r="B30" s="49" t="n">
+        <v>90</v>
+      </c>
+      <c r="B30" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A30)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D30)</f>
-        <v>3.95583333333333</v>
+        <v>3.65388888888889</v>
       </c>
       <c r="C30" s="45"/>
-      <c r="D30" s="49" t="n">
-        <v>4</v>
+      <c r="D30" s="48" t="n">
+        <v>3.7</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="48" t="s">
-        <v>92</v>
+        <v>46</v>
       </c>
       <c r="B31" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A31)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D31)</f>
-        <v>2.94666666666667</v>
+        <v>3.95583333333333</v>
       </c>
       <c r="C31" s="45"/>
       <c r="D31" s="49" t="n">
-        <v>2.9</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="48" t="s">
-        <v>40</v>
+        <v>92</v>
       </c>
       <c r="B32" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A32)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D32)</f>
+        <v>2.94666666666667</v>
+      </c>
+      <c r="C32" s="45"/>
+      <c r="D32" s="49" t="n">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="48" t="s">
+        <v>40</v>
+      </c>
+      <c r="B33" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A33)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D33)</f>
         <v>3.935</v>
       </c>
-      <c r="C32" s="45" t="s">
+      <c r="C33" s="45" t="s">
         <v>104</v>
       </c>
-      <c r="D32" s="49" t="n">
+      <c r="D33" s="49" t="n">
         <v>3.9</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="46" t="s">
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="B33" s="47" t="n">
-        <f aca="false">AVERAGE(B34:B44)</f>
+      <c r="B34" s="47" t="n">
+        <f aca="false">AVERAGE(B35:B45)</f>
         <v>3.26275505050505</v>
       </c>
-      <c r="C33" s="45"/>
-    </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="48" t="s">
-        <v>36</v>
-      </c>
-      <c r="B34" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A34)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D34)</f>
-        <v>3.5</v>
-      </c>
       <c r="C34" s="45"/>
-      <c r="D34" s="48" t="n">
-        <v>3.5</v>
-      </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="48" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="B35" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A35)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D35)</f>
-        <v>3.43088888888889</v>
+        <v>3.5</v>
       </c>
       <c r="C35" s="45"/>
       <c r="D35" s="48" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="48" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="B36" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A36)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D36)</f>
-        <v>3.7</v>
+        <v>3.43088888888889</v>
       </c>
       <c r="C36" s="45"/>
       <c r="D36" s="48" t="n">
-        <v>3.7</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="48" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="B37" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A37)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D37)</f>
-        <v>2.6</v>
+        <v>3.7</v>
       </c>
       <c r="C37" s="45"/>
       <c r="D37" s="48" t="n">
-        <v>2.6</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="48" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="B38" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A38)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D38)</f>
-        <v>3.77816666666667</v>
+        <v>2.6</v>
       </c>
       <c r="C38" s="45"/>
       <c r="D38" s="48" t="n">
-        <v>3.8</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="48" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="B39" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A39)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D39)</f>
-        <v>2.59388888888889</v>
+        <v>3.77816666666667</v>
       </c>
       <c r="C39" s="45"/>
       <c r="D39" s="48" t="n">
-        <v>2.6</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="48" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="B40" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A40)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D40)</f>
-        <v>3.23902777777778</v>
+        <v>2.59388888888889</v>
       </c>
       <c r="C40" s="45"/>
       <c r="D40" s="48" t="n">
-        <v>3.6</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="48" t="s">
-        <v>87</v>
+        <v>54</v>
       </c>
       <c r="B41" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A41)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D41)</f>
-        <v>2.6</v>
+        <v>3.23902777777778</v>
       </c>
       <c r="C41" s="45"/>
       <c r="D41" s="48" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="48" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B42" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A42)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D42)</f>
-        <v>3.58416666666667</v>
+        <v>2.6</v>
       </c>
       <c r="C42" s="45"/>
       <c r="D42" s="48" t="n">
-        <v>3.6</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="48" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B43" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A43)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D43)</f>
-        <v>2.94083333333333</v>
+        <v>3.58416666666667</v>
       </c>
       <c r="C43" s="45"/>
       <c r="D43" s="48" t="n">
-        <v>2.9</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="48" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B44" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A44)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D44)</f>
-        <v>3.92333333333333</v>
+        <v>2.94083333333333</v>
       </c>
       <c r="C44" s="45"/>
       <c r="D44" s="48" t="n">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="48" t="s">
+        <v>97</v>
+      </c>
+      <c r="B45" s="48" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A45)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D45)</f>
+        <v>3.92333333333333</v>
+      </c>
+      <c r="C45" s="45"/>
+      <c r="D45" s="48" t="n">
         <v>3.9</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="46" t="s">
+    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="46" t="s">
         <v>70</v>
       </c>
-      <c r="B45" s="47" t="n">
-        <f aca="false">AVERAGE(B46:B50)</f>
+      <c r="B46" s="47" t="n">
+        <f aca="false">AVERAGE(B47:B51)</f>
         <v>3.2865</v>
       </c>
-      <c r="C45" s="45"/>
-    </row>
-    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="48" t="s">
-        <v>71</v>
-      </c>
-      <c r="B46" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A46)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D46)</f>
-        <v>3.6</v>
-      </c>
-      <c r="C46" s="45" t="s">
-        <v>103</v>
-      </c>
-      <c r="D46" s="48" t="n">
-        <v>3.6</v>
-      </c>
+      <c r="C46" s="45"/>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="48" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B47" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A47)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D47)</f>
-        <v>3.33761111111111</v>
+        <v>3.6</v>
       </c>
       <c r="C47" s="45" t="s">
         <v>103</v>
       </c>
       <c r="D47" s="48" t="n">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="48" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="B48" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A48)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D48)</f>
-        <v>3.2</v>
-      </c>
-      <c r="C48" s="45"/>
+        <v>3.33761111111111</v>
+      </c>
+      <c r="C48" s="45" t="s">
+        <v>103</v>
+      </c>
       <c r="D48" s="48" t="n">
-        <v>3.2</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="48" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B49" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A49)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D49)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C49" s="45" t="s">
-        <v>104</v>
-      </c>
+        <v>3.2</v>
+      </c>
+      <c r="C49" s="45"/>
       <c r="D49" s="48" t="n">
-        <v>3.9</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="48" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="B50" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A50)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D50)</f>
+        <v>3.9</v>
+      </c>
+      <c r="C50" s="45" t="s">
+        <v>104</v>
+      </c>
+      <c r="D50" s="48" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="48" t="s">
+        <v>93</v>
+      </c>
+      <c r="B51" s="48" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A51)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D51)</f>
         <v>2.39488888888889</v>
       </c>
-      <c r="C50" s="45"/>
-      <c r="D50" s="48" t="n">
+      <c r="C51" s="45"/>
+      <c r="D51" s="48" t="n">
         <v>2.4</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="46" t="s">
+    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="46" t="s">
         <v>38</v>
       </c>
-      <c r="B51" s="47" t="n">
-        <f aca="false">AVERAGE(B52:B56)</f>
+      <c r="B52" s="47" t="n">
+        <f aca="false">AVERAGE(B53:B57)</f>
         <v>3.42807</v>
       </c>
-      <c r="C51" s="45"/>
-    </row>
-    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="48" t="s">
-        <v>49</v>
-      </c>
-      <c r="B52" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A52)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D52)</f>
-        <v>3.6</v>
-      </c>
       <c r="C52" s="45"/>
-      <c r="D52" s="48" t="n">
-        <v>3.6</v>
-      </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="48" t="s">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="B53" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A53)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D53)</f>
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
       <c r="C53" s="45"/>
       <c r="D53" s="48" t="n">
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="48" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B54" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A54)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D54)</f>
-        <v>2.7</v>
+        <v>3.8</v>
       </c>
       <c r="C54" s="45"/>
       <c r="D54" s="48" t="n">
-        <v>2.7</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="48" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="B55" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A55)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D55)</f>
-        <v>3.3</v>
+        <v>2.7</v>
       </c>
       <c r="C55" s="45"/>
       <c r="D55" s="48" t="n">
-        <v>3.3</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="48" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B56" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A56)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D56)</f>
-        <v>3.74035</v>
+        <v>3.3</v>
       </c>
       <c r="C56" s="45"/>
       <c r="D56" s="48" t="n">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="48" t="s">
+        <v>63</v>
+      </c>
+      <c r="B57" s="48" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A57)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D57)</f>
+        <v>3.74035</v>
+      </c>
+      <c r="C57" s="45"/>
+      <c r="D57" s="48" t="n">
         <v>3.7</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="46" t="s">
+    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="46" t="s">
         <v>59</v>
       </c>
-      <c r="B57" s="47" t="n">
-        <f aca="false">AVERAGE(B58:B59)</f>
+      <c r="B58" s="47" t="n">
+        <f aca="false">AVERAGE(B59:B60)</f>
         <v>3.05</v>
       </c>
-      <c r="C57" s="45"/>
-    </row>
-    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="48" t="s">
-        <v>33</v>
-      </c>
-      <c r="B58" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A58)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D58)</f>
-        <v>2.7</v>
-      </c>
       <c r="C58" s="45"/>
-      <c r="D58" s="48" t="n">
-        <v>2.7</v>
-      </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="48" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="B59" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A59)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D59)</f>
-        <v>3.4</v>
+        <v>2.7</v>
       </c>
       <c r="C59" s="45"/>
       <c r="D59" s="48" t="n">
-        <v>3.4</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="48" t="s">
+        <v>69</v>
+      </c>
+      <c r="B60" s="48" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A60)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D60)</f>
+        <v>3.4</v>
+      </c>
+      <c r="C60" s="45"/>
+      <c r="D60" s="48" t="n">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="48" t="s">
         <v>84</v>
       </c>
-      <c r="B60" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A60)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D60)</f>
-        <v>1</v>
-      </c>
-      <c r="C60" s="45"/>
-      <c r="D60" s="49" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="46" t="s">
+      <c r="B61" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A61)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D61)</f>
+        <v>1</v>
+      </c>
+      <c r="C61" s="45"/>
+      <c r="D61" s="49" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="46" t="s">
         <v>51</v>
       </c>
-      <c r="B61" s="47" t="n">
-        <f aca="false">AVERAGE(B62:B63)</f>
+      <c r="B62" s="47" t="n">
+        <f aca="false">AVERAGE(B63:B64)</f>
         <v>2.25194444444444</v>
       </c>
-      <c r="C61" s="45"/>
-    </row>
-    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="48" t="s">
-        <v>52</v>
-      </c>
-      <c r="B62" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A62)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D62)</f>
-        <v>2.30388888888889</v>
-      </c>
       <c r="C62" s="45"/>
-      <c r="D62" s="48" t="n">
-        <v>2.5</v>
-      </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="48" t="s">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="B63" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A63)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D63)</f>
-        <v>2.2</v>
+        <v>2.30388888888889</v>
       </c>
       <c r="C63" s="45"/>
       <c r="D63" s="48" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="48" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="B64" s="48" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A64)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D64)</f>
+        <v>2.2</v>
+      </c>
+      <c r="C64" s="45"/>
+      <c r="D64" s="48" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="48" t="s">
+        <v>96</v>
+      </c>
+      <c r="B65" s="48" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A65)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D65)</f>
         <v>2.43069444444444</v>
       </c>
-      <c r="D64" s="48" t="n">
+      <c r="D65" s="48" t="n">
         <v>2.4</v>
       </c>
     </row>
@@ -26519,7 +26534,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D65"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="29.89"/>
@@ -26627,60 +26642,62 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="46" t="s">
+    <row r="7" spans="1:4">
+      <c r="A7" s="48" t="inlineStr">
+        <is>
+          <t>ZZ Test New Deck</t>
+        </is>
+      </c>
+      <c r="B7" s="48">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A7)</f>
+        <v>0</v>
+      </c>
+      <c r="C7" s="48">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A7,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D7" s="48">
+        <f>IFERROR(C7/B7,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A7)</f>
+      <c r="B8" s="47" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A8)</f>
         <v>14</v>
       </c>
-      <c r="C7" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A7,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+      <c r="C8" s="47" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A8,'Game Log Season 3'!$F$3:$F$1000,1)</f>
         <v>4</v>
       </c>
-      <c r="D7" s="47" t="n">
-        <f aca="false">IFERROR(C7/B7,0)</f>
+      <c r="D8" s="47" t="n">
+        <f aca="false">IFERROR(C8/B8,0)</f>
         <v>0.285714285714286</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="48" t="s">
-        <v>68</v>
-      </c>
-      <c r="B8" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A8)</f>
-        <v>4</v>
-      </c>
-      <c r="C8" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A8,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>2</v>
-      </c>
-      <c r="D8" s="48" t="n">
-        <f aca="false">IFERROR(C8/B8,0)</f>
-        <v>0.5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="48" t="s">
-        <v>42</v>
+        <v>68</v>
       </c>
       <c r="B9" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A9)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C9" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A9,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D9" s="48" t="n">
         <f aca="false">IFERROR(C9/B9,0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="48" t="s">
-        <v>67</v>
+        <v>42</v>
       </c>
       <c r="B10" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A10)</f>
@@ -26697,7 +26714,7 @@
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="48" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="B11" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A11)</f>
@@ -26714,7 +26731,7 @@
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="48" t="s">
-        <v>44</v>
+        <v>82</v>
       </c>
       <c r="B12" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A12)</f>
@@ -26731,11 +26748,11 @@
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="48" t="s">
-        <v>88</v>
+        <v>44</v>
       </c>
       <c r="B13" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A13)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C13" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A13,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -26748,11 +26765,11 @@
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="48" t="s">
-        <v>48</v>
+        <v>88</v>
       </c>
       <c r="B14" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A14)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C14" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A14,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -26765,28 +26782,28 @@
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="48" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="B15" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A15)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C15" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A15,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" s="48" t="n">
         <f aca="false">IFERROR(C15/B15,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="48" t="s">
-        <v>91</v>
+        <v>37</v>
       </c>
       <c r="B16" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A16)</f>
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C16" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A16,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -26794,63 +26811,63 @@
       </c>
       <c r="D16" s="48" t="n">
         <f aca="false">IFERROR(C16/B16,0)</f>
-        <v>0.166666666666667</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="48" t="s">
-        <v>47</v>
+        <v>91</v>
       </c>
       <c r="B17" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A17)</f>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C17" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A17,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" s="48" t="n">
         <f aca="false">IFERROR(C17/B17,0)</f>
-        <v>0</v>
+        <v>0.166666666666667</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="46" t="s">
+      <c r="A18" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A18)</f>
+        <v>1</v>
+      </c>
+      <c r="C18" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A18,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="48" t="n">
+        <f aca="false">IFERROR(C18/B18,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A18)</f>
+      <c r="B19" s="47" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A19)</f>
         <v>12</v>
       </c>
-      <c r="C18" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A18,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+      <c r="C19" s="47" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A19,'Game Log Season 3'!$F$3:$F$1000,1)</f>
         <v>5</v>
       </c>
-      <c r="D18" s="47" t="n">
-        <f aca="false">IFERROR(C18/B18,0)</f>
+      <c r="D19" s="47" t="n">
+        <f aca="false">IFERROR(C19/B19,0)</f>
         <v>0.416666666666667</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="48" t="s">
-        <v>73</v>
-      </c>
-      <c r="B19" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A19)</f>
-        <v>0</v>
-      </c>
-      <c r="C19" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A19,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D19" s="48" t="n">
-        <f aca="false">IFERROR(C19/B19,0)</f>
-        <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="48" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B20" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A20)</f>
@@ -26867,11 +26884,11 @@
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="48" t="s">
-        <v>31</v>
+        <v>66</v>
       </c>
       <c r="B21" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A21)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C21" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A21,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -26884,11 +26901,11 @@
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="48" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B22" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A22)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C22" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A22,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -26901,7 +26918,7 @@
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="48" t="s">
-        <v>74</v>
+        <v>34</v>
       </c>
       <c r="B23" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A23)</f>
@@ -26918,7 +26935,7 @@
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="48" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="B24" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A24)</f>
@@ -26935,7 +26952,7 @@
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="48" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
       <c r="B25" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A25)</f>
@@ -26952,7 +26969,7 @@
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="48" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B26" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A26)</f>
@@ -26969,11 +26986,11 @@
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="48" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B27" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A27)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C27" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A27,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -26986,7 +27003,7 @@
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="48" t="s">
-        <v>48</v>
+        <v>83</v>
       </c>
       <c r="B28" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A28)</f>
@@ -26994,122 +27011,122 @@
       </c>
       <c r="C28" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A28,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D28" s="48" t="n">
         <f aca="false">IFERROR(C28/B28,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="48" t="s">
-        <v>90</v>
+        <v>48</v>
       </c>
       <c r="B29" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A29)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C29" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A29,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D29" s="48" t="n">
         <f aca="false">IFERROR(C29/B29,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="48" t="s">
-        <v>46</v>
+        <v>90</v>
       </c>
       <c r="B30" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A30)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C30" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A30,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D30" s="48" t="n">
         <f aca="false">IFERROR(C30/B30,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="48" t="s">
-        <v>92</v>
+        <v>46</v>
       </c>
       <c r="B31" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A31)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C31" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A31,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D31" s="48" t="n">
         <f aca="false">IFERROR(C31/B31,0)</f>
-        <v>0.666666666666667</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="48" t="s">
-        <v>40</v>
+        <v>92</v>
       </c>
       <c r="B32" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A32)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C32" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A32,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" s="48" t="n">
         <f aca="false">IFERROR(C32/B32,0)</f>
-        <v>1</v>
+        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="46" t="s">
+      <c r="A33" s="48" t="s">
+        <v>40</v>
+      </c>
+      <c r="B33" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A33)</f>
+        <v>1</v>
+      </c>
+      <c r="C33" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A33,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>1</v>
+      </c>
+      <c r="D33" s="48" t="n">
+        <f aca="false">IFERROR(C33/B33,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="B33" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A33)</f>
+      <c r="B34" s="47" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A34)</f>
         <v>11</v>
       </c>
-      <c r="C33" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A33,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>3</v>
-      </c>
-      <c r="D33" s="47" t="n">
-        <f aca="false">IFERROR(C33/B33,0)</f>
+      <c r="C34" s="47" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A34,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>3</v>
+      </c>
+      <c r="D34" s="47" t="n">
+        <f aca="false">IFERROR(C34/B34,0)</f>
         <v>0.272727272727273</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="48" t="s">
-        <v>36</v>
-      </c>
-      <c r="B34" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A34)</f>
-        <v>0</v>
-      </c>
-      <c r="C34" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A34,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D34" s="48" t="n">
-        <f aca="false">IFERROR(C34/B34,0)</f>
-        <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="48" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="B35" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A35)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C35" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A35,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27122,11 +27139,11 @@
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="48" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="B36" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A36)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C36" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A36,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27139,7 +27156,7 @@
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="48" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="B37" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A37)</f>
@@ -27156,24 +27173,24 @@
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="48" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="B38" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A38)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C38" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A38,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D38" s="48" t="n">
         <f aca="false">IFERROR(C38/B38,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="48" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="B39" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A39)</f>
@@ -27181,20 +27198,20 @@
       </c>
       <c r="C39" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A39,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D39" s="48" t="n">
         <f aca="false">IFERROR(C39/B39,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="48" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="B40" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A40)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C40" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A40,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27207,11 +27224,11 @@
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="48" t="s">
-        <v>87</v>
+        <v>54</v>
       </c>
       <c r="B41" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A41)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C41" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A41,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27224,11 +27241,11 @@
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="48" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B42" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A42)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C42" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A42,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27241,7 +27258,7 @@
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="48" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B43" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A43)</f>
@@ -27249,16 +27266,16 @@
       </c>
       <c r="C43" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A43,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D43" s="48" t="n">
         <f aca="false">IFERROR(C43/B43,0)</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="48" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B44" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A44)</f>
@@ -27274,46 +27291,46 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="46" t="s">
+      <c r="A45" s="48" t="s">
+        <v>97</v>
+      </c>
+      <c r="B45" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A45)</f>
+        <v>2</v>
+      </c>
+      <c r="C45" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A45,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>1</v>
+      </c>
+      <c r="D45" s="48" t="n">
+        <f aca="false">IFERROR(C45/B45,0)</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="46" t="s">
         <v>70</v>
       </c>
-      <c r="B45" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A45)</f>
-        <v>2</v>
-      </c>
-      <c r="C45" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A45,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D45" s="47" t="n">
-        <f aca="false">IFERROR(C45/B45,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="48" t="s">
-        <v>71</v>
-      </c>
-      <c r="B46" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A46)</f>
-        <v>0</v>
-      </c>
-      <c r="C46" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A46,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D46" s="48" t="n">
+      <c r="B46" s="47" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A46)</f>
+        <v>2</v>
+      </c>
+      <c r="C46" s="47" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A46,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D46" s="47" t="n">
         <f aca="false">IFERROR(C46/B46,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="48" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B47" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A47)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C47" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A47,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27326,11 +27343,11 @@
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="48" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="B48" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A48)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C48" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A48,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27343,7 +27360,7 @@
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="48" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B49" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A49)</f>
@@ -27360,11 +27377,11 @@
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="48" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="B50" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A50)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C50" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A50,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27376,42 +27393,42 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="46" t="s">
+      <c r="A51" s="48" t="s">
+        <v>93</v>
+      </c>
+      <c r="B51" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A51)</f>
+        <v>1</v>
+      </c>
+      <c r="C51" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A51,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D51" s="48" t="n">
+        <f aca="false">IFERROR(C51/B51,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="46" t="s">
         <v>38</v>
       </c>
-      <c r="B51" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A51)</f>
-        <v>1</v>
-      </c>
-      <c r="C51" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A51,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D51" s="47" t="n">
-        <f aca="false">IFERROR(C51/B51,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="48" t="s">
-        <v>49</v>
-      </c>
-      <c r="B52" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A52)</f>
-        <v>0</v>
-      </c>
-      <c r="C52" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A52,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D52" s="48" t="n">
+      <c r="B52" s="47" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A52)</f>
+        <v>1</v>
+      </c>
+      <c r="C52" s="47" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A52,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D52" s="47" t="n">
         <f aca="false">IFERROR(C52/B52,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="48" t="s">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="B53" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A53)</f>
@@ -27428,7 +27445,7 @@
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="48" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B54" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A54)</f>
@@ -27445,7 +27462,7 @@
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="48" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="B55" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A55)</f>
@@ -27462,11 +27479,11 @@
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="48" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B56" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A56)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C56" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A56,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27478,42 +27495,42 @@
       </c>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="46" t="s">
+      <c r="A57" s="48" t="s">
+        <v>63</v>
+      </c>
+      <c r="B57" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A57)</f>
+        <v>1</v>
+      </c>
+      <c r="C57" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A57,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D57" s="48" t="n">
+        <f aca="false">IFERROR(C57/B57,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="46" t="s">
         <v>59</v>
       </c>
-      <c r="B57" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A57)</f>
-        <v>0</v>
-      </c>
-      <c r="C57" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A57,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D57" s="47" t="n">
-        <f aca="false">IFERROR(C57/B57,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="48" t="s">
-        <v>33</v>
-      </c>
-      <c r="B58" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A58)</f>
-        <v>0</v>
-      </c>
-      <c r="C58" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A58,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D58" s="48" t="n">
+      <c r="B58" s="47" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A58)</f>
+        <v>0</v>
+      </c>
+      <c r="C58" s="47" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A58,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D58" s="47" t="n">
         <f aca="false">IFERROR(C58/B58,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="48" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="B59" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A59)</f>
@@ -27530,7 +27547,7 @@
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="48" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="B60" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A60)</f>
@@ -27546,46 +27563,46 @@
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="46" t="s">
+      <c r="A61" s="48" t="s">
+        <v>84</v>
+      </c>
+      <c r="B61" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A61)</f>
+        <v>0</v>
+      </c>
+      <c r="C61" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A61,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D61" s="48" t="n">
+        <f aca="false">IFERROR(C61/B61,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="46" t="s">
         <v>51</v>
       </c>
-      <c r="B61" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A61)</f>
+      <c r="B62" s="47" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A62)</f>
         <v>4</v>
       </c>
-      <c r="C61" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A61,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D61" s="47" t="n">
-        <f aca="false">IFERROR(C61/B61,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="48" t="s">
-        <v>52</v>
-      </c>
-      <c r="B62" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A62)</f>
-        <v>3</v>
-      </c>
-      <c r="C62" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A62,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D62" s="48" t="n">
+      <c r="C62" s="47" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A62,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D62" s="47" t="n">
         <f aca="false">IFERROR(C62/B62,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="48" t="s">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="B63" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A63)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C63" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A63,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27598,11 +27615,11 @@
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="48" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="B64" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A64)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C64" s="48" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A64,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27610,6 +27627,23 @@
       </c>
       <c r="D64" s="48" t="n">
         <f aca="false">IFERROR(C64/B64,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="48" t="s">
+        <v>96</v>
+      </c>
+      <c r="B65" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A65)</f>
+        <v>1</v>
+      </c>
+      <c r="C65" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A65,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D65" s="48" t="n">
+        <f aca="false">IFERROR(C65/B65,0)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
test: season_rollover.py dry run to Season 4 (to be reverted)
</commit_message>
<xml_diff>
--- a/deck-strength.xlsx
+++ b/deck-strength.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Game Log Season 1" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Game Log Season 2" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Game Log Season 3" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Game Log Season 4" sheetId="7" r:id="rId10"/>
     <sheet name="Current Deck Strength" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Deck Win Rates" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Player Adjusted Ranks" sheetId="6" state="visible" r:id="rId8"/>
@@ -25706,12 +25707,12 @@
         <v>45</v>
       </c>
       <c r="B3" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Becca")*('Game Log Season 3'!$D$3:$D$1000=A3)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D3)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Becca")*('Game Log Season 4'!$D$3:$D$1000=A3)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D3)</f>
         <v>2.40388888888889</v>
       </c>
       <c r="C3" s="45"/>
       <c r="D3" s="48" t="n">
-        <v>2.4</v>
+        <v>2.40388888888889</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25719,7 +25720,7 @@
         <v>27</v>
       </c>
       <c r="B4" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Becca")*('Game Log Season 3'!$D$3:$D$1000=A4)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D4)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Becca")*('Game Log Season 4'!$D$3:$D$1000=A4)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D4)</f>
         <v>3.7</v>
       </c>
       <c r="C4" s="45" t="s">
@@ -25734,12 +25735,12 @@
         <v>75</v>
       </c>
       <c r="B5" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Becca")*('Game Log Season 3'!$D$3:$D$1000=A5)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D5)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Becca")*('Game Log Season 4'!$D$3:$D$1000=A5)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D5)</f>
         <v>2.30388888888889</v>
       </c>
       <c r="C5" s="45"/>
       <c r="D5" s="48" t="n">
-        <v>2.3</v>
+        <v>2.30388888888889</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25747,12 +25748,12 @@
         <v>95</v>
       </c>
       <c r="B6" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Becca")*('Game Log Season 3'!$D$3:$D$1000=A6)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D6)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Becca")*('Game Log Season 4'!$D$3:$D$1000=A6)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D6)</f>
         <v>2.48375</v>
       </c>
       <c r="C6" s="45"/>
       <c r="D6" s="48" t="n">
-        <v>2.5</v>
+        <v>2.48375</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25770,12 +25771,12 @@
         <v>68</v>
       </c>
       <c r="B8" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A8)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D8)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Manny")*('Game Log Season 4'!$D$3:$D$1000=A8)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D8)</f>
         <v>3.83916666666667</v>
       </c>
       <c r="C8" s="45"/>
       <c r="D8" s="48" t="n">
-        <v>3.8</v>
+        <v>3.83916666666667</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25783,7 +25784,7 @@
         <v>42</v>
       </c>
       <c r="B9" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A9)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D9)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Manny")*('Game Log Season 4'!$D$3:$D$1000=A9)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D9)</f>
         <v>3.9</v>
       </c>
       <c r="C9" s="45"/>
@@ -25796,7 +25797,7 @@
         <v>67</v>
       </c>
       <c r="B10" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A10)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D10)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Manny")*('Game Log Season 4'!$D$3:$D$1000=A10)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D10)</f>
         <v>3.4</v>
       </c>
       <c r="C10" s="45" t="s">
@@ -25811,7 +25812,7 @@
         <v>82</v>
       </c>
       <c r="B11" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A11)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D11)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Manny")*('Game Log Season 4'!$D$3:$D$1000=A11)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D11)</f>
         <v>2.6</v>
       </c>
       <c r="C11" s="45"/>
@@ -25824,7 +25825,7 @@
         <v>44</v>
       </c>
       <c r="B12" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A12)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D12)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Manny")*('Game Log Season 4'!$D$3:$D$1000=A12)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D12)</f>
         <v>3.5</v>
       </c>
       <c r="C12" s="45" t="s">
@@ -25839,12 +25840,12 @@
         <v>88</v>
       </c>
       <c r="B13" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A13)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D13)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Manny")*('Game Log Season 4'!$D$3:$D$1000=A13)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D13)</f>
         <v>2.65388888888889</v>
       </c>
       <c r="C13" s="45"/>
       <c r="D13" s="48" t="n">
-        <v>2.7</v>
+        <v>2.65388888888889</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25852,7 +25853,7 @@
         <v>48</v>
       </c>
       <c r="B14" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A14)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D14)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Manny")*('Game Log Season 4'!$D$3:$D$1000=A14)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D14)</f>
         <v>2.6</v>
       </c>
       <c r="C14" s="45"/>
@@ -25865,12 +25866,12 @@
         <v>37</v>
       </c>
       <c r="B15" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A15)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D15)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Manny")*('Game Log Season 4'!$D$3:$D$1000=A15)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D15)</f>
         <v>3.91083333333333</v>
       </c>
       <c r="C15" s="45"/>
       <c r="D15" s="48" t="n">
-        <v>3.9</v>
+        <v>3.91083333333333</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25878,12 +25879,12 @@
         <v>91</v>
       </c>
       <c r="B16" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A16)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D16)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Manny")*('Game Log Season 4'!$D$3:$D$1000=A16)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D16)</f>
         <v>2.94083333333333</v>
       </c>
       <c r="C16" s="45"/>
       <c r="D16" s="48" t="n">
-        <v>2.3</v>
+        <v>2.94083333333333</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25891,12 +25892,12 @@
         <v>47</v>
       </c>
       <c r="B17" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A17)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D17)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Manny")*('Game Log Season 4'!$D$3:$D$1000=A17)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D17)</f>
         <v>3.49347222222222</v>
       </c>
       <c r="C17" s="45"/>
       <c r="D17" s="48" t="n">
-        <v>3.5</v>
+        <v>3.49347222222222</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25914,7 +25915,7 @@
         <v>73</v>
       </c>
       <c r="B19" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A19)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D19)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Mateo")*('Game Log Season 4'!$D$3:$D$1000=A19)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D19)</f>
         <v>2.4</v>
       </c>
       <c r="C19" s="45"/>
@@ -25927,7 +25928,7 @@
         <v>66</v>
       </c>
       <c r="B20" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A20)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D20)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Mateo")*('Game Log Season 4'!$D$3:$D$1000=A20)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D20)</f>
         <v>2.6</v>
       </c>
       <c r="C20" s="45"/>
@@ -25940,12 +25941,12 @@
         <v>31</v>
       </c>
       <c r="B21" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A21)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D21)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Mateo")*('Game Log Season 4'!$D$3:$D$1000=A21)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D21)</f>
         <v>3.57402777777778</v>
       </c>
       <c r="C21" s="45"/>
       <c r="D21" s="48" t="n">
-        <v>3.6</v>
+        <v>3.57402777777778</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25953,7 +25954,7 @@
         <v>34</v>
       </c>
       <c r="B22" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A22)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D22)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Mateo")*('Game Log Season 4'!$D$3:$D$1000=A22)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D22)</f>
         <v>3.6</v>
       </c>
       <c r="C22" s="45"/>
@@ -25966,7 +25967,7 @@
         <v>74</v>
       </c>
       <c r="B23" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A23)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D23)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Mateo")*('Game Log Season 4'!$D$3:$D$1000=A23)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D23)</f>
         <v>2.9</v>
       </c>
       <c r="C23" s="45"/>
@@ -25979,7 +25980,7 @@
         <v>57</v>
       </c>
       <c r="B24" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A24)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D24)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Mateo")*('Game Log Season 4'!$D$3:$D$1000=A24)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D24)</f>
         <v>3.9</v>
       </c>
       <c r="C24" s="45" t="s">
@@ -25994,7 +25995,7 @@
         <v>80</v>
       </c>
       <c r="B25" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A25)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D25)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Mateo")*('Game Log Season 4'!$D$3:$D$1000=A25)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D25)</f>
         <v>2.8</v>
       </c>
       <c r="C25" s="45"/>
@@ -26007,7 +26008,7 @@
         <v>81</v>
       </c>
       <c r="B26" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A26)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D26)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Mateo")*('Game Log Season 4'!$D$3:$D$1000=A26)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D26)</f>
         <v>2.6</v>
       </c>
       <c r="C26" s="45"/>
@@ -26020,14 +26021,14 @@
         <v>83</v>
       </c>
       <c r="B27" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A27)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D27)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Mateo")*('Game Log Season 4'!$D$3:$D$1000=A27)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D27)</f>
         <v>3.59875</v>
       </c>
       <c r="C27" s="45" t="s">
         <v>103</v>
       </c>
       <c r="D27" s="48" t="n">
-        <v>3.6</v>
+        <v>3.59875</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26035,12 +26036,12 @@
         <v>48</v>
       </c>
       <c r="B28" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A28)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D28)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Mateo")*('Game Log Season 4'!$D$3:$D$1000=A28)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D28)</f>
         <v>3.94083333333333</v>
       </c>
       <c r="C28" s="45"/>
       <c r="D28" s="48" t="n">
-        <v>3.9</v>
+        <v>3.94083333333333</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26048,12 +26049,12 @@
         <v>90</v>
       </c>
       <c r="B29" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A29)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D29)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Mateo")*('Game Log Season 4'!$D$3:$D$1000=A29)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D29)</f>
         <v>3.65388888888889</v>
       </c>
       <c r="C29" s="45"/>
       <c r="D29" s="48" t="n">
-        <v>3.7</v>
+        <v>3.65388888888889</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26061,12 +26062,12 @@
         <v>46</v>
       </c>
       <c r="B30" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A30)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D30)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Mateo")*('Game Log Season 4'!$D$3:$D$1000=A30)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D30)</f>
         <v>3.95583333333333</v>
       </c>
       <c r="C30" s="45"/>
       <c r="D30" s="49" t="n">
-        <v>4</v>
+        <v>3.95583333333333</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26074,12 +26075,12 @@
         <v>92</v>
       </c>
       <c r="B31" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A31)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D31)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Mateo")*('Game Log Season 4'!$D$3:$D$1000=A31)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D31)</f>
         <v>2.94666666666667</v>
       </c>
       <c r="C31" s="45"/>
       <c r="D31" s="49" t="n">
-        <v>2.9</v>
+        <v>2.94666666666667</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26087,14 +26088,14 @@
         <v>40</v>
       </c>
       <c r="B32" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A32)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D32)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Mateo")*('Game Log Season 4'!$D$3:$D$1000=A32)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D32)</f>
         <v>3.935</v>
       </c>
       <c r="C32" s="45" t="s">
         <v>104</v>
       </c>
       <c r="D32" s="49" t="n">
-        <v>3.9</v>
+        <v>3.935</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26112,7 +26113,7 @@
         <v>36</v>
       </c>
       <c r="B34" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A34)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D34)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Ryan")*('Game Log Season 4'!$D$3:$D$1000=A34)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D34)</f>
         <v>3.5</v>
       </c>
       <c r="C34" s="45"/>
@@ -26125,12 +26126,12 @@
         <v>62</v>
       </c>
       <c r="B35" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A35)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D35)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Ryan")*('Game Log Season 4'!$D$3:$D$1000=A35)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D35)</f>
         <v>3.43088888888889</v>
       </c>
       <c r="C35" s="45"/>
       <c r="D35" s="48" t="n">
-        <v>3.4</v>
+        <v>3.43088888888889</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26138,7 +26139,7 @@
         <v>33</v>
       </c>
       <c r="B36" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A36)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D36)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Ryan")*('Game Log Season 4'!$D$3:$D$1000=A36)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D36)</f>
         <v>3.7</v>
       </c>
       <c r="C36" s="45"/>
@@ -26151,7 +26152,7 @@
         <v>61</v>
       </c>
       <c r="B37" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A37)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D37)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Ryan")*('Game Log Season 4'!$D$3:$D$1000=A37)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D37)</f>
         <v>2.6</v>
       </c>
       <c r="C37" s="45"/>
@@ -26164,12 +26165,12 @@
         <v>41</v>
       </c>
       <c r="B38" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A38)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D38)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Ryan")*('Game Log Season 4'!$D$3:$D$1000=A38)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D38)</f>
         <v>3.77816666666667</v>
       </c>
       <c r="C38" s="45"/>
       <c r="D38" s="48" t="n">
-        <v>3.8</v>
+        <v>3.77816666666667</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26177,12 +26178,12 @@
         <v>79</v>
       </c>
       <c r="B39" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A39)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D39)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Ryan")*('Game Log Season 4'!$D$3:$D$1000=A39)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D39)</f>
         <v>2.59388888888889</v>
       </c>
       <c r="C39" s="45"/>
       <c r="D39" s="48" t="n">
-        <v>2.6</v>
+        <v>2.59388888888889</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26190,12 +26191,12 @@
         <v>54</v>
       </c>
       <c r="B40" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A40)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D40)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Ryan")*('Game Log Season 4'!$D$3:$D$1000=A40)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D40)</f>
         <v>3.23902777777778</v>
       </c>
       <c r="C40" s="45"/>
       <c r="D40" s="48" t="n">
-        <v>3.6</v>
+        <v>3.23902777777778</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26203,7 +26204,7 @@
         <v>87</v>
       </c>
       <c r="B41" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A41)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D41)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Ryan")*('Game Log Season 4'!$D$3:$D$1000=A41)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D41)</f>
         <v>2.6</v>
       </c>
       <c r="C41" s="45"/>
@@ -26216,12 +26217,12 @@
         <v>89</v>
       </c>
       <c r="B42" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A42)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D42)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Ryan")*('Game Log Season 4'!$D$3:$D$1000=A42)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D42)</f>
         <v>3.58416666666667</v>
       </c>
       <c r="C42" s="45"/>
       <c r="D42" s="48" t="n">
-        <v>3.6</v>
+        <v>3.58416666666667</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26229,12 +26230,12 @@
         <v>94</v>
       </c>
       <c r="B43" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A43)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D43)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Ryan")*('Game Log Season 4'!$D$3:$D$1000=A43)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D43)</f>
         <v>2.94083333333333</v>
       </c>
       <c r="C43" s="45"/>
       <c r="D43" s="48" t="n">
-        <v>2.9</v>
+        <v>2.94083333333333</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26242,12 +26243,12 @@
         <v>97</v>
       </c>
       <c r="B44" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A44)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D44)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Ryan")*('Game Log Season 4'!$D$3:$D$1000=A44)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D44)</f>
         <v>3.92333333333333</v>
       </c>
       <c r="C44" s="45"/>
       <c r="D44" s="48" t="n">
-        <v>3.9</v>
+        <v>3.92333333333333</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26265,7 +26266,7 @@
         <v>71</v>
       </c>
       <c r="B46" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A46)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D46)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Kristy")*('Game Log Season 4'!$D$3:$D$1000=A46)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D46)</f>
         <v>3.6</v>
       </c>
       <c r="C46" s="45" t="s">
@@ -26280,14 +26281,14 @@
         <v>57</v>
       </c>
       <c r="B47" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A47)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D47)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Kristy")*('Game Log Season 4'!$D$3:$D$1000=A47)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D47)</f>
         <v>3.33761111111111</v>
       </c>
       <c r="C47" s="45" t="s">
         <v>103</v>
       </c>
       <c r="D47" s="48" t="n">
-        <v>3.3</v>
+        <v>3.33761111111111</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26295,7 +26296,7 @@
         <v>78</v>
       </c>
       <c r="B48" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A48)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D48)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Kristy")*('Game Log Season 4'!$D$3:$D$1000=A48)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D48)</f>
         <v>3.2</v>
       </c>
       <c r="C48" s="45"/>
@@ -26308,7 +26309,7 @@
         <v>85</v>
       </c>
       <c r="B49" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A49)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D49)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Kristy")*('Game Log Season 4'!$D$3:$D$1000=A49)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D49)</f>
         <v>3.9</v>
       </c>
       <c r="C49" s="45" t="s">
@@ -26323,12 +26324,12 @@
         <v>93</v>
       </c>
       <c r="B50" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A50)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D50)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Kristy")*('Game Log Season 4'!$D$3:$D$1000=A50)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D50)</f>
         <v>2.39488888888889</v>
       </c>
       <c r="C50" s="45"/>
       <c r="D50" s="48" t="n">
-        <v>2.4</v>
+        <v>2.39488888888889</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26346,7 +26347,7 @@
         <v>49</v>
       </c>
       <c r="B52" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A52)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D52)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Joseph")*('Game Log Season 4'!$D$3:$D$1000=A52)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D52)</f>
         <v>3.6</v>
       </c>
       <c r="C52" s="45"/>
@@ -26359,7 +26360,7 @@
         <v>76</v>
       </c>
       <c r="B53" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A53)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D53)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Joseph")*('Game Log Season 4'!$D$3:$D$1000=A53)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D53)</f>
         <v>3.8</v>
       </c>
       <c r="C53" s="45"/>
@@ -26372,7 +26373,7 @@
         <v>77</v>
       </c>
       <c r="B54" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A54)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D54)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Joseph")*('Game Log Season 4'!$D$3:$D$1000=A54)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D54)</f>
         <v>2.7</v>
       </c>
       <c r="C54" s="45"/>
@@ -26385,7 +26386,7 @@
         <v>64</v>
       </c>
       <c r="B55" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A55)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D55)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Joseph")*('Game Log Season 4'!$D$3:$D$1000=A55)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D55)</f>
         <v>3.3</v>
       </c>
       <c r="C55" s="45"/>
@@ -26398,12 +26399,12 @@
         <v>63</v>
       </c>
       <c r="B56" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A56)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D56)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Joseph")*('Game Log Season 4'!$D$3:$D$1000=A56)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D56)</f>
         <v>3.74035</v>
       </c>
       <c r="C56" s="45"/>
       <c r="D56" s="48" t="n">
-        <v>3.7</v>
+        <v>3.74035</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26421,7 +26422,7 @@
         <v>33</v>
       </c>
       <c r="B58" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A58)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D58)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Red")*('Game Log Season 4'!$D$3:$D$1000=A58)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D58)</f>
         <v>2.7</v>
       </c>
       <c r="C58" s="45"/>
@@ -26434,7 +26435,7 @@
         <v>69</v>
       </c>
       <c r="B59" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A59)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D59)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Red")*('Game Log Season 4'!$D$3:$D$1000=A59)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D59)</f>
         <v>3.4</v>
       </c>
       <c r="C59" s="45"/>
@@ -26447,7 +26448,7 @@
         <v>84</v>
       </c>
       <c r="B60" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A60)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D60)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Red")*('Game Log Season 4'!$D$3:$D$1000=A60)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D60)</f>
         <v>1</v>
       </c>
       <c r="C60" s="45"/>
@@ -26470,12 +26471,12 @@
         <v>52</v>
       </c>
       <c r="B62" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A62)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D62)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Michelle")*('Game Log Season 4'!$D$3:$D$1000=A62)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D62)</f>
         <v>2.30388888888889</v>
       </c>
       <c r="C62" s="45"/>
       <c r="D62" s="48" t="n">
-        <v>2.5</v>
+        <v>2.30388888888889</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26483,7 +26484,7 @@
         <v>86</v>
       </c>
       <c r="B63" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A63)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D63)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Michelle")*('Game Log Season 4'!$D$3:$D$1000=A63)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D63)</f>
         <v>2.2</v>
       </c>
       <c r="C63" s="45"/>
@@ -26496,11 +26497,11 @@
         <v>96</v>
       </c>
       <c r="B64" s="48" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A64)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D64)</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 4'!$C$3:$C$1000="Michelle")*('Game Log Season 4'!$D$3:$D$1000=A64)*('Game Log Season 4'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 4'!$X$3:$X$1000), D64)</f>
         <v>2.43069444444444</v>
       </c>
       <c r="D64" s="48" t="n">
-        <v>2.4</v>
+        <v>2.43069444444444</v>
       </c>
     </row>
   </sheetData>
@@ -26547,11 +26548,11 @@
         <v>26</v>
       </c>
       <c r="B2" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A2)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,A2)</f>
         <v>7</v>
       </c>
       <c r="C2" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A2,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,A2,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>2</v>
       </c>
       <c r="D2" s="47" t="n">
@@ -26564,11 +26565,11 @@
         <v>45</v>
       </c>
       <c r="B3" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A3)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Becca",'Game Log Season 4'!$D$3:$D$1000,A3)</f>
         <v>3</v>
       </c>
       <c r="C3" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A3,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Becca",'Game Log Season 4'!$D$3:$D$1000,A3,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>1</v>
       </c>
       <c r="D3" s="48" t="n">
@@ -26581,11 +26582,11 @@
         <v>27</v>
       </c>
       <c r="B4" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A4)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Becca",'Game Log Season 4'!$D$3:$D$1000,A4)</f>
         <v>0</v>
       </c>
       <c r="C4" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A4,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Becca",'Game Log Season 4'!$D$3:$D$1000,A4,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D4" s="48" t="n">
@@ -26598,11 +26599,11 @@
         <v>75</v>
       </c>
       <c r="B5" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A5)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Becca",'Game Log Season 4'!$D$3:$D$1000,A5)</f>
         <v>3</v>
       </c>
       <c r="C5" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A5,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Becca",'Game Log Season 4'!$D$3:$D$1000,A5,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>1</v>
       </c>
       <c r="D5" s="48" t="n">
@@ -26615,11 +26616,11 @@
         <v>95</v>
       </c>
       <c r="B6" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A6)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Becca",'Game Log Season 4'!$D$3:$D$1000,A6)</f>
         <v>1</v>
       </c>
       <c r="C6" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A6,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Becca",'Game Log Season 4'!$D$3:$D$1000,A6,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D6" s="48" t="n">
@@ -26632,11 +26633,11 @@
         <v>28</v>
       </c>
       <c r="B7" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A7)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,A7)</f>
         <v>14</v>
       </c>
       <c r="C7" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A7,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,A7,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>4</v>
       </c>
       <c r="D7" s="47" t="n">
@@ -26649,11 +26650,11 @@
         <v>68</v>
       </c>
       <c r="B8" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A8)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Manny",'Game Log Season 4'!$D$3:$D$1000,A8)</f>
         <v>4</v>
       </c>
       <c r="C8" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A8,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Manny",'Game Log Season 4'!$D$3:$D$1000,A8,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>2</v>
       </c>
       <c r="D8" s="48" t="n">
@@ -26666,11 +26667,11 @@
         <v>42</v>
       </c>
       <c r="B9" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A9)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Manny",'Game Log Season 4'!$D$3:$D$1000,A9)</f>
         <v>0</v>
       </c>
       <c r="C9" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A9,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Manny",'Game Log Season 4'!$D$3:$D$1000,A9,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D9" s="48" t="n">
@@ -26683,11 +26684,11 @@
         <v>67</v>
       </c>
       <c r="B10" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A10)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Manny",'Game Log Season 4'!$D$3:$D$1000,A10)</f>
         <v>0</v>
       </c>
       <c r="C10" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A10,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Manny",'Game Log Season 4'!$D$3:$D$1000,A10,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D10" s="48" t="n">
@@ -26700,11 +26701,11 @@
         <v>82</v>
       </c>
       <c r="B11" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A11)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Manny",'Game Log Season 4'!$D$3:$D$1000,A11)</f>
         <v>0</v>
       </c>
       <c r="C11" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A11,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Manny",'Game Log Season 4'!$D$3:$D$1000,A11,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D11" s="48" t="n">
@@ -26717,11 +26718,11 @@
         <v>44</v>
       </c>
       <c r="B12" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A12)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Manny",'Game Log Season 4'!$D$3:$D$1000,A12)</f>
         <v>0</v>
       </c>
       <c r="C12" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A12,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Manny",'Game Log Season 4'!$D$3:$D$1000,A12,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D12" s="48" t="n">
@@ -26734,11 +26735,11 @@
         <v>88</v>
       </c>
       <c r="B13" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A13)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Manny",'Game Log Season 4'!$D$3:$D$1000,A13)</f>
         <v>2</v>
       </c>
       <c r="C13" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A13,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Manny",'Game Log Season 4'!$D$3:$D$1000,A13,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D13" s="48" t="n">
@@ -26751,11 +26752,11 @@
         <v>48</v>
       </c>
       <c r="B14" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A14)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Manny",'Game Log Season 4'!$D$3:$D$1000,A14)</f>
         <v>0</v>
       </c>
       <c r="C14" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A14,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Manny",'Game Log Season 4'!$D$3:$D$1000,A14,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D14" s="48" t="n">
@@ -26768,11 +26769,11 @@
         <v>37</v>
       </c>
       <c r="B15" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A15)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Manny",'Game Log Season 4'!$D$3:$D$1000,A15)</f>
         <v>1</v>
       </c>
       <c r="C15" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A15,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Manny",'Game Log Season 4'!$D$3:$D$1000,A15,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>1</v>
       </c>
       <c r="D15" s="48" t="n">
@@ -26785,11 +26786,11 @@
         <v>91</v>
       </c>
       <c r="B16" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A16)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Manny",'Game Log Season 4'!$D$3:$D$1000,A16)</f>
         <v>6</v>
       </c>
       <c r="C16" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A16,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Manny",'Game Log Season 4'!$D$3:$D$1000,A16,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>1</v>
       </c>
       <c r="D16" s="48" t="n">
@@ -26802,11 +26803,11 @@
         <v>47</v>
       </c>
       <c r="B17" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A17)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Manny",'Game Log Season 4'!$D$3:$D$1000,A17)</f>
         <v>1</v>
       </c>
       <c r="C17" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A17,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Manny",'Game Log Season 4'!$D$3:$D$1000,A17,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D17" s="48" t="n">
@@ -26819,11 +26820,11 @@
         <v>30</v>
       </c>
       <c r="B18" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A18)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,A18)</f>
         <v>12</v>
       </c>
       <c r="C18" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A18,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,A18,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>5</v>
       </c>
       <c r="D18" s="47" t="n">
@@ -26836,11 +26837,11 @@
         <v>73</v>
       </c>
       <c r="B19" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A19)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A19)</f>
         <v>0</v>
       </c>
       <c r="C19" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A19,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A19,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D19" s="48" t="n">
@@ -26853,11 +26854,11 @@
         <v>66</v>
       </c>
       <c r="B20" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A20)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A20)</f>
         <v>0</v>
       </c>
       <c r="C20" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A20,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A20,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D20" s="48" t="n">
@@ -26870,11 +26871,11 @@
         <v>31</v>
       </c>
       <c r="B21" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A21)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A21)</f>
         <v>1</v>
       </c>
       <c r="C21" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A21,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A21,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D21" s="48" t="n">
@@ -26887,11 +26888,11 @@
         <v>34</v>
       </c>
       <c r="B22" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A22)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A22)</f>
         <v>0</v>
       </c>
       <c r="C22" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A22,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A22,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D22" s="48" t="n">
@@ -26904,11 +26905,11 @@
         <v>74</v>
       </c>
       <c r="B23" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A23)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A23)</f>
         <v>0</v>
       </c>
       <c r="C23" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A23,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A23,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D23" s="48" t="n">
@@ -26921,11 +26922,11 @@
         <v>57</v>
       </c>
       <c r="B24" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A24)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A24)</f>
         <v>0</v>
       </c>
       <c r="C24" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A24,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A24,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D24" s="48" t="n">
@@ -26938,11 +26939,11 @@
         <v>80</v>
       </c>
       <c r="B25" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A25)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A25)</f>
         <v>0</v>
       </c>
       <c r="C25" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A25,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A25,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D25" s="48" t="n">
@@ -26955,11 +26956,11 @@
         <v>81</v>
       </c>
       <c r="B26" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A26)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A26)</f>
         <v>0</v>
       </c>
       <c r="C26" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A26,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A26,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D26" s="48" t="n">
@@ -26972,11 +26973,11 @@
         <v>83</v>
       </c>
       <c r="B27" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A27)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A27)</f>
         <v>1</v>
       </c>
       <c r="C27" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A27,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A27,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D27" s="48" t="n">
@@ -26989,11 +26990,11 @@
         <v>48</v>
       </c>
       <c r="B28" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A28)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A28)</f>
         <v>1</v>
       </c>
       <c r="C28" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A28,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A28,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>1</v>
       </c>
       <c r="D28" s="48" t="n">
@@ -27006,11 +27007,11 @@
         <v>90</v>
       </c>
       <c r="B29" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A29)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A29)</f>
         <v>4</v>
       </c>
       <c r="C29" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A29,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A29,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D29" s="48" t="n">
@@ -27023,11 +27024,11 @@
         <v>46</v>
       </c>
       <c r="B30" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A30)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A30)</f>
         <v>1</v>
       </c>
       <c r="C30" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A30,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A30,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>1</v>
       </c>
       <c r="D30" s="48" t="n">
@@ -27040,11 +27041,11 @@
         <v>92</v>
       </c>
       <c r="B31" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A31)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A31)</f>
         <v>3</v>
       </c>
       <c r="C31" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A31,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A31,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>2</v>
       </c>
       <c r="D31" s="48" t="n">
@@ -27057,11 +27058,11 @@
         <v>40</v>
       </c>
       <c r="B32" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A32)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A32)</f>
         <v>1</v>
       </c>
       <c r="C32" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A32,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Mateo",'Game Log Season 4'!$D$3:$D$1000,A32,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>1</v>
       </c>
       <c r="D32" s="48" t="n">
@@ -27074,11 +27075,11 @@
         <v>32</v>
       </c>
       <c r="B33" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A33)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,A33)</f>
         <v>11</v>
       </c>
       <c r="C33" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A33,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,A33,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>3</v>
       </c>
       <c r="D33" s="47" t="n">
@@ -27091,11 +27092,11 @@
         <v>36</v>
       </c>
       <c r="B34" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A34)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A34)</f>
         <v>0</v>
       </c>
       <c r="C34" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A34,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A34,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D34" s="48" t="n">
@@ -27108,11 +27109,11 @@
         <v>62</v>
       </c>
       <c r="B35" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A35)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A35)</f>
         <v>1</v>
       </c>
       <c r="C35" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A35,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A35,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D35" s="48" t="n">
@@ -27125,11 +27126,11 @@
         <v>33</v>
       </c>
       <c r="B36" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A36)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A36)</f>
         <v>0</v>
       </c>
       <c r="C36" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A36,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A36,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D36" s="48" t="n">
@@ -27142,11 +27143,11 @@
         <v>61</v>
       </c>
       <c r="B37" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A37)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A37)</f>
         <v>0</v>
       </c>
       <c r="C37" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A37,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A37,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D37" s="48" t="n">
@@ -27159,11 +27160,11 @@
         <v>41</v>
       </c>
       <c r="B38" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A38)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A38)</f>
         <v>1</v>
       </c>
       <c r="C38" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A38,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A38,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>1</v>
       </c>
       <c r="D38" s="48" t="n">
@@ -27176,11 +27177,11 @@
         <v>79</v>
       </c>
       <c r="B39" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A39)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A39)</f>
         <v>1</v>
       </c>
       <c r="C39" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A39,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A39,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D39" s="48" t="n">
@@ -27193,11 +27194,11 @@
         <v>54</v>
       </c>
       <c r="B40" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A40)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A40)</f>
         <v>2</v>
       </c>
       <c r="C40" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A40,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A40,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D40" s="48" t="n">
@@ -27210,11 +27211,11 @@
         <v>87</v>
       </c>
       <c r="B41" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A41)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A41)</f>
         <v>0</v>
       </c>
       <c r="C41" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A41,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A41,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D41" s="48" t="n">
@@ -27227,11 +27228,11 @@
         <v>89</v>
       </c>
       <c r="B42" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A42)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A42)</f>
         <v>2</v>
       </c>
       <c r="C42" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A42,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A42,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D42" s="48" t="n">
@@ -27244,11 +27245,11 @@
         <v>94</v>
       </c>
       <c r="B43" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A43)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A43)</f>
         <v>2</v>
       </c>
       <c r="C43" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A43,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A43,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>1</v>
       </c>
       <c r="D43" s="48" t="n">
@@ -27261,11 +27262,11 @@
         <v>97</v>
       </c>
       <c r="B44" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A44)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A44)</f>
         <v>2</v>
       </c>
       <c r="C44" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A44,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Ryan",'Game Log Season 4'!$D$3:$D$1000,A44,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>1</v>
       </c>
       <c r="D44" s="48" t="n">
@@ -27278,11 +27279,11 @@
         <v>70</v>
       </c>
       <c r="B45" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A45)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,A45)</f>
         <v>2</v>
       </c>
       <c r="C45" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A45,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,A45,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D45" s="47" t="n">
@@ -27295,11 +27296,11 @@
         <v>71</v>
       </c>
       <c r="B46" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A46)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Kristy",'Game Log Season 4'!$D$3:$D$1000,A46)</f>
         <v>0</v>
       </c>
       <c r="C46" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A46,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Kristy",'Game Log Season 4'!$D$3:$D$1000,A46,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D46" s="48" t="n">
@@ -27312,11 +27313,11 @@
         <v>57</v>
       </c>
       <c r="B47" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A47)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Kristy",'Game Log Season 4'!$D$3:$D$1000,A47)</f>
         <v>1</v>
       </c>
       <c r="C47" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A47,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Kristy",'Game Log Season 4'!$D$3:$D$1000,A47,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D47" s="48" t="n">
@@ -27329,11 +27330,11 @@
         <v>78</v>
       </c>
       <c r="B48" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A48)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Kristy",'Game Log Season 4'!$D$3:$D$1000,A48)</f>
         <v>0</v>
       </c>
       <c r="C48" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A48,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Kristy",'Game Log Season 4'!$D$3:$D$1000,A48,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D48" s="48" t="n">
@@ -27346,11 +27347,11 @@
         <v>85</v>
       </c>
       <c r="B49" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A49)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Kristy",'Game Log Season 4'!$D$3:$D$1000,A49)</f>
         <v>0</v>
       </c>
       <c r="C49" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A49,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Kristy",'Game Log Season 4'!$D$3:$D$1000,A49,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D49" s="48" t="n">
@@ -27363,11 +27364,11 @@
         <v>93</v>
       </c>
       <c r="B50" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A50)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Kristy",'Game Log Season 4'!$D$3:$D$1000,A50)</f>
         <v>1</v>
       </c>
       <c r="C50" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A50,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Kristy",'Game Log Season 4'!$D$3:$D$1000,A50,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D50" s="48" t="n">
@@ -27380,11 +27381,11 @@
         <v>38</v>
       </c>
       <c r="B51" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A51)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,A51)</f>
         <v>1</v>
       </c>
       <c r="C51" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A51,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,A51,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D51" s="47" t="n">
@@ -27397,11 +27398,11 @@
         <v>49</v>
       </c>
       <c r="B52" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A52)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Joseph",'Game Log Season 4'!$D$3:$D$1000,A52)</f>
         <v>0</v>
       </c>
       <c r="C52" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A52,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Joseph",'Game Log Season 4'!$D$3:$D$1000,A52,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D52" s="48" t="n">
@@ -27414,11 +27415,11 @@
         <v>76</v>
       </c>
       <c r="B53" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A53)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Joseph",'Game Log Season 4'!$D$3:$D$1000,A53)</f>
         <v>0</v>
       </c>
       <c r="C53" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A53,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Joseph",'Game Log Season 4'!$D$3:$D$1000,A53,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D53" s="48" t="n">
@@ -27431,11 +27432,11 @@
         <v>77</v>
       </c>
       <c r="B54" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A54)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Joseph",'Game Log Season 4'!$D$3:$D$1000,A54)</f>
         <v>0</v>
       </c>
       <c r="C54" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A54,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Joseph",'Game Log Season 4'!$D$3:$D$1000,A54,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D54" s="48" t="n">
@@ -27448,11 +27449,11 @@
         <v>64</v>
       </c>
       <c r="B55" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A55)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Joseph",'Game Log Season 4'!$D$3:$D$1000,A55)</f>
         <v>0</v>
       </c>
       <c r="C55" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A55,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Joseph",'Game Log Season 4'!$D$3:$D$1000,A55,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D55" s="48" t="n">
@@ -27465,11 +27466,11 @@
         <v>63</v>
       </c>
       <c r="B56" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A56)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Joseph",'Game Log Season 4'!$D$3:$D$1000,A56)</f>
         <v>1</v>
       </c>
       <c r="C56" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A56,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Joseph",'Game Log Season 4'!$D$3:$D$1000,A56,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D56" s="48" t="n">
@@ -27482,11 +27483,11 @@
         <v>59</v>
       </c>
       <c r="B57" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A57)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,A57)</f>
         <v>0</v>
       </c>
       <c r="C57" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A57,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,A57,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D57" s="47" t="n">
@@ -27499,11 +27500,11 @@
         <v>33</v>
       </c>
       <c r="B58" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A58)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Red",'Game Log Season 4'!$D$3:$D$1000,A58)</f>
         <v>0</v>
       </c>
       <c r="C58" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A58,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Red",'Game Log Season 4'!$D$3:$D$1000,A58,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D58" s="48" t="n">
@@ -27516,11 +27517,11 @@
         <v>69</v>
       </c>
       <c r="B59" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A59)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Red",'Game Log Season 4'!$D$3:$D$1000,A59)</f>
         <v>0</v>
       </c>
       <c r="C59" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A59,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Red",'Game Log Season 4'!$D$3:$D$1000,A59,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D59" s="48" t="n">
@@ -27533,11 +27534,11 @@
         <v>84</v>
       </c>
       <c r="B60" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A60)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Red",'Game Log Season 4'!$D$3:$D$1000,A60)</f>
         <v>0</v>
       </c>
       <c r="C60" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A60,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Red",'Game Log Season 4'!$D$3:$D$1000,A60,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D60" s="48" t="n">
@@ -27550,11 +27551,11 @@
         <v>51</v>
       </c>
       <c r="B61" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A61)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,A61)</f>
         <v>4</v>
       </c>
       <c r="C61" s="47" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A61,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,A61,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D61" s="47" t="n">
@@ -27567,11 +27568,11 @@
         <v>52</v>
       </c>
       <c r="B62" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A62)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Michelle",'Game Log Season 4'!$D$3:$D$1000,A62)</f>
         <v>3</v>
       </c>
       <c r="C62" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A62,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Michelle",'Game Log Season 4'!$D$3:$D$1000,A62,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D62" s="48" t="n">
@@ -27584,11 +27585,11 @@
         <v>86</v>
       </c>
       <c r="B63" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A63)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Michelle",'Game Log Season 4'!$D$3:$D$1000,A63)</f>
         <v>0</v>
       </c>
       <c r="C63" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A63,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Michelle",'Game Log Season 4'!$D$3:$D$1000,A63,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D63" s="48" t="n">
@@ -27601,11 +27602,11 @@
         <v>96</v>
       </c>
       <c r="B64" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A64)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Michelle",'Game Log Season 4'!$D$3:$D$1000,A64)</f>
         <v>1</v>
       </c>
       <c r="C64" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A64,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$1000,"Michelle",'Game Log Season 4'!$D$3:$D$1000,A64,'Game Log Season 4'!$F$3:$F$1000,1)</f>
         <v>0</v>
       </c>
       <c r="D64" s="48" t="n">
@@ -27693,11 +27694,11 @@
         <v>0.371988902467902</v>
       </c>
       <c r="C2" s="14" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$126, "Mateo", 'Game Log Season 3'!$F$3:$F$126, 1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$126, "Mateo", 'Game Log Season 4'!$F$3:$F$126, 1)</f>
         <v>5</v>
       </c>
       <c r="D2" s="14" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$126, "Mateo", 'Game Log Season 3'!$F$3:$F$126, 0)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$126, "Mateo", 'Game Log Season 4'!$F$3:$F$126, 0)</f>
         <v>7</v>
       </c>
       <c r="E2" s="17" t="n">
@@ -27705,11 +27706,11 @@
         <v>0.416666666666667</v>
       </c>
       <c r="F2" s="14" t="n">
-        <f aca="false">SUMIFS('Game Log Season 3'!$J$3:$J$126, 'Game Log Season 3'!$C$3:$C$126, "Mateo", 'Game Log Season 3'!$F$3:$F$126, 1)</f>
+        <f aca="false">SUMIFS('Game Log Season 4'!$J$3:$J$126, 'Game Log Season 4'!$C$3:$C$126, "Mateo", 'Game Log Season 4'!$F$3:$F$126, 1)</f>
         <v>3.55</v>
       </c>
       <c r="G2" s="14" t="n">
-        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 3'!$J$3:$J$126, 'Game Log Season 3'!$C$3:$C$126, "Mateo", 'Game Log Season 3'!$F$3:$F$126, 0)*-1))*D2,0)</f>
+        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 4'!$J$3:$J$126, 'Game Log Season 4'!$C$3:$C$126, "Mateo", 'Game Log Season 4'!$F$3:$F$126, 0)*-1))*D2,0)</f>
         <v>5.13333333333333</v>
       </c>
       <c r="H2" s="17" t="n">
@@ -27717,15 +27718,15 @@
         <v>0.408829174664108</v>
       </c>
       <c r="I2" s="17" t="n">
-        <f aca="false">IF(C2&lt;&gt;0,AVERAGEIF('Game Log Season 3'!$C$3:$C$126, "Mateo", 'Game Log Season 3'!$K$3:$K$126),0)</f>
+        <f aca="false">IF(C2&lt;&gt;0,AVERAGEIF('Game Log Season 4'!$C$3:$C$126, "Mateo", 'Game Log Season 4'!$K$3:$K$126),0)</f>
         <v>0.238611111111111</v>
       </c>
       <c r="J2" s="14" t="n">
-        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 3'!$M$3:$M$126, 'Game Log Season 3'!$C$3:$C$126, "Mateo", 'Game Log Season 3'!$F$3:$F$126, 1)-0.5))*C2, 0)</f>
+        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 4'!$M$3:$M$126, 'Game Log Season 4'!$C$3:$C$126, "Mateo", 'Game Log Season 4'!$F$3:$F$126, 1)-0.5))*C2, 0)</f>
         <v>5.01575</v>
       </c>
       <c r="K2" s="14" t="n">
-        <f aca="false">IFERROR((1+(AVERAGEIFS('Game Log Season 3'!$M$3:$M$126, 'Game Log Season 3'!$C$3:$C$126, "Mateo", 'Game Log Season 3'!$F$3:$F$126, 0)-0.5))*D2, 0)</f>
+        <f aca="false">IFERROR((1+(AVERAGEIFS('Game Log Season 4'!$M$3:$M$126, 'Game Log Season 4'!$C$3:$C$126, "Mateo", 'Game Log Season 4'!$F$3:$F$126, 0)-0.5))*D2, 0)</f>
         <v>7.423</v>
       </c>
       <c r="L2" s="17" t="n">
@@ -27742,11 +27743,11 @@
         <v>0.249788769042654</v>
       </c>
       <c r="C3" s="14" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$126, "Ryan", 'Game Log Season 3'!$F$3:$F$126, 1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$126, "Ryan", 'Game Log Season 4'!$F$3:$F$126, 1)</f>
         <v>3</v>
       </c>
       <c r="D3" s="14" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$126, "Ryan", 'Game Log Season 3'!$F$3:$F$126, 0)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$126, "Ryan", 'Game Log Season 4'!$F$3:$F$126, 0)</f>
         <v>8</v>
       </c>
       <c r="E3" s="17" t="n">
@@ -27754,11 +27755,11 @@
         <v>0.272727272727273</v>
       </c>
       <c r="F3" s="14" t="n">
-        <f aca="false">SUMIFS('Game Log Season 3'!$J$3:$J$126, 'Game Log Season 3'!$C$3:$C$126, "Ryan", 'Game Log Season 3'!$F$3:$F$126, 1)</f>
+        <f aca="false">SUMIFS('Game Log Season 4'!$J$3:$J$126, 'Game Log Season 4'!$C$3:$C$126, "Ryan", 'Game Log Season 4'!$F$3:$F$126, 1)</f>
         <v>2.13333333333333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 3'!$J$3:$J$126, 'Game Log Season 3'!$C$3:$C$126, "Ryan", 'Game Log Season 3'!$F$3:$F$126, 0)*-1))*D3,0)</f>
+        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 4'!$J$3:$J$126, 'Game Log Season 4'!$C$3:$C$126, "Ryan", 'Game Log Season 4'!$F$3:$F$126, 0)*-1))*D3,0)</f>
         <v>5.71666666666667</v>
       </c>
       <c r="H3" s="17" t="n">
@@ -27766,15 +27767,15 @@
         <v>0.271762208067941</v>
       </c>
       <c r="I3" s="17" t="n">
-        <f aca="false">IF(C3&lt;&gt;0,AVERAGEIF('Game Log Season 3'!$C$3:$C$126, "Ryan", 'Game Log Season 3'!$K$3:$K$126),0)</f>
+        <f aca="false">IF(C3&lt;&gt;0,AVERAGEIF('Game Log Season 4'!$C$3:$C$126, "Ryan", 'Game Log Season 4'!$K$3:$K$126),0)</f>
         <v>0.187575757575758</v>
       </c>
       <c r="J3" s="14" t="n">
-        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 3'!$M$3:$M$126, 'Game Log Season 3'!$C$3:$C$126, "Ryan", 'Game Log Season 3'!$F$3:$F$126, 1)-0.5))*C3, 0)</f>
+        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 4'!$M$3:$M$126, 'Game Log Season 4'!$C$3:$C$126, "Ryan", 'Game Log Season 4'!$F$3:$F$126, 1)-0.5))*C3, 0)</f>
         <v>2.9415</v>
       </c>
       <c r="K3" s="14" t="n">
-        <f aca="false">IFERROR((1+(AVERAGEIFS('Game Log Season 3'!$M$3:$M$126, 'Game Log Season 3'!$C$3:$C$126, "Ryan", 'Game Log Season 3'!$F$3:$F$126, 0)-0.5))*D3, 0)</f>
+        <f aca="false">IFERROR((1+(AVERAGEIFS('Game Log Season 4'!$M$3:$M$126, 'Game Log Season 4'!$C$3:$C$126, "Ryan", 'Game Log Season 4'!$F$3:$F$126, 0)-0.5))*D3, 0)</f>
         <v>8.3075</v>
       </c>
       <c r="L3" s="17" t="n">
@@ -27791,11 +27792,11 @@
         <v>0.257655970198026</v>
       </c>
       <c r="C4" s="14" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$126, "Becca", 'Game Log Season 3'!$F$3:$F$126, 1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$126, "Becca", 'Game Log Season 4'!$F$3:$F$126, 1)</f>
         <v>2</v>
       </c>
       <c r="D4" s="14" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$126, "Becca", 'Game Log Season 3'!$F$3:$F$126, 0)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$126, "Becca", 'Game Log Season 4'!$F$3:$F$126, 0)</f>
         <v>5</v>
       </c>
       <c r="E4" s="17" t="n">
@@ -27803,11 +27804,11 @@
         <v>0.285714285714286</v>
       </c>
       <c r="F4" s="14" t="n">
-        <f aca="false">SUMIFS('Game Log Season 3'!$J$3:$J$126, 'Game Log Season 3'!$C$3:$C$126, "Becca", 'Game Log Season 3'!$F$3:$F$126, 1)</f>
+        <f aca="false">SUMIFS('Game Log Season 4'!$J$3:$J$126, 'Game Log Season 4'!$C$3:$C$126, "Becca", 'Game Log Season 4'!$F$3:$F$126, 1)</f>
         <v>1.5</v>
       </c>
       <c r="G4" s="14" t="n">
-        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 3'!$J$3:$J$126, 'Game Log Season 3'!$C$3:$C$126, "Becca", 'Game Log Season 3'!$F$3:$F$126, 0)*-1))*D4,0)</f>
+        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 4'!$J$3:$J$126, 'Game Log Season 4'!$C$3:$C$126, "Becca", 'Game Log Season 4'!$F$3:$F$126, 0)*-1))*D4,0)</f>
         <v>3.63333333333333</v>
       </c>
       <c r="H4" s="17" t="n">
@@ -27815,15 +27816,15 @@
         <v>0.292207792207792</v>
       </c>
       <c r="I4" s="17" t="n">
-        <f aca="false">IF(C4&lt;&gt;0,AVERAGEIF('Game Log Season 3'!$C$3:$C$126, "Becca", 'Game Log Season 3'!$K$3:$K$126),0)</f>
+        <f aca="false">IF(C4&lt;&gt;0,AVERAGEIF('Game Log Season 4'!$C$3:$C$126, "Becca", 'Game Log Season 4'!$K$3:$K$126),0)</f>
         <v>0.0771428571428572</v>
       </c>
       <c r="J4" s="14" t="n">
-        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 3'!$M$3:$M$126, 'Game Log Season 3'!$C$3:$C$126, "Becca", 'Game Log Season 3'!$F$3:$F$126, 1)-0.5))*C4, 0)</f>
+        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 4'!$M$3:$M$126, 'Game Log Season 4'!$C$3:$C$126, "Becca", 'Game Log Season 4'!$F$3:$F$126, 1)-0.5))*C4, 0)</f>
         <v>2.15</v>
       </c>
       <c r="K4" s="14" t="n">
-        <f aca="false">IFERROR((1+(AVERAGEIFS('Game Log Season 3'!$M$3:$M$126, 'Game Log Season 3'!$C$3:$C$126, "Becca", 'Game Log Season 3'!$F$3:$F$126, 0)-0.5))*D4, 0)</f>
+        <f aca="false">IFERROR((1+(AVERAGEIFS('Game Log Season 4'!$M$3:$M$126, 'Game Log Season 4'!$C$3:$C$126, "Becca", 'Game Log Season 4'!$F$3:$F$126, 0)-0.5))*D4, 0)</f>
         <v>4.805</v>
       </c>
       <c r="L4" s="17" t="n">
@@ -27840,11 +27841,11 @@
         <v>0.259653014766718</v>
       </c>
       <c r="C5" s="14" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$126, "Manny", 'Game Log Season 3'!$F$3:$F$126, 1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$126, "Manny", 'Game Log Season 4'!$F$3:$F$126, 1)</f>
         <v>4</v>
       </c>
       <c r="D5" s="14" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$126, "Manny", 'Game Log Season 3'!$F$3:$F$126, 0)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$126, "Manny", 'Game Log Season 4'!$F$3:$F$126, 0)</f>
         <v>10</v>
       </c>
       <c r="E5" s="17" t="n">
@@ -27852,11 +27853,11 @@
         <v>0.285714285714286</v>
       </c>
       <c r="F5" s="14" t="n">
-        <f aca="false">SUMIFS('Game Log Season 3'!$J$3:$J$126, 'Game Log Season 3'!$C$3:$C$126, "Manny", 'Game Log Season 3'!$F$3:$F$126, 1)</f>
+        <f aca="false">SUMIFS('Game Log Season 4'!$J$3:$J$126, 'Game Log Season 4'!$C$3:$C$126, "Manny", 'Game Log Season 4'!$F$3:$F$126, 1)</f>
         <v>2.83333333333333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 3'!$J$3:$J$126, 'Game Log Season 3'!$C$3:$C$126, "Manny", 'Game Log Season 3'!$F$3:$F$126, 0)*-1))*D5,0)</f>
+        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 4'!$J$3:$J$126, 'Game Log Season 4'!$C$3:$C$126, "Manny", 'Game Log Season 4'!$F$3:$F$126, 0)*-1))*D5,0)</f>
         <v>7.18333333333333</v>
       </c>
       <c r="H5" s="17" t="n">
@@ -27864,15 +27865,15 @@
         <v>0.282861896838602</v>
       </c>
       <c r="I5" s="17" t="n">
-        <f aca="false">IF(C5&lt;&gt;0,AVERAGEIF('Game Log Season 3'!$C$3:$C$126, "Manny", 'Game Log Season 3'!$K$3:$K$126),0)</f>
+        <f aca="false">IF(C5&lt;&gt;0,AVERAGEIF('Game Log Season 4'!$C$3:$C$126, "Manny", 'Game Log Season 4'!$K$3:$K$126),0)</f>
         <v>0.166428571428571</v>
       </c>
       <c r="J5" s="14" t="n">
-        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 3'!$M$3:$M$126, 'Game Log Season 3'!$C$3:$C$126, "Manny", 'Game Log Season 3'!$F$3:$F$126, 1)-0.5))*C5, 0)</f>
+        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 4'!$M$3:$M$126, 'Game Log Season 4'!$C$3:$C$126, "Manny", 'Game Log Season 4'!$F$3:$F$126, 1)-0.5))*C5, 0)</f>
         <v>3.8005</v>
       </c>
       <c r="K5" s="14" t="n">
-        <f aca="false">IFERROR((1+(AVERAGEIFS('Game Log Season 3'!$M$3:$M$126, 'Game Log Season 3'!$C$3:$C$126, "Manny", 'Game Log Season 3'!$F$3:$F$126, 0)-0.5))*D5, 0)</f>
+        <f aca="false">IFERROR((1+(AVERAGEIFS('Game Log Season 4'!$M$3:$M$126, 'Game Log Season 4'!$C$3:$C$126, "Manny", 'Game Log Season 4'!$F$3:$F$126, 0)-0.5))*D5, 0)</f>
         <v>9.628</v>
       </c>
       <c r="L5" s="17" t="n">
@@ -27889,11 +27890,11 @@
         <v>0</v>
       </c>
       <c r="C6" s="14" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$126, "Kristy", 'Game Log Season 3'!$F$3:$F$126, 1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$126, "Kristy", 'Game Log Season 4'!$F$3:$F$126, 1)</f>
         <v>0</v>
       </c>
       <c r="D6" s="14" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$126, "Kristy", 'Game Log Season 3'!$F$3:$F$126, 0)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$126, "Kristy", 'Game Log Season 4'!$F$3:$F$126, 0)</f>
         <v>2</v>
       </c>
       <c r="E6" s="17" t="n">
@@ -27901,11 +27902,11 @@
         <v>0</v>
       </c>
       <c r="F6" s="14" t="n">
-        <f aca="false">SUMIFS('Game Log Season 3'!$J$3:$J$126, 'Game Log Season 3'!$C$3:$C$126, "Kristy", 'Game Log Season 3'!$F$3:$F$126, 1)</f>
+        <f aca="false">SUMIFS('Game Log Season 4'!$J$3:$J$126, 'Game Log Season 4'!$C$3:$C$126, "Kristy", 'Game Log Season 4'!$F$3:$F$126, 1)</f>
         <v>0</v>
       </c>
       <c r="G6" s="14" t="n">
-        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 3'!$J$3:$J$126, 'Game Log Season 3'!$C$3:$C$126, "Kristy", 'Game Log Season 3'!$F$3:$F$126, 0)*-1))*D6,0)</f>
+        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 4'!$J$3:$J$126, 'Game Log Season 4'!$C$3:$C$126, "Kristy", 'Game Log Season 4'!$F$3:$F$126, 0)*-1))*D6,0)</f>
         <v>1.6</v>
       </c>
       <c r="H6" s="17" t="n">
@@ -27913,15 +27914,15 @@
         <v>0</v>
       </c>
       <c r="I6" s="17" t="n">
-        <f aca="false">IF(C6&lt;&gt;0,AVERAGEIF('Game Log Season 3'!$C$3:$C$126, "Kristy", 'Game Log Season 3'!$K$3:$K$126),0)</f>
+        <f aca="false">IF(C6&lt;&gt;0,AVERAGEIF('Game Log Season 4'!$C$3:$C$126, "Kristy", 'Game Log Season 4'!$K$3:$K$126),0)</f>
         <v>0</v>
       </c>
       <c r="J6" s="14" t="n">
-        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 3'!$M$3:$M$126, 'Game Log Season 3'!$C$3:$C$126, "Kristy", 'Game Log Season 3'!$F$3:$F$126, 1)-0.5))*C6, 0)</f>
+        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 4'!$M$3:$M$126, 'Game Log Season 4'!$C$3:$C$126, "Kristy", 'Game Log Season 4'!$F$3:$F$126, 1)-0.5))*C6, 0)</f>
         <v>0</v>
       </c>
       <c r="K6" s="14" t="n">
-        <f aca="false">IFERROR((1+(AVERAGEIFS('Game Log Season 3'!$M$3:$M$126, 'Game Log Season 3'!$C$3:$C$126, "Kristy", 'Game Log Season 3'!$F$3:$F$126, 0)-0.5))*D6, 0)</f>
+        <f aca="false">IFERROR((1+(AVERAGEIFS('Game Log Season 4'!$M$3:$M$126, 'Game Log Season 4'!$C$3:$C$126, "Kristy", 'Game Log Season 4'!$F$3:$F$126, 0)-0.5))*D6, 0)</f>
         <v>1.955</v>
       </c>
       <c r="L6" s="17" t="n">
@@ -27938,11 +27939,11 @@
         <v>0</v>
       </c>
       <c r="C7" s="14" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$126, "Joseph", 'Game Log Season 3'!$F$3:$F$126, 1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$126, "Joseph", 'Game Log Season 4'!$F$3:$F$126, 1)</f>
         <v>0</v>
       </c>
       <c r="D7" s="14" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$126, "Joseph", 'Game Log Season 3'!$F$3:$F$126, 0)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$126, "Joseph", 'Game Log Season 4'!$F$3:$F$126, 0)</f>
         <v>1</v>
       </c>
       <c r="E7" s="17" t="n">
@@ -27950,11 +27951,11 @@
         <v>0</v>
       </c>
       <c r="F7" s="14" t="n">
-        <f aca="false">SUMIFS('Game Log Season 3'!$J$3:$J$126, 'Game Log Season 3'!$C$3:$C$126, "Joseph", 'Game Log Season 3'!$F$3:$F$126, 1)</f>
+        <f aca="false">SUMIFS('Game Log Season 4'!$J$3:$J$126, 'Game Log Season 4'!$C$3:$C$126, "Joseph", 'Game Log Season 4'!$F$3:$F$126, 1)</f>
         <v>0</v>
       </c>
       <c r="G7" s="14" t="n">
-        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 3'!$J$3:$J$126, 'Game Log Season 3'!$C$3:$C$126, "Joseph", 'Game Log Season 3'!$F$3:$F$126, 0)*-1))*D7,0)</f>
+        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 4'!$J$3:$J$126, 'Game Log Season 4'!$C$3:$C$126, "Joseph", 'Game Log Season 4'!$F$3:$F$126, 0)*-1))*D7,0)</f>
         <v>0.8</v>
       </c>
       <c r="H7" s="17" t="n">
@@ -27962,15 +27963,15 @@
         <v>0</v>
       </c>
       <c r="I7" s="17" t="n">
-        <f aca="false">IF(C7&lt;&gt;0,AVERAGEIF('Game Log Season 3'!$C$3:$C$126, "Joseph", 'Game Log Season 3'!$K$3:$K$126),0)</f>
+        <f aca="false">IF(C7&lt;&gt;0,AVERAGEIF('Game Log Season 4'!$C$3:$C$126, "Joseph", 'Game Log Season 4'!$K$3:$K$126),0)</f>
         <v>0</v>
       </c>
       <c r="J7" s="14" t="n">
-        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 3'!$M$3:$M$126, 'Game Log Season 3'!$C$3:$C$126, "Joseph", 'Game Log Season 3'!$F$3:$F$126, 1)-0.5))*C7, 0)</f>
+        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 4'!$M$3:$M$126, 'Game Log Season 4'!$C$3:$C$126, "Joseph", 'Game Log Season 4'!$F$3:$F$126, 1)-0.5))*C7, 0)</f>
         <v>0</v>
       </c>
       <c r="K7" s="14" t="n">
-        <f aca="false">IFERROR((1+(AVERAGEIFS('Game Log Season 3'!$M$3:$M$126, 'Game Log Season 3'!$C$3:$C$126, "Joseph", 'Game Log Season 3'!$F$3:$F$126, 0)-0.5))*D7, 0)</f>
+        <f aca="false">IFERROR((1+(AVERAGEIFS('Game Log Season 4'!$M$3:$M$126, 'Game Log Season 4'!$C$3:$C$126, "Joseph", 'Game Log Season 4'!$F$3:$F$126, 0)-0.5))*D7, 0)</f>
         <v>1.04275</v>
       </c>
       <c r="L7" s="17" t="n">
@@ -27987,11 +27988,11 @@
         <v>0</v>
       </c>
       <c r="C8" s="14" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$126, "Michelle", 'Game Log Season 3'!$F$3:$F$126, 1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$126, "Michelle", 'Game Log Season 4'!$F$3:$F$126, 1)</f>
         <v>0</v>
       </c>
       <c r="D8" s="14" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$126, "Michelle", 'Game Log Season 3'!$F$3:$F$126, 0)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$126, "Michelle", 'Game Log Season 4'!$F$3:$F$126, 0)</f>
         <v>4</v>
       </c>
       <c r="E8" s="17" t="n">
@@ -27999,11 +28000,11 @@
         <v>0</v>
       </c>
       <c r="F8" s="14" t="n">
-        <f aca="false">SUMIFS('Game Log Season 3'!$J$3:$J$126, 'Game Log Season 3'!$C$3:$C$126, "Michelle", 'Game Log Season 3'!$F$3:$F$126, 1)</f>
+        <f aca="false">SUMIFS('Game Log Season 4'!$J$3:$J$126, 'Game Log Season 4'!$C$3:$C$126, "Michelle", 'Game Log Season 4'!$F$3:$F$126, 1)</f>
         <v>0</v>
       </c>
       <c r="G8" s="14" t="n">
-        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 3'!$J$3:$J$126, 'Game Log Season 3'!$C$3:$C$126, "Michelle", 'Game Log Season 3'!$F$3:$F$126, 0)*-1))*D8,0)</f>
+        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 4'!$J$3:$J$126, 'Game Log Season 4'!$C$3:$C$126, "Michelle", 'Game Log Season 4'!$F$3:$F$126, 0)*-1))*D8,0)</f>
         <v>2.91666666666667</v>
       </c>
       <c r="H8" s="17" t="n">
@@ -28011,15 +28012,15 @@
         <v>0</v>
       </c>
       <c r="I8" s="17" t="n">
-        <f aca="false">IF(C8&lt;&gt;0,AVERAGEIF('Game Log Season 3'!$C$3:$C$126, "Michelle", 'Game Log Season 3'!$K$3:$K$126),0)</f>
+        <f aca="false">IF(C8&lt;&gt;0,AVERAGEIF('Game Log Season 4'!$C$3:$C$126, "Michelle", 'Game Log Season 4'!$K$3:$K$126),0)</f>
         <v>0</v>
       </c>
       <c r="J8" s="14" t="n">
-        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 3'!$M$3:$M$126, 'Game Log Season 3'!$C$3:$C$126, "Michelle", 'Game Log Season 3'!$F$3:$F$126, 1)-0.5))*C8, 0)</f>
+        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 4'!$M$3:$M$126, 'Game Log Season 4'!$C$3:$C$126, "Michelle", 'Game Log Season 4'!$F$3:$F$126, 1)-0.5))*C8, 0)</f>
         <v>0</v>
       </c>
       <c r="K8" s="14" t="n">
-        <f aca="false">IFERROR((1+(AVERAGEIFS('Game Log Season 3'!$M$3:$M$126, 'Game Log Season 3'!$C$3:$C$126, "Michelle", 'Game Log Season 3'!$F$3:$F$126, 0)-0.5))*D8, 0)</f>
+        <f aca="false">IFERROR((1+(AVERAGEIFS('Game Log Season 4'!$M$3:$M$126, 'Game Log Season 4'!$C$3:$C$126, "Michelle", 'Game Log Season 4'!$F$3:$F$126, 0)-0.5))*D8, 0)</f>
         <v>3.7465</v>
       </c>
       <c r="L8" s="17" t="n">
@@ -28036,11 +28037,11 @@
         <v>0</v>
       </c>
       <c r="C9" s="14" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$126, "Red", 'Game Log Season 3'!$F$3:$F$126, 1)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$126, "Red", 'Game Log Season 4'!$F$3:$F$126, 1)</f>
         <v>0</v>
       </c>
       <c r="D9" s="14" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$126, "Red", 'Game Log Season 3'!$F$3:$F$126, 0)</f>
+        <f aca="false">COUNTIFS('Game Log Season 4'!$C$3:$C$126, "Red", 'Game Log Season 4'!$F$3:$F$126, 0)</f>
         <v>0</v>
       </c>
       <c r="E9" s="17" t="n">
@@ -28048,11 +28049,11 @@
         <v>0</v>
       </c>
       <c r="F9" s="14" t="n">
-        <f aca="false">SUMIFS('Game Log Season 3'!$J$3:$J$126, 'Game Log Season 3'!$C$3:$C$126, "Red", 'Game Log Season 3'!$F$3:$F$126, 1)</f>
+        <f aca="false">SUMIFS('Game Log Season 4'!$J$3:$J$126, 'Game Log Season 4'!$C$3:$C$126, "Red", 'Game Log Season 4'!$F$3:$F$126, 1)</f>
         <v>0</v>
       </c>
       <c r="G9" s="14" t="n">
-        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 3'!$J$3:$J$126, 'Game Log Season 3'!$C$3:$C$126, "Red", 'Game Log Season 3'!$F$3:$F$126, 0)*-1))*D9,0)</f>
+        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 4'!$J$3:$J$126, 'Game Log Season 4'!$C$3:$C$126, "Red", 'Game Log Season 4'!$F$3:$F$126, 0)*-1))*D9,0)</f>
         <v>0</v>
       </c>
       <c r="H9" s="17" t="n">
@@ -28060,15 +28061,15 @@
         <v>0</v>
       </c>
       <c r="I9" s="17" t="n">
-        <f aca="false">IF(C9&lt;&gt;0,AVERAGEIF('Game Log Season 3'!$C$3:$C$126, "Red", 'Game Log Season 3'!$K$3:$K$126),0)</f>
+        <f aca="false">IF(C9&lt;&gt;0,AVERAGEIF('Game Log Season 4'!$C$3:$C$126, "Red", 'Game Log Season 4'!$K$3:$K$126),0)</f>
         <v>0</v>
       </c>
       <c r="J9" s="14" t="n">
-        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 3'!$M$3:$M$126, 'Game Log Season 3'!$C$3:$C$126, "Red", 'Game Log Season 3'!$F$3:$F$126, 1)-0.5))*C9, 0)</f>
+        <f aca="false">IFERROR((1-(AVERAGEIFS('Game Log Season 4'!$M$3:$M$126, 'Game Log Season 4'!$C$3:$C$126, "Red", 'Game Log Season 4'!$F$3:$F$126, 1)-0.5))*C9, 0)</f>
         <v>0</v>
       </c>
       <c r="K9" s="14" t="n">
-        <f aca="false">IFERROR((1+(AVERAGEIFS('Game Log Season 3'!$M$3:$M$126, 'Game Log Season 3'!$C$3:$C$126, "Red", 'Game Log Season 3'!$F$3:$F$126, 0)-0.5))*D9, 0)</f>
+        <f aca="false">IFERROR((1+(AVERAGEIFS('Game Log Season 4'!$M$3:$M$126, 'Game Log Season 4'!$C$3:$C$126, "Red", 'Game Log Season 4'!$F$3:$F$126, 0)-0.5))*D9, 0)</f>
         <v>0</v>
       </c>
       <c r="L9" s="17" t="n">
@@ -28085,4 +28086,162 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:X2"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="48.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="21.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="9.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="28.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="11" style="0" width="32.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="29.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="0" width="20.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="17" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="10.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="20" style="0" width="19.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="22" style="0" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="26.78"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
+      <c r="N1" s="3"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="W1" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="X1" s="6"/>
+    </row>
+    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="L2" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="M2" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="N2" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="O2" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="P2" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q2" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="R2" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="S2" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="T2" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="U2" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="V2" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="W2" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="X2" s="12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:X34"/>
+  <mergeCells count="4">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="P1:Q1"/>
+    <mergeCell ref="S1:U1"/>
+    <mergeCell ref="W1:X1"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
test: Phase 2 dry run (add_player.py + add_deck.py with column E) -- to be reverted
</commit_message>
<xml_diff>
--- a/deck-strength.xlsx
+++ b/deck-strength.xlsx
@@ -25781,7 +25781,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40.33"/>
@@ -25810,7 +25810,7 @@
         <v>26</v>
       </c>
       <c r="B2" s="48" t="n">
-        <f aca="false">AVERAGE(B3:B6)</f>
+        <f aca="false">AVERAGE(B3:B7)</f>
         <v>2.72288194444444</v>
       </c>
       <c r="C2" s="46"/>
@@ -25878,864 +25878,932 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="47" t="s">
+    <row r="7" spans="1:5">
+      <c r="A7" s="49" t="inlineStr">
+        <is>
+          <t>ZZ Test Deck With ID</t>
+        </is>
+      </c>
+      <c r="B7" s="49">
+        <f>IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Becca")*('Game Log Season 3'!$D$3:$D$1000=A7)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D7)</f>
+        <v>2.9</v>
+      </c>
+      <c r="C7" s="46"/>
+      <c r="D7" s="49">
+        <v>2.9</v>
+      </c>
+      <c r="E7" s="47" t="inlineStr">
+        <is>
+          <t>999002</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="48" t="n">
-        <f aca="false">AVERAGE(B8:B17)</f>
+      <c r="B8" s="48" t="n">
+        <f aca="false">AVERAGE(B9:B18)</f>
         <v>3.28381944444444</v>
       </c>
-      <c r="C7" s="46"/>
-    </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="49" t="s">
-        <v>68</v>
-      </c>
-      <c r="B8" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A8)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D8)</f>
-        <v>3.83916666666667</v>
-      </c>
       <c r="C8" s="46"/>
-      <c r="D8" s="49" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="E8" s="47" t="s">
-        <v>106</v>
-      </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="49" t="s">
-        <v>42</v>
+        <v>68</v>
       </c>
       <c r="B9" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A9)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D9)</f>
-        <v>3.9</v>
+        <v>3.83916666666667</v>
       </c>
       <c r="C9" s="46"/>
       <c r="D9" s="49" t="n">
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
       <c r="E9" s="47" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="49" t="s">
-        <v>67</v>
+        <v>42</v>
       </c>
       <c r="B10" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A10)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D10)</f>
-        <v>3.4</v>
-      </c>
-      <c r="C10" s="46" t="s">
-        <v>108</v>
-      </c>
+        <v>3.9</v>
+      </c>
+      <c r="C10" s="46"/>
       <c r="D10" s="49" t="n">
-        <v>3.4</v>
+        <v>3.9</v>
       </c>
       <c r="E10" s="47" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="49" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="B11" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A11)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D11)</f>
-        <v>2.6</v>
-      </c>
-      <c r="C11" s="46"/>
+        <v>3.4</v>
+      </c>
+      <c r="C11" s="46" t="s">
+        <v>108</v>
+      </c>
       <c r="D11" s="49" t="n">
-        <v>2.6</v>
+        <v>3.4</v>
       </c>
       <c r="E11" s="47" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="49" t="s">
-        <v>44</v>
+        <v>82</v>
       </c>
       <c r="B12" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A12)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D12)</f>
-        <v>3.5</v>
-      </c>
-      <c r="C12" s="46" t="s">
-        <v>103</v>
-      </c>
+        <v>2.6</v>
+      </c>
+      <c r="C12" s="46"/>
       <c r="D12" s="49" t="n">
-        <v>3.5</v>
+        <v>2.6</v>
       </c>
       <c r="E12" s="47" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="49" t="s">
-        <v>88</v>
+        <v>44</v>
       </c>
       <c r="B13" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A13)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D13)</f>
-        <v>2.65388888888889</v>
-      </c>
-      <c r="C13" s="46"/>
+        <v>3.5</v>
+      </c>
+      <c r="C13" s="46" t="s">
+        <v>103</v>
+      </c>
       <c r="D13" s="49" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="E13" s="47" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="49" t="s">
-        <v>48</v>
+        <v>88</v>
       </c>
       <c r="B14" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A14)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D14)</f>
-        <v>2.6</v>
+        <v>2.65388888888889</v>
       </c>
       <c r="C14" s="46"/>
       <c r="D14" s="49" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="E14" s="47" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="49" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="B15" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A15)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D15)</f>
-        <v>3.91083333333333</v>
+        <v>2.6</v>
       </c>
       <c r="C15" s="46"/>
       <c r="D15" s="49" t="n">
-        <v>3.9</v>
+        <v>2.6</v>
       </c>
       <c r="E15" s="47" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="49" t="s">
-        <v>91</v>
+        <v>37</v>
       </c>
       <c r="B16" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A16)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D16)</f>
-        <v>2.94083333333333</v>
+        <v>3.91083333333333</v>
       </c>
       <c r="C16" s="46"/>
       <c r="D16" s="49" t="n">
-        <v>2.3</v>
+        <v>3.9</v>
       </c>
       <c r="E16" s="47" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="49" t="s">
-        <v>47</v>
+        <v>91</v>
       </c>
       <c r="B17" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A17)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D17)</f>
-        <v>3.49347222222222</v>
+        <v>2.94083333333333</v>
       </c>
       <c r="C17" s="46"/>
       <c r="D17" s="49" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E17" s="47" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="49" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A18)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D18)</f>
+        <v>3.49347222222222</v>
+      </c>
+      <c r="C18" s="46"/>
+      <c r="D18" s="49" t="n">
         <v>3.5</v>
       </c>
-      <c r="E17" s="47" t="s">
+      <c r="E18" s="47" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="47" t="s">
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="47" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="48" t="n">
-        <f aca="false">AVERAGE(B19:B32)</f>
+      <c r="B19" s="48" t="n">
+        <f aca="false">AVERAGE(B20:B33)</f>
         <v>3.31464285714286</v>
       </c>
-      <c r="C18" s="46"/>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="49" t="s">
-        <v>73</v>
-      </c>
-      <c r="B19" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A19)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D19)</f>
-        <v>2.4</v>
-      </c>
       <c r="C19" s="46"/>
-      <c r="D19" s="49" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="E19" s="47" t="s">
-        <v>117</v>
-      </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="49" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B20" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A20)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D20)</f>
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="C20" s="46"/>
       <c r="D20" s="49" t="n">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="E20" s="47" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="49" t="s">
-        <v>31</v>
+        <v>66</v>
       </c>
       <c r="B21" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A21)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D21)</f>
-        <v>3.57402777777778</v>
+        <v>2.6</v>
       </c>
       <c r="C21" s="46"/>
       <c r="D21" s="49" t="n">
-        <v>3.6</v>
+        <v>2.6</v>
       </c>
       <c r="E21" s="47" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="49" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B22" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A22)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D22)</f>
-        <v>3.6</v>
+        <v>3.57402777777778</v>
       </c>
       <c r="C22" s="46"/>
       <c r="D22" s="49" t="n">
         <v>3.6</v>
       </c>
       <c r="E22" s="47" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="49" t="s">
-        <v>74</v>
+        <v>34</v>
       </c>
       <c r="B23" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A23)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D23)</f>
-        <v>2.9</v>
+        <v>3.6</v>
       </c>
       <c r="C23" s="46"/>
       <c r="D23" s="49" t="n">
-        <v>2.9</v>
+        <v>3.6</v>
       </c>
       <c r="E23" s="47" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="49" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="B24" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A24)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D24)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C24" s="46" t="s">
-        <v>103</v>
-      </c>
+        <v>2.9</v>
+      </c>
+      <c r="C24" s="46"/>
       <c r="D24" s="49" t="n">
-        <v>3.9</v>
+        <v>2.9</v>
       </c>
       <c r="E24" s="47" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="49" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
       <c r="B25" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A25)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D25)</f>
-        <v>2.8</v>
-      </c>
-      <c r="C25" s="46"/>
+        <v>3.9</v>
+      </c>
+      <c r="C25" s="46" t="s">
+        <v>103</v>
+      </c>
       <c r="D25" s="49" t="n">
-        <v>2.8</v>
+        <v>3.9</v>
+      </c>
+      <c r="E25" s="47" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="49" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B26" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A26)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D26)</f>
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="C26" s="46"/>
       <c r="D26" s="49" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="E26" s="47" t="s">
-        <v>123</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="49" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B27" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A27)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D27)</f>
-        <v>3.59875</v>
-      </c>
-      <c r="C27" s="46" t="s">
-        <v>124</v>
-      </c>
+        <v>2.6</v>
+      </c>
+      <c r="C27" s="46"/>
       <c r="D27" s="49" t="n">
-        <v>3.6</v>
+        <v>2.6</v>
       </c>
       <c r="E27" s="47" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="49" t="s">
-        <v>48</v>
+        <v>83</v>
       </c>
       <c r="B28" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A28)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D28)</f>
-        <v>3.94083333333333</v>
-      </c>
-      <c r="C28" s="46"/>
+        <v>3.59875</v>
+      </c>
+      <c r="C28" s="46" t="s">
+        <v>124</v>
+      </c>
       <c r="D28" s="49" t="n">
-        <v>3.9</v>
+        <v>3.6</v>
       </c>
       <c r="E28" s="47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="49" t="s">
-        <v>90</v>
+        <v>48</v>
       </c>
       <c r="B29" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A29)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D29)</f>
-        <v>3.65388888888889</v>
+        <v>3.94083333333333</v>
       </c>
       <c r="C29" s="46"/>
       <c r="D29" s="49" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="E29" s="47" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="49" t="s">
-        <v>46</v>
-      </c>
-      <c r="B30" s="50" t="n">
+        <v>90</v>
+      </c>
+      <c r="B30" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A30)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D30)</f>
-        <v>3.95583333333333</v>
+        <v>3.65388888888889</v>
       </c>
       <c r="C30" s="46"/>
-      <c r="D30" s="50" t="n">
-        <v>4</v>
+      <c r="D30" s="49" t="n">
+        <v>3.7</v>
       </c>
       <c r="E30" s="47" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="49" t="s">
-        <v>92</v>
+        <v>46</v>
       </c>
       <c r="B31" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A31)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D31)</f>
-        <v>2.94666666666667</v>
+        <v>3.95583333333333</v>
       </c>
       <c r="C31" s="46"/>
       <c r="D31" s="50" t="n">
-        <v>2.9</v>
+        <v>4</v>
       </c>
       <c r="E31" s="47" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="49" t="s">
-        <v>40</v>
+        <v>92</v>
       </c>
       <c r="B32" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A32)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D32)</f>
+        <v>2.94666666666667</v>
+      </c>
+      <c r="C32" s="46"/>
+      <c r="D32" s="50" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="E32" s="47" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="49" t="s">
+        <v>40</v>
+      </c>
+      <c r="B33" s="50" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A33)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D33)</f>
         <v>3.935</v>
       </c>
-      <c r="C32" s="46" t="s">
+      <c r="C33" s="46" t="s">
         <v>130</v>
       </c>
-      <c r="D32" s="50" t="n">
+      <c r="D33" s="50" t="n">
         <v>3.9</v>
       </c>
-      <c r="E32" s="47" t="s">
+      <c r="E33" s="47" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="47" t="s">
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="47" t="s">
         <v>32</v>
       </c>
-      <c r="B33" s="48" t="n">
-        <f aca="false">AVERAGE(B34:B44)</f>
+      <c r="B34" s="48" t="n">
+        <f aca="false">AVERAGE(B35:B45)</f>
         <v>3.26275505050505</v>
       </c>
-      <c r="C33" s="46"/>
-    </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="49" t="s">
-        <v>36</v>
-      </c>
-      <c r="B34" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A34)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D34)</f>
-        <v>3.5</v>
-      </c>
       <c r="C34" s="46"/>
-      <c r="D34" s="49" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="E34" s="47" t="s">
-        <v>132</v>
-      </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="49" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="B35" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A35)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D35)</f>
-        <v>3.43088888888889</v>
+        <v>3.5</v>
       </c>
       <c r="C35" s="46"/>
       <c r="D35" s="49" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="E35" s="47" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="49" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="B36" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A36)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D36)</f>
-        <v>3.7</v>
+        <v>3.43088888888889</v>
       </c>
       <c r="C36" s="46"/>
       <c r="D36" s="49" t="n">
-        <v>3.7</v>
+        <v>3.4</v>
       </c>
       <c r="E36" s="47" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="49" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="B37" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A37)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D37)</f>
-        <v>2.6</v>
+        <v>3.7</v>
       </c>
       <c r="C37" s="46"/>
       <c r="D37" s="49" t="n">
-        <v>2.6</v>
+        <v>3.7</v>
       </c>
       <c r="E37" s="47" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="49" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="B38" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A38)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D38)</f>
-        <v>3.77816666666667</v>
+        <v>2.6</v>
       </c>
       <c r="C38" s="46"/>
       <c r="D38" s="49" t="n">
-        <v>3.8</v>
+        <v>2.6</v>
       </c>
       <c r="E38" s="47" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="49" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="B39" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A39)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D39)</f>
-        <v>2.59388888888889</v>
+        <v>3.77816666666667</v>
       </c>
       <c r="C39" s="46"/>
       <c r="D39" s="49" t="n">
-        <v>2.6</v>
+        <v>3.8</v>
       </c>
       <c r="E39" s="47" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="49" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="B40" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A40)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D40)</f>
-        <v>3.23902777777778</v>
+        <v>2.59388888888889</v>
       </c>
       <c r="C40" s="46"/>
       <c r="D40" s="49" t="n">
-        <v>3.6</v>
+        <v>2.6</v>
       </c>
       <c r="E40" s="47" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="49" t="s">
-        <v>87</v>
+        <v>54</v>
       </c>
       <c r="B41" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A41)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D41)</f>
-        <v>2.6</v>
+        <v>3.23902777777778</v>
       </c>
       <c r="C41" s="46"/>
       <c r="D41" s="49" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="E41" s="47" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="49" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B42" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A42)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D42)</f>
-        <v>3.58416666666667</v>
+        <v>2.6</v>
       </c>
       <c r="C42" s="46"/>
       <c r="D42" s="49" t="n">
-        <v>3.6</v>
+        <v>2.6</v>
+      </c>
+      <c r="E42" s="47" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="49" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B43" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A43)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D43)</f>
-        <v>2.94083333333333</v>
+        <v>3.58416666666667</v>
       </c>
       <c r="C43" s="46"/>
       <c r="D43" s="49" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="E43" s="47" t="s">
-        <v>140</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="49" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B44" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A44)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D44)</f>
-        <v>3.92333333333333</v>
+        <v>2.94083333333333</v>
       </c>
       <c r="C44" s="46"/>
       <c r="D44" s="49" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="E44" s="47" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="49" t="s">
+        <v>97</v>
+      </c>
+      <c r="B45" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A45)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D45)</f>
+        <v>3.92333333333333</v>
+      </c>
+      <c r="C45" s="46"/>
+      <c r="D45" s="49" t="n">
         <v>3.9</v>
       </c>
-      <c r="E44" s="47" t="s">
+      <c r="E45" s="47" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="47" t="s">
+    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="47" t="s">
         <v>70</v>
       </c>
-      <c r="B45" s="48" t="n">
-        <f aca="false">AVERAGE(B46:B50)</f>
+      <c r="B46" s="48" t="n">
+        <f aca="false">AVERAGE(B47:B51)</f>
         <v>3.2865</v>
       </c>
-      <c r="C45" s="46"/>
-    </row>
-    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="49" t="s">
-        <v>71</v>
-      </c>
-      <c r="B46" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A46)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D46)</f>
-        <v>3.6</v>
-      </c>
-      <c r="C46" s="46" t="s">
-        <v>124</v>
-      </c>
-      <c r="D46" s="49" t="n">
-        <v>3.6</v>
-      </c>
+      <c r="C46" s="46"/>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="49" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B47" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A47)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D47)</f>
-        <v>3.33761111111111</v>
+        <v>3.6</v>
       </c>
       <c r="C47" s="46" t="s">
         <v>124</v>
       </c>
       <c r="D47" s="49" t="n">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="49" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="B48" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A48)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D48)</f>
-        <v>3.2</v>
-      </c>
-      <c r="C48" s="46"/>
+        <v>3.33761111111111</v>
+      </c>
+      <c r="C48" s="46" t="s">
+        <v>124</v>
+      </c>
       <c r="D48" s="49" t="n">
-        <v>3.2</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="49" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B49" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A49)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D49)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C49" s="46" t="s">
-        <v>130</v>
-      </c>
+        <v>3.2</v>
+      </c>
+      <c r="C49" s="46"/>
       <c r="D49" s="49" t="n">
-        <v>3.9</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="49" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="B50" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A50)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D50)</f>
+        <v>3.9</v>
+      </c>
+      <c r="C50" s="46" t="s">
+        <v>130</v>
+      </c>
+      <c r="D50" s="49" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="49" t="s">
+        <v>93</v>
+      </c>
+      <c r="B51" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A51)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D51)</f>
         <v>2.39488888888889</v>
       </c>
-      <c r="C50" s="46"/>
-      <c r="D50" s="49" t="n">
+      <c r="C51" s="46"/>
+      <c r="D51" s="49" t="n">
         <v>2.4</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="47" t="s">
+    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="47" t="s">
         <v>38</v>
       </c>
-      <c r="B51" s="48" t="n">
-        <f aca="false">AVERAGE(B52:B56)</f>
+      <c r="B52" s="48" t="n">
+        <f aca="false">AVERAGE(B53:B57)</f>
         <v>3.42807</v>
       </c>
-      <c r="C51" s="46"/>
-    </row>
-    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="49" t="s">
-        <v>49</v>
-      </c>
-      <c r="B52" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A52)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D52)</f>
-        <v>3.6</v>
-      </c>
       <c r="C52" s="46"/>
-      <c r="D52" s="49" t="n">
-        <v>3.6</v>
-      </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="49" t="s">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="B53" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A53)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D53)</f>
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
       <c r="C53" s="46"/>
       <c r="D53" s="49" t="n">
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="49" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B54" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A54)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D54)</f>
-        <v>2.7</v>
+        <v>3.8</v>
       </c>
       <c r="C54" s="46"/>
       <c r="D54" s="49" t="n">
-        <v>2.7</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="49" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="B55" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A55)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D55)</f>
-        <v>3.3</v>
+        <v>2.7</v>
       </c>
       <c r="C55" s="46"/>
       <c r="D55" s="49" t="n">
-        <v>3.3</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="49" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B56" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A56)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D56)</f>
-        <v>3.74035</v>
+        <v>3.3</v>
       </c>
       <c r="C56" s="46"/>
       <c r="D56" s="49" t="n">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="49" t="s">
+        <v>63</v>
+      </c>
+      <c r="B57" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A57)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D57)</f>
+        <v>3.74035</v>
+      </c>
+      <c r="C57" s="46"/>
+      <c r="D57" s="49" t="n">
         <v>3.7</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="47" t="s">
+    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="47" t="s">
         <v>59</v>
       </c>
-      <c r="B57" s="48" t="n">
-        <f aca="false">AVERAGE(B58:B59)</f>
+      <c r="B58" s="48" t="n">
+        <f aca="false">AVERAGE(B59:B60)</f>
         <v>3.05</v>
       </c>
-      <c r="C57" s="46"/>
-    </row>
-    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="49" t="s">
-        <v>33</v>
-      </c>
-      <c r="B58" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A58)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D58)</f>
-        <v>2.7</v>
-      </c>
       <c r="C58" s="46"/>
-      <c r="D58" s="49" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="E58" s="47" t="s">
-        <v>142</v>
-      </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="49" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="B59" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A59)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D59)</f>
-        <v>3.4</v>
+        <v>2.7</v>
       </c>
       <c r="C59" s="46"/>
       <c r="D59" s="49" t="n">
-        <v>3.4</v>
+        <v>2.7</v>
       </c>
       <c r="E59" s="47" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="49" t="s">
+        <v>69</v>
+      </c>
+      <c r="B60" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A60)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D60)</f>
+        <v>3.4</v>
+      </c>
+      <c r="C60" s="46"/>
+      <c r="D60" s="49" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="E60" s="47" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="49" t="s">
         <v>84</v>
       </c>
-      <c r="B60" s="50" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A60)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D60)</f>
-        <v>1</v>
-      </c>
-      <c r="C60" s="46"/>
-      <c r="D60" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E60" s="47" t="s">
+      <c r="B61" s="50" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A61)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D61)</f>
+        <v>1</v>
+      </c>
+      <c r="C61" s="46"/>
+      <c r="D61" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" s="47" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="47" t="s">
+    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="47" t="s">
         <v>51</v>
       </c>
-      <c r="B61" s="48" t="n">
-        <f aca="false">AVERAGE(B62:B63)</f>
+      <c r="B62" s="48" t="n">
+        <f aca="false">AVERAGE(B63:B64)</f>
         <v>2.25194444444444</v>
       </c>
-      <c r="C61" s="46"/>
-    </row>
-    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="49" t="s">
-        <v>52</v>
-      </c>
-      <c r="B62" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A62)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D62)</f>
-        <v>2.30388888888889</v>
-      </c>
       <c r="C62" s="46"/>
-      <c r="D62" s="49" t="n">
-        <v>2.5</v>
-      </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="49" t="s">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="B63" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A63)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D63)</f>
-        <v>2.2</v>
+        <v>2.30388888888889</v>
       </c>
       <c r="C63" s="46"/>
       <c r="D63" s="49" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="E63" s="47" t="s">
-        <v>145</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="49" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="B64" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A64)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D64)</f>
+        <v>2.2</v>
+      </c>
+      <c r="C64" s="46"/>
+      <c r="D64" s="49" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E64" s="47" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="49" t="s">
+        <v>96</v>
+      </c>
+      <c r="B65" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A65)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D65)</f>
         <v>2.43069444444444</v>
       </c>
-      <c r="D64" s="49" t="n">
+      <c r="D65" s="49" t="n">
         <v>2.4</v>
       </c>
+    </row>
+    <row r="66" spans="1:5">
+      <c r="A66" s="47" t="inlineStr">
+        <is>
+          <t>ZZTestPlayer2</t>
+        </is>
+      </c>
+      <c r="B66" s="48">
+        <f>AVERAGE(B67:B68)</f>
+        <v>2.85</v>
+      </c>
+      <c r="C66" s="46"/>
+    </row>
+    <row r="67" spans="1:5">
+      <c r="A67" s="49" t="inlineStr">
+        <is>
+          <t>Test Commander A</t>
+        </is>
+      </c>
+      <c r="B67" s="49">
+        <f>IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="ZZTestPlayer2")*('Game Log Season 3'!$D$3:$D$1000=A67)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D67)</f>
+        <v>3</v>
+      </c>
+      <c r="C67" s="46"/>
+      <c r="D67" s="49">
+        <v>3</v>
+      </c>
+      <c r="E67" s="47" t="inlineStr">
+        <is>
+          <t>999001</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" spans="1:5">
+      <c r="A68" s="49" t="inlineStr">
+        <is>
+          <t>Test Commander B</t>
+        </is>
+      </c>
+      <c r="B68" s="49">
+        <f>IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="ZZTestPlayer2")*('Game Log Season 3'!$D$3:$D$1000=A68)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D68)</f>
+        <v>2.7</v>
+      </c>
+      <c r="C68" s="46"/>
+      <c r="D68" s="49">
+        <v>2.7</v>
+      </c>
+      <c r="E68" s="47"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -26753,7 +26821,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D68"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.89"/>
@@ -26861,60 +26929,62 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="47" t="s">
+    <row r="7" spans="1:4">
+      <c r="A7" s="49" t="inlineStr">
+        <is>
+          <t>ZZ Test Deck With ID</t>
+        </is>
+      </c>
+      <c r="B7" s="49">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A7)</f>
+        <v>0</v>
+      </c>
+      <c r="C7" s="49">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A7,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D7" s="49">
+        <f>IFERROR(C7/B7,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A7)</f>
+      <c r="B8" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A8)</f>
         <v>14</v>
       </c>
-      <c r="C7" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A7,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+      <c r="C8" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A8,'Game Log Season 3'!$F$3:$F$1000,1)</f>
         <v>4</v>
       </c>
-      <c r="D7" s="48" t="n">
-        <f aca="false">IFERROR(C7/B7,0)</f>
+      <c r="D8" s="48" t="n">
+        <f aca="false">IFERROR(C8/B8,0)</f>
         <v>0.285714285714286</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="49" t="s">
-        <v>68</v>
-      </c>
-      <c r="B8" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A8)</f>
-        <v>4</v>
-      </c>
-      <c r="C8" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A8,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>2</v>
-      </c>
-      <c r="D8" s="49" t="n">
-        <f aca="false">IFERROR(C8/B8,0)</f>
-        <v>0.5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="49" t="s">
-        <v>42</v>
+        <v>68</v>
       </c>
       <c r="B9" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A9)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C9" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A9,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D9" s="49" t="n">
         <f aca="false">IFERROR(C9/B9,0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="49" t="s">
-        <v>67</v>
+        <v>42</v>
       </c>
       <c r="B10" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A10)</f>
@@ -26931,7 +27001,7 @@
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="49" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="B11" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A11)</f>
@@ -26948,7 +27018,7 @@
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="49" t="s">
-        <v>44</v>
+        <v>82</v>
       </c>
       <c r="B12" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A12)</f>
@@ -26965,11 +27035,11 @@
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="49" t="s">
-        <v>88</v>
+        <v>44</v>
       </c>
       <c r="B13" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A13)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C13" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A13,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -26982,11 +27052,11 @@
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="49" t="s">
-        <v>48</v>
+        <v>88</v>
       </c>
       <c r="B14" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A14)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C14" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A14,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -26999,28 +27069,28 @@
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="49" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="B15" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A15)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C15" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A15,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" s="49" t="n">
         <f aca="false">IFERROR(C15/B15,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="49" t="s">
-        <v>91</v>
+        <v>37</v>
       </c>
       <c r="B16" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A16)</f>
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C16" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A16,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27028,63 +27098,63 @@
       </c>
       <c r="D16" s="49" t="n">
         <f aca="false">IFERROR(C16/B16,0)</f>
-        <v>0.166666666666667</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="49" t="s">
-        <v>47</v>
+        <v>91</v>
       </c>
       <c r="B17" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A17)</f>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C17" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A17,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" s="49" t="n">
         <f aca="false">IFERROR(C17/B17,0)</f>
-        <v>0</v>
+        <v>0.166666666666667</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="47" t="s">
+      <c r="A18" s="49" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A18)</f>
+        <v>1</v>
+      </c>
+      <c r="C18" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A18,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="49" t="n">
+        <f aca="false">IFERROR(C18/B18,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="47" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A18)</f>
+      <c r="B19" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A19)</f>
         <v>12</v>
       </c>
-      <c r="C18" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A18,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+      <c r="C19" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A19,'Game Log Season 3'!$F$3:$F$1000,1)</f>
         <v>5</v>
       </c>
-      <c r="D18" s="48" t="n">
-        <f aca="false">IFERROR(C18/B18,0)</f>
+      <c r="D19" s="48" t="n">
+        <f aca="false">IFERROR(C19/B19,0)</f>
         <v>0.416666666666667</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="49" t="s">
-        <v>73</v>
-      </c>
-      <c r="B19" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A19)</f>
-        <v>0</v>
-      </c>
-      <c r="C19" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A19,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D19" s="49" t="n">
-        <f aca="false">IFERROR(C19/B19,0)</f>
-        <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="49" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B20" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A20)</f>
@@ -27101,11 +27171,11 @@
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="49" t="s">
-        <v>31</v>
+        <v>66</v>
       </c>
       <c r="B21" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A21)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C21" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A21,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27118,11 +27188,11 @@
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="49" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B22" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A22)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C22" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A22,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27135,7 +27205,7 @@
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="49" t="s">
-        <v>74</v>
+        <v>34</v>
       </c>
       <c r="B23" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A23)</f>
@@ -27152,7 +27222,7 @@
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="49" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="B24" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A24)</f>
@@ -27169,7 +27239,7 @@
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="49" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
       <c r="B25" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A25)</f>
@@ -27186,7 +27256,7 @@
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="49" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B26" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A26)</f>
@@ -27203,11 +27273,11 @@
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="49" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B27" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A27)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C27" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A27,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27220,7 +27290,7 @@
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="49" t="s">
-        <v>48</v>
+        <v>83</v>
       </c>
       <c r="B28" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A28)</f>
@@ -27228,122 +27298,122 @@
       </c>
       <c r="C28" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A28,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D28" s="49" t="n">
         <f aca="false">IFERROR(C28/B28,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="49" t="s">
-        <v>90</v>
+        <v>48</v>
       </c>
       <c r="B29" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A29)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C29" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A29,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D29" s="49" t="n">
         <f aca="false">IFERROR(C29/B29,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="49" t="s">
-        <v>46</v>
+        <v>90</v>
       </c>
       <c r="B30" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A30)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C30" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A30,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D30" s="49" t="n">
         <f aca="false">IFERROR(C30/B30,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="49" t="s">
-        <v>92</v>
+        <v>46</v>
       </c>
       <c r="B31" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A31)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C31" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A31,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D31" s="49" t="n">
         <f aca="false">IFERROR(C31/B31,0)</f>
-        <v>0.666666666666667</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="49" t="s">
-        <v>40</v>
+        <v>92</v>
       </c>
       <c r="B32" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A32)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C32" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A32,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" s="49" t="n">
         <f aca="false">IFERROR(C32/B32,0)</f>
-        <v>1</v>
+        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="47" t="s">
+      <c r="A33" s="49" t="s">
+        <v>40</v>
+      </c>
+      <c r="B33" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A33)</f>
+        <v>1</v>
+      </c>
+      <c r="C33" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A33,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>1</v>
+      </c>
+      <c r="D33" s="49" t="n">
+        <f aca="false">IFERROR(C33/B33,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="47" t="s">
         <v>32</v>
       </c>
-      <c r="B33" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A33)</f>
+      <c r="B34" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A34)</f>
         <v>11</v>
       </c>
-      <c r="C33" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A33,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>3</v>
-      </c>
-      <c r="D33" s="48" t="n">
-        <f aca="false">IFERROR(C33/B33,0)</f>
+      <c r="C34" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A34,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>3</v>
+      </c>
+      <c r="D34" s="48" t="n">
+        <f aca="false">IFERROR(C34/B34,0)</f>
         <v>0.272727272727273</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="49" t="s">
-        <v>36</v>
-      </c>
-      <c r="B34" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A34)</f>
-        <v>0</v>
-      </c>
-      <c r="C34" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A34,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D34" s="49" t="n">
-        <f aca="false">IFERROR(C34/B34,0)</f>
-        <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="49" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="B35" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A35)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C35" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A35,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27356,11 +27426,11 @@
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="49" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="B36" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A36)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C36" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A36,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27373,7 +27443,7 @@
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="49" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="B37" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A37)</f>
@@ -27390,24 +27460,24 @@
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="49" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="B38" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A38)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C38" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A38,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D38" s="49" t="n">
         <f aca="false">IFERROR(C38/B38,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="49" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="B39" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A39)</f>
@@ -27415,20 +27485,20 @@
       </c>
       <c r="C39" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A39,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D39" s="49" t="n">
         <f aca="false">IFERROR(C39/B39,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="49" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="B40" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A40)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C40" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A40,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27441,11 +27511,11 @@
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="49" t="s">
-        <v>87</v>
+        <v>54</v>
       </c>
       <c r="B41" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A41)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C41" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A41,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27458,11 +27528,11 @@
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="49" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B42" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A42)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C42" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A42,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27475,7 +27545,7 @@
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="49" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B43" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A43)</f>
@@ -27483,16 +27553,16 @@
       </c>
       <c r="C43" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A43,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D43" s="49" t="n">
         <f aca="false">IFERROR(C43/B43,0)</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="49" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B44" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A44)</f>
@@ -27508,46 +27578,46 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="47" t="s">
+      <c r="A45" s="49" t="s">
+        <v>97</v>
+      </c>
+      <c r="B45" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A45)</f>
+        <v>2</v>
+      </c>
+      <c r="C45" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A45,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>1</v>
+      </c>
+      <c r="D45" s="49" t="n">
+        <f aca="false">IFERROR(C45/B45,0)</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="47" t="s">
         <v>70</v>
       </c>
-      <c r="B45" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A45)</f>
-        <v>2</v>
-      </c>
-      <c r="C45" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A45,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D45" s="48" t="n">
-        <f aca="false">IFERROR(C45/B45,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="49" t="s">
-        <v>71</v>
-      </c>
-      <c r="B46" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A46)</f>
-        <v>0</v>
-      </c>
-      <c r="C46" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A46,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D46" s="49" t="n">
+      <c r="B46" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A46)</f>
+        <v>2</v>
+      </c>
+      <c r="C46" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A46,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D46" s="48" t="n">
         <f aca="false">IFERROR(C46/B46,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="49" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B47" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A47)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C47" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A47,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27560,11 +27630,11 @@
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="49" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="B48" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A48)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C48" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A48,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27577,7 +27647,7 @@
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="49" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B49" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A49)</f>
@@ -27594,11 +27664,11 @@
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="49" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="B50" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A50)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C50" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A50,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27610,42 +27680,42 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="47" t="s">
+      <c r="A51" s="49" t="s">
+        <v>93</v>
+      </c>
+      <c r="B51" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A51)</f>
+        <v>1</v>
+      </c>
+      <c r="C51" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A51,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D51" s="49" t="n">
+        <f aca="false">IFERROR(C51/B51,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="47" t="s">
         <v>38</v>
       </c>
-      <c r="B51" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A51)</f>
-        <v>1</v>
-      </c>
-      <c r="C51" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A51,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D51" s="48" t="n">
-        <f aca="false">IFERROR(C51/B51,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="49" t="s">
-        <v>49</v>
-      </c>
-      <c r="B52" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A52)</f>
-        <v>0</v>
-      </c>
-      <c r="C52" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A52,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D52" s="49" t="n">
+      <c r="B52" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A52)</f>
+        <v>1</v>
+      </c>
+      <c r="C52" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A52,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D52" s="48" t="n">
         <f aca="false">IFERROR(C52/B52,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="49" t="s">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="B53" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A53)</f>
@@ -27662,7 +27732,7 @@
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="49" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B54" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A54)</f>
@@ -27679,7 +27749,7 @@
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="49" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="B55" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A55)</f>
@@ -27696,11 +27766,11 @@
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="49" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B56" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A56)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C56" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A56,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27712,42 +27782,42 @@
       </c>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="47" t="s">
+      <c r="A57" s="49" t="s">
+        <v>63</v>
+      </c>
+      <c r="B57" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A57)</f>
+        <v>1</v>
+      </c>
+      <c r="C57" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A57,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D57" s="49" t="n">
+        <f aca="false">IFERROR(C57/B57,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="47" t="s">
         <v>59</v>
       </c>
-      <c r="B57" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A57)</f>
-        <v>0</v>
-      </c>
-      <c r="C57" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A57,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D57" s="48" t="n">
-        <f aca="false">IFERROR(C57/B57,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="49" t="s">
-        <v>33</v>
-      </c>
-      <c r="B58" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A58)</f>
-        <v>0</v>
-      </c>
-      <c r="C58" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A58,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D58" s="49" t="n">
+      <c r="B58" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A58)</f>
+        <v>0</v>
+      </c>
+      <c r="C58" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A58,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D58" s="48" t="n">
         <f aca="false">IFERROR(C58/B58,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="49" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="B59" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A59)</f>
@@ -27764,7 +27834,7 @@
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="49" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="B60" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A60)</f>
@@ -27780,46 +27850,46 @@
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="47" t="s">
+      <c r="A61" s="49" t="s">
+        <v>84</v>
+      </c>
+      <c r="B61" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A61)</f>
+        <v>0</v>
+      </c>
+      <c r="C61" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A61,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D61" s="49" t="n">
+        <f aca="false">IFERROR(C61/B61,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="47" t="s">
         <v>51</v>
       </c>
-      <c r="B61" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A61)</f>
+      <c r="B62" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A62)</f>
         <v>4</v>
       </c>
-      <c r="C61" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A61,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D61" s="48" t="n">
-        <f aca="false">IFERROR(C61/B61,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="49" t="s">
-        <v>52</v>
-      </c>
-      <c r="B62" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A62)</f>
-        <v>3</v>
-      </c>
-      <c r="C62" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A62,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D62" s="49" t="n">
+      <c r="C62" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A62,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D62" s="48" t="n">
         <f aca="false">IFERROR(C62/B62,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="49" t="s">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="B63" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A63)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C63" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A63,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27832,11 +27902,11 @@
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="49" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="B64" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A64)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C64" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A64,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27844,6 +27914,80 @@
       </c>
       <c r="D64" s="49" t="n">
         <f aca="false">IFERROR(C64/B64,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="49" t="s">
+        <v>96</v>
+      </c>
+      <c r="B65" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A65)</f>
+        <v>1</v>
+      </c>
+      <c r="C65" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A65,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D65" s="49" t="n">
+        <f aca="false">IFERROR(C65/B65,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66" s="47" t="inlineStr">
+        <is>
+          <t>ZZTestPlayer2</t>
+        </is>
+      </c>
+      <c r="B66" s="48">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A66)</f>
+        <v>0</v>
+      </c>
+      <c r="C66" s="48">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A66,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D66" s="48">
+        <f>IFERROR(C66/B66,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
+      <c r="A67" s="49" t="inlineStr">
+        <is>
+          <t>Test Commander A</t>
+        </is>
+      </c>
+      <c r="B67" s="49">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"ZZTestPlayer2",'Game Log Season 3'!$D$3:$D$1000,A67)</f>
+        <v>0</v>
+      </c>
+      <c r="C67" s="49">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"ZZTestPlayer2",'Game Log Season 3'!$D$3:$D$1000,A67,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D67" s="49">
+        <f>IFERROR(C67/B67,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4">
+      <c r="A68" s="49" t="inlineStr">
+        <is>
+          <t>Test Commander B</t>
+        </is>
+      </c>
+      <c r="B68" s="49">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"ZZTestPlayer2",'Game Log Season 3'!$D$3:$D$1000,A68)</f>
+        <v>0</v>
+      </c>
+      <c r="C68" s="49">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"ZZTestPlayer2",'Game Log Season 3'!$D$3:$D$1000,A68,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D68" s="49">
+        <f>IFERROR(C68/B68,0)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert Phase 2 test data -- add_player.py/add_deck.py column E support validated
Confirmed via a real LibreOffice recalculation: new player + new deck
(with and without a playgroup ID) both wrote correct column E values,
existing IDs on unrelated rows survived row-shifting untouched, and
Becca's average correctly recomputed to include the new deck. The two
scripts themselves stay updated -- only the test rows are reverted.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deck-strength.xlsx
+++ b/deck-strength.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="883" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="161">
   <si>
     <t xml:space="preserve">Base Game Info</t>
   </si>
@@ -350,12 +350,6 @@
     <t xml:space="preserve">648625</t>
   </si>
   <si>
-    <t xml:space="preserve">ZZ Test Deck With ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">999002</t>
-  </si>
-  <si>
     <t xml:space="preserve">626865</t>
   </si>
   <si>
@@ -474,18 +468,6 @@
   </si>
   <si>
     <t xml:space="preserve">576574</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZZTestPlayer2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test Commander A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">999001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test Commander B</t>
   </si>
   <si>
     <t xml:space="preserve">Player / Deck</t>
@@ -25799,7 +25781,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40.33"/>
@@ -25828,8 +25810,8 @@
         <v>26</v>
       </c>
       <c r="B2" s="48" t="n">
-        <f aca="false">AVERAGE(B3:B7)</f>
-        <v>2.75830555555556</v>
+        <f aca="false">AVERAGE(B3:B6)</f>
+        <v>2.72288194444444</v>
       </c>
       <c r="C2" s="46"/>
     </row>
@@ -25897,327 +25879,329 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="49" t="s">
+      <c r="A7" s="47" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="48" t="n">
+        <f aca="false">AVERAGE(B8:B17)</f>
+        <v>3.28381944444444</v>
+      </c>
+      <c r="C7" s="46"/>
+    </row>
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="49" t="s">
+        <v>68</v>
+      </c>
+      <c r="B8" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A8)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D8)</f>
+        <v>3.83916666666667</v>
+      </c>
+      <c r="C8" s="46"/>
+      <c r="D8" s="49" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="E8" s="47" t="s">
         <v>106</v>
       </c>
-      <c r="B7" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Becca")*('Game Log Season 3'!$D$3:$D$1000=A7)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D7)</f>
-        <v>2.9</v>
-      </c>
-      <c r="C7" s="46"/>
-      <c r="D7" s="49" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="E7" s="47" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="47" t="s">
-        <v>28</v>
-      </c>
-      <c r="B8" s="48" t="n">
-        <f aca="false">AVERAGE(B9:B18)</f>
-        <v>3.28381944444444</v>
-      </c>
-      <c r="C8" s="46"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="49" t="s">
-        <v>68</v>
+        <v>42</v>
       </c>
       <c r="B9" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A9)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D9)</f>
-        <v>3.83916666666667</v>
+        <v>3.9</v>
       </c>
       <c r="C9" s="46"/>
       <c r="D9" s="49" t="n">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
       <c r="E9" s="47" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="49" t="s">
-        <v>42</v>
+        <v>67</v>
       </c>
       <c r="B10" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A10)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D10)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C10" s="46"/>
+        <v>3.4</v>
+      </c>
+      <c r="C10" s="46" t="s">
+        <v>108</v>
+      </c>
       <c r="D10" s="49" t="n">
-        <v>3.9</v>
+        <v>3.4</v>
       </c>
       <c r="E10" s="47" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="49" t="s">
-        <v>67</v>
+        <v>82</v>
       </c>
       <c r="B11" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A11)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D11)</f>
-        <v>3.4</v>
-      </c>
-      <c r="C11" s="46" t="s">
+        <v>2.6</v>
+      </c>
+      <c r="C11" s="46"/>
+      <c r="D11" s="49" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E11" s="47" t="s">
         <v>110</v>
       </c>
-      <c r="D11" s="49" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="E11" s="47" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="49" t="s">
-        <v>82</v>
+        <v>44</v>
       </c>
       <c r="B12" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A12)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D12)</f>
-        <v>2.6</v>
-      </c>
-      <c r="C12" s="46"/>
+        <v>3.5</v>
+      </c>
+      <c r="C12" s="46" t="s">
+        <v>103</v>
+      </c>
       <c r="D12" s="49" t="n">
-        <v>2.6</v>
+        <v>3.5</v>
       </c>
       <c r="E12" s="47" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="49" t="s">
-        <v>44</v>
+        <v>88</v>
       </c>
       <c r="B13" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A13)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D13)</f>
-        <v>3.5</v>
-      </c>
-      <c r="C13" s="46" t="s">
-        <v>103</v>
-      </c>
+        <v>2.65388888888889</v>
+      </c>
+      <c r="C13" s="46"/>
       <c r="D13" s="49" t="n">
-        <v>3.5</v>
+        <v>2.7</v>
       </c>
       <c r="E13" s="47" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="49" t="s">
-        <v>88</v>
+        <v>48</v>
       </c>
       <c r="B14" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A14)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D14)</f>
-        <v>2.65388888888889</v>
+        <v>2.6</v>
       </c>
       <c r="C14" s="46"/>
       <c r="D14" s="49" t="n">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
       <c r="E14" s="47" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="49" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="B15" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A15)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D15)</f>
-        <v>2.6</v>
+        <v>3.91083333333333</v>
       </c>
       <c r="C15" s="46"/>
       <c r="D15" s="49" t="n">
-        <v>2.6</v>
+        <v>3.9</v>
       </c>
       <c r="E15" s="47" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="49" t="s">
-        <v>37</v>
+        <v>91</v>
       </c>
       <c r="B16" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A16)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D16)</f>
-        <v>3.91083333333333</v>
+        <v>2.94083333333333</v>
       </c>
       <c r="C16" s="46"/>
       <c r="D16" s="49" t="n">
-        <v>3.9</v>
+        <v>2.3</v>
       </c>
       <c r="E16" s="47" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="49" t="s">
-        <v>91</v>
+        <v>47</v>
       </c>
       <c r="B17" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A17)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D17)</f>
-        <v>2.94083333333333</v>
+        <v>3.49347222222222</v>
       </c>
       <c r="C17" s="46"/>
       <c r="D17" s="49" t="n">
-        <v>2.3</v>
+        <v>3.5</v>
       </c>
       <c r="E17" s="47" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="47" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="48" t="n">
+        <f aca="false">AVERAGE(B19:B32)</f>
+        <v>3.31464285714286</v>
+      </c>
+      <c r="C18" s="46"/>
+    </row>
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="49" t="s">
+        <v>73</v>
+      </c>
+      <c r="B19" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A19)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D19)</f>
+        <v>2.4</v>
+      </c>
+      <c r="C19" s="46"/>
+      <c r="D19" s="49" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E19" s="47" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="49" t="s">
-        <v>47</v>
-      </c>
-      <c r="B18" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A18)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D18)</f>
-        <v>3.49347222222222</v>
-      </c>
-      <c r="C18" s="46"/>
-      <c r="D18" s="49" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="E18" s="47" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="47" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" s="48" t="n">
-        <f aca="false">AVERAGE(B20:B33)</f>
-        <v>3.31464285714286</v>
-      </c>
-      <c r="C19" s="46"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="49" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="B20" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A20)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D20)</f>
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="C20" s="46"/>
       <c r="D20" s="49" t="n">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="E20" s="47" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="49" t="s">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="B21" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A21)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D21)</f>
-        <v>2.6</v>
+        <v>3.57402777777778</v>
       </c>
       <c r="C21" s="46"/>
       <c r="D21" s="49" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="E21" s="47" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="49" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B22" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A22)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D22)</f>
-        <v>3.57402777777778</v>
+        <v>3.6</v>
       </c>
       <c r="C22" s="46"/>
       <c r="D22" s="49" t="n">
         <v>3.6</v>
       </c>
       <c r="E22" s="47" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="49" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="B23" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A23)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D23)</f>
-        <v>3.6</v>
+        <v>2.9</v>
       </c>
       <c r="C23" s="46"/>
       <c r="D23" s="49" t="n">
-        <v>3.6</v>
+        <v>2.9</v>
       </c>
       <c r="E23" s="47" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="49" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="B24" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A24)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D24)</f>
-        <v>2.9</v>
-      </c>
-      <c r="C24" s="46"/>
+        <v>3.9</v>
+      </c>
+      <c r="C24" s="46" t="s">
+        <v>103</v>
+      </c>
       <c r="D24" s="49" t="n">
-        <v>2.9</v>
+        <v>3.9</v>
       </c>
       <c r="E24" s="47" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="49" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="B25" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A25)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D25)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C25" s="46" t="s">
-        <v>103</v>
-      </c>
+        <v>2.8</v>
+      </c>
+      <c r="C25" s="46"/>
       <c r="D25" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E25" s="47" t="s">
-        <v>124</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="49" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B26" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A26)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D26)</f>
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="C26" s="46"/>
       <c r="D26" s="49" t="n">
-        <v>2.8</v>
+        <v>2.6</v>
+      </c>
+      <c r="E26" s="47" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="49" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B27" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A27)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D27)</f>
-        <v>2.6</v>
-      </c>
-      <c r="C27" s="46"/>
+        <v>3.59875</v>
+      </c>
+      <c r="C27" s="46" t="s">
+        <v>124</v>
+      </c>
       <c r="D27" s="49" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="E27" s="47" t="s">
         <v>125</v>
@@ -26225,591 +26209,533 @@
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="49" t="s">
-        <v>83</v>
+        <v>48</v>
       </c>
       <c r="B28" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A28)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D28)</f>
-        <v>3.59875</v>
-      </c>
-      <c r="C28" s="46" t="s">
+        <v>3.94083333333333</v>
+      </c>
+      <c r="C28" s="46"/>
+      <c r="D28" s="49" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="E28" s="47" t="s">
         <v>126</v>
-      </c>
-      <c r="D28" s="49" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="E28" s="47" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="49" t="s">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="B29" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A29)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D29)</f>
-        <v>3.94083333333333</v>
+        <v>3.65388888888889</v>
       </c>
       <c r="C29" s="46"/>
       <c r="D29" s="49" t="n">
-        <v>3.9</v>
+        <v>3.7</v>
       </c>
       <c r="E29" s="47" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="49" t="s">
-        <v>90</v>
-      </c>
-      <c r="B30" s="49" t="n">
+        <v>46</v>
+      </c>
+      <c r="B30" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A30)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D30)</f>
-        <v>3.65388888888889</v>
+        <v>3.95583333333333</v>
       </c>
       <c r="C30" s="46"/>
-      <c r="D30" s="49" t="n">
-        <v>3.7</v>
+      <c r="D30" s="50" t="n">
+        <v>4</v>
       </c>
       <c r="E30" s="47" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="49" t="s">
-        <v>46</v>
+        <v>92</v>
       </c>
       <c r="B31" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A31)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D31)</f>
-        <v>3.95583333333333</v>
+        <v>2.94666666666667</v>
       </c>
       <c r="C31" s="46"/>
       <c r="D31" s="50" t="n">
-        <v>4</v>
+        <v>2.9</v>
       </c>
       <c r="E31" s="47" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="49" t="s">
-        <v>92</v>
+        <v>40</v>
       </c>
       <c r="B32" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A32)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D32)</f>
-        <v>2.94666666666667</v>
-      </c>
-      <c r="C32" s="46"/>
+        <v>3.935</v>
+      </c>
+      <c r="C32" s="46" t="s">
+        <v>130</v>
+      </c>
       <c r="D32" s="50" t="n">
-        <v>2.9</v>
+        <v>3.9</v>
       </c>
       <c r="E32" s="47" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="49" t="s">
-        <v>40</v>
-      </c>
-      <c r="B33" s="50" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A33)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D33)</f>
-        <v>3.935</v>
-      </c>
-      <c r="C33" s="46" t="s">
+    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" s="48" t="n">
+        <f aca="false">AVERAGE(B34:B44)</f>
+        <v>3.26275505050505</v>
+      </c>
+      <c r="C33" s="46"/>
+    </row>
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="49" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A34)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D34)</f>
+        <v>3.5</v>
+      </c>
+      <c r="C34" s="46"/>
+      <c r="D34" s="49" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E34" s="47" t="s">
         <v>132</v>
       </c>
-      <c r="D33" s="50" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E33" s="47" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="47" t="s">
-        <v>32</v>
-      </c>
-      <c r="B34" s="48" t="n">
-        <f aca="false">AVERAGE(B35:B45)</f>
-        <v>3.26275505050505</v>
-      </c>
-      <c r="C34" s="46"/>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="49" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="B35" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A35)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D35)</f>
-        <v>3.5</v>
+        <v>3.43088888888889</v>
       </c>
       <c r="C35" s="46"/>
       <c r="D35" s="49" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="E35" s="47" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="49" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="B36" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A36)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D36)</f>
-        <v>3.43088888888889</v>
+        <v>3.7</v>
       </c>
       <c r="C36" s="46"/>
       <c r="D36" s="49" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="E36" s="47" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="49" t="s">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="B37" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A37)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D37)</f>
-        <v>3.7</v>
+        <v>2.6</v>
       </c>
       <c r="C37" s="46"/>
       <c r="D37" s="49" t="n">
-        <v>3.7</v>
+        <v>2.6</v>
       </c>
       <c r="E37" s="47" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="49" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="B38" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A38)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D38)</f>
-        <v>2.6</v>
+        <v>3.77816666666667</v>
       </c>
       <c r="C38" s="46"/>
       <c r="D38" s="49" t="n">
-        <v>2.6</v>
+        <v>3.8</v>
       </c>
       <c r="E38" s="47" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="49" t="s">
-        <v>41</v>
+        <v>79</v>
       </c>
       <c r="B39" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A39)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D39)</f>
-        <v>3.77816666666667</v>
+        <v>2.59388888888889</v>
       </c>
       <c r="C39" s="46"/>
       <c r="D39" s="49" t="n">
-        <v>3.8</v>
+        <v>2.6</v>
       </c>
       <c r="E39" s="47" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="49" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="B40" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A40)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D40)</f>
-        <v>2.59388888888889</v>
+        <v>3.23902777777778</v>
       </c>
       <c r="C40" s="46"/>
       <c r="D40" s="49" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="E40" s="47" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="49" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="B41" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A41)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D41)</f>
-        <v>3.23902777777778</v>
+        <v>2.6</v>
       </c>
       <c r="C41" s="46"/>
       <c r="D41" s="49" t="n">
-        <v>3.6</v>
+        <v>2.6</v>
       </c>
       <c r="E41" s="47" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="49" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B42" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A42)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D42)</f>
-        <v>2.6</v>
+        <v>3.58416666666667</v>
       </c>
       <c r="C42" s="46"/>
       <c r="D42" s="49" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="E42" s="47" t="s">
-        <v>141</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="49" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B43" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A43)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D43)</f>
-        <v>3.58416666666667</v>
+        <v>2.94083333333333</v>
       </c>
       <c r="C43" s="46"/>
       <c r="D43" s="49" t="n">
-        <v>3.6</v>
+        <v>2.9</v>
+      </c>
+      <c r="E43" s="47" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="49" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B44" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A44)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D44)</f>
-        <v>2.94083333333333</v>
+        <v>3.92333333333333</v>
       </c>
       <c r="C44" s="46"/>
       <c r="D44" s="49" t="n">
-        <v>2.9</v>
+        <v>3.9</v>
       </c>
       <c r="E44" s="47" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="49" t="s">
-        <v>97</v>
-      </c>
-      <c r="B45" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A45)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D45)</f>
-        <v>3.92333333333333</v>
+      <c r="A45" s="47" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45" s="48" t="n">
+        <f aca="false">AVERAGE(B46:B50)</f>
+        <v>3.2865</v>
       </c>
       <c r="C45" s="46"/>
-      <c r="D45" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E45" s="47" t="s">
-        <v>143</v>
-      </c>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="47" t="s">
-        <v>70</v>
-      </c>
-      <c r="B46" s="48" t="n">
-        <f aca="false">AVERAGE(B47:B51)</f>
-        <v>3.2865</v>
-      </c>
-      <c r="C46" s="46"/>
+      <c r="A46" s="49" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A46)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D46)</f>
+        <v>3.6</v>
+      </c>
+      <c r="C46" s="46" t="s">
+        <v>124</v>
+      </c>
+      <c r="D46" s="49" t="n">
+        <v>3.6</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="49" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="B47" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A47)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D47)</f>
-        <v>3.6</v>
+        <v>3.33761111111111</v>
       </c>
       <c r="C47" s="46" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D47" s="49" t="n">
-        <v>3.6</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="49" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="B48" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A48)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D48)</f>
-        <v>3.33761111111111</v>
-      </c>
-      <c r="C48" s="46" t="s">
-        <v>126</v>
-      </c>
+        <v>3.2</v>
+      </c>
+      <c r="C48" s="46"/>
       <c r="D48" s="49" t="n">
-        <v>3.3</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="49" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B49" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A49)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D49)</f>
-        <v>3.2</v>
-      </c>
-      <c r="C49" s="46"/>
+        <v>3.9</v>
+      </c>
+      <c r="C49" s="46" t="s">
+        <v>130</v>
+      </c>
       <c r="D49" s="49" t="n">
-        <v>3.2</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="49" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B50" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A50)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D50)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C50" s="46" t="s">
-        <v>132</v>
-      </c>
+        <v>2.39488888888889</v>
+      </c>
+      <c r="C50" s="46"/>
       <c r="D50" s="49" t="n">
-        <v>3.9</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="49" t="s">
-        <v>93</v>
-      </c>
-      <c r="B51" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A51)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D51)</f>
-        <v>2.39488888888889</v>
+      <c r="A51" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="B51" s="48" t="n">
+        <f aca="false">AVERAGE(B52:B56)</f>
+        <v>3.42807</v>
       </c>
       <c r="C51" s="46"/>
-      <c r="D51" s="49" t="n">
-        <v>2.4</v>
-      </c>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="47" t="s">
-        <v>38</v>
-      </c>
-      <c r="B52" s="48" t="n">
-        <f aca="false">AVERAGE(B53:B57)</f>
-        <v>3.42807</v>
+      <c r="A52" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="B52" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A52)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D52)</f>
+        <v>3.6</v>
       </c>
       <c r="C52" s="46"/>
+      <c r="D52" s="49" t="n">
+        <v>3.6</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="49" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="B53" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A53)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D53)</f>
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
       <c r="C53" s="46"/>
       <c r="D53" s="49" t="n">
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="49" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B54" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A54)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D54)</f>
-        <v>3.8</v>
+        <v>2.7</v>
       </c>
       <c r="C54" s="46"/>
       <c r="D54" s="49" t="n">
-        <v>3.8</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="49" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="B55" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A55)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D55)</f>
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
       <c r="C55" s="46"/>
       <c r="D55" s="49" t="n">
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B56" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A56)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D56)</f>
-        <v>3.3</v>
+        <v>3.74035</v>
       </c>
       <c r="C56" s="46"/>
       <c r="D56" s="49" t="n">
-        <v>3.3</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="49" t="s">
-        <v>63</v>
-      </c>
-      <c r="B57" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A57)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D57)</f>
-        <v>3.74035</v>
+      <c r="A57" s="47" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="48" t="n">
+        <f aca="false">AVERAGE(B58:B59)</f>
+        <v>3.05</v>
       </c>
       <c r="C57" s="46"/>
-      <c r="D57" s="49" t="n">
-        <v>3.7</v>
-      </c>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="47" t="s">
-        <v>59</v>
-      </c>
-      <c r="B58" s="48" t="n">
-        <f aca="false">AVERAGE(B59:B60)</f>
-        <v>3.05</v>
+      <c r="A58" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="B58" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A58)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D58)</f>
+        <v>2.7</v>
       </c>
       <c r="C58" s="46"/>
+      <c r="D58" s="49" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E58" s="47" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="49" t="s">
-        <v>33</v>
+        <v>69</v>
       </c>
       <c r="B59" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A59)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D59)</f>
-        <v>2.7</v>
+        <v>3.4</v>
       </c>
       <c r="C59" s="46"/>
       <c r="D59" s="49" t="n">
-        <v>2.7</v>
+        <v>3.4</v>
       </c>
       <c r="E59" s="47" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="49" t="s">
-        <v>69</v>
-      </c>
-      <c r="B60" s="49" t="n">
+        <v>84</v>
+      </c>
+      <c r="B60" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A60)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D60)</f>
-        <v>3.4</v>
+        <v>1</v>
       </c>
       <c r="C60" s="46"/>
-      <c r="D60" s="49" t="n">
-        <v>3.4</v>
+      <c r="D60" s="50" t="n">
+        <v>1</v>
       </c>
       <c r="E60" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="49" t="s">
-        <v>84</v>
-      </c>
-      <c r="B61" s="50" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A61)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D61)</f>
-        <v>1</v>
+      <c r="A61" s="47" t="s">
+        <v>51</v>
+      </c>
+      <c r="B61" s="48" t="n">
+        <f aca="false">AVERAGE(B62:B63)</f>
+        <v>2.25194444444444</v>
       </c>
       <c r="C61" s="46"/>
-      <c r="D61" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E61" s="47" t="s">
-        <v>146</v>
-      </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="47" t="s">
-        <v>51</v>
-      </c>
-      <c r="B62" s="48" t="n">
-        <f aca="false">AVERAGE(B63:B64)</f>
-        <v>2.25194444444444</v>
+      <c r="A62" s="49" t="s">
+        <v>52</v>
+      </c>
+      <c r="B62" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A62)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D62)</f>
+        <v>2.30388888888889</v>
       </c>
       <c r="C62" s="46"/>
+      <c r="D62" s="49" t="n">
+        <v>2.5</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="49" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B63" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A63)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D63)</f>
-        <v>2.30388888888889</v>
+        <v>2.2</v>
       </c>
       <c r="C63" s="46"/>
       <c r="D63" s="49" t="n">
-        <v>2.5</v>
+        <v>2.2</v>
+      </c>
+      <c r="E63" s="47" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="49" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="B64" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A64)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D64)</f>
-        <v>2.2</v>
-      </c>
-      <c r="C64" s="46"/>
+        <v>2.43069444444444</v>
+      </c>
       <c r="D64" s="49" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="E64" s="47" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="49" t="s">
-        <v>96</v>
-      </c>
-      <c r="B65" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A65)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D65)</f>
-        <v>2.43069444444444</v>
-      </c>
-      <c r="D65" s="49" t="n">
         <v>2.4</v>
       </c>
-    </row>
-    <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="47" t="s">
-        <v>148</v>
-      </c>
-      <c r="B66" s="48" t="n">
-        <f aca="false">AVERAGE(B67:B68)</f>
-        <v>2.85</v>
-      </c>
-      <c r="C66" s="46"/>
-    </row>
-    <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="49" t="s">
-        <v>149</v>
-      </c>
-      <c r="B67" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="ZZTestPlayer2")*('Game Log Season 3'!$D$3:$D$1000=A67)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D67)</f>
-        <v>3</v>
-      </c>
-      <c r="C67" s="46"/>
-      <c r="D67" s="49" t="n">
-        <v>3</v>
-      </c>
-      <c r="E67" s="47" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="49" t="s">
-        <v>151</v>
-      </c>
-      <c r="B68" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="ZZTestPlayer2")*('Game Log Season 3'!$D$3:$D$1000=A68)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D68)</f>
-        <v>2.7</v>
-      </c>
-      <c r="C68" s="46"/>
-      <c r="D68" s="49" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="E68" s="47"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -26827,7 +26753,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D68"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.89"/>
@@ -26838,16 +26764,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="45" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="B1" s="45" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="C1" s="45" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="D1" s="45" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26936,59 +26862,59 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="49" t="s">
-        <v>106</v>
-      </c>
-      <c r="B7" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A7)</f>
-        <v>0</v>
-      </c>
-      <c r="C7" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Becca",'Game Log Season 3'!$D$3:$D$1000,A7,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D7" s="49" t="n">
+      <c r="A7" s="47" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A7)</f>
+        <v>14</v>
+      </c>
+      <c r="C7" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A7,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>4</v>
+      </c>
+      <c r="D7" s="48" t="n">
         <f aca="false">IFERROR(C7/B7,0)</f>
-        <v>0</v>
+        <v>0.285714285714286</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="47" t="s">
-        <v>28</v>
-      </c>
-      <c r="B8" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A8)</f>
-        <v>14</v>
-      </c>
-      <c r="C8" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A8,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+      <c r="A8" s="49" t="s">
+        <v>68</v>
+      </c>
+      <c r="B8" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A8)</f>
         <v>4</v>
       </c>
-      <c r="D8" s="48" t="n">
+      <c r="C8" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A8,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>2</v>
+      </c>
+      <c r="D8" s="49" t="n">
         <f aca="false">IFERROR(C8/B8,0)</f>
-        <v>0.285714285714286</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="49" t="s">
-        <v>68</v>
+        <v>42</v>
       </c>
       <c r="B9" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A9)</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C9" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A9,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D9" s="49" t="n">
         <f aca="false">IFERROR(C9/B9,0)</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="49" t="s">
-        <v>42</v>
+        <v>67</v>
       </c>
       <c r="B10" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A10)</f>
@@ -27005,7 +26931,7 @@
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="49" t="s">
-        <v>67</v>
+        <v>82</v>
       </c>
       <c r="B11" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A11)</f>
@@ -27022,7 +26948,7 @@
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="49" t="s">
-        <v>82</v>
+        <v>44</v>
       </c>
       <c r="B12" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A12)</f>
@@ -27039,11 +26965,11 @@
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="49" t="s">
-        <v>44</v>
+        <v>88</v>
       </c>
       <c r="B13" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A13)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C13" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A13,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27056,11 +26982,11 @@
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="49" t="s">
-        <v>88</v>
+        <v>48</v>
       </c>
       <c r="B14" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A14)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C14" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A14,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27073,28 +26999,28 @@
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="49" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="B15" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A15)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C15" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A15,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" s="49" t="n">
         <f aca="false">IFERROR(C15/B15,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="49" t="s">
-        <v>37</v>
+        <v>91</v>
       </c>
       <c r="B16" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A16)</f>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C16" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A16,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27102,63 +27028,63 @@
       </c>
       <c r="D16" s="49" t="n">
         <f aca="false">IFERROR(C16/B16,0)</f>
-        <v>1</v>
+        <v>0.166666666666667</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="49" t="s">
-        <v>91</v>
+        <v>47</v>
       </c>
       <c r="B17" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A17)</f>
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C17" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A17,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D17" s="49" t="n">
         <f aca="false">IFERROR(C17/B17,0)</f>
-        <v>0.166666666666667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="49" t="s">
-        <v>47</v>
-      </c>
-      <c r="B18" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A18)</f>
-        <v>1</v>
-      </c>
-      <c r="C18" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A18,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D18" s="49" t="n">
+      <c r="A18" s="47" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A18)</f>
+        <v>12</v>
+      </c>
+      <c r="C18" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A18,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>5</v>
+      </c>
+      <c r="D18" s="48" t="n">
         <f aca="false">IFERROR(C18/B18,0)</f>
-        <v>0</v>
+        <v>0.416666666666667</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="47" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A19)</f>
-        <v>12</v>
-      </c>
-      <c r="C19" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A19,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>5</v>
-      </c>
-      <c r="D19" s="48" t="n">
+      <c r="A19" s="49" t="s">
+        <v>73</v>
+      </c>
+      <c r="B19" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A19)</f>
+        <v>0</v>
+      </c>
+      <c r="C19" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A19,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D19" s="49" t="n">
         <f aca="false">IFERROR(C19/B19,0)</f>
-        <v>0.416666666666667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="49" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="B20" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A20)</f>
@@ -27175,11 +27101,11 @@
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="49" t="s">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="B21" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A21)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C21" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A21,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27192,11 +27118,11 @@
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="49" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B22" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A22)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C22" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A22,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27209,7 +27135,7 @@
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="49" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="B23" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A23)</f>
@@ -27226,7 +27152,7 @@
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="49" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="B24" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A24)</f>
@@ -27243,7 +27169,7 @@
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="49" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="B25" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A25)</f>
@@ -27260,7 +27186,7 @@
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="49" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B26" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A26)</f>
@@ -27277,11 +27203,11 @@
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="49" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B27" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A27)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C27" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A27,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27294,7 +27220,7 @@
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="49" t="s">
-        <v>83</v>
+        <v>48</v>
       </c>
       <c r="B28" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A28)</f>
@@ -27302,122 +27228,122 @@
       </c>
       <c r="C28" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A28,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D28" s="49" t="n">
         <f aca="false">IFERROR(C28/B28,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="49" t="s">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="B29" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A29)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C29" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A29,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D29" s="49" t="n">
         <f aca="false">IFERROR(C29/B29,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="49" t="s">
-        <v>90</v>
+        <v>46</v>
       </c>
       <c r="B30" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A30)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C30" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A30,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D30" s="49" t="n">
         <f aca="false">IFERROR(C30/B30,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="49" t="s">
-        <v>46</v>
+        <v>92</v>
       </c>
       <c r="B31" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A31)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C31" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A31,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D31" s="49" t="n">
         <f aca="false">IFERROR(C31/B31,0)</f>
-        <v>1</v>
+        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="49" t="s">
-        <v>92</v>
+        <v>40</v>
       </c>
       <c r="B32" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A32)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C32" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A32,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D32" s="49" t="n">
         <f aca="false">IFERROR(C32/B32,0)</f>
-        <v>0.666666666666667</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="49" t="s">
-        <v>40</v>
-      </c>
-      <c r="B33" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A33)</f>
-        <v>1</v>
-      </c>
-      <c r="C33" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A33,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
-      </c>
-      <c r="D33" s="49" t="n">
+      <c r="A33" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A33)</f>
+        <v>11</v>
+      </c>
+      <c r="C33" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A33,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>3</v>
+      </c>
+      <c r="D33" s="48" t="n">
         <f aca="false">IFERROR(C33/B33,0)</f>
-        <v>1</v>
+        <v>0.272727272727273</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="47" t="s">
-        <v>32</v>
-      </c>
-      <c r="B34" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A34)</f>
-        <v>11</v>
-      </c>
-      <c r="C34" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A34,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>3</v>
-      </c>
-      <c r="D34" s="48" t="n">
+      <c r="A34" s="49" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A34)</f>
+        <v>0</v>
+      </c>
+      <c r="C34" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A34,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D34" s="49" t="n">
         <f aca="false">IFERROR(C34/B34,0)</f>
-        <v>0.272727272727273</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="49" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="B35" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A35)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C35" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A35,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27430,11 +27356,11 @@
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="49" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="B36" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A36)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C36" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A36,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27447,7 +27373,7 @@
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="49" t="s">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="B37" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A37)</f>
@@ -27464,24 +27390,24 @@
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="49" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="B38" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A38)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C38" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A38,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D38" s="49" t="n">
         <f aca="false">IFERROR(C38/B38,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="49" t="s">
-        <v>41</v>
+        <v>79</v>
       </c>
       <c r="B39" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A39)</f>
@@ -27489,20 +27415,20 @@
       </c>
       <c r="C39" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A39,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D39" s="49" t="n">
         <f aca="false">IFERROR(C39/B39,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="49" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="B40" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A40)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C40" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A40,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27515,11 +27441,11 @@
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="49" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="B41" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A41)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C41" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A41,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27532,11 +27458,11 @@
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="49" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B42" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A42)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C42" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A42,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27549,7 +27475,7 @@
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="49" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B43" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A43)</f>
@@ -27557,16 +27483,16 @@
       </c>
       <c r="C43" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A43,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D43" s="49" t="n">
         <f aca="false">IFERROR(C43/B43,0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="49" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B44" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A44)</f>
@@ -27582,46 +27508,46 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="49" t="s">
-        <v>97</v>
-      </c>
-      <c r="B45" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A45)</f>
-        <v>2</v>
-      </c>
-      <c r="C45" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A45,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
-      </c>
-      <c r="D45" s="49" t="n">
+      <c r="A45" s="47" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A45)</f>
+        <v>2</v>
+      </c>
+      <c r="C45" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A45,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D45" s="48" t="n">
         <f aca="false">IFERROR(C45/B45,0)</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="47" t="s">
-        <v>70</v>
-      </c>
-      <c r="B46" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A46)</f>
-        <v>2</v>
-      </c>
-      <c r="C46" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A46,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D46" s="48" t="n">
+      <c r="A46" s="49" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A46)</f>
+        <v>0</v>
+      </c>
+      <c r="C46" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A46,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D46" s="49" t="n">
         <f aca="false">IFERROR(C46/B46,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="49" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="B47" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A47)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C47" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A47,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27634,11 +27560,11 @@
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="49" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="B48" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A48)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C48" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A48,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27651,7 +27577,7 @@
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="49" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B49" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A49)</f>
@@ -27668,11 +27594,11 @@
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="49" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B50" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A50)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C50" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A50,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27684,42 +27610,42 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="49" t="s">
-        <v>93</v>
-      </c>
-      <c r="B51" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A51)</f>
-        <v>1</v>
-      </c>
-      <c r="C51" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A51,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D51" s="49" t="n">
+      <c r="A51" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="B51" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A51)</f>
+        <v>1</v>
+      </c>
+      <c r="C51" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A51,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D51" s="48" t="n">
         <f aca="false">IFERROR(C51/B51,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="47" t="s">
-        <v>38</v>
-      </c>
-      <c r="B52" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A52)</f>
-        <v>1</v>
-      </c>
-      <c r="C52" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A52,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D52" s="48" t="n">
+      <c r="A52" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="B52" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A52)</f>
+        <v>0</v>
+      </c>
+      <c r="C52" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A52,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D52" s="49" t="n">
         <f aca="false">IFERROR(C52/B52,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="49" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="B53" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A53)</f>
@@ -27736,7 +27662,7 @@
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="49" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B54" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A54)</f>
@@ -27753,7 +27679,7 @@
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="49" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="B55" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A55)</f>
@@ -27770,11 +27696,11 @@
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B56" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A56)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C56" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A56,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27786,42 +27712,42 @@
       </c>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="49" t="s">
-        <v>63</v>
-      </c>
-      <c r="B57" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A57)</f>
-        <v>1</v>
-      </c>
-      <c r="C57" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A57,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D57" s="49" t="n">
+      <c r="A57" s="47" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A57)</f>
+        <v>0</v>
+      </c>
+      <c r="C57" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A57,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D57" s="48" t="n">
         <f aca="false">IFERROR(C57/B57,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="47" t="s">
-        <v>59</v>
-      </c>
-      <c r="B58" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A58)</f>
-        <v>0</v>
-      </c>
-      <c r="C58" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A58,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D58" s="48" t="n">
+      <c r="A58" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="B58" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A58)</f>
+        <v>0</v>
+      </c>
+      <c r="C58" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A58,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D58" s="49" t="n">
         <f aca="false">IFERROR(C58/B58,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="49" t="s">
-        <v>33</v>
+        <v>69</v>
       </c>
       <c r="B59" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A59)</f>
@@ -27838,7 +27764,7 @@
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="49" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="B60" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A60)</f>
@@ -27854,46 +27780,46 @@
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="49" t="s">
-        <v>84</v>
-      </c>
-      <c r="B61" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A61)</f>
-        <v>0</v>
-      </c>
-      <c r="C61" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A61,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D61" s="49" t="n">
+      <c r="A61" s="47" t="s">
+        <v>51</v>
+      </c>
+      <c r="B61" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A61)</f>
+        <v>4</v>
+      </c>
+      <c r="C61" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A61,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D61" s="48" t="n">
         <f aca="false">IFERROR(C61/B61,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="47" t="s">
-        <v>51</v>
-      </c>
-      <c r="B62" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A62)</f>
-        <v>4</v>
-      </c>
-      <c r="C62" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A62,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D62" s="48" t="n">
+      <c r="A62" s="49" t="s">
+        <v>52</v>
+      </c>
+      <c r="B62" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A62)</f>
+        <v>3</v>
+      </c>
+      <c r="C62" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A62,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D62" s="49" t="n">
         <f aca="false">IFERROR(C62/B62,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="49" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B63" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A63)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C63" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A63,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27906,11 +27832,11 @@
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="49" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="B64" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A64)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C64" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A64,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27918,74 +27844,6 @@
       </c>
       <c r="D64" s="49" t="n">
         <f aca="false">IFERROR(C64/B64,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="49" t="s">
-        <v>96</v>
-      </c>
-      <c r="B65" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A65)</f>
-        <v>1</v>
-      </c>
-      <c r="C65" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A65,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D65" s="49" t="n">
-        <f aca="false">IFERROR(C65/B65,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="47" t="s">
-        <v>148</v>
-      </c>
-      <c r="B66" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A66)</f>
-        <v>0</v>
-      </c>
-      <c r="C66" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A66,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D66" s="48" t="n">
-        <f aca="false">IFERROR(C66/B66,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="49" t="s">
-        <v>149</v>
-      </c>
-      <c r="B67" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"ZZTestPlayer2",'Game Log Season 3'!$D$3:$D$1000,A67)</f>
-        <v>0</v>
-      </c>
-      <c r="C67" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"ZZTestPlayer2",'Game Log Season 3'!$D$3:$D$1000,A67,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D67" s="49" t="n">
-        <f aca="false">IFERROR(C67/B67,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="49" t="s">
-        <v>151</v>
-      </c>
-      <c r="B68" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"ZZTestPlayer2",'Game Log Season 3'!$D$3:$D$1000,A68)</f>
-        <v>0</v>
-      </c>
-      <c r="C68" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"ZZTestPlayer2",'Game Log Season 3'!$D$3:$D$1000,A68,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D68" s="49" t="n">
-        <f aca="false">IFERROR(C68/B68,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -28024,40 +27882,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="51" t="s">
+        <v>150</v>
+      </c>
+      <c r="B1" s="51" t="s">
+        <v>151</v>
+      </c>
+      <c r="C1" s="51" t="s">
+        <v>152</v>
+      </c>
+      <c r="D1" s="51" t="s">
+        <v>153</v>
+      </c>
+      <c r="E1" s="51" t="s">
+        <v>149</v>
+      </c>
+      <c r="F1" s="51" t="s">
+        <v>154</v>
+      </c>
+      <c r="G1" s="51" t="s">
+        <v>155</v>
+      </c>
+      <c r="H1" s="51" t="s">
         <v>156</v>
       </c>
-      <c r="B1" s="51" t="s">
+      <c r="I1" s="51" t="s">
         <v>157</v>
       </c>
-      <c r="C1" s="51" t="s">
+      <c r="J1" s="51" t="s">
         <v>158</v>
       </c>
-      <c r="D1" s="51" t="s">
+      <c r="K1" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="E1" s="51" t="s">
-        <v>155</v>
-      </c>
-      <c r="F1" s="51" t="s">
+      <c r="L1" s="51" t="s">
         <v>160</v>
-      </c>
-      <c r="G1" s="51" t="s">
-        <v>161</v>
-      </c>
-      <c r="H1" s="51" t="s">
-        <v>162</v>
-      </c>
-      <c r="I1" s="51" t="s">
-        <v>163</v>
-      </c>
-      <c r="J1" s="51" t="s">
-        <v>164</v>
-      </c>
-      <c r="K1" s="51" t="s">
-        <v>165</v>
-      </c>
-      <c r="L1" s="51" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
test: Phase 3 dry run (apply_roster_update.py, new player + new deck) -- to be reverted
</commit_message>
<xml_diff>
--- a/deck-strength.xlsx
+++ b/deck-strength.xlsx
@@ -25781,7 +25781,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40.33"/>
@@ -25883,7 +25883,7 @@
         <v>28</v>
       </c>
       <c r="B7" s="48" t="n">
-        <f aca="false">AVERAGE(B8:B17)</f>
+        <f aca="false">AVERAGE(B8:B18)</f>
         <v>3.28381944444444</v>
       </c>
       <c r="C7" s="46"/>
@@ -26052,689 +26052,761 @@
         <v>116</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="47" t="s">
+    <row r="18" spans="1:5">
+      <c r="A18" s="49" t="inlineStr">
+        <is>
+          <t>ZZ Test Batch Deck</t>
+        </is>
+      </c>
+      <c r="B18" s="49">
+        <f>IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A18)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D18)</f>
+        <v>2.8</v>
+      </c>
+      <c r="C18" s="46"/>
+      <c r="D18" s="49">
+        <v>2.8</v>
+      </c>
+      <c r="E18" s="47" t="inlineStr">
+        <is>
+          <t>999003</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="47" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="48" t="n">
-        <f aca="false">AVERAGE(B19:B32)</f>
+      <c r="B19" s="48" t="n">
+        <f aca="false">AVERAGE(B20:B33)</f>
         <v>3.31464285714286</v>
       </c>
-      <c r="C18" s="46"/>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="49" t="s">
-        <v>73</v>
-      </c>
-      <c r="B19" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A19)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D19)</f>
-        <v>2.4</v>
-      </c>
       <c r="C19" s="46"/>
-      <c r="D19" s="49" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="E19" s="47" t="s">
-        <v>117</v>
-      </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="49" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B20" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A20)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D20)</f>
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="C20" s="46"/>
       <c r="D20" s="49" t="n">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="E20" s="47" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="49" t="s">
-        <v>31</v>
+        <v>66</v>
       </c>
       <c r="B21" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A21)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D21)</f>
-        <v>3.57402777777778</v>
+        <v>2.6</v>
       </c>
       <c r="C21" s="46"/>
       <c r="D21" s="49" t="n">
-        <v>3.6</v>
+        <v>2.6</v>
       </c>
       <c r="E21" s="47" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="49" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B22" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A22)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D22)</f>
-        <v>3.6</v>
+        <v>3.57402777777778</v>
       </c>
       <c r="C22" s="46"/>
       <c r="D22" s="49" t="n">
         <v>3.6</v>
       </c>
       <c r="E22" s="47" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="49" t="s">
-        <v>74</v>
+        <v>34</v>
       </c>
       <c r="B23" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A23)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D23)</f>
-        <v>2.9</v>
+        <v>3.6</v>
       </c>
       <c r="C23" s="46"/>
       <c r="D23" s="49" t="n">
-        <v>2.9</v>
+        <v>3.6</v>
       </c>
       <c r="E23" s="47" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="49" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="B24" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A24)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D24)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C24" s="46" t="s">
-        <v>103</v>
-      </c>
+        <v>2.9</v>
+      </c>
+      <c r="C24" s="46"/>
       <c r="D24" s="49" t="n">
-        <v>3.9</v>
+        <v>2.9</v>
       </c>
       <c r="E24" s="47" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="49" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
       <c r="B25" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A25)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D25)</f>
-        <v>2.8</v>
-      </c>
-      <c r="C25" s="46"/>
+        <v>3.9</v>
+      </c>
+      <c r="C25" s="46" t="s">
+        <v>103</v>
+      </c>
       <c r="D25" s="49" t="n">
-        <v>2.8</v>
+        <v>3.9</v>
+      </c>
+      <c r="E25" s="47" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="49" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B26" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A26)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D26)</f>
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="C26" s="46"/>
       <c r="D26" s="49" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="E26" s="47" t="s">
-        <v>123</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="49" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B27" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A27)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D27)</f>
-        <v>3.59875</v>
-      </c>
-      <c r="C27" s="46" t="s">
-        <v>124</v>
-      </c>
+        <v>2.6</v>
+      </c>
+      <c r="C27" s="46"/>
       <c r="D27" s="49" t="n">
-        <v>3.6</v>
+        <v>2.6</v>
       </c>
       <c r="E27" s="47" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="49" t="s">
-        <v>48</v>
+        <v>83</v>
       </c>
       <c r="B28" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A28)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D28)</f>
-        <v>3.94083333333333</v>
-      </c>
-      <c r="C28" s="46"/>
+        <v>3.59875</v>
+      </c>
+      <c r="C28" s="46" t="s">
+        <v>124</v>
+      </c>
       <c r="D28" s="49" t="n">
-        <v>3.9</v>
+        <v>3.6</v>
       </c>
       <c r="E28" s="47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="49" t="s">
-        <v>90</v>
+        <v>48</v>
       </c>
       <c r="B29" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A29)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D29)</f>
-        <v>3.65388888888889</v>
+        <v>3.94083333333333</v>
       </c>
       <c r="C29" s="46"/>
       <c r="D29" s="49" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="E29" s="47" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="49" t="s">
-        <v>46</v>
-      </c>
-      <c r="B30" s="50" t="n">
+        <v>90</v>
+      </c>
+      <c r="B30" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A30)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D30)</f>
-        <v>3.95583333333333</v>
+        <v>3.65388888888889</v>
       </c>
       <c r="C30" s="46"/>
-      <c r="D30" s="50" t="n">
-        <v>4</v>
+      <c r="D30" s="49" t="n">
+        <v>3.7</v>
       </c>
       <c r="E30" s="47" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="49" t="s">
-        <v>92</v>
+        <v>46</v>
       </c>
       <c r="B31" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A31)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D31)</f>
-        <v>2.94666666666667</v>
+        <v>3.95583333333333</v>
       </c>
       <c r="C31" s="46"/>
       <c r="D31" s="50" t="n">
-        <v>2.9</v>
+        <v>4</v>
       </c>
       <c r="E31" s="47" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="49" t="s">
-        <v>40</v>
+        <v>92</v>
       </c>
       <c r="B32" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A32)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D32)</f>
+        <v>2.94666666666667</v>
+      </c>
+      <c r="C32" s="46"/>
+      <c r="D32" s="50" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="E32" s="47" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="49" t="s">
+        <v>40</v>
+      </c>
+      <c r="B33" s="50" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A33)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D33)</f>
         <v>3.935</v>
       </c>
-      <c r="C32" s="46" t="s">
+      <c r="C33" s="46" t="s">
         <v>130</v>
       </c>
-      <c r="D32" s="50" t="n">
+      <c r="D33" s="50" t="n">
         <v>3.9</v>
       </c>
-      <c r="E32" s="47" t="s">
+      <c r="E33" s="47" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="47" t="s">
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="47" t="s">
         <v>32</v>
       </c>
-      <c r="B33" s="48" t="n">
-        <f aca="false">AVERAGE(B34:B44)</f>
+      <c r="B34" s="48" t="n">
+        <f aca="false">AVERAGE(B35:B45)</f>
         <v>3.26275505050505</v>
       </c>
-      <c r="C33" s="46"/>
-    </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="49" t="s">
-        <v>36</v>
-      </c>
-      <c r="B34" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A34)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D34)</f>
-        <v>3.5</v>
-      </c>
       <c r="C34" s="46"/>
-      <c r="D34" s="49" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="E34" s="47" t="s">
-        <v>132</v>
-      </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="49" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="B35" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A35)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D35)</f>
-        <v>3.43088888888889</v>
+        <v>3.5</v>
       </c>
       <c r="C35" s="46"/>
       <c r="D35" s="49" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="E35" s="47" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="49" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="B36" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A36)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D36)</f>
-        <v>3.7</v>
+        <v>3.43088888888889</v>
       </c>
       <c r="C36" s="46"/>
       <c r="D36" s="49" t="n">
-        <v>3.7</v>
+        <v>3.4</v>
       </c>
       <c r="E36" s="47" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="49" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="B37" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A37)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D37)</f>
-        <v>2.6</v>
+        <v>3.7</v>
       </c>
       <c r="C37" s="46"/>
       <c r="D37" s="49" t="n">
-        <v>2.6</v>
+        <v>3.7</v>
       </c>
       <c r="E37" s="47" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="49" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="B38" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A38)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D38)</f>
-        <v>3.77816666666667</v>
+        <v>2.6</v>
       </c>
       <c r="C38" s="46"/>
       <c r="D38" s="49" t="n">
-        <v>3.8</v>
+        <v>2.6</v>
       </c>
       <c r="E38" s="47" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="49" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="B39" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A39)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D39)</f>
-        <v>2.59388888888889</v>
+        <v>3.77816666666667</v>
       </c>
       <c r="C39" s="46"/>
       <c r="D39" s="49" t="n">
-        <v>2.6</v>
+        <v>3.8</v>
       </c>
       <c r="E39" s="47" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="49" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="B40" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A40)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D40)</f>
-        <v>3.23902777777778</v>
+        <v>2.59388888888889</v>
       </c>
       <c r="C40" s="46"/>
       <c r="D40" s="49" t="n">
-        <v>3.6</v>
+        <v>2.6</v>
       </c>
       <c r="E40" s="47" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="49" t="s">
-        <v>87</v>
+        <v>54</v>
       </c>
       <c r="B41" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A41)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D41)</f>
-        <v>2.6</v>
+        <v>3.23902777777778</v>
       </c>
       <c r="C41" s="46"/>
       <c r="D41" s="49" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="E41" s="47" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="49" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B42" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A42)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D42)</f>
-        <v>3.58416666666667</v>
+        <v>2.6</v>
       </c>
       <c r="C42" s="46"/>
       <c r="D42" s="49" t="n">
-        <v>3.6</v>
+        <v>2.6</v>
+      </c>
+      <c r="E42" s="47" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="49" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B43" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A43)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D43)</f>
-        <v>2.94083333333333</v>
+        <v>3.58416666666667</v>
       </c>
       <c r="C43" s="46"/>
       <c r="D43" s="49" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="E43" s="47" t="s">
-        <v>140</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="49" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B44" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A44)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D44)</f>
-        <v>3.92333333333333</v>
+        <v>2.94083333333333</v>
       </c>
       <c r="C44" s="46"/>
       <c r="D44" s="49" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="E44" s="47" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="49" t="s">
+        <v>97</v>
+      </c>
+      <c r="B45" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A45)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D45)</f>
+        <v>3.92333333333333</v>
+      </c>
+      <c r="C45" s="46"/>
+      <c r="D45" s="49" t="n">
         <v>3.9</v>
       </c>
-      <c r="E44" s="47" t="s">
+      <c r="E45" s="47" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="47" t="s">
+    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="47" t="s">
         <v>70</v>
       </c>
-      <c r="B45" s="48" t="n">
-        <f aca="false">AVERAGE(B46:B50)</f>
+      <c r="B46" s="48" t="n">
+        <f aca="false">AVERAGE(B47:B51)</f>
         <v>3.2865</v>
       </c>
-      <c r="C45" s="46"/>
-    </row>
-    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="49" t="s">
-        <v>71</v>
-      </c>
-      <c r="B46" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A46)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D46)</f>
-        <v>3.6</v>
-      </c>
-      <c r="C46" s="46" t="s">
-        <v>124</v>
-      </c>
-      <c r="D46" s="49" t="n">
-        <v>3.6</v>
-      </c>
+      <c r="C46" s="46"/>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="49" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B47" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A47)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D47)</f>
-        <v>3.33761111111111</v>
+        <v>3.6</v>
       </c>
       <c r="C47" s="46" t="s">
         <v>124</v>
       </c>
       <c r="D47" s="49" t="n">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="49" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="B48" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A48)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D48)</f>
-        <v>3.2</v>
-      </c>
-      <c r="C48" s="46"/>
+        <v>3.33761111111111</v>
+      </c>
+      <c r="C48" s="46" t="s">
+        <v>124</v>
+      </c>
       <c r="D48" s="49" t="n">
-        <v>3.2</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="49" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B49" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A49)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D49)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C49" s="46" t="s">
-        <v>130</v>
-      </c>
+        <v>3.2</v>
+      </c>
+      <c r="C49" s="46"/>
       <c r="D49" s="49" t="n">
-        <v>3.9</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="49" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="B50" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A50)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D50)</f>
+        <v>3.9</v>
+      </c>
+      <c r="C50" s="46" t="s">
+        <v>130</v>
+      </c>
+      <c r="D50" s="49" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="49" t="s">
+        <v>93</v>
+      </c>
+      <c r="B51" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A51)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D51)</f>
         <v>2.39488888888889</v>
       </c>
-      <c r="C50" s="46"/>
-      <c r="D50" s="49" t="n">
+      <c r="C51" s="46"/>
+      <c r="D51" s="49" t="n">
         <v>2.4</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="47" t="s">
+    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="47" t="s">
         <v>38</v>
       </c>
-      <c r="B51" s="48" t="n">
-        <f aca="false">AVERAGE(B52:B56)</f>
+      <c r="B52" s="48" t="n">
+        <f aca="false">AVERAGE(B53:B57)</f>
         <v>3.42807</v>
       </c>
-      <c r="C51" s="46"/>
-    </row>
-    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="49" t="s">
-        <v>49</v>
-      </c>
-      <c r="B52" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A52)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D52)</f>
-        <v>3.6</v>
-      </c>
       <c r="C52" s="46"/>
-      <c r="D52" s="49" t="n">
-        <v>3.6</v>
-      </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="49" t="s">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="B53" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A53)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D53)</f>
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
       <c r="C53" s="46"/>
       <c r="D53" s="49" t="n">
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="49" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B54" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A54)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D54)</f>
-        <v>2.7</v>
+        <v>3.8</v>
       </c>
       <c r="C54" s="46"/>
       <c r="D54" s="49" t="n">
-        <v>2.7</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="49" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="B55" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A55)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D55)</f>
-        <v>3.3</v>
+        <v>2.7</v>
       </c>
       <c r="C55" s="46"/>
       <c r="D55" s="49" t="n">
-        <v>3.3</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="49" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B56" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A56)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D56)</f>
-        <v>3.74035</v>
+        <v>3.3</v>
       </c>
       <c r="C56" s="46"/>
       <c r="D56" s="49" t="n">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="49" t="s">
+        <v>63</v>
+      </c>
+      <c r="B57" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A57)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D57)</f>
+        <v>3.74035</v>
+      </c>
+      <c r="C57" s="46"/>
+      <c r="D57" s="49" t="n">
         <v>3.7</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="47" t="s">
+    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="47" t="s">
         <v>59</v>
       </c>
-      <c r="B57" s="48" t="n">
-        <f aca="false">AVERAGE(B58:B59)</f>
+      <c r="B58" s="48" t="n">
+        <f aca="false">AVERAGE(B59:B60)</f>
         <v>3.05</v>
       </c>
-      <c r="C57" s="46"/>
-    </row>
-    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="49" t="s">
-        <v>33</v>
-      </c>
-      <c r="B58" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A58)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D58)</f>
-        <v>2.7</v>
-      </c>
       <c r="C58" s="46"/>
-      <c r="D58" s="49" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="E58" s="47" t="s">
-        <v>142</v>
-      </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="49" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="B59" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A59)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D59)</f>
-        <v>3.4</v>
+        <v>2.7</v>
       </c>
       <c r="C59" s="46"/>
       <c r="D59" s="49" t="n">
-        <v>3.4</v>
+        <v>2.7</v>
       </c>
       <c r="E59" s="47" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="49" t="s">
+        <v>69</v>
+      </c>
+      <c r="B60" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A60)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D60)</f>
+        <v>3.4</v>
+      </c>
+      <c r="C60" s="46"/>
+      <c r="D60" s="49" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="E60" s="47" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="49" t="s">
         <v>84</v>
       </c>
-      <c r="B60" s="50" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A60)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D60)</f>
-        <v>1</v>
-      </c>
-      <c r="C60" s="46"/>
-      <c r="D60" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E60" s="47" t="s">
+      <c r="B61" s="50" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A61)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D61)</f>
+        <v>1</v>
+      </c>
+      <c r="C61" s="46"/>
+      <c r="D61" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" s="47" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="47" t="s">
+    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="47" t="s">
         <v>51</v>
       </c>
-      <c r="B61" s="48" t="n">
-        <f aca="false">AVERAGE(B62:B63)</f>
+      <c r="B62" s="48" t="n">
+        <f aca="false">AVERAGE(B63:B64)</f>
         <v>2.25194444444444</v>
       </c>
-      <c r="C61" s="46"/>
-    </row>
-    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="49" t="s">
-        <v>52</v>
-      </c>
-      <c r="B62" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A62)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D62)</f>
-        <v>2.30388888888889</v>
-      </c>
       <c r="C62" s="46"/>
-      <c r="D62" s="49" t="n">
-        <v>2.5</v>
-      </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="49" t="s">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="B63" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A63)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D63)</f>
-        <v>2.2</v>
+        <v>2.30388888888889</v>
       </c>
       <c r="C63" s="46"/>
       <c r="D63" s="49" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="E63" s="47" t="s">
-        <v>145</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="49" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="B64" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A64)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D64)</f>
+        <v>2.2</v>
+      </c>
+      <c r="C64" s="46"/>
+      <c r="D64" s="49" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E64" s="47" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="49" t="s">
+        <v>96</v>
+      </c>
+      <c r="B65" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A65)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D65)</f>
         <v>2.43069444444444</v>
       </c>
-      <c r="D64" s="49" t="n">
+      <c r="D65" s="49" t="n">
         <v>2.4</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5">
+      <c r="A66" s="47" t="inlineStr">
+        <is>
+          <t>ZZTestAlex</t>
+        </is>
+      </c>
+      <c r="B66" s="48">
+        <f>AVERAGE(B67:B68)</f>
+        <v>3.1</v>
+      </c>
+      <c r="C66" s="46"/>
+    </row>
+    <row r="67" spans="1:5">
+      <c r="A67" s="49" t="inlineStr">
+        <is>
+          <t>Aragorn, the Uniter</t>
+        </is>
+      </c>
+      <c r="B67" s="49">
+        <f>IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="ZZTestAlex")*('Game Log Season 3'!$D$3:$D$1000=A67)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D67)</f>
+        <v>3.2</v>
+      </c>
+      <c r="C67" s="46"/>
+      <c r="D67" s="49">
+        <v>3.2</v>
+      </c>
+      <c r="E67" s="47" t="inlineStr">
+        <is>
+          <t>763457</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" spans="1:5">
+      <c r="A68" s="49" t="inlineStr">
+        <is>
+          <t>Kruphix, God of Horizons</t>
+        </is>
+      </c>
+      <c r="B68" s="49">
+        <f>IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="ZZTestAlex")*('Game Log Season 3'!$D$3:$D$1000=A68)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D68)</f>
+        <v>3</v>
+      </c>
+      <c r="C68" s="46"/>
+      <c r="D68" s="49">
+        <v>3</v>
+      </c>
+      <c r="E68" s="47" t="inlineStr">
+        <is>
+          <t>763449</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -26753,7 +26825,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D68"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.89"/>
@@ -27048,43 +27120,45 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="47" t="s">
+    <row r="18" spans="1:4">
+      <c r="A18" s="49" t="inlineStr">
+        <is>
+          <t>ZZ Test Batch Deck</t>
+        </is>
+      </c>
+      <c r="B18" s="49">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A18)</f>
+        <v>0</v>
+      </c>
+      <c r="C18" s="49">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A18,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="49">
+        <f>IFERROR(C18/B18,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="47" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A18)</f>
+      <c r="B19" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A19)</f>
         <v>12</v>
       </c>
-      <c r="C18" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A18,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+      <c r="C19" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A19,'Game Log Season 3'!$F$3:$F$1000,1)</f>
         <v>5</v>
       </c>
-      <c r="D18" s="48" t="n">
-        <f aca="false">IFERROR(C18/B18,0)</f>
+      <c r="D19" s="48" t="n">
+        <f aca="false">IFERROR(C19/B19,0)</f>
         <v>0.416666666666667</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="49" t="s">
-        <v>73</v>
-      </c>
-      <c r="B19" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A19)</f>
-        <v>0</v>
-      </c>
-      <c r="C19" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A19,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D19" s="49" t="n">
-        <f aca="false">IFERROR(C19/B19,0)</f>
-        <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="49" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B20" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A20)</f>
@@ -27101,11 +27175,11 @@
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="49" t="s">
-        <v>31</v>
+        <v>66</v>
       </c>
       <c r="B21" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A21)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C21" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A21,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27118,11 +27192,11 @@
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="49" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B22" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A22)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C22" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A22,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27135,7 +27209,7 @@
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="49" t="s">
-        <v>74</v>
+        <v>34</v>
       </c>
       <c r="B23" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A23)</f>
@@ -27152,7 +27226,7 @@
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="49" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="B24" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A24)</f>
@@ -27169,7 +27243,7 @@
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="49" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
       <c r="B25" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A25)</f>
@@ -27186,7 +27260,7 @@
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="49" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B26" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A26)</f>
@@ -27203,11 +27277,11 @@
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="49" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B27" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A27)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C27" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A27,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27220,7 +27294,7 @@
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="49" t="s">
-        <v>48</v>
+        <v>83</v>
       </c>
       <c r="B28" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A28)</f>
@@ -27228,122 +27302,122 @@
       </c>
       <c r="C28" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A28,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D28" s="49" t="n">
         <f aca="false">IFERROR(C28/B28,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="49" t="s">
-        <v>90</v>
+        <v>48</v>
       </c>
       <c r="B29" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A29)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C29" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A29,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D29" s="49" t="n">
         <f aca="false">IFERROR(C29/B29,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="49" t="s">
-        <v>46</v>
+        <v>90</v>
       </c>
       <c r="B30" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A30)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C30" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A30,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D30" s="49" t="n">
         <f aca="false">IFERROR(C30/B30,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="49" t="s">
-        <v>92</v>
+        <v>46</v>
       </c>
       <c r="B31" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A31)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C31" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A31,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D31" s="49" t="n">
         <f aca="false">IFERROR(C31/B31,0)</f>
-        <v>0.666666666666667</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="49" t="s">
-        <v>40</v>
+        <v>92</v>
       </c>
       <c r="B32" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A32)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C32" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A32,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" s="49" t="n">
         <f aca="false">IFERROR(C32/B32,0)</f>
-        <v>1</v>
+        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="47" t="s">
+      <c r="A33" s="49" t="s">
+        <v>40</v>
+      </c>
+      <c r="B33" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A33)</f>
+        <v>1</v>
+      </c>
+      <c r="C33" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A33,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>1</v>
+      </c>
+      <c r="D33" s="49" t="n">
+        <f aca="false">IFERROR(C33/B33,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="47" t="s">
         <v>32</v>
       </c>
-      <c r="B33" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A33)</f>
+      <c r="B34" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A34)</f>
         <v>11</v>
       </c>
-      <c r="C33" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A33,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>3</v>
-      </c>
-      <c r="D33" s="48" t="n">
-        <f aca="false">IFERROR(C33/B33,0)</f>
+      <c r="C34" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A34,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>3</v>
+      </c>
+      <c r="D34" s="48" t="n">
+        <f aca="false">IFERROR(C34/B34,0)</f>
         <v>0.272727272727273</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="49" t="s">
-        <v>36</v>
-      </c>
-      <c r="B34" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A34)</f>
-        <v>0</v>
-      </c>
-      <c r="C34" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A34,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D34" s="49" t="n">
-        <f aca="false">IFERROR(C34/B34,0)</f>
-        <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="49" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="B35" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A35)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C35" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A35,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27356,11 +27430,11 @@
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="49" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="B36" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A36)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C36" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A36,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27373,7 +27447,7 @@
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="49" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="B37" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A37)</f>
@@ -27390,24 +27464,24 @@
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="49" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="B38" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A38)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C38" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A38,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D38" s="49" t="n">
         <f aca="false">IFERROR(C38/B38,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="49" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="B39" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A39)</f>
@@ -27415,20 +27489,20 @@
       </c>
       <c r="C39" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A39,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D39" s="49" t="n">
         <f aca="false">IFERROR(C39/B39,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="49" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="B40" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A40)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C40" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A40,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27441,11 +27515,11 @@
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="49" t="s">
-        <v>87</v>
+        <v>54</v>
       </c>
       <c r="B41" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A41)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C41" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A41,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27458,11 +27532,11 @@
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="49" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B42" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A42)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C42" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A42,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27475,7 +27549,7 @@
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="49" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B43" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A43)</f>
@@ -27483,16 +27557,16 @@
       </c>
       <c r="C43" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A43,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D43" s="49" t="n">
         <f aca="false">IFERROR(C43/B43,0)</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="49" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B44" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A44)</f>
@@ -27508,46 +27582,46 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="47" t="s">
+      <c r="A45" s="49" t="s">
+        <v>97</v>
+      </c>
+      <c r="B45" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A45)</f>
+        <v>2</v>
+      </c>
+      <c r="C45" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A45,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>1</v>
+      </c>
+      <c r="D45" s="49" t="n">
+        <f aca="false">IFERROR(C45/B45,0)</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="47" t="s">
         <v>70</v>
       </c>
-      <c r="B45" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A45)</f>
-        <v>2</v>
-      </c>
-      <c r="C45" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A45,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D45" s="48" t="n">
-        <f aca="false">IFERROR(C45/B45,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="49" t="s">
-        <v>71</v>
-      </c>
-      <c r="B46" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A46)</f>
-        <v>0</v>
-      </c>
-      <c r="C46" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A46,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D46" s="49" t="n">
+      <c r="B46" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A46)</f>
+        <v>2</v>
+      </c>
+      <c r="C46" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A46,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D46" s="48" t="n">
         <f aca="false">IFERROR(C46/B46,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="49" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B47" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A47)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C47" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A47,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27560,11 +27634,11 @@
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="49" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="B48" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A48)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C48" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A48,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27577,7 +27651,7 @@
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="49" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B49" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A49)</f>
@@ -27594,11 +27668,11 @@
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="49" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="B50" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A50)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C50" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A50,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27610,42 +27684,42 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="47" t="s">
+      <c r="A51" s="49" t="s">
+        <v>93</v>
+      </c>
+      <c r="B51" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A51)</f>
+        <v>1</v>
+      </c>
+      <c r="C51" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A51,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D51" s="49" t="n">
+        <f aca="false">IFERROR(C51/B51,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="47" t="s">
         <v>38</v>
       </c>
-      <c r="B51" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A51)</f>
-        <v>1</v>
-      </c>
-      <c r="C51" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A51,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D51" s="48" t="n">
-        <f aca="false">IFERROR(C51/B51,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="49" t="s">
-        <v>49</v>
-      </c>
-      <c r="B52" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A52)</f>
-        <v>0</v>
-      </c>
-      <c r="C52" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A52,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D52" s="49" t="n">
+      <c r="B52" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A52)</f>
+        <v>1</v>
+      </c>
+      <c r="C52" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A52,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D52" s="48" t="n">
         <f aca="false">IFERROR(C52/B52,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="49" t="s">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="B53" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A53)</f>
@@ -27662,7 +27736,7 @@
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="49" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B54" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A54)</f>
@@ -27679,7 +27753,7 @@
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="49" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="B55" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A55)</f>
@@ -27696,11 +27770,11 @@
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="49" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B56" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A56)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C56" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A56,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27712,42 +27786,42 @@
       </c>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="47" t="s">
+      <c r="A57" s="49" t="s">
+        <v>63</v>
+      </c>
+      <c r="B57" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A57)</f>
+        <v>1</v>
+      </c>
+      <c r="C57" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A57,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D57" s="49" t="n">
+        <f aca="false">IFERROR(C57/B57,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="47" t="s">
         <v>59</v>
       </c>
-      <c r="B57" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A57)</f>
-        <v>0</v>
-      </c>
-      <c r="C57" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A57,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D57" s="48" t="n">
-        <f aca="false">IFERROR(C57/B57,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="49" t="s">
-        <v>33</v>
-      </c>
-      <c r="B58" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A58)</f>
-        <v>0</v>
-      </c>
-      <c r="C58" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A58,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D58" s="49" t="n">
+      <c r="B58" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A58)</f>
+        <v>0</v>
+      </c>
+      <c r="C58" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A58,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D58" s="48" t="n">
         <f aca="false">IFERROR(C58/B58,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="49" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="B59" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A59)</f>
@@ -27764,7 +27838,7 @@
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="49" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="B60" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A60)</f>
@@ -27780,46 +27854,46 @@
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="47" t="s">
+      <c r="A61" s="49" t="s">
+        <v>84</v>
+      </c>
+      <c r="B61" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A61)</f>
+        <v>0</v>
+      </c>
+      <c r="C61" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A61,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D61" s="49" t="n">
+        <f aca="false">IFERROR(C61/B61,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="47" t="s">
         <v>51</v>
       </c>
-      <c r="B61" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A61)</f>
+      <c r="B62" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A62)</f>
         <v>4</v>
       </c>
-      <c r="C61" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A61,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D61" s="48" t="n">
-        <f aca="false">IFERROR(C61/B61,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="49" t="s">
-        <v>52</v>
-      </c>
-      <c r="B62" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A62)</f>
-        <v>3</v>
-      </c>
-      <c r="C62" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A62,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D62" s="49" t="n">
+      <c r="C62" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A62,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D62" s="48" t="n">
         <f aca="false">IFERROR(C62/B62,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="49" t="s">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="B63" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A63)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C63" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A63,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27832,11 +27906,11 @@
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="49" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="B64" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A64)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C64" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A64,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27844,6 +27918,80 @@
       </c>
       <c r="D64" s="49" t="n">
         <f aca="false">IFERROR(C64/B64,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="49" t="s">
+        <v>96</v>
+      </c>
+      <c r="B65" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A65)</f>
+        <v>1</v>
+      </c>
+      <c r="C65" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A65,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D65" s="49" t="n">
+        <f aca="false">IFERROR(C65/B65,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66" s="47" t="inlineStr">
+        <is>
+          <t>ZZTestAlex</t>
+        </is>
+      </c>
+      <c r="B66" s="48">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A66)</f>
+        <v>0</v>
+      </c>
+      <c r="C66" s="48">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A66,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D66" s="48">
+        <f>IFERROR(C66/B66,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
+      <c r="A67" s="49" t="inlineStr">
+        <is>
+          <t>Aragorn, the Uniter</t>
+        </is>
+      </c>
+      <c r="B67" s="49">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"ZZTestAlex",'Game Log Season 3'!$D$3:$D$1000,A67)</f>
+        <v>0</v>
+      </c>
+      <c r="C67" s="49">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"ZZTestAlex",'Game Log Season 3'!$D$3:$D$1000,A67,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D67" s="49">
+        <f>IFERROR(C67/B67,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4">
+      <c r="A68" s="49" t="inlineStr">
+        <is>
+          <t>Kruphix, God of Horizons</t>
+        </is>
+      </c>
+      <c r="B68" s="49">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"ZZTestAlex",'Game Log Season 3'!$D$3:$D$1000,A68)</f>
+        <v>0</v>
+      </c>
+      <c r="C68" s="49">
+        <f>COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"ZZTestAlex",'Game Log Season 3'!$D$3:$D$1000,A68,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D68" s="49">
+        <f>IFERROR(C68/B68,0)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert Phase 3 test data -- apply_roster_update.py validated end to end
Confirmed via a real LibreOffice recalculation: a batch adding one new
player (2 decks) and one new deck for an existing player, in a single
pass, produced correct rows/formulas/IDs and correctly appended to
relay.js's USERNAME_TO_PLAYER. apply_roster_update.py itself stays --
only the test rows and the test relay.js entry are reverted.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deck-strength.xlsx
+++ b/deck-strength.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="884" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="161">
   <si>
     <t xml:space="preserve">Base Game Info</t>
   </si>
@@ -383,12 +383,6 @@
     <t xml:space="preserve">560535</t>
   </si>
   <si>
-    <t xml:space="preserve">ZZ Test Batch Deck</t>
-  </si>
-  <si>
-    <t xml:space="preserve">999003</t>
-  </si>
-  <si>
     <t xml:space="preserve">639396</t>
   </si>
   <si>
@@ -474,15 +468,6 @@
   </si>
   <si>
     <t xml:space="preserve">576574</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZZTestAlex</t>
-  </si>
-  <si>
-    <t xml:space="preserve">763457</t>
-  </si>
-  <si>
-    <t xml:space="preserve">763449</t>
   </si>
   <si>
     <t xml:space="preserve">Player / Deck</t>
@@ -25796,7 +25781,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40.33"/>
@@ -25898,8 +25883,8 @@
         <v>28</v>
       </c>
       <c r="B7" s="48" t="n">
-        <f aca="false">AVERAGE(B8:B18)</f>
-        <v>3.23983585858586</v>
+        <f aca="false">AVERAGE(B8:B17)</f>
+        <v>3.28381944444444</v>
       </c>
       <c r="C7" s="46"/>
     </row>
@@ -26068,153 +26053,155 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="49" t="s">
+      <c r="A18" s="47" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="48" t="n">
+        <f aca="false">AVERAGE(B19:B32)</f>
+        <v>3.31464285714286</v>
+      </c>
+      <c r="C18" s="46"/>
+    </row>
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="49" t="s">
+        <v>73</v>
+      </c>
+      <c r="B19" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A19)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D19)</f>
+        <v>2.4</v>
+      </c>
+      <c r="C19" s="46"/>
+      <c r="D19" s="49" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E19" s="47" t="s">
         <v>117</v>
       </c>
-      <c r="B18" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A18)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D18)</f>
-        <v>2.8</v>
-      </c>
-      <c r="C18" s="46"/>
-      <c r="D18" s="49" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="E18" s="47" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="47" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" s="48" t="n">
-        <f aca="false">AVERAGE(B20:B33)</f>
-        <v>3.31464285714286</v>
-      </c>
-      <c r="C19" s="46"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="49" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="B20" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A20)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D20)</f>
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="C20" s="46"/>
       <c r="D20" s="49" t="n">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="E20" s="47" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="49" t="s">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="B21" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A21)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D21)</f>
-        <v>2.6</v>
+        <v>3.57402777777778</v>
       </c>
       <c r="C21" s="46"/>
       <c r="D21" s="49" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="E21" s="47" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="49" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B22" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A22)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D22)</f>
-        <v>3.57402777777778</v>
+        <v>3.6</v>
       </c>
       <c r="C22" s="46"/>
       <c r="D22" s="49" t="n">
         <v>3.6</v>
       </c>
       <c r="E22" s="47" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="49" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="B23" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A23)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D23)</f>
-        <v>3.6</v>
+        <v>2.9</v>
       </c>
       <c r="C23" s="46"/>
       <c r="D23" s="49" t="n">
-        <v>3.6</v>
+        <v>2.9</v>
       </c>
       <c r="E23" s="47" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="49" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="B24" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A24)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D24)</f>
-        <v>2.9</v>
-      </c>
-      <c r="C24" s="46"/>
+        <v>3.9</v>
+      </c>
+      <c r="C24" s="46" t="s">
+        <v>103</v>
+      </c>
       <c r="D24" s="49" t="n">
-        <v>2.9</v>
+        <v>3.9</v>
       </c>
       <c r="E24" s="47" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="49" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="B25" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A25)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D25)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C25" s="46" t="s">
-        <v>103</v>
-      </c>
+        <v>2.8</v>
+      </c>
+      <c r="C25" s="46"/>
       <c r="D25" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E25" s="47" t="s">
-        <v>124</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="49" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B26" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A26)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D26)</f>
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="C26" s="46"/>
       <c r="D26" s="49" t="n">
-        <v>2.8</v>
+        <v>2.6</v>
+      </c>
+      <c r="E26" s="47" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="49" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B27" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A27)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D27)</f>
-        <v>2.6</v>
-      </c>
-      <c r="C27" s="46"/>
+        <v>3.59875</v>
+      </c>
+      <c r="C27" s="46" t="s">
+        <v>124</v>
+      </c>
       <c r="D27" s="49" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="E27" s="47" t="s">
         <v>125</v>
@@ -26222,592 +26209,532 @@
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="49" t="s">
-        <v>83</v>
+        <v>48</v>
       </c>
       <c r="B28" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A28)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D28)</f>
-        <v>3.59875</v>
-      </c>
-      <c r="C28" s="46" t="s">
+        <v>3.94083333333333</v>
+      </c>
+      <c r="C28" s="46"/>
+      <c r="D28" s="49" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="E28" s="47" t="s">
         <v>126</v>
-      </c>
-      <c r="D28" s="49" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="E28" s="47" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="49" t="s">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="B29" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A29)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D29)</f>
-        <v>3.94083333333333</v>
+        <v>3.65388888888889</v>
       </c>
       <c r="C29" s="46"/>
       <c r="D29" s="49" t="n">
-        <v>3.9</v>
+        <v>3.7</v>
       </c>
       <c r="E29" s="47" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="49" t="s">
-        <v>90</v>
-      </c>
-      <c r="B30" s="49" t="n">
+        <v>46</v>
+      </c>
+      <c r="B30" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A30)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D30)</f>
-        <v>3.65388888888889</v>
+        <v>3.95583333333333</v>
       </c>
       <c r="C30" s="46"/>
-      <c r="D30" s="49" t="n">
-        <v>3.7</v>
+      <c r="D30" s="50" t="n">
+        <v>4</v>
       </c>
       <c r="E30" s="47" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="49" t="s">
-        <v>46</v>
+        <v>92</v>
       </c>
       <c r="B31" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A31)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D31)</f>
-        <v>3.95583333333333</v>
+        <v>2.94666666666667</v>
       </c>
       <c r="C31" s="46"/>
       <c r="D31" s="50" t="n">
-        <v>4</v>
+        <v>2.9</v>
       </c>
       <c r="E31" s="47" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="49" t="s">
-        <v>92</v>
+        <v>40</v>
       </c>
       <c r="B32" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A32)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D32)</f>
-        <v>2.94666666666667</v>
-      </c>
-      <c r="C32" s="46"/>
+        <v>3.935</v>
+      </c>
+      <c r="C32" s="46" t="s">
+        <v>130</v>
+      </c>
       <c r="D32" s="50" t="n">
-        <v>2.9</v>
+        <v>3.9</v>
       </c>
       <c r="E32" s="47" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="49" t="s">
-        <v>40</v>
-      </c>
-      <c r="B33" s="50" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A33)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D33)</f>
-        <v>3.935</v>
-      </c>
-      <c r="C33" s="46" t="s">
+    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" s="48" t="n">
+        <f aca="false">AVERAGE(B34:B44)</f>
+        <v>3.26275505050505</v>
+      </c>
+      <c r="C33" s="46"/>
+    </row>
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="49" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A34)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D34)</f>
+        <v>3.5</v>
+      </c>
+      <c r="C34" s="46"/>
+      <c r="D34" s="49" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E34" s="47" t="s">
         <v>132</v>
       </c>
-      <c r="D33" s="50" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E33" s="47" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="47" t="s">
-        <v>32</v>
-      </c>
-      <c r="B34" s="48" t="n">
-        <f aca="false">AVERAGE(B35:B45)</f>
-        <v>3.26275505050505</v>
-      </c>
-      <c r="C34" s="46"/>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="49" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="B35" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A35)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D35)</f>
-        <v>3.5</v>
+        <v>3.43088888888889</v>
       </c>
       <c r="C35" s="46"/>
       <c r="D35" s="49" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="E35" s="47" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="49" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="B36" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A36)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D36)</f>
-        <v>3.43088888888889</v>
+        <v>3.7</v>
       </c>
       <c r="C36" s="46"/>
       <c r="D36" s="49" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="E36" s="47" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="49" t="s">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="B37" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A37)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D37)</f>
-        <v>3.7</v>
+        <v>2.6</v>
       </c>
       <c r="C37" s="46"/>
       <c r="D37" s="49" t="n">
-        <v>3.7</v>
+        <v>2.6</v>
       </c>
       <c r="E37" s="47" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="49" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="B38" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A38)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D38)</f>
-        <v>2.6</v>
+        <v>3.77816666666667</v>
       </c>
       <c r="C38" s="46"/>
       <c r="D38" s="49" t="n">
-        <v>2.6</v>
+        <v>3.8</v>
       </c>
       <c r="E38" s="47" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="49" t="s">
-        <v>41</v>
+        <v>79</v>
       </c>
       <c r="B39" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A39)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D39)</f>
-        <v>3.77816666666667</v>
+        <v>2.59388888888889</v>
       </c>
       <c r="C39" s="46"/>
       <c r="D39" s="49" t="n">
-        <v>3.8</v>
+        <v>2.6</v>
       </c>
       <c r="E39" s="47" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="49" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="B40" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A40)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D40)</f>
-        <v>2.59388888888889</v>
+        <v>3.23902777777778</v>
       </c>
       <c r="C40" s="46"/>
       <c r="D40" s="49" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="E40" s="47" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="49" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="B41" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A41)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D41)</f>
-        <v>3.23902777777778</v>
+        <v>2.6</v>
       </c>
       <c r="C41" s="46"/>
       <c r="D41" s="49" t="n">
-        <v>3.6</v>
+        <v>2.6</v>
       </c>
       <c r="E41" s="47" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="49" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B42" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A42)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D42)</f>
-        <v>2.6</v>
+        <v>3.58416666666667</v>
       </c>
       <c r="C42" s="46"/>
       <c r="D42" s="49" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="E42" s="47" t="s">
-        <v>141</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="49" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B43" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A43)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D43)</f>
-        <v>3.58416666666667</v>
+        <v>2.94083333333333</v>
       </c>
       <c r="C43" s="46"/>
       <c r="D43" s="49" t="n">
-        <v>3.6</v>
+        <v>2.9</v>
+      </c>
+      <c r="E43" s="47" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="49" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B44" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A44)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D44)</f>
-        <v>2.94083333333333</v>
+        <v>3.92333333333333</v>
       </c>
       <c r="C44" s="46"/>
       <c r="D44" s="49" t="n">
-        <v>2.9</v>
+        <v>3.9</v>
       </c>
       <c r="E44" s="47" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="49" t="s">
-        <v>97</v>
-      </c>
-      <c r="B45" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A45)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D45)</f>
-        <v>3.92333333333333</v>
+      <c r="A45" s="47" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45" s="48" t="n">
+        <f aca="false">AVERAGE(B46:B50)</f>
+        <v>3.2865</v>
       </c>
       <c r="C45" s="46"/>
-      <c r="D45" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E45" s="47" t="s">
-        <v>143</v>
-      </c>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="47" t="s">
-        <v>70</v>
-      </c>
-      <c r="B46" s="48" t="n">
-        <f aca="false">AVERAGE(B47:B51)</f>
-        <v>3.2865</v>
-      </c>
-      <c r="C46" s="46"/>
+      <c r="A46" s="49" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A46)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D46)</f>
+        <v>3.6</v>
+      </c>
+      <c r="C46" s="46" t="s">
+        <v>124</v>
+      </c>
+      <c r="D46" s="49" t="n">
+        <v>3.6</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="49" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="B47" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A47)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D47)</f>
-        <v>3.6</v>
+        <v>3.33761111111111</v>
       </c>
       <c r="C47" s="46" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D47" s="49" t="n">
-        <v>3.6</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="49" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="B48" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A48)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D48)</f>
-        <v>3.33761111111111</v>
-      </c>
-      <c r="C48" s="46" t="s">
-        <v>126</v>
-      </c>
+        <v>3.2</v>
+      </c>
+      <c r="C48" s="46"/>
       <c r="D48" s="49" t="n">
-        <v>3.3</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="49" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B49" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A49)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D49)</f>
-        <v>3.2</v>
-      </c>
-      <c r="C49" s="46"/>
+        <v>3.9</v>
+      </c>
+      <c r="C49" s="46" t="s">
+        <v>130</v>
+      </c>
       <c r="D49" s="49" t="n">
-        <v>3.2</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="49" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B50" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A50)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D50)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C50" s="46" t="s">
-        <v>132</v>
-      </c>
+        <v>2.39488888888889</v>
+      </c>
+      <c r="C50" s="46"/>
       <c r="D50" s="49" t="n">
-        <v>3.9</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="49" t="s">
-        <v>93</v>
-      </c>
-      <c r="B51" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A51)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D51)</f>
-        <v>2.39488888888889</v>
+      <c r="A51" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="B51" s="48" t="n">
+        <f aca="false">AVERAGE(B52:B56)</f>
+        <v>3.42807</v>
       </c>
       <c r="C51" s="46"/>
-      <c r="D51" s="49" t="n">
-        <v>2.4</v>
-      </c>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="47" t="s">
-        <v>38</v>
-      </c>
-      <c r="B52" s="48" t="n">
-        <f aca="false">AVERAGE(B53:B57)</f>
-        <v>3.42807</v>
+      <c r="A52" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="B52" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A52)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D52)</f>
+        <v>3.6</v>
       </c>
       <c r="C52" s="46"/>
+      <c r="D52" s="49" t="n">
+        <v>3.6</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="49" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="B53" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A53)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D53)</f>
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
       <c r="C53" s="46"/>
       <c r="D53" s="49" t="n">
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="49" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B54" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A54)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D54)</f>
-        <v>3.8</v>
+        <v>2.7</v>
       </c>
       <c r="C54" s="46"/>
       <c r="D54" s="49" t="n">
-        <v>3.8</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="49" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="B55" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A55)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D55)</f>
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
       <c r="C55" s="46"/>
       <c r="D55" s="49" t="n">
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B56" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A56)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D56)</f>
-        <v>3.3</v>
+        <v>3.74035</v>
       </c>
       <c r="C56" s="46"/>
       <c r="D56" s="49" t="n">
-        <v>3.3</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="49" t="s">
-        <v>63</v>
-      </c>
-      <c r="B57" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A57)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D57)</f>
-        <v>3.74035</v>
+      <c r="A57" s="47" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="48" t="n">
+        <f aca="false">AVERAGE(B58:B59)</f>
+        <v>3.05</v>
       </c>
       <c r="C57" s="46"/>
-      <c r="D57" s="49" t="n">
-        <v>3.7</v>
-      </c>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="47" t="s">
-        <v>59</v>
-      </c>
-      <c r="B58" s="48" t="n">
-        <f aca="false">AVERAGE(B59:B60)</f>
-        <v>3.05</v>
+      <c r="A58" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="B58" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A58)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D58)</f>
+        <v>2.7</v>
       </c>
       <c r="C58" s="46"/>
+      <c r="D58" s="49" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E58" s="47" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="49" t="s">
-        <v>33</v>
+        <v>69</v>
       </c>
       <c r="B59" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A59)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D59)</f>
-        <v>2.7</v>
+        <v>3.4</v>
       </c>
       <c r="C59" s="46"/>
       <c r="D59" s="49" t="n">
-        <v>2.7</v>
+        <v>3.4</v>
       </c>
       <c r="E59" s="47" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="49" t="s">
-        <v>69</v>
-      </c>
-      <c r="B60" s="49" t="n">
+        <v>84</v>
+      </c>
+      <c r="B60" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A60)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D60)</f>
-        <v>3.4</v>
+        <v>1</v>
       </c>
       <c r="C60" s="46"/>
-      <c r="D60" s="49" t="n">
-        <v>3.4</v>
+      <c r="D60" s="50" t="n">
+        <v>1</v>
       </c>
       <c r="E60" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="49" t="s">
-        <v>84</v>
-      </c>
-      <c r="B61" s="50" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A61)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D61)</f>
-        <v>1</v>
+      <c r="A61" s="47" t="s">
+        <v>51</v>
+      </c>
+      <c r="B61" s="48" t="n">
+        <f aca="false">AVERAGE(B62:B63)</f>
+        <v>2.25194444444444</v>
       </c>
       <c r="C61" s="46"/>
-      <c r="D61" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E61" s="47" t="s">
-        <v>146</v>
-      </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="47" t="s">
-        <v>51</v>
-      </c>
-      <c r="B62" s="48" t="n">
-        <f aca="false">AVERAGE(B63:B64)</f>
-        <v>2.25194444444444</v>
+      <c r="A62" s="49" t="s">
+        <v>52</v>
+      </c>
+      <c r="B62" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A62)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D62)</f>
+        <v>2.30388888888889</v>
       </c>
       <c r="C62" s="46"/>
+      <c r="D62" s="49" t="n">
+        <v>2.5</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="49" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B63" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A63)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D63)</f>
-        <v>2.30388888888889</v>
+        <v>2.2</v>
       </c>
       <c r="C63" s="46"/>
       <c r="D63" s="49" t="n">
-        <v>2.5</v>
+        <v>2.2</v>
+      </c>
+      <c r="E63" s="47" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="49" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="B64" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A64)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D64)</f>
-        <v>2.2</v>
-      </c>
-      <c r="C64" s="46"/>
+        <v>2.43069444444444</v>
+      </c>
       <c r="D64" s="49" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="E64" s="47" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="49" t="s">
-        <v>96</v>
-      </c>
-      <c r="B65" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A65)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D65)</f>
-        <v>2.43069444444444</v>
-      </c>
-      <c r="D65" s="49" t="n">
         <v>2.4</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="47" t="s">
-        <v>148</v>
-      </c>
-      <c r="B66" s="48" t="n">
-        <f aca="false">AVERAGE(B67:B68)</f>
-        <v>3.1</v>
-      </c>
-      <c r="C66" s="46"/>
-    </row>
-    <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="49" t="s">
-        <v>37</v>
-      </c>
-      <c r="B67" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="ZZTestAlex")*('Game Log Season 3'!$D$3:$D$1000=A67)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D67)</f>
-        <v>3.2</v>
-      </c>
-      <c r="C67" s="46"/>
-      <c r="D67" s="49" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="E67" s="47" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="49" t="s">
-        <v>91</v>
-      </c>
-      <c r="B68" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="ZZTestAlex")*('Game Log Season 3'!$D$3:$D$1000=A68)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D68)</f>
-        <v>3</v>
-      </c>
-      <c r="C68" s="46"/>
-      <c r="D68" s="49" t="n">
-        <v>3</v>
-      </c>
-      <c r="E68" s="47" t="s">
-        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -26826,7 +26753,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D68"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.89"/>
@@ -26837,16 +26764,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="45" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="B1" s="45" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="C1" s="45" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="D1" s="45" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27122,42 +27049,42 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="49" t="s">
-        <v>117</v>
-      </c>
-      <c r="B18" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A18)</f>
-        <v>0</v>
-      </c>
-      <c r="C18" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A18,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D18" s="49" t="n">
+      <c r="A18" s="47" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A18)</f>
+        <v>12</v>
+      </c>
+      <c r="C18" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A18,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>5</v>
+      </c>
+      <c r="D18" s="48" t="n">
         <f aca="false">IFERROR(C18/B18,0)</f>
-        <v>0</v>
+        <v>0.416666666666667</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="47" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A19)</f>
-        <v>12</v>
-      </c>
-      <c r="C19" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A19,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>5</v>
-      </c>
-      <c r="D19" s="48" t="n">
+      <c r="A19" s="49" t="s">
+        <v>73</v>
+      </c>
+      <c r="B19" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A19)</f>
+        <v>0</v>
+      </c>
+      <c r="C19" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A19,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D19" s="49" t="n">
         <f aca="false">IFERROR(C19/B19,0)</f>
-        <v>0.416666666666667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="49" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="B20" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A20)</f>
@@ -27174,11 +27101,11 @@
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="49" t="s">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="B21" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A21)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C21" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A21,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27191,11 +27118,11 @@
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="49" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B22" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A22)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C22" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A22,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27208,7 +27135,7 @@
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="49" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="B23" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A23)</f>
@@ -27225,7 +27152,7 @@
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="49" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="B24" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A24)</f>
@@ -27242,7 +27169,7 @@
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="49" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="B25" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A25)</f>
@@ -27259,7 +27186,7 @@
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="49" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B26" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A26)</f>
@@ -27276,11 +27203,11 @@
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="49" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B27" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A27)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C27" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A27,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27293,7 +27220,7 @@
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="49" t="s">
-        <v>83</v>
+        <v>48</v>
       </c>
       <c r="B28" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A28)</f>
@@ -27301,122 +27228,122 @@
       </c>
       <c r="C28" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A28,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D28" s="49" t="n">
         <f aca="false">IFERROR(C28/B28,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="49" t="s">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="B29" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A29)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C29" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A29,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D29" s="49" t="n">
         <f aca="false">IFERROR(C29/B29,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="49" t="s">
-        <v>90</v>
+        <v>46</v>
       </c>
       <c r="B30" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A30)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C30" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A30,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D30" s="49" t="n">
         <f aca="false">IFERROR(C30/B30,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="49" t="s">
-        <v>46</v>
+        <v>92</v>
       </c>
       <c r="B31" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A31)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C31" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A31,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D31" s="49" t="n">
         <f aca="false">IFERROR(C31/B31,0)</f>
-        <v>1</v>
+        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="49" t="s">
-        <v>92</v>
+        <v>40</v>
       </c>
       <c r="B32" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A32)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C32" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A32,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D32" s="49" t="n">
         <f aca="false">IFERROR(C32/B32,0)</f>
-        <v>0.666666666666667</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="49" t="s">
-        <v>40</v>
-      </c>
-      <c r="B33" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A33)</f>
-        <v>1</v>
-      </c>
-      <c r="C33" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A33,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
-      </c>
-      <c r="D33" s="49" t="n">
+      <c r="A33" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A33)</f>
+        <v>11</v>
+      </c>
+      <c r="C33" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A33,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>3</v>
+      </c>
+      <c r="D33" s="48" t="n">
         <f aca="false">IFERROR(C33/B33,0)</f>
-        <v>1</v>
+        <v>0.272727272727273</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="47" t="s">
-        <v>32</v>
-      </c>
-      <c r="B34" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A34)</f>
-        <v>11</v>
-      </c>
-      <c r="C34" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A34,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>3</v>
-      </c>
-      <c r="D34" s="48" t="n">
+      <c r="A34" s="49" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A34)</f>
+        <v>0</v>
+      </c>
+      <c r="C34" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A34,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D34" s="49" t="n">
         <f aca="false">IFERROR(C34/B34,0)</f>
-        <v>0.272727272727273</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="49" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="B35" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A35)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C35" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A35,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27429,11 +27356,11 @@
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="49" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="B36" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A36)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C36" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A36,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27446,7 +27373,7 @@
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="49" t="s">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="B37" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A37)</f>
@@ -27463,24 +27390,24 @@
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="49" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="B38" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A38)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C38" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A38,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D38" s="49" t="n">
         <f aca="false">IFERROR(C38/B38,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="49" t="s">
-        <v>41</v>
+        <v>79</v>
       </c>
       <c r="B39" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A39)</f>
@@ -27488,20 +27415,20 @@
       </c>
       <c r="C39" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A39,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D39" s="49" t="n">
         <f aca="false">IFERROR(C39/B39,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="49" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="B40" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A40)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C40" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A40,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27514,11 +27441,11 @@
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="49" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="B41" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A41)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C41" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A41,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27531,11 +27458,11 @@
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="49" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B42" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A42)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C42" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A42,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27548,7 +27475,7 @@
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="49" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B43" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A43)</f>
@@ -27556,16 +27483,16 @@
       </c>
       <c r="C43" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A43,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D43" s="49" t="n">
         <f aca="false">IFERROR(C43/B43,0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="49" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B44" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A44)</f>
@@ -27581,46 +27508,46 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="49" t="s">
-        <v>97</v>
-      </c>
-      <c r="B45" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A45)</f>
-        <v>2</v>
-      </c>
-      <c r="C45" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A45,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
-      </c>
-      <c r="D45" s="49" t="n">
+      <c r="A45" s="47" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A45)</f>
+        <v>2</v>
+      </c>
+      <c r="C45" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A45,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D45" s="48" t="n">
         <f aca="false">IFERROR(C45/B45,0)</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="47" t="s">
-        <v>70</v>
-      </c>
-      <c r="B46" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A46)</f>
-        <v>2</v>
-      </c>
-      <c r="C46" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A46,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D46" s="48" t="n">
+      <c r="A46" s="49" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A46)</f>
+        <v>0</v>
+      </c>
+      <c r="C46" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A46,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D46" s="49" t="n">
         <f aca="false">IFERROR(C46/B46,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="49" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="B47" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A47)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C47" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A47,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27633,11 +27560,11 @@
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="49" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="B48" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A48)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C48" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A48,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27650,7 +27577,7 @@
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="49" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B49" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A49)</f>
@@ -27667,11 +27594,11 @@
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="49" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B50" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A50)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C50" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A50,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27683,42 +27610,42 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="49" t="s">
-        <v>93</v>
-      </c>
-      <c r="B51" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A51)</f>
-        <v>1</v>
-      </c>
-      <c r="C51" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A51,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D51" s="49" t="n">
+      <c r="A51" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="B51" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A51)</f>
+        <v>1</v>
+      </c>
+      <c r="C51" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A51,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D51" s="48" t="n">
         <f aca="false">IFERROR(C51/B51,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="47" t="s">
-        <v>38</v>
-      </c>
-      <c r="B52" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A52)</f>
-        <v>1</v>
-      </c>
-      <c r="C52" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A52,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D52" s="48" t="n">
+      <c r="A52" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="B52" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A52)</f>
+        <v>0</v>
+      </c>
+      <c r="C52" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A52,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D52" s="49" t="n">
         <f aca="false">IFERROR(C52/B52,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="49" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="B53" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A53)</f>
@@ -27735,7 +27662,7 @@
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="49" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B54" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A54)</f>
@@ -27752,7 +27679,7 @@
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="49" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="B55" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A55)</f>
@@ -27769,11 +27696,11 @@
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B56" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A56)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C56" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A56,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27785,42 +27712,42 @@
       </c>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="49" t="s">
-        <v>63</v>
-      </c>
-      <c r="B57" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A57)</f>
-        <v>1</v>
-      </c>
-      <c r="C57" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A57,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D57" s="49" t="n">
+      <c r="A57" s="47" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A57)</f>
+        <v>0</v>
+      </c>
+      <c r="C57" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A57,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D57" s="48" t="n">
         <f aca="false">IFERROR(C57/B57,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="47" t="s">
-        <v>59</v>
-      </c>
-      <c r="B58" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A58)</f>
-        <v>0</v>
-      </c>
-      <c r="C58" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A58,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D58" s="48" t="n">
+      <c r="A58" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="B58" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A58)</f>
+        <v>0</v>
+      </c>
+      <c r="C58" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A58,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D58" s="49" t="n">
         <f aca="false">IFERROR(C58/B58,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="49" t="s">
-        <v>33</v>
+        <v>69</v>
       </c>
       <c r="B59" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A59)</f>
@@ -27837,7 +27764,7 @@
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="49" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="B60" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A60)</f>
@@ -27853,46 +27780,46 @@
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="49" t="s">
-        <v>84</v>
-      </c>
-      <c r="B61" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A61)</f>
-        <v>0</v>
-      </c>
-      <c r="C61" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A61,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D61" s="49" t="n">
+      <c r="A61" s="47" t="s">
+        <v>51</v>
+      </c>
+      <c r="B61" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A61)</f>
+        <v>4</v>
+      </c>
+      <c r="C61" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A61,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D61" s="48" t="n">
         <f aca="false">IFERROR(C61/B61,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="47" t="s">
-        <v>51</v>
-      </c>
-      <c r="B62" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A62)</f>
-        <v>4</v>
-      </c>
-      <c r="C62" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A62,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D62" s="48" t="n">
+      <c r="A62" s="49" t="s">
+        <v>52</v>
+      </c>
+      <c r="B62" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A62)</f>
+        <v>3</v>
+      </c>
+      <c r="C62" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A62,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D62" s="49" t="n">
         <f aca="false">IFERROR(C62/B62,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="49" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B63" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A63)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C63" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A63,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27905,11 +27832,11 @@
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="49" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="B64" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A64)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C64" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A64,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27917,74 +27844,6 @@
       </c>
       <c r="D64" s="49" t="n">
         <f aca="false">IFERROR(C64/B64,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="49" t="s">
-        <v>96</v>
-      </c>
-      <c r="B65" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A65)</f>
-        <v>1</v>
-      </c>
-      <c r="C65" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A65,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D65" s="49" t="n">
-        <f aca="false">IFERROR(C65/B65,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="47" t="s">
-        <v>148</v>
-      </c>
-      <c r="B66" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A66)</f>
-        <v>0</v>
-      </c>
-      <c r="C66" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A66,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D66" s="48" t="n">
-        <f aca="false">IFERROR(C66/B66,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="49" t="s">
-        <v>37</v>
-      </c>
-      <c r="B67" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"ZZTestAlex",'Game Log Season 3'!$D$3:$D$1000,A67)</f>
-        <v>0</v>
-      </c>
-      <c r="C67" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"ZZTestAlex",'Game Log Season 3'!$D$3:$D$1000,A67,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D67" s="49" t="n">
-        <f aca="false">IFERROR(C67/B67,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="49" t="s">
-        <v>91</v>
-      </c>
-      <c r="B68" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"ZZTestAlex",'Game Log Season 3'!$D$3:$D$1000,A68)</f>
-        <v>0</v>
-      </c>
-      <c r="C68" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"ZZTestAlex",'Game Log Season 3'!$D$3:$D$1000,A68,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D68" s="49" t="n">
-        <f aca="false">IFERROR(C68/B68,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -28023,40 +27882,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="51" t="s">
+        <v>150</v>
+      </c>
+      <c r="B1" s="51" t="s">
+        <v>151</v>
+      </c>
+      <c r="C1" s="51" t="s">
+        <v>152</v>
+      </c>
+      <c r="D1" s="51" t="s">
+        <v>153</v>
+      </c>
+      <c r="E1" s="51" t="s">
+        <v>149</v>
+      </c>
+      <c r="F1" s="51" t="s">
+        <v>154</v>
+      </c>
+      <c r="G1" s="51" t="s">
         <v>155</v>
       </c>
-      <c r="B1" s="51" t="s">
+      <c r="H1" s="51" t="s">
         <v>156</v>
       </c>
-      <c r="C1" s="51" t="s">
+      <c r="I1" s="51" t="s">
         <v>157</v>
       </c>
-      <c r="D1" s="51" t="s">
+      <c r="J1" s="51" t="s">
         <v>158</v>
       </c>
-      <c r="E1" s="51" t="s">
-        <v>154</v>
-      </c>
-      <c r="F1" s="51" t="s">
+      <c r="K1" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="G1" s="51" t="s">
+      <c r="L1" s="51" t="s">
         <v>160</v>
-      </c>
-      <c r="H1" s="51" t="s">
-        <v>161</v>
-      </c>
-      <c r="I1" s="51" t="s">
-        <v>162</v>
-      </c>
-      <c r="J1" s="51" t="s">
-        <v>163</v>
-      </c>
-      <c r="K1" s="51" t="s">
-        <v>164</v>
-      </c>
-      <c r="L1" s="51" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Revert ZZ Test Workflow Deck -- roster-update.yml validated via a real dispatch
Manually fired a repository_dispatch event end to end: the workflow ran
apply_roster_update.py, recalculated for real, correctly determined
relay.js hadn't changed (deck-only payload, no new player), and
correctly skipped the Worker redeploy step rather than failing on the
still-missing Cloudflare secrets. The workflow itself stays -- only the
test deck is reverted.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deck-strength.xlsx
+++ b/deck-strength.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="876" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="161">
   <si>
     <t xml:space="preserve">Base Game Info</t>
   </si>
@@ -381,12 +381,6 @@
   </si>
   <si>
     <t xml:space="preserve">560535</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZZ Test Workflow Deck</t>
-  </si>
-  <si>
-    <t xml:space="preserve">999004</t>
   </si>
   <si>
     <t xml:space="preserve">639396</t>
@@ -25787,7 +25781,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40.33"/>
@@ -25889,8 +25883,8 @@
         <v>28</v>
       </c>
       <c r="B7" s="48" t="n">
-        <f aca="false">AVERAGE(B8:B18)</f>
-        <v>3.22165404040404</v>
+        <f aca="false">AVERAGE(B8:B17)</f>
+        <v>3.28381944444444</v>
       </c>
       <c r="C7" s="46"/>
     </row>
@@ -26059,153 +26053,155 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="49" t="s">
+      <c r="A18" s="47" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="48" t="n">
+        <f aca="false">AVERAGE(B19:B32)</f>
+        <v>3.31464285714286</v>
+      </c>
+      <c r="C18" s="46"/>
+    </row>
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="49" t="s">
+        <v>73</v>
+      </c>
+      <c r="B19" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A19)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D19)</f>
+        <v>2.4</v>
+      </c>
+      <c r="C19" s="46"/>
+      <c r="D19" s="49" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E19" s="47" t="s">
         <v>117</v>
       </c>
-      <c r="B18" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A18)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D18)</f>
-        <v>2.6</v>
-      </c>
-      <c r="C18" s="46"/>
-      <c r="D18" s="49" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="E18" s="47" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="47" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" s="48" t="n">
-        <f aca="false">AVERAGE(B20:B33)</f>
-        <v>3.31464285714286</v>
-      </c>
-      <c r="C19" s="46"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="49" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="B20" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A20)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D20)</f>
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="C20" s="46"/>
       <c r="D20" s="49" t="n">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="E20" s="47" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="49" t="s">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="B21" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A21)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D21)</f>
-        <v>2.6</v>
+        <v>3.57402777777778</v>
       </c>
       <c r="C21" s="46"/>
       <c r="D21" s="49" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="E21" s="47" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="49" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B22" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A22)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D22)</f>
-        <v>3.57402777777778</v>
+        <v>3.6</v>
       </c>
       <c r="C22" s="46"/>
       <c r="D22" s="49" t="n">
         <v>3.6</v>
       </c>
       <c r="E22" s="47" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="49" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="B23" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A23)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D23)</f>
-        <v>3.6</v>
+        <v>2.9</v>
       </c>
       <c r="C23" s="46"/>
       <c r="D23" s="49" t="n">
-        <v>3.6</v>
+        <v>2.9</v>
       </c>
       <c r="E23" s="47" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="49" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="B24" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A24)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D24)</f>
-        <v>2.9</v>
-      </c>
-      <c r="C24" s="46"/>
+        <v>3.9</v>
+      </c>
+      <c r="C24" s="46" t="s">
+        <v>103</v>
+      </c>
       <c r="D24" s="49" t="n">
-        <v>2.9</v>
+        <v>3.9</v>
       </c>
       <c r="E24" s="47" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="49" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="B25" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A25)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D25)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C25" s="46" t="s">
-        <v>103</v>
-      </c>
+        <v>2.8</v>
+      </c>
+      <c r="C25" s="46"/>
       <c r="D25" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E25" s="47" t="s">
-        <v>124</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="49" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B26" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A26)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D26)</f>
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="C26" s="46"/>
       <c r="D26" s="49" t="n">
-        <v>2.8</v>
+        <v>2.6</v>
+      </c>
+      <c r="E26" s="47" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="49" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B27" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A27)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D27)</f>
-        <v>2.6</v>
-      </c>
-      <c r="C27" s="46"/>
+        <v>3.59875</v>
+      </c>
+      <c r="C27" s="46" t="s">
+        <v>124</v>
+      </c>
       <c r="D27" s="49" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="E27" s="47" t="s">
         <v>125</v>
@@ -26213,549 +26209,531 @@
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="49" t="s">
-        <v>83</v>
+        <v>48</v>
       </c>
       <c r="B28" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A28)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D28)</f>
-        <v>3.59875</v>
-      </c>
-      <c r="C28" s="46" t="s">
+        <v>3.94083333333333</v>
+      </c>
+      <c r="C28" s="46"/>
+      <c r="D28" s="49" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="E28" s="47" t="s">
         <v>126</v>
-      </c>
-      <c r="D28" s="49" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="E28" s="47" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="49" t="s">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="B29" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A29)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D29)</f>
-        <v>3.94083333333333</v>
+        <v>3.65388888888889</v>
       </c>
       <c r="C29" s="46"/>
       <c r="D29" s="49" t="n">
-        <v>3.9</v>
+        <v>3.7</v>
       </c>
       <c r="E29" s="47" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="49" t="s">
-        <v>90</v>
-      </c>
-      <c r="B30" s="49" t="n">
+        <v>46</v>
+      </c>
+      <c r="B30" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A30)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D30)</f>
-        <v>3.65388888888889</v>
+        <v>3.95583333333333</v>
       </c>
       <c r="C30" s="46"/>
-      <c r="D30" s="49" t="n">
-        <v>3.7</v>
+      <c r="D30" s="50" t="n">
+        <v>4</v>
       </c>
       <c r="E30" s="47" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="49" t="s">
-        <v>46</v>
+        <v>92</v>
       </c>
       <c r="B31" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A31)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D31)</f>
-        <v>3.95583333333333</v>
+        <v>2.94666666666667</v>
       </c>
       <c r="C31" s="46"/>
       <c r="D31" s="50" t="n">
-        <v>4</v>
+        <v>2.9</v>
       </c>
       <c r="E31" s="47" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="49" t="s">
-        <v>92</v>
+        <v>40</v>
       </c>
       <c r="B32" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A32)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D32)</f>
-        <v>2.94666666666667</v>
-      </c>
-      <c r="C32" s="46"/>
+        <v>3.935</v>
+      </c>
+      <c r="C32" s="46" t="s">
+        <v>130</v>
+      </c>
       <c r="D32" s="50" t="n">
-        <v>2.9</v>
+        <v>3.9</v>
       </c>
       <c r="E32" s="47" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="49" t="s">
-        <v>40</v>
-      </c>
-      <c r="B33" s="50" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A33)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D33)</f>
-        <v>3.935</v>
-      </c>
-      <c r="C33" s="46" t="s">
+    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" s="48" t="n">
+        <f aca="false">AVERAGE(B34:B44)</f>
+        <v>3.26275505050505</v>
+      </c>
+      <c r="C33" s="46"/>
+    </row>
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="49" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A34)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D34)</f>
+        <v>3.5</v>
+      </c>
+      <c r="C34" s="46"/>
+      <c r="D34" s="49" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E34" s="47" t="s">
         <v>132</v>
       </c>
-      <c r="D33" s="50" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E33" s="47" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="47" t="s">
-        <v>32</v>
-      </c>
-      <c r="B34" s="48" t="n">
-        <f aca="false">AVERAGE(B35:B45)</f>
-        <v>3.26275505050505</v>
-      </c>
-      <c r="C34" s="46"/>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="49" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="B35" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A35)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D35)</f>
-        <v>3.5</v>
+        <v>3.43088888888889</v>
       </c>
       <c r="C35" s="46"/>
       <c r="D35" s="49" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="E35" s="47" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="49" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="B36" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A36)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D36)</f>
-        <v>3.43088888888889</v>
+        <v>3.7</v>
       </c>
       <c r="C36" s="46"/>
       <c r="D36" s="49" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="E36" s="47" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="49" t="s">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="B37" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A37)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D37)</f>
-        <v>3.7</v>
+        <v>2.6</v>
       </c>
       <c r="C37" s="46"/>
       <c r="D37" s="49" t="n">
-        <v>3.7</v>
+        <v>2.6</v>
       </c>
       <c r="E37" s="47" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="49" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="B38" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A38)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D38)</f>
-        <v>2.6</v>
+        <v>3.77816666666667</v>
       </c>
       <c r="C38" s="46"/>
       <c r="D38" s="49" t="n">
-        <v>2.6</v>
+        <v>3.8</v>
       </c>
       <c r="E38" s="47" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="49" t="s">
-        <v>41</v>
+        <v>79</v>
       </c>
       <c r="B39" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A39)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D39)</f>
-        <v>3.77816666666667</v>
+        <v>2.59388888888889</v>
       </c>
       <c r="C39" s="46"/>
       <c r="D39" s="49" t="n">
-        <v>3.8</v>
+        <v>2.6</v>
       </c>
       <c r="E39" s="47" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="49" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="B40" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A40)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D40)</f>
-        <v>2.59388888888889</v>
+        <v>3.23902777777778</v>
       </c>
       <c r="C40" s="46"/>
       <c r="D40" s="49" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="E40" s="47" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="49" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="B41" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A41)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D41)</f>
-        <v>3.23902777777778</v>
+        <v>2.6</v>
       </c>
       <c r="C41" s="46"/>
       <c r="D41" s="49" t="n">
-        <v>3.6</v>
+        <v>2.6</v>
       </c>
       <c r="E41" s="47" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="49" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B42" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A42)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D42)</f>
-        <v>2.6</v>
+        <v>3.58416666666667</v>
       </c>
       <c r="C42" s="46"/>
       <c r="D42" s="49" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="E42" s="47" t="s">
-        <v>141</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="49" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B43" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A43)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D43)</f>
-        <v>3.58416666666667</v>
+        <v>2.94083333333333</v>
       </c>
       <c r="C43" s="46"/>
       <c r="D43" s="49" t="n">
-        <v>3.6</v>
+        <v>2.9</v>
+      </c>
+      <c r="E43" s="47" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="49" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B44" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A44)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D44)</f>
-        <v>2.94083333333333</v>
+        <v>3.92333333333333</v>
       </c>
       <c r="C44" s="46"/>
       <c r="D44" s="49" t="n">
-        <v>2.9</v>
+        <v>3.9</v>
       </c>
       <c r="E44" s="47" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="49" t="s">
-        <v>97</v>
-      </c>
-      <c r="B45" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A45)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D45)</f>
-        <v>3.92333333333333</v>
+      <c r="A45" s="47" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45" s="48" t="n">
+        <f aca="false">AVERAGE(B46:B50)</f>
+        <v>3.2865</v>
       </c>
       <c r="C45" s="46"/>
-      <c r="D45" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E45" s="47" t="s">
-        <v>143</v>
-      </c>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="47" t="s">
-        <v>70</v>
-      </c>
-      <c r="B46" s="48" t="n">
-        <f aca="false">AVERAGE(B47:B51)</f>
-        <v>3.2865</v>
-      </c>
-      <c r="C46" s="46"/>
+      <c r="A46" s="49" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A46)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D46)</f>
+        <v>3.6</v>
+      </c>
+      <c r="C46" s="46" t="s">
+        <v>124</v>
+      </c>
+      <c r="D46" s="49" t="n">
+        <v>3.6</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="49" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="B47" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A47)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D47)</f>
-        <v>3.6</v>
+        <v>3.33761111111111</v>
       </c>
       <c r="C47" s="46" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D47" s="49" t="n">
-        <v>3.6</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="49" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="B48" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A48)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D48)</f>
-        <v>3.33761111111111</v>
-      </c>
-      <c r="C48" s="46" t="s">
-        <v>126</v>
-      </c>
+        <v>3.2</v>
+      </c>
+      <c r="C48" s="46"/>
       <c r="D48" s="49" t="n">
-        <v>3.3</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="49" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B49" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A49)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D49)</f>
-        <v>3.2</v>
-      </c>
-      <c r="C49" s="46"/>
+        <v>3.9</v>
+      </c>
+      <c r="C49" s="46" t="s">
+        <v>130</v>
+      </c>
       <c r="D49" s="49" t="n">
-        <v>3.2</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="49" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B50" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A50)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D50)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C50" s="46" t="s">
-        <v>132</v>
-      </c>
+        <v>2.39488888888889</v>
+      </c>
+      <c r="C50" s="46"/>
       <c r="D50" s="49" t="n">
-        <v>3.9</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="49" t="s">
-        <v>93</v>
-      </c>
-      <c r="B51" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A51)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D51)</f>
-        <v>2.39488888888889</v>
+      <c r="A51" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="B51" s="48" t="n">
+        <f aca="false">AVERAGE(B52:B56)</f>
+        <v>3.42807</v>
       </c>
       <c r="C51" s="46"/>
-      <c r="D51" s="49" t="n">
-        <v>2.4</v>
-      </c>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="47" t="s">
-        <v>38</v>
-      </c>
-      <c r="B52" s="48" t="n">
-        <f aca="false">AVERAGE(B53:B57)</f>
-        <v>3.42807</v>
+      <c r="A52" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="B52" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A52)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D52)</f>
+        <v>3.6</v>
       </c>
       <c r="C52" s="46"/>
+      <c r="D52" s="49" t="n">
+        <v>3.6</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="49" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="B53" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A53)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D53)</f>
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
       <c r="C53" s="46"/>
       <c r="D53" s="49" t="n">
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="49" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B54" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A54)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D54)</f>
-        <v>3.8</v>
+        <v>2.7</v>
       </c>
       <c r="C54" s="46"/>
       <c r="D54" s="49" t="n">
-        <v>3.8</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="49" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="B55" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A55)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D55)</f>
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
       <c r="C55" s="46"/>
       <c r="D55" s="49" t="n">
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B56" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A56)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D56)</f>
-        <v>3.3</v>
+        <v>3.74035</v>
       </c>
       <c r="C56" s="46"/>
       <c r="D56" s="49" t="n">
-        <v>3.3</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="49" t="s">
-        <v>63</v>
-      </c>
-      <c r="B57" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A57)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D57)</f>
-        <v>3.74035</v>
+      <c r="A57" s="47" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="48" t="n">
+        <f aca="false">AVERAGE(B58:B59)</f>
+        <v>3.05</v>
       </c>
       <c r="C57" s="46"/>
-      <c r="D57" s="49" t="n">
-        <v>3.7</v>
-      </c>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="47" t="s">
-        <v>59</v>
-      </c>
-      <c r="B58" s="48" t="n">
-        <f aca="false">AVERAGE(B59:B60)</f>
-        <v>3.05</v>
+      <c r="A58" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="B58" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A58)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D58)</f>
+        <v>2.7</v>
       </c>
       <c r="C58" s="46"/>
+      <c r="D58" s="49" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E58" s="47" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="49" t="s">
-        <v>33</v>
+        <v>69</v>
       </c>
       <c r="B59" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A59)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D59)</f>
-        <v>2.7</v>
+        <v>3.4</v>
       </c>
       <c r="C59" s="46"/>
       <c r="D59" s="49" t="n">
-        <v>2.7</v>
+        <v>3.4</v>
       </c>
       <c r="E59" s="47" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="49" t="s">
-        <v>69</v>
-      </c>
-      <c r="B60" s="49" t="n">
+        <v>84</v>
+      </c>
+      <c r="B60" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A60)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D60)</f>
-        <v>3.4</v>
+        <v>1</v>
       </c>
       <c r="C60" s="46"/>
-      <c r="D60" s="49" t="n">
-        <v>3.4</v>
+      <c r="D60" s="50" t="n">
+        <v>1</v>
       </c>
       <c r="E60" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="49" t="s">
-        <v>84</v>
-      </c>
-      <c r="B61" s="50" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A61)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D61)</f>
-        <v>1</v>
+      <c r="A61" s="47" t="s">
+        <v>51</v>
+      </c>
+      <c r="B61" s="48" t="n">
+        <f aca="false">AVERAGE(B62:B63)</f>
+        <v>2.25194444444444</v>
       </c>
       <c r="C61" s="46"/>
-      <c r="D61" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E61" s="47" t="s">
-        <v>146</v>
-      </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="47" t="s">
-        <v>51</v>
-      </c>
-      <c r="B62" s="48" t="n">
-        <f aca="false">AVERAGE(B63:B64)</f>
-        <v>2.25194444444444</v>
+      <c r="A62" s="49" t="s">
+        <v>52</v>
+      </c>
+      <c r="B62" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A62)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D62)</f>
+        <v>2.30388888888889</v>
       </c>
       <c r="C62" s="46"/>
+      <c r="D62" s="49" t="n">
+        <v>2.5</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="49" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B63" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A63)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D63)</f>
-        <v>2.30388888888889</v>
+        <v>2.2</v>
       </c>
       <c r="C63" s="46"/>
       <c r="D63" s="49" t="n">
-        <v>2.5</v>
+        <v>2.2</v>
+      </c>
+      <c r="E63" s="47" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="49" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="B64" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A64)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D64)</f>
-        <v>2.2</v>
-      </c>
-      <c r="C64" s="46"/>
+        <v>2.43069444444444</v>
+      </c>
       <c r="D64" s="49" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="E64" s="47" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="49" t="s">
-        <v>96</v>
-      </c>
-      <c r="B65" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A65)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D65)</f>
-        <v>2.43069444444444</v>
-      </c>
-      <c r="D65" s="49" t="n">
         <v>2.4</v>
       </c>
     </row>
@@ -26775,7 +26753,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D65"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.89"/>
@@ -26786,16 +26764,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="45" t="s">
+        <v>146</v>
+      </c>
+      <c r="B1" s="45" t="s">
+        <v>147</v>
+      </c>
+      <c r="C1" s="45" t="s">
         <v>148</v>
       </c>
-      <c r="B1" s="45" t="s">
+      <c r="D1" s="45" t="s">
         <v>149</v>
-      </c>
-      <c r="C1" s="45" t="s">
-        <v>150</v>
-      </c>
-      <c r="D1" s="45" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27071,42 +27049,42 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="49" t="s">
-        <v>117</v>
-      </c>
-      <c r="B18" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A18)</f>
-        <v>0</v>
-      </c>
-      <c r="C18" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Manny",'Game Log Season 3'!$D$3:$D$1000,A18,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D18" s="49" t="n">
+      <c r="A18" s="47" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A18)</f>
+        <v>12</v>
+      </c>
+      <c r="C18" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A18,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>5</v>
+      </c>
+      <c r="D18" s="48" t="n">
         <f aca="false">IFERROR(C18/B18,0)</f>
-        <v>0</v>
+        <v>0.416666666666667</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="47" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A19)</f>
-        <v>12</v>
-      </c>
-      <c r="C19" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A19,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>5</v>
-      </c>
-      <c r="D19" s="48" t="n">
+      <c r="A19" s="49" t="s">
+        <v>73</v>
+      </c>
+      <c r="B19" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A19)</f>
+        <v>0</v>
+      </c>
+      <c r="C19" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A19,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D19" s="49" t="n">
         <f aca="false">IFERROR(C19/B19,0)</f>
-        <v>0.416666666666667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="49" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="B20" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A20)</f>
@@ -27123,11 +27101,11 @@
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="49" t="s">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="B21" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A21)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C21" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A21,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27140,11 +27118,11 @@
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="49" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B22" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A22)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C22" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A22,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27157,7 +27135,7 @@
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="49" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="B23" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A23)</f>
@@ -27174,7 +27152,7 @@
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="49" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="B24" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A24)</f>
@@ -27191,7 +27169,7 @@
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="49" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="B25" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A25)</f>
@@ -27208,7 +27186,7 @@
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="49" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B26" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A26)</f>
@@ -27225,11 +27203,11 @@
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="49" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B27" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A27)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C27" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A27,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27242,7 +27220,7 @@
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="49" t="s">
-        <v>83</v>
+        <v>48</v>
       </c>
       <c r="B28" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A28)</f>
@@ -27250,122 +27228,122 @@
       </c>
       <c r="C28" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A28,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D28" s="49" t="n">
         <f aca="false">IFERROR(C28/B28,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="49" t="s">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="B29" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A29)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C29" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A29,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D29" s="49" t="n">
         <f aca="false">IFERROR(C29/B29,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="49" t="s">
-        <v>90</v>
+        <v>46</v>
       </c>
       <c r="B30" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A30)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C30" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A30,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D30" s="49" t="n">
         <f aca="false">IFERROR(C30/B30,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="49" t="s">
-        <v>46</v>
+        <v>92</v>
       </c>
       <c r="B31" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A31)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C31" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A31,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D31" s="49" t="n">
         <f aca="false">IFERROR(C31/B31,0)</f>
-        <v>1</v>
+        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="49" t="s">
-        <v>92</v>
+        <v>40</v>
       </c>
       <c r="B32" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A32)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C32" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A32,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D32" s="49" t="n">
         <f aca="false">IFERROR(C32/B32,0)</f>
-        <v>0.666666666666667</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="49" t="s">
-        <v>40</v>
-      </c>
-      <c r="B33" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A33)</f>
-        <v>1</v>
-      </c>
-      <c r="C33" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A33,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
-      </c>
-      <c r="D33" s="49" t="n">
+      <c r="A33" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A33)</f>
+        <v>11</v>
+      </c>
+      <c r="C33" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A33,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>3</v>
+      </c>
+      <c r="D33" s="48" t="n">
         <f aca="false">IFERROR(C33/B33,0)</f>
-        <v>1</v>
+        <v>0.272727272727273</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="47" t="s">
-        <v>32</v>
-      </c>
-      <c r="B34" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A34)</f>
-        <v>11</v>
-      </c>
-      <c r="C34" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A34,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>3</v>
-      </c>
-      <c r="D34" s="48" t="n">
+      <c r="A34" s="49" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A34)</f>
+        <v>0</v>
+      </c>
+      <c r="C34" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A34,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D34" s="49" t="n">
         <f aca="false">IFERROR(C34/B34,0)</f>
-        <v>0.272727272727273</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="49" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="B35" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A35)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C35" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A35,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27378,11 +27356,11 @@
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="49" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="B36" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A36)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C36" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A36,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27395,7 +27373,7 @@
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="49" t="s">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="B37" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A37)</f>
@@ -27412,24 +27390,24 @@
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="49" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="B38" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A38)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C38" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A38,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D38" s="49" t="n">
         <f aca="false">IFERROR(C38/B38,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="49" t="s">
-        <v>41</v>
+        <v>79</v>
       </c>
       <c r="B39" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A39)</f>
@@ -27437,20 +27415,20 @@
       </c>
       <c r="C39" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A39,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D39" s="49" t="n">
         <f aca="false">IFERROR(C39/B39,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="49" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="B40" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A40)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C40" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A40,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27463,11 +27441,11 @@
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="49" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="B41" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A41)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C41" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A41,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27480,11 +27458,11 @@
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="49" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B42" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A42)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C42" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A42,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27497,7 +27475,7 @@
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="49" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B43" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A43)</f>
@@ -27505,16 +27483,16 @@
       </c>
       <c r="C43" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A43,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D43" s="49" t="n">
         <f aca="false">IFERROR(C43/B43,0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="49" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B44" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A44)</f>
@@ -27530,46 +27508,46 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="49" t="s">
-        <v>97</v>
-      </c>
-      <c r="B45" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A45)</f>
-        <v>2</v>
-      </c>
-      <c r="C45" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A45,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
-      </c>
-      <c r="D45" s="49" t="n">
+      <c r="A45" s="47" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A45)</f>
+        <v>2</v>
+      </c>
+      <c r="C45" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A45,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D45" s="48" t="n">
         <f aca="false">IFERROR(C45/B45,0)</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="47" t="s">
-        <v>70</v>
-      </c>
-      <c r="B46" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A46)</f>
-        <v>2</v>
-      </c>
-      <c r="C46" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A46,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D46" s="48" t="n">
+      <c r="A46" s="49" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A46)</f>
+        <v>0</v>
+      </c>
+      <c r="C46" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A46,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D46" s="49" t="n">
         <f aca="false">IFERROR(C46/B46,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="49" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="B47" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A47)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C47" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A47,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27582,11 +27560,11 @@
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="49" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="B48" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A48)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C48" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A48,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27599,7 +27577,7 @@
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="49" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B49" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A49)</f>
@@ -27616,11 +27594,11 @@
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="49" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B50" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A50)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C50" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A50,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27632,42 +27610,42 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="49" t="s">
-        <v>93</v>
-      </c>
-      <c r="B51" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A51)</f>
-        <v>1</v>
-      </c>
-      <c r="C51" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A51,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D51" s="49" t="n">
+      <c r="A51" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="B51" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A51)</f>
+        <v>1</v>
+      </c>
+      <c r="C51" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A51,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D51" s="48" t="n">
         <f aca="false">IFERROR(C51/B51,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="47" t="s">
-        <v>38</v>
-      </c>
-      <c r="B52" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A52)</f>
-        <v>1</v>
-      </c>
-      <c r="C52" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A52,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D52" s="48" t="n">
+      <c r="A52" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="B52" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A52)</f>
+        <v>0</v>
+      </c>
+      <c r="C52" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A52,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D52" s="49" t="n">
         <f aca="false">IFERROR(C52/B52,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="49" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="B53" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A53)</f>
@@ -27684,7 +27662,7 @@
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="49" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B54" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A54)</f>
@@ -27701,7 +27679,7 @@
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="49" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="B55" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A55)</f>
@@ -27718,11 +27696,11 @@
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B56" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A56)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C56" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A56,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27734,42 +27712,42 @@
       </c>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="49" t="s">
-        <v>63</v>
-      </c>
-      <c r="B57" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A57)</f>
-        <v>1</v>
-      </c>
-      <c r="C57" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A57,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D57" s="49" t="n">
+      <c r="A57" s="47" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A57)</f>
+        <v>0</v>
+      </c>
+      <c r="C57" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A57,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D57" s="48" t="n">
         <f aca="false">IFERROR(C57/B57,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="47" t="s">
-        <v>59</v>
-      </c>
-      <c r="B58" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A58)</f>
-        <v>0</v>
-      </c>
-      <c r="C58" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A58,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D58" s="48" t="n">
+      <c r="A58" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="B58" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A58)</f>
+        <v>0</v>
+      </c>
+      <c r="C58" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A58,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D58" s="49" t="n">
         <f aca="false">IFERROR(C58/B58,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="49" t="s">
-        <v>33</v>
+        <v>69</v>
       </c>
       <c r="B59" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A59)</f>
@@ -27786,7 +27764,7 @@
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="49" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="B60" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A60)</f>
@@ -27802,46 +27780,46 @@
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="49" t="s">
-        <v>84</v>
-      </c>
-      <c r="B61" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A61)</f>
-        <v>0</v>
-      </c>
-      <c r="C61" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A61,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D61" s="49" t="n">
+      <c r="A61" s="47" t="s">
+        <v>51</v>
+      </c>
+      <c r="B61" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A61)</f>
+        <v>4</v>
+      </c>
+      <c r="C61" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A61,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D61" s="48" t="n">
         <f aca="false">IFERROR(C61/B61,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="47" t="s">
-        <v>51</v>
-      </c>
-      <c r="B62" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A62)</f>
-        <v>4</v>
-      </c>
-      <c r="C62" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A62,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D62" s="48" t="n">
+      <c r="A62" s="49" t="s">
+        <v>52</v>
+      </c>
+      <c r="B62" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A62)</f>
+        <v>3</v>
+      </c>
+      <c r="C62" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A62,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D62" s="49" t="n">
         <f aca="false">IFERROR(C62/B62,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="49" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B63" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A63)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C63" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A63,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27854,11 +27832,11 @@
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="49" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="B64" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A64)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C64" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A64,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27866,23 +27844,6 @@
       </c>
       <c r="D64" s="49" t="n">
         <f aca="false">IFERROR(C64/B64,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="49" t="s">
-        <v>96</v>
-      </c>
-      <c r="B65" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A65)</f>
-        <v>1</v>
-      </c>
-      <c r="C65" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A65,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D65" s="49" t="n">
-        <f aca="false">IFERROR(C65/B65,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -27921,40 +27882,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="51" t="s">
+        <v>150</v>
+      </c>
+      <c r="B1" s="51" t="s">
+        <v>151</v>
+      </c>
+      <c r="C1" s="51" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="51" t="s">
+      <c r="D1" s="51" t="s">
         <v>153</v>
       </c>
-      <c r="C1" s="51" t="s">
+      <c r="E1" s="51" t="s">
+        <v>149</v>
+      </c>
+      <c r="F1" s="51" t="s">
         <v>154</v>
       </c>
-      <c r="D1" s="51" t="s">
+      <c r="G1" s="51" t="s">
         <v>155</v>
       </c>
-      <c r="E1" s="51" t="s">
-        <v>151</v>
-      </c>
-      <c r="F1" s="51" t="s">
+      <c r="H1" s="51" t="s">
         <v>156</v>
       </c>
-      <c r="G1" s="51" t="s">
+      <c r="I1" s="51" t="s">
         <v>157</v>
       </c>
-      <c r="H1" s="51" t="s">
+      <c r="J1" s="51" t="s">
         <v>158</v>
       </c>
-      <c r="I1" s="51" t="s">
+      <c r="K1" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="J1" s="51" t="s">
+      <c r="L1" s="51" t="s">
         <v>160</v>
-      </c>
-      <c r="K1" s="51" t="s">
-        <v>161</v>
-      </c>
-      <c r="L1" s="51" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Remove Mateo's stale 'Leonardo, the Balance/Michelangelo, the Heart' deck row
That partner-pairing deck (playgroup ID 614175) no longer exists on
playgroup.gg -- it was split into a standalone 'Michelangelo, the
Heart' deck (ID 743883), which Update the App already correctly
detected and added as a separate new deck in the last batch. This
removes the now-orphaned old row so Pod Validator doesn't show a dead
deck alongside its replacement.

Adds scripts/remove_deck.py, the mirror-image of add_deck.py, for
future cases where a deck gets deleted/restructured on playgroup.gg.
</commit_message>
<xml_diff>
--- a/deck-strength.xlsx
+++ b/deck-strength.xlsx
@@ -25886,7 +25886,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E88"/>
+  <dimension ref="A1:E87"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40.33"/>
@@ -26226,7 +26226,7 @@
         <v>30</v>
       </c>
       <c r="B22" s="48" t="n">
-        <f aca="false">AVERAGE(B23:B40)</f>
+        <f aca="false">AVERAGE(B23:B39)</f>
         <v>3.28916666666667</v>
       </c>
       <c r="C22" s="46"/>
@@ -26249,250 +26249,250 @@
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="49" t="s">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="B24" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A24)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D24)</f>
-        <v>2.6</v>
+        <v>3.57402777777778</v>
       </c>
       <c r="C24" s="46"/>
       <c r="D24" s="49" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="E24" s="47" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="49" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B25" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A25)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D25)</f>
-        <v>3.57402777777778</v>
+        <v>3.6</v>
       </c>
       <c r="C25" s="46"/>
       <c r="D25" s="49" t="n">
         <v>3.6</v>
       </c>
       <c r="E25" s="47" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="49" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="B26" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A26)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D26)</f>
-        <v>3.6</v>
+        <v>2.9</v>
       </c>
       <c r="C26" s="46"/>
       <c r="D26" s="49" t="n">
-        <v>3.6</v>
+        <v>2.9</v>
       </c>
       <c r="E26" s="47" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="49" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="B27" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A27)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D27)</f>
-        <v>2.9</v>
-      </c>
-      <c r="C27" s="46"/>
+        <v>3.9</v>
+      </c>
+      <c r="C27" s="46" t="s">
+        <v>103</v>
+      </c>
       <c r="D27" s="49" t="n">
-        <v>2.9</v>
+        <v>3.9</v>
       </c>
       <c r="E27" s="47" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="49" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="B28" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A28)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D28)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C28" s="46" t="s">
-        <v>103</v>
-      </c>
+        <v>2.8</v>
+      </c>
+      <c r="C28" s="46"/>
       <c r="D28" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E28" s="47" t="s">
-        <v>130</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="49" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B29" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A29)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D29)</f>
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="C29" s="46"/>
       <c r="D29" s="49" t="n">
-        <v>2.8</v>
+        <v>2.6</v>
+      </c>
+      <c r="E29" s="47" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="49" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B30" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A30)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D30)</f>
-        <v>2.6</v>
-      </c>
-      <c r="C30" s="46"/>
+        <v>3.59875</v>
+      </c>
+      <c r="C30" s="46" t="s">
+        <v>132</v>
+      </c>
       <c r="D30" s="49" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="E30" s="47" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="49" t="s">
-        <v>83</v>
+        <v>48</v>
       </c>
       <c r="B31" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A31)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D31)</f>
-        <v>3.59875</v>
-      </c>
-      <c r="C31" s="46" t="s">
-        <v>132</v>
-      </c>
+        <v>3.94083333333333</v>
+      </c>
+      <c r="C31" s="46"/>
       <c r="D31" s="49" t="n">
-        <v>3.6</v>
+        <v>3.9</v>
       </c>
       <c r="E31" s="47" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="49" t="s">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="B32" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A32)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D32)</f>
-        <v>3.94083333333333</v>
+        <v>3.65388888888889</v>
       </c>
       <c r="C32" s="46"/>
       <c r="D32" s="49" t="n">
-        <v>3.9</v>
+        <v>3.7</v>
       </c>
       <c r="E32" s="47" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="49" t="s">
-        <v>90</v>
-      </c>
-      <c r="B33" s="49" t="n">
+        <v>46</v>
+      </c>
+      <c r="B33" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A33)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D33)</f>
-        <v>3.65388888888889</v>
+        <v>3.95583333333333</v>
       </c>
       <c r="C33" s="46"/>
-      <c r="D33" s="49" t="n">
-        <v>3.7</v>
+      <c r="D33" s="50" t="n">
+        <v>4</v>
       </c>
       <c r="E33" s="47" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="49" t="s">
-        <v>46</v>
+        <v>92</v>
       </c>
       <c r="B34" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A34)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D34)</f>
-        <v>3.95583333333333</v>
+        <v>2.94666666666667</v>
       </c>
       <c r="C34" s="46"/>
       <c r="D34" s="50" t="n">
-        <v>4</v>
+        <v>2.9</v>
       </c>
       <c r="E34" s="47" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="49" t="s">
-        <v>92</v>
+        <v>40</v>
       </c>
       <c r="B35" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A35)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D35)</f>
-        <v>2.94666666666667</v>
-      </c>
-      <c r="C35" s="46"/>
+        <v>3.935</v>
+      </c>
+      <c r="C35" s="46" t="s">
+        <v>138</v>
+      </c>
       <c r="D35" s="50" t="n">
-        <v>2.9</v>
+        <v>3.9</v>
       </c>
       <c r="E35" s="47" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="49" t="s">
-        <v>40</v>
-      </c>
-      <c r="B36" s="50" t="n">
+        <v>140</v>
+      </c>
+      <c r="B36" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A36)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D36)</f>
-        <v>3.935</v>
-      </c>
-      <c r="C36" s="46" t="s">
-        <v>138</v>
-      </c>
-      <c r="D36" s="50" t="n">
-        <v>3.9</v>
+        <v>3</v>
+      </c>
+      <c r="C36" s="46"/>
+      <c r="D36" s="49" t="n">
+        <v>3</v>
       </c>
       <c r="E36" s="47" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="49" t="s">
-        <v>140</v>
+        <v>93</v>
       </c>
       <c r="B37" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A37)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D37)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C37" s="46"/>
       <c r="D37" s="49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E37" s="47" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="49" t="s">
-        <v>93</v>
+        <v>143</v>
       </c>
       <c r="B38" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A38)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D38)</f>
-        <v>2</v>
+        <v>3.9</v>
       </c>
       <c r="C38" s="46"/>
       <c r="D38" s="49" t="n">
-        <v>2</v>
+        <v>3.9</v>
       </c>
       <c r="E38" s="47" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="49" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B39" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A39)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D39)</f>
@@ -26503,534 +26503,534 @@
         <v>3.9</v>
       </c>
       <c r="E39" s="47" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="49" t="s">
-        <v>145</v>
-      </c>
-      <c r="B40" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A40)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D40)</f>
-        <v>3.9</v>
+      <c r="A40" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="B40" s="48" t="n">
+        <f aca="false">AVERAGE(B41:B54)</f>
+        <v>3.33502182539683</v>
       </c>
       <c r="C40" s="46"/>
-      <c r="D40" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E40" s="47" t="s">
-        <v>146</v>
-      </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="47" t="s">
-        <v>32</v>
-      </c>
-      <c r="B41" s="48" t="n">
-        <f aca="false">AVERAGE(B42:B55)</f>
-        <v>3.33502182539683</v>
+      <c r="A41" s="49" t="s">
+        <v>36</v>
+      </c>
+      <c r="B41" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A41)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D41)</f>
+        <v>3.5</v>
       </c>
       <c r="C41" s="46"/>
+      <c r="D41" s="49" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E41" s="47" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="49" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="B42" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A42)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D42)</f>
-        <v>3.5</v>
+        <v>3.43088888888889</v>
       </c>
       <c r="C42" s="46"/>
       <c r="D42" s="49" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="E42" s="47" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="49" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="B43" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A43)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D43)</f>
-        <v>3.43088888888889</v>
+        <v>3.7</v>
       </c>
       <c r="C43" s="46"/>
       <c r="D43" s="49" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="E43" s="47" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="49" t="s">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="B44" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A44)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D44)</f>
-        <v>3.7</v>
+        <v>2.6</v>
       </c>
       <c r="C44" s="46"/>
       <c r="D44" s="49" t="n">
-        <v>3.7</v>
+        <v>2.6</v>
       </c>
       <c r="E44" s="47" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="49" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="B45" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A45)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D45)</f>
-        <v>2.6</v>
+        <v>3.77816666666667</v>
       </c>
       <c r="C45" s="46"/>
       <c r="D45" s="49" t="n">
-        <v>2.6</v>
+        <v>3.8</v>
       </c>
       <c r="E45" s="47" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="49" t="s">
-        <v>41</v>
+        <v>79</v>
       </c>
       <c r="B46" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A46)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D46)</f>
-        <v>3.77816666666667</v>
+        <v>2.59388888888889</v>
       </c>
       <c r="C46" s="46"/>
       <c r="D46" s="49" t="n">
-        <v>3.8</v>
+        <v>2.6</v>
       </c>
       <c r="E46" s="47" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="49" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="B47" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A47)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D47)</f>
-        <v>2.59388888888889</v>
+        <v>3.23902777777778</v>
       </c>
       <c r="C47" s="46"/>
       <c r="D47" s="49" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="E47" s="47" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="49" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="B48" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A48)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D48)</f>
-        <v>3.23902777777778</v>
+        <v>2.6</v>
       </c>
       <c r="C48" s="46"/>
       <c r="D48" s="49" t="n">
-        <v>3.6</v>
+        <v>2.6</v>
       </c>
       <c r="E48" s="47" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="49" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B49" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A49)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D49)</f>
-        <v>2.6</v>
+        <v>3.58416666666667</v>
       </c>
       <c r="C49" s="46"/>
       <c r="D49" s="49" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="E49" s="47" t="s">
-        <v>154</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="49" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B50" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A50)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D50)</f>
-        <v>3.58416666666667</v>
+        <v>2.94083333333333</v>
       </c>
       <c r="C50" s="46"/>
       <c r="D50" s="49" t="n">
-        <v>3.6</v>
+        <v>2.9</v>
+      </c>
+      <c r="E50" s="47" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="49" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B51" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A51)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D51)</f>
-        <v>2.94083333333333</v>
+        <v>3.92333333333333</v>
       </c>
       <c r="C51" s="46"/>
       <c r="D51" s="49" t="n">
-        <v>2.9</v>
+        <v>3.9</v>
       </c>
       <c r="E51" s="47" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="49" t="s">
-        <v>97</v>
+        <v>157</v>
       </c>
       <c r="B52" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A52)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D52)</f>
-        <v>3.92333333333333</v>
+        <v>3.7</v>
       </c>
       <c r="C52" s="46"/>
       <c r="D52" s="49" t="n">
-        <v>3.9</v>
+        <v>3.7</v>
       </c>
       <c r="E52" s="47" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="49" t="s">
-        <v>157</v>
+        <v>43</v>
       </c>
       <c r="B53" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A53)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D53)</f>
-        <v>3.7</v>
+        <v>3.2</v>
       </c>
       <c r="C53" s="46"/>
       <c r="D53" s="49" t="n">
-        <v>3.7</v>
+        <v>3.2</v>
       </c>
       <c r="E53" s="47" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="49" t="s">
-        <v>43</v>
+        <v>160</v>
       </c>
       <c r="B54" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A54)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D54)</f>
-        <v>3.2</v>
+        <v>3.9</v>
       </c>
       <c r="C54" s="46"/>
       <c r="D54" s="49" t="n">
-        <v>3.2</v>
+        <v>3.9</v>
       </c>
       <c r="E54" s="47" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="49" t="s">
-        <v>160</v>
-      </c>
-      <c r="B55" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A55)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D55)</f>
-        <v>3.9</v>
+      <c r="A55" s="47" t="s">
+        <v>70</v>
+      </c>
+      <c r="B55" s="48" t="n">
+        <f aca="false">AVERAGE(B56:B60)</f>
+        <v>3.2865</v>
       </c>
       <c r="C55" s="46"/>
-      <c r="D55" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E55" s="47" t="s">
-        <v>161</v>
-      </c>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="47" t="s">
-        <v>70</v>
-      </c>
-      <c r="B56" s="48" t="n">
-        <f aca="false">AVERAGE(B57:B61)</f>
-        <v>3.2865</v>
-      </c>
-      <c r="C56" s="46"/>
+      <c r="A56" s="49" t="s">
+        <v>71</v>
+      </c>
+      <c r="B56" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A56)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D56)</f>
+        <v>3.6</v>
+      </c>
+      <c r="C56" s="46" t="s">
+        <v>132</v>
+      </c>
+      <c r="D56" s="49" t="n">
+        <v>3.6</v>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="49" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="B57" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A57)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D57)</f>
-        <v>3.6</v>
+        <v>3.33761111111111</v>
       </c>
       <c r="C57" s="46" t="s">
         <v>132</v>
       </c>
       <c r="D57" s="49" t="n">
-        <v>3.6</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="49" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="B58" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A58)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D58)</f>
-        <v>3.33761111111111</v>
-      </c>
-      <c r="C58" s="46" t="s">
-        <v>132</v>
-      </c>
+        <v>3.2</v>
+      </c>
+      <c r="C58" s="46"/>
       <c r="D58" s="49" t="n">
-        <v>3.3</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="49" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B59" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A59)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D59)</f>
-        <v>3.2</v>
-      </c>
-      <c r="C59" s="46"/>
+        <v>3.9</v>
+      </c>
+      <c r="C59" s="46" t="s">
+        <v>138</v>
+      </c>
       <c r="D59" s="49" t="n">
-        <v>3.2</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="49" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B60" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A60)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D60)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C60" s="46" t="s">
-        <v>138</v>
-      </c>
+        <v>2.39488888888889</v>
+      </c>
+      <c r="C60" s="46"/>
       <c r="D60" s="49" t="n">
-        <v>3.9</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="49" t="s">
-        <v>93</v>
-      </c>
-      <c r="B61" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A61)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D61)</f>
-        <v>2.39488888888889</v>
+      <c r="A61" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="B61" s="48" t="n">
+        <f aca="false">AVERAGE(B62:B66)</f>
+        <v>3.42807</v>
       </c>
       <c r="C61" s="46"/>
-      <c r="D61" s="49" t="n">
-        <v>2.4</v>
-      </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="47" t="s">
-        <v>38</v>
-      </c>
-      <c r="B62" s="48" t="n">
-        <f aca="false">AVERAGE(B63:B67)</f>
-        <v>3.42807</v>
+      <c r="A62" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="B62" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A62)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D62)</f>
+        <v>3.6</v>
       </c>
       <c r="C62" s="46"/>
+      <c r="D62" s="49" t="n">
+        <v>3.6</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="49" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="B63" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A63)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D63)</f>
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
       <c r="C63" s="46"/>
       <c r="D63" s="49" t="n">
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="49" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B64" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A64)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D64)</f>
-        <v>3.8</v>
+        <v>2.7</v>
       </c>
       <c r="C64" s="46"/>
       <c r="D64" s="49" t="n">
-        <v>3.8</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="49" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="B65" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A65)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D65)</f>
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
       <c r="C65" s="46"/>
       <c r="D65" s="49" t="n">
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B66" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A66)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D66)</f>
-        <v>3.3</v>
+        <v>3.74035</v>
       </c>
       <c r="C66" s="46"/>
       <c r="D66" s="49" t="n">
-        <v>3.3</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="49" t="s">
-        <v>63</v>
-      </c>
-      <c r="B67" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A67)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D67)</f>
-        <v>3.74035</v>
+      <c r="A67" s="47" t="s">
+        <v>59</v>
+      </c>
+      <c r="B67" s="48" t="n">
+        <f aca="false">AVERAGE(B68:B69)</f>
+        <v>3.05</v>
       </c>
       <c r="C67" s="46"/>
-      <c r="D67" s="49" t="n">
-        <v>3.7</v>
-      </c>
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="47" t="s">
-        <v>59</v>
-      </c>
-      <c r="B68" s="48" t="n">
-        <f aca="false">AVERAGE(B69:B70)</f>
-        <v>3.05</v>
+      <c r="A68" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="B68" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A68)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D68)</f>
+        <v>2.7</v>
       </c>
       <c r="C68" s="46"/>
+      <c r="D68" s="49" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E68" s="47" t="s">
+        <v>162</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="49" t="s">
-        <v>33</v>
+        <v>69</v>
       </c>
       <c r="B69" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A69)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D69)</f>
-        <v>2.7</v>
+        <v>3.4</v>
       </c>
       <c r="C69" s="46"/>
       <c r="D69" s="49" t="n">
-        <v>2.7</v>
+        <v>3.4</v>
       </c>
       <c r="E69" s="47" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="49" t="s">
-        <v>69</v>
-      </c>
-      <c r="B70" s="49" t="n">
+        <v>84</v>
+      </c>
+      <c r="B70" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A70)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D70)</f>
-        <v>3.4</v>
+        <v>1</v>
       </c>
       <c r="C70" s="46"/>
-      <c r="D70" s="49" t="n">
-        <v>3.4</v>
+      <c r="D70" s="50" t="n">
+        <v>1</v>
       </c>
       <c r="E70" s="47" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="49" t="s">
-        <v>84</v>
-      </c>
-      <c r="B71" s="50" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A71)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D71)</f>
-        <v>1</v>
+      <c r="A71" s="47" t="s">
+        <v>51</v>
+      </c>
+      <c r="B71" s="48" t="n">
+        <f aca="false">AVERAGE(B72:B73)</f>
+        <v>2.25194444444444</v>
       </c>
       <c r="C71" s="46"/>
-      <c r="D71" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E71" s="47" t="s">
-        <v>164</v>
-      </c>
     </row>
     <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="47" t="s">
-        <v>51</v>
-      </c>
-      <c r="B72" s="48" t="n">
-        <f aca="false">AVERAGE(B73:B74)</f>
-        <v>2.25194444444444</v>
+      <c r="A72" s="49" t="s">
+        <v>52</v>
+      </c>
+      <c r="B72" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A72)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D72)</f>
+        <v>2.30388888888889</v>
       </c>
       <c r="C72" s="46"/>
+      <c r="D72" s="49" t="n">
+        <v>2.5</v>
+      </c>
     </row>
     <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="49" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B73" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A73)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D73)</f>
-        <v>2.30388888888889</v>
+        <v>2.2</v>
       </c>
       <c r="C73" s="46"/>
       <c r="D73" s="49" t="n">
-        <v>2.5</v>
+        <v>2.2</v>
+      </c>
+      <c r="E73" s="47" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="49" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="B74" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A74)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D74)</f>
-        <v>2.2</v>
-      </c>
-      <c r="C74" s="46"/>
+        <v>2.43069444444444</v>
+      </c>
       <c r="D74" s="49" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="E74" s="47" t="s">
-        <v>165</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="49" t="s">
-        <v>96</v>
-      </c>
-      <c r="B75" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A75)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D75)</f>
-        <v>2.43069444444444</v>
-      </c>
-      <c r="D75" s="49" t="n">
-        <v>2.4</v>
-      </c>
+      <c r="A75" s="47" t="s">
+        <v>166</v>
+      </c>
+      <c r="B75" s="48" t="n">
+        <f aca="false">AVERAGE(B76:B87)</f>
+        <v>3.88333333333333</v>
+      </c>
+      <c r="C75" s="46"/>
     </row>
     <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="47" t="s">
-        <v>166</v>
-      </c>
-      <c r="B76" s="48" t="n">
-        <f aca="false">AVERAGE(B77:B88)</f>
-        <v>3.88333333333333</v>
+      <c r="A76" s="49" t="s">
+        <v>37</v>
+      </c>
+      <c r="B76" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A76)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D76)</f>
+        <v>3.9</v>
       </c>
       <c r="C76" s="46"/>
+      <c r="D76" s="49" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="E76" s="47" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="49" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="B77" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A77)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D77)</f>
@@ -27041,12 +27041,12 @@
         <v>3.9</v>
       </c>
       <c r="E77" s="47" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="49" t="s">
-        <v>48</v>
+        <v>169</v>
       </c>
       <c r="B78" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A78)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D78)</f>
@@ -27057,12 +27057,12 @@
         <v>3.9</v>
       </c>
       <c r="E78" s="47" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="49" t="s">
-        <v>169</v>
+        <v>119</v>
       </c>
       <c r="B79" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A79)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D79)</f>
@@ -27073,12 +27073,12 @@
         <v>3.9</v>
       </c>
       <c r="E79" s="47" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="49" t="s">
-        <v>119</v>
+        <v>68</v>
       </c>
       <c r="B80" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A80)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D80)</f>
@@ -27089,12 +27089,12 @@
         <v>3.9</v>
       </c>
       <c r="E80" s="47" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="49" t="s">
-        <v>68</v>
+        <v>91</v>
       </c>
       <c r="B81" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A81)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D81)</f>
@@ -27105,44 +27105,44 @@
         <v>3.9</v>
       </c>
       <c r="E81" s="47" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="49" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="B82" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A82)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D82)</f>
-        <v>3.9</v>
+        <v>3.7</v>
       </c>
       <c r="C82" s="46"/>
       <c r="D82" s="49" t="n">
-        <v>3.9</v>
+        <v>3.7</v>
       </c>
       <c r="E82" s="47" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="49" t="s">
-        <v>82</v>
+        <v>121</v>
       </c>
       <c r="B83" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A83)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D83)</f>
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="C83" s="46"/>
       <c r="D83" s="49" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="E83" s="47" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="49" t="s">
-        <v>121</v>
+        <v>176</v>
       </c>
       <c r="B84" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A84)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D84)</f>
@@ -27153,12 +27153,12 @@
         <v>3.9</v>
       </c>
       <c r="E84" s="47" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="49" t="s">
-        <v>176</v>
+        <v>123</v>
       </c>
       <c r="B85" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A85)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D85)</f>
@@ -27169,12 +27169,12 @@
         <v>3.9</v>
       </c>
       <c r="E85" s="47" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="49" t="s">
-        <v>123</v>
+        <v>157</v>
       </c>
       <c r="B86" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A86)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D86)</f>
@@ -27185,12 +27185,12 @@
         <v>3.9</v>
       </c>
       <c r="E86" s="47" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="49" t="s">
-        <v>157</v>
+        <v>88</v>
       </c>
       <c r="B87" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A87)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D87)</f>
@@ -27201,22 +27201,6 @@
         <v>3.9</v>
       </c>
       <c r="E87" s="47" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="49" t="s">
-        <v>88</v>
-      </c>
-      <c r="B88" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A88)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D88)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C88" s="46"/>
-      <c r="D88" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E88" s="47" t="s">
         <v>180</v>
       </c>
     </row>
@@ -27236,7 +27220,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D88"/>
+  <dimension ref="A1:D87"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.89"/>
@@ -27635,11 +27619,11 @@
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="49" t="s">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="B24" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A24)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C24" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A24,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27652,11 +27636,11 @@
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="49" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B25" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A25)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C25" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A25,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27669,7 +27653,7 @@
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="49" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="B26" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A26)</f>
@@ -27686,7 +27670,7 @@
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="49" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="B27" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A27)</f>
@@ -27703,7 +27687,7 @@
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="49" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="B28" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A28)</f>
@@ -27720,7 +27704,7 @@
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="49" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B29" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A29)</f>
@@ -27737,11 +27721,11 @@
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="49" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B30" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A30)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C30" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A30,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27754,7 +27738,7 @@
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="49" t="s">
-        <v>83</v>
+        <v>48</v>
       </c>
       <c r="B31" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A31)</f>
@@ -27762,101 +27746,101 @@
       </c>
       <c r="C31" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A31,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D31" s="49" t="n">
         <f aca="false">IFERROR(C31/B31,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="49" t="s">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="B32" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A32)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C32" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A32,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D32" s="49" t="n">
         <f aca="false">IFERROR(C32/B32,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="49" t="s">
-        <v>90</v>
+        <v>46</v>
       </c>
       <c r="B33" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A33)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C33" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A33,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D33" s="49" t="n">
         <f aca="false">IFERROR(C33/B33,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="49" t="s">
-        <v>46</v>
+        <v>92</v>
       </c>
       <c r="B34" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A34)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C34" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A34,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D34" s="49" t="n">
         <f aca="false">IFERROR(C34/B34,0)</f>
-        <v>1</v>
+        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="49" t="s">
-        <v>92</v>
+        <v>40</v>
       </c>
       <c r="B35" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A35)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C35" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A35,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D35" s="49" t="n">
         <f aca="false">IFERROR(C35/B35,0)</f>
-        <v>0.666666666666667</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="49" t="s">
-        <v>40</v>
+        <v>140</v>
       </c>
       <c r="B36" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A36)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C36" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A36,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D36" s="49" t="n">
         <f aca="false">IFERROR(C36/B36,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="49" t="s">
-        <v>140</v>
+        <v>93</v>
       </c>
       <c r="B37" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A37)</f>
@@ -27873,7 +27857,7 @@
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="49" t="s">
-        <v>93</v>
+        <v>143</v>
       </c>
       <c r="B38" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A38)</f>
@@ -27890,7 +27874,7 @@
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="49" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B39" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A39)</f>
@@ -27906,46 +27890,46 @@
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="49" t="s">
-        <v>145</v>
-      </c>
-      <c r="B40" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A40)</f>
-        <v>0</v>
-      </c>
-      <c r="C40" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A40,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D40" s="49" t="n">
+      <c r="A40" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="B40" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A40)</f>
+        <v>11</v>
+      </c>
+      <c r="C40" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A40,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>3</v>
+      </c>
+      <c r="D40" s="48" t="n">
         <f aca="false">IFERROR(C40/B40,0)</f>
-        <v>0</v>
+        <v>0.272727272727273</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="47" t="s">
-        <v>32</v>
-      </c>
-      <c r="B41" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A41)</f>
-        <v>11</v>
-      </c>
-      <c r="C41" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A41,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>3</v>
-      </c>
-      <c r="D41" s="48" t="n">
+      <c r="A41" s="49" t="s">
+        <v>36</v>
+      </c>
+      <c r="B41" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A41)</f>
+        <v>0</v>
+      </c>
+      <c r="C41" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A41,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D41" s="49" t="n">
         <f aca="false">IFERROR(C41/B41,0)</f>
-        <v>0.272727272727273</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="49" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="B42" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A42)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C42" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A42,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27958,11 +27942,11 @@
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="49" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="B43" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A43)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C43" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A43,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27975,7 +27959,7 @@
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="49" t="s">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="B44" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A44)</f>
@@ -27992,24 +27976,24 @@
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="49" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="B45" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A45)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C45" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A45,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D45" s="49" t="n">
         <f aca="false">IFERROR(C45/B45,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="49" t="s">
-        <v>41</v>
+        <v>79</v>
       </c>
       <c r="B46" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A46)</f>
@@ -28017,20 +28001,20 @@
       </c>
       <c r="C46" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A46,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D46" s="49" t="n">
         <f aca="false">IFERROR(C46/B46,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="49" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="B47" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A47)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C47" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A47,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -28043,11 +28027,11 @@
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="49" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="B48" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A48)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C48" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A48,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -28060,11 +28044,11 @@
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="49" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B49" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A49)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C49" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A49,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -28077,7 +28061,7 @@
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="49" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B50" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A50)</f>
@@ -28085,16 +28069,16 @@
       </c>
       <c r="C50" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A50,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D50" s="49" t="n">
         <f aca="false">IFERROR(C50/B50,0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="49" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B51" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A51)</f>
@@ -28111,24 +28095,24 @@
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="49" t="s">
-        <v>97</v>
+        <v>157</v>
       </c>
       <c r="B52" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A52)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C52" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A52,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D52" s="49" t="n">
         <f aca="false">IFERROR(C52/B52,0)</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="49" t="s">
-        <v>157</v>
+        <v>43</v>
       </c>
       <c r="B53" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A53)</f>
@@ -28145,7 +28129,7 @@
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="49" t="s">
-        <v>43</v>
+        <v>160</v>
       </c>
       <c r="B54" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A54)</f>
@@ -28161,46 +28145,46 @@
       </c>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="49" t="s">
-        <v>160</v>
-      </c>
-      <c r="B55" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A55)</f>
-        <v>0</v>
-      </c>
-      <c r="C55" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A55,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D55" s="49" t="n">
+      <c r="A55" s="47" t="s">
+        <v>70</v>
+      </c>
+      <c r="B55" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A55)</f>
+        <v>2</v>
+      </c>
+      <c r="C55" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A55,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D55" s="48" t="n">
         <f aca="false">IFERROR(C55/B55,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="47" t="s">
-        <v>70</v>
-      </c>
-      <c r="B56" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A56)</f>
-        <v>2</v>
-      </c>
-      <c r="C56" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A56,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D56" s="48" t="n">
+      <c r="A56" s="49" t="s">
+        <v>71</v>
+      </c>
+      <c r="B56" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A56)</f>
+        <v>0</v>
+      </c>
+      <c r="C56" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A56,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D56" s="49" t="n">
         <f aca="false">IFERROR(C56/B56,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="49" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="B57" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A57)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C57" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A57,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -28213,11 +28197,11 @@
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="49" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="B58" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A58)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C58" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A58,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -28230,7 +28214,7 @@
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="49" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B59" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A59)</f>
@@ -28247,11 +28231,11 @@
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="49" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B60" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A60)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C60" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A60,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -28263,42 +28247,42 @@
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="49" t="s">
-        <v>93</v>
-      </c>
-      <c r="B61" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A61)</f>
-        <v>1</v>
-      </c>
-      <c r="C61" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A61,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D61" s="49" t="n">
+      <c r="A61" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="B61" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A61)</f>
+        <v>1</v>
+      </c>
+      <c r="C61" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A61,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D61" s="48" t="n">
         <f aca="false">IFERROR(C61/B61,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="47" t="s">
-        <v>38</v>
-      </c>
-      <c r="B62" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A62)</f>
-        <v>1</v>
-      </c>
-      <c r="C62" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A62,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D62" s="48" t="n">
+      <c r="A62" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="B62" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A62)</f>
+        <v>0</v>
+      </c>
+      <c r="C62" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A62,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D62" s="49" t="n">
         <f aca="false">IFERROR(C62/B62,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="49" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="B63" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A63)</f>
@@ -28315,7 +28299,7 @@
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="49" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B64" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A64)</f>
@@ -28332,7 +28316,7 @@
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="49" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="B65" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A65)</f>
@@ -28349,11 +28333,11 @@
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B66" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A66)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C66" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A66,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -28365,42 +28349,42 @@
       </c>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="49" t="s">
-        <v>63</v>
-      </c>
-      <c r="B67" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A67)</f>
-        <v>1</v>
-      </c>
-      <c r="C67" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A67,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D67" s="49" t="n">
+      <c r="A67" s="47" t="s">
+        <v>59</v>
+      </c>
+      <c r="B67" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A67)</f>
+        <v>0</v>
+      </c>
+      <c r="C67" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A67,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D67" s="48" t="n">
         <f aca="false">IFERROR(C67/B67,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="47" t="s">
-        <v>59</v>
-      </c>
-      <c r="B68" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A68)</f>
-        <v>0</v>
-      </c>
-      <c r="C68" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A68,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D68" s="48" t="n">
+      <c r="A68" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="B68" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A68)</f>
+        <v>0</v>
+      </c>
+      <c r="C68" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A68,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D68" s="49" t="n">
         <f aca="false">IFERROR(C68/B68,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="49" t="s">
-        <v>33</v>
+        <v>69</v>
       </c>
       <c r="B69" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A69)</f>
@@ -28417,7 +28401,7 @@
     </row>
     <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="49" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="B70" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A70)</f>
@@ -28433,46 +28417,46 @@
       </c>
     </row>
     <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="49" t="s">
-        <v>84</v>
-      </c>
-      <c r="B71" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A71)</f>
-        <v>0</v>
-      </c>
-      <c r="C71" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A71,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D71" s="49" t="n">
+      <c r="A71" s="47" t="s">
+        <v>51</v>
+      </c>
+      <c r="B71" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A71)</f>
+        <v>4</v>
+      </c>
+      <c r="C71" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A71,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D71" s="48" t="n">
         <f aca="false">IFERROR(C71/B71,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="47" t="s">
-        <v>51</v>
-      </c>
-      <c r="B72" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A72)</f>
-        <v>4</v>
-      </c>
-      <c r="C72" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A72,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D72" s="48" t="n">
+      <c r="A72" s="49" t="s">
+        <v>52</v>
+      </c>
+      <c r="B72" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A72)</f>
+        <v>3</v>
+      </c>
+      <c r="C72" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A72,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D72" s="49" t="n">
         <f aca="false">IFERROR(C72/B72,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="49" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B73" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A73)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C73" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A73,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -28485,11 +28469,11 @@
     </row>
     <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="49" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="B74" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A74)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C74" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A74,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -28501,42 +28485,42 @@
       </c>
     </row>
     <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="49" t="s">
-        <v>96</v>
-      </c>
-      <c r="B75" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A75)</f>
-        <v>1</v>
-      </c>
-      <c r="C75" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A75,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D75" s="49" t="n">
+      <c r="A75" s="47" t="s">
+        <v>166</v>
+      </c>
+      <c r="B75" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A75)</f>
+        <v>0</v>
+      </c>
+      <c r="C75" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A75,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D75" s="48" t="n">
         <f aca="false">IFERROR(C75/B75,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="47" t="s">
-        <v>166</v>
-      </c>
-      <c r="B76" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A76)</f>
-        <v>0</v>
-      </c>
-      <c r="C76" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A76,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D76" s="48" t="n">
+      <c r="A76" s="49" t="s">
+        <v>37</v>
+      </c>
+      <c r="B76" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A76)</f>
+        <v>0</v>
+      </c>
+      <c r="C76" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A76,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D76" s="49" t="n">
         <f aca="false">IFERROR(C76/B76,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="49" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="B77" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A77)</f>
@@ -28553,7 +28537,7 @@
     </row>
     <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="49" t="s">
-        <v>48</v>
+        <v>169</v>
       </c>
       <c r="B78" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A78)</f>
@@ -28570,7 +28554,7 @@
     </row>
     <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="49" t="s">
-        <v>169</v>
+        <v>119</v>
       </c>
       <c r="B79" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A79)</f>
@@ -28587,7 +28571,7 @@
     </row>
     <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="49" t="s">
-        <v>119</v>
+        <v>68</v>
       </c>
       <c r="B80" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A80)</f>
@@ -28604,7 +28588,7 @@
     </row>
     <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="49" t="s">
-        <v>68</v>
+        <v>91</v>
       </c>
       <c r="B81" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A81)</f>
@@ -28621,7 +28605,7 @@
     </row>
     <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="49" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="B82" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A82)</f>
@@ -28638,7 +28622,7 @@
     </row>
     <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="49" t="s">
-        <v>82</v>
+        <v>121</v>
       </c>
       <c r="B83" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A83)</f>
@@ -28655,7 +28639,7 @@
     </row>
     <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="49" t="s">
-        <v>121</v>
+        <v>176</v>
       </c>
       <c r="B84" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A84)</f>
@@ -28672,7 +28656,7 @@
     </row>
     <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="49" t="s">
-        <v>176</v>
+        <v>123</v>
       </c>
       <c r="B85" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A85)</f>
@@ -28689,7 +28673,7 @@
     </row>
     <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="49" t="s">
-        <v>123</v>
+        <v>157</v>
       </c>
       <c r="B86" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A86)</f>
@@ -28706,7 +28690,7 @@
     </row>
     <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="49" t="s">
-        <v>157</v>
+        <v>88</v>
       </c>
       <c r="B87" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A87)</f>
@@ -28718,23 +28702,6 @@
       </c>
       <c r="D87" s="49" t="n">
         <f aca="false">IFERROR(C87/B87,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="49" t="s">
-        <v>88</v>
-      </c>
-      <c r="B88" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A88)</f>
-        <v>0</v>
-      </c>
-      <c r="C88" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A88,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D88" s="49" t="n">
-        <f aca="false">IFERROR(C88/B88,0)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove Hiccup_The_Hero and Mateo's Michelangelo, the Heart deck
Per request. Hiccup_The_Hero (all 12 decks) removed from both sheets
and relay.js's USERNAME_TO_PLAYER again -- Worker needs a redeploy for
this to take effect. Mateo's "Michelangelo, the Heart" (playgroup ID
743883) removed as a standalone deck row.

Both verified against a scratch copy first: sheets shrink from 87 to
73 rows (13 + 1 removed), every remaining player's block stays intact
and correctly ordered, no stale references left anywhere.
</commit_message>
<xml_diff>
--- a/deck-strength.xlsx
+++ b/deck-strength.xlsx
@@ -25883,7 +25883,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E87"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40.33"/>
@@ -26223,7 +26223,7 @@
         <v>30</v>
       </c>
       <c r="B22" s="48" t="n">
-        <f aca="false">AVERAGE(B23:B39)</f>
+        <f aca="false">AVERAGE(B23:B38)</f>
         <v>3.32970588235294</v>
       </c>
       <c r="C22" s="46"/>
@@ -26488,717 +26488,499 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="49" t="s">
-        <v>144</v>
-      </c>
-      <c r="B39" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A39)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D39)</f>
-        <v>3.9</v>
+      <c r="A39" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="B39" s="48" t="n">
+        <f aca="false">AVERAGE(B40:B53)</f>
+        <v>3.33502182539683</v>
       </c>
       <c r="C39" s="46"/>
-      <c r="D39" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E39" s="47" t="s">
-        <v>145</v>
-      </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="47" t="s">
-        <v>32</v>
-      </c>
-      <c r="B40" s="48" t="n">
-        <f aca="false">AVERAGE(B41:B54)</f>
-        <v>3.33502182539683</v>
+      <c r="A40" s="49" t="s">
+        <v>36</v>
+      </c>
+      <c r="B40" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A40)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D40)</f>
+        <v>3.5</v>
       </c>
       <c r="C40" s="46"/>
+      <c r="D40" s="49" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E40" s="47" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="49" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="B41" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A41)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D41)</f>
-        <v>3.5</v>
+        <v>3.43088888888889</v>
       </c>
       <c r="C41" s="46"/>
       <c r="D41" s="49" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="E41" s="47" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="49" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="B42" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A42)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D42)</f>
-        <v>3.43088888888889</v>
+        <v>3.7</v>
       </c>
       <c r="C42" s="46"/>
       <c r="D42" s="49" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="E42" s="47" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="49" t="s">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="B43" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A43)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D43)</f>
-        <v>3.7</v>
+        <v>2.6</v>
       </c>
       <c r="C43" s="46"/>
       <c r="D43" s="49" t="n">
-        <v>3.7</v>
+        <v>2.6</v>
       </c>
       <c r="E43" s="47" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="49" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="B44" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A44)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D44)</f>
-        <v>2.6</v>
+        <v>3.77816666666667</v>
       </c>
       <c r="C44" s="46"/>
       <c r="D44" s="49" t="n">
-        <v>2.6</v>
+        <v>3.8</v>
       </c>
       <c r="E44" s="47" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="49" t="s">
-        <v>41</v>
+        <v>79</v>
       </c>
       <c r="B45" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A45)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D45)</f>
-        <v>3.77816666666667</v>
+        <v>2.59388888888889</v>
       </c>
       <c r="C45" s="46"/>
       <c r="D45" s="49" t="n">
-        <v>3.8</v>
+        <v>2.6</v>
       </c>
       <c r="E45" s="47" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="49" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="B46" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A46)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D46)</f>
-        <v>2.59388888888889</v>
+        <v>3.23902777777778</v>
       </c>
       <c r="C46" s="46"/>
       <c r="D46" s="49" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="E46" s="47" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="49" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="B47" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A47)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D47)</f>
-        <v>3.23902777777778</v>
+        <v>2.6</v>
       </c>
       <c r="C47" s="46"/>
       <c r="D47" s="49" t="n">
-        <v>3.6</v>
+        <v>2.6</v>
       </c>
       <c r="E47" s="47" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="49" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B48" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A48)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D48)</f>
-        <v>2.6</v>
+        <v>3.58416666666667</v>
       </c>
       <c r="C48" s="46"/>
       <c r="D48" s="49" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="E48" s="47" t="s">
-        <v>153</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="49" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B49" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A49)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D49)</f>
-        <v>3.58416666666667</v>
+        <v>2.94083333333333</v>
       </c>
       <c r="C49" s="46"/>
       <c r="D49" s="49" t="n">
-        <v>3.6</v>
+        <v>2.9</v>
+      </c>
+      <c r="E49" s="47" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="49" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B50" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A50)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D50)</f>
-        <v>2.94083333333333</v>
+        <v>3.92333333333333</v>
       </c>
       <c r="C50" s="46"/>
       <c r="D50" s="49" t="n">
-        <v>2.9</v>
+        <v>3.9</v>
       </c>
       <c r="E50" s="47" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="49" t="s">
-        <v>97</v>
+        <v>156</v>
       </c>
       <c r="B51" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A51)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D51)</f>
-        <v>3.92333333333333</v>
+        <v>3.7</v>
       </c>
       <c r="C51" s="46"/>
       <c r="D51" s="49" t="n">
-        <v>3.9</v>
+        <v>3.7</v>
       </c>
       <c r="E51" s="47" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="49" t="s">
-        <v>156</v>
+        <v>43</v>
       </c>
       <c r="B52" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A52)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D52)</f>
-        <v>3.7</v>
+        <v>3.2</v>
       </c>
       <c r="C52" s="46"/>
       <c r="D52" s="49" t="n">
-        <v>3.7</v>
+        <v>3.2</v>
       </c>
       <c r="E52" s="47" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="49" t="s">
-        <v>43</v>
+        <v>159</v>
       </c>
       <c r="B53" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A53)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D53)</f>
-        <v>3.2</v>
+        <v>3.9</v>
       </c>
       <c r="C53" s="46"/>
       <c r="D53" s="49" t="n">
-        <v>3.2</v>
+        <v>3.9</v>
       </c>
       <c r="E53" s="47" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="49" t="s">
-        <v>159</v>
-      </c>
-      <c r="B54" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A54)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D54)</f>
-        <v>3.9</v>
+      <c r="A54" s="47" t="s">
+        <v>70</v>
+      </c>
+      <c r="B54" s="48" t="n">
+        <f aca="false">AVERAGE(B55:B59)</f>
+        <v>3.2865</v>
       </c>
       <c r="C54" s="46"/>
-      <c r="D54" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E54" s="47" t="s">
-        <v>160</v>
-      </c>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="47" t="s">
-        <v>70</v>
-      </c>
-      <c r="B55" s="48" t="n">
-        <f aca="false">AVERAGE(B56:B60)</f>
-        <v>3.2865</v>
-      </c>
-      <c r="C55" s="46"/>
+      <c r="A55" s="49" t="s">
+        <v>71</v>
+      </c>
+      <c r="B55" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A55)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D55)</f>
+        <v>3.6</v>
+      </c>
+      <c r="C55" s="46" t="s">
+        <v>131</v>
+      </c>
+      <c r="D55" s="49" t="n">
+        <v>3.6</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="49" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="B56" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A56)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D56)</f>
-        <v>3.6</v>
+        <v>3.33761111111111</v>
       </c>
       <c r="C56" s="46" t="s">
         <v>131</v>
       </c>
       <c r="D56" s="49" t="n">
-        <v>3.6</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="49" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="B57" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A57)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D57)</f>
-        <v>3.33761111111111</v>
-      </c>
-      <c r="C57" s="46" t="s">
-        <v>131</v>
-      </c>
+        <v>3.2</v>
+      </c>
+      <c r="C57" s="46"/>
       <c r="D57" s="49" t="n">
-        <v>3.3</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="49" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B58" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A58)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D58)</f>
-        <v>3.2</v>
-      </c>
-      <c r="C58" s="46"/>
+        <v>3.9</v>
+      </c>
+      <c r="C58" s="46" t="s">
+        <v>137</v>
+      </c>
       <c r="D58" s="49" t="n">
-        <v>3.2</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="49" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B59" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A59)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D59)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C59" s="46" t="s">
-        <v>137</v>
-      </c>
+        <v>2.39488888888889</v>
+      </c>
+      <c r="C59" s="46"/>
       <c r="D59" s="49" t="n">
-        <v>3.9</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="49" t="s">
-        <v>93</v>
-      </c>
-      <c r="B60" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Kristy")*('Game Log Season 3'!$D$3:$D$1000=A60)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D60)</f>
-        <v>2.39488888888889</v>
+      <c r="A60" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="B60" s="48" t="n">
+        <f aca="false">AVERAGE(B61:B65)</f>
+        <v>3.42807</v>
       </c>
       <c r="C60" s="46"/>
-      <c r="D60" s="49" t="n">
-        <v>2.4</v>
-      </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="47" t="s">
-        <v>38</v>
-      </c>
-      <c r="B61" s="48" t="n">
-        <f aca="false">AVERAGE(B62:B66)</f>
-        <v>3.42807</v>
+      <c r="A61" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="B61" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A61)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D61)</f>
+        <v>3.6</v>
       </c>
       <c r="C61" s="46"/>
+      <c r="D61" s="49" t="n">
+        <v>3.6</v>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="49" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="B62" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A62)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D62)</f>
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
       <c r="C62" s="46"/>
       <c r="D62" s="49" t="n">
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="49" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B63" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A63)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D63)</f>
-        <v>3.8</v>
+        <v>2.7</v>
       </c>
       <c r="C63" s="46"/>
       <c r="D63" s="49" t="n">
-        <v>3.8</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="49" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="B64" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A64)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D64)</f>
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
       <c r="C64" s="46"/>
       <c r="D64" s="49" t="n">
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B65" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A65)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D65)</f>
-        <v>3.3</v>
+        <v>3.74035</v>
       </c>
       <c r="C65" s="46"/>
       <c r="D65" s="49" t="n">
-        <v>3.3</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="49" t="s">
-        <v>63</v>
-      </c>
-      <c r="B66" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Joseph")*('Game Log Season 3'!$D$3:$D$1000=A66)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D66)</f>
-        <v>3.74035</v>
+      <c r="A66" s="47" t="s">
+        <v>59</v>
+      </c>
+      <c r="B66" s="48" t="n">
+        <f aca="false">AVERAGE(B67:B68)</f>
+        <v>3.05</v>
       </c>
       <c r="C66" s="46"/>
-      <c r="D66" s="49" t="n">
-        <v>3.7</v>
-      </c>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="47" t="s">
-        <v>59</v>
-      </c>
-      <c r="B67" s="48" t="n">
-        <f aca="false">AVERAGE(B68:B69)</f>
-        <v>3.05</v>
+      <c r="A67" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="B67" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A67)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D67)</f>
+        <v>2.7</v>
       </c>
       <c r="C67" s="46"/>
+      <c r="D67" s="49" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E67" s="47" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="49" t="s">
-        <v>33</v>
+        <v>69</v>
       </c>
       <c r="B68" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A68)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D68)</f>
-        <v>2.7</v>
+        <v>3.4</v>
       </c>
       <c r="C68" s="46"/>
       <c r="D68" s="49" t="n">
-        <v>2.7</v>
+        <v>3.4</v>
       </c>
       <c r="E68" s="47" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="49" t="s">
-        <v>69</v>
-      </c>
-      <c r="B69" s="49" t="n">
+        <v>84</v>
+      </c>
+      <c r="B69" s="50" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A69)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D69)</f>
-        <v>3.4</v>
+        <v>1</v>
       </c>
       <c r="C69" s="46"/>
-      <c r="D69" s="49" t="n">
-        <v>3.4</v>
+      <c r="D69" s="50" t="n">
+        <v>1</v>
       </c>
       <c r="E69" s="47" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="49" t="s">
-        <v>84</v>
-      </c>
-      <c r="B70" s="50" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Red")*('Game Log Season 3'!$D$3:$D$1000=A70)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D70)</f>
-        <v>1</v>
+      <c r="A70" s="47" t="s">
+        <v>51</v>
+      </c>
+      <c r="B70" s="48" t="n">
+        <f aca="false">AVERAGE(B71:B72)</f>
+        <v>2.25194444444444</v>
       </c>
       <c r="C70" s="46"/>
-      <c r="D70" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E70" s="47" t="s">
-        <v>163</v>
-      </c>
     </row>
     <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="47" t="s">
-        <v>51</v>
-      </c>
-      <c r="B71" s="48" t="n">
-        <f aca="false">AVERAGE(B72:B73)</f>
-        <v>2.25194444444444</v>
+      <c r="A71" s="49" t="s">
+        <v>52</v>
+      </c>
+      <c r="B71" s="49" t="n">
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A71)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D71)</f>
+        <v>2.30388888888889</v>
       </c>
       <c r="C71" s="46"/>
+      <c r="D71" s="49" t="n">
+        <v>2.5</v>
+      </c>
     </row>
     <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="49" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B72" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A72)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D72)</f>
-        <v>2.30388888888889</v>
+        <v>2.2</v>
       </c>
       <c r="C72" s="46"/>
       <c r="D72" s="49" t="n">
-        <v>2.5</v>
+        <v>2.2</v>
+      </c>
+      <c r="E72" s="47" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="49" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="B73" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A73)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D73)</f>
-        <v>2.2</v>
-      </c>
-      <c r="C73" s="46"/>
+        <v>2.43069444444444</v>
+      </c>
       <c r="D73" s="49" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="E73" s="47" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="49" t="s">
-        <v>96</v>
-      </c>
-      <c r="B74" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Michelle")*('Game Log Season 3'!$D$3:$D$1000=A74)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D74)</f>
-        <v>2.43069444444444</v>
-      </c>
-      <c r="D74" s="49" t="n">
         <v>2.4</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="47" t="s">
-        <v>165</v>
-      </c>
-      <c r="B75" s="48" t="n">
-        <f aca="false">AVERAGE(B76:B87)</f>
-        <v>3.88333333333333</v>
-      </c>
-      <c r="C75" s="46"/>
-    </row>
-    <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="49" t="s">
-        <v>37</v>
-      </c>
-      <c r="B76" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A76)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D76)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C76" s="46"/>
-      <c r="D76" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E76" s="47" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="49" t="s">
-        <v>48</v>
-      </c>
-      <c r="B77" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A77)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D77)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C77" s="46"/>
-      <c r="D77" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E77" s="47" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="49" t="s">
-        <v>168</v>
-      </c>
-      <c r="B78" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A78)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D78)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C78" s="46"/>
-      <c r="D78" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E78" s="47" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="49" t="s">
-        <v>119</v>
-      </c>
-      <c r="B79" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A79)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D79)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C79" s="46"/>
-      <c r="D79" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E79" s="47" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="49" t="s">
-        <v>68</v>
-      </c>
-      <c r="B80" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A80)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D80)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C80" s="46"/>
-      <c r="D80" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E80" s="47" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="49" t="s">
-        <v>91</v>
-      </c>
-      <c r="B81" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A81)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D81)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C81" s="46"/>
-      <c r="D81" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E81" s="47" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="49" t="s">
-        <v>82</v>
-      </c>
-      <c r="B82" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A82)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D82)</f>
-        <v>3.7</v>
-      </c>
-      <c r="C82" s="46"/>
-      <c r="D82" s="49" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="E82" s="47" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="49" t="s">
-        <v>121</v>
-      </c>
-      <c r="B83" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A83)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D83)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C83" s="46"/>
-      <c r="D83" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E83" s="47" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="49" t="s">
-        <v>175</v>
-      </c>
-      <c r="B84" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A84)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D84)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C84" s="46"/>
-      <c r="D84" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E84" s="47" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="49" t="s">
-        <v>123</v>
-      </c>
-      <c r="B85" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A85)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D85)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C85" s="46"/>
-      <c r="D85" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E85" s="47" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="49" t="s">
-        <v>156</v>
-      </c>
-      <c r="B86" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A86)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D86)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C86" s="46"/>
-      <c r="D86" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E86" s="47" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="49" t="s">
-        <v>88</v>
-      </c>
-      <c r="B87" s="49" t="n">
-        <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Hiccup_The_Hero")*('Game Log Season 3'!$D$3:$D$1000=A87)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D87)</f>
-        <v>3.9</v>
-      </c>
-      <c r="C87" s="46"/>
-      <c r="D87" s="49" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E87" s="47" t="s">
-        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -27217,7 +26999,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D87"/>
+  <dimension ref="A1:D73"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.89"/>
@@ -27870,46 +27652,46 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="49" t="s">
-        <v>144</v>
-      </c>
-      <c r="B39" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A39)</f>
-        <v>0</v>
-      </c>
-      <c r="C39" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A39,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D39" s="49" t="n">
+      <c r="A39" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="B39" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A39)</f>
+        <v>11</v>
+      </c>
+      <c r="C39" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A39,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>3</v>
+      </c>
+      <c r="D39" s="48" t="n">
         <f aca="false">IFERROR(C39/B39,0)</f>
-        <v>0</v>
+        <v>0.272727272727273</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="47" t="s">
-        <v>32</v>
-      </c>
-      <c r="B40" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A40)</f>
-        <v>11</v>
-      </c>
-      <c r="C40" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A40,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>3</v>
-      </c>
-      <c r="D40" s="48" t="n">
+      <c r="A40" s="49" t="s">
+        <v>36</v>
+      </c>
+      <c r="B40" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A40)</f>
+        <v>0</v>
+      </c>
+      <c r="C40" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A40,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D40" s="49" t="n">
         <f aca="false">IFERROR(C40/B40,0)</f>
-        <v>0.272727272727273</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="49" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="B41" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A41)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C41" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A41,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27922,11 +27704,11 @@
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="49" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="B42" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A42)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C42" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A42,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -27939,7 +27721,7 @@
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="49" t="s">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="B43" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A43)</f>
@@ -27956,24 +27738,24 @@
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="49" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="B44" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A44)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C44" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A44,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D44" s="49" t="n">
         <f aca="false">IFERROR(C44/B44,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="49" t="s">
-        <v>41</v>
+        <v>79</v>
       </c>
       <c r="B45" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A45)</f>
@@ -27981,20 +27763,20 @@
       </c>
       <c r="C45" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A45,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D45" s="49" t="n">
         <f aca="false">IFERROR(C45/B45,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="49" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="B46" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A46)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C46" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A46,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -28007,11 +27789,11 @@
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="49" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="B47" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A47)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C47" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A47,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -28024,11 +27806,11 @@
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="49" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B48" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A48)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C48" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A48,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -28041,7 +27823,7 @@
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="49" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B49" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A49)</f>
@@ -28049,16 +27831,16 @@
       </c>
       <c r="C49" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A49,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D49" s="49" t="n">
         <f aca="false">IFERROR(C49/B49,0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="49" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B50" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A50)</f>
@@ -28075,24 +27857,24 @@
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="49" t="s">
-        <v>97</v>
+        <v>156</v>
       </c>
       <c r="B51" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A51)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C51" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A51,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D51" s="49" t="n">
         <f aca="false">IFERROR(C51/B51,0)</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="49" t="s">
-        <v>156</v>
+        <v>43</v>
       </c>
       <c r="B52" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A52)</f>
@@ -28109,7 +27891,7 @@
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="49" t="s">
-        <v>43</v>
+        <v>159</v>
       </c>
       <c r="B53" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A53)</f>
@@ -28125,46 +27907,46 @@
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="49" t="s">
-        <v>159</v>
-      </c>
-      <c r="B54" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A54)</f>
-        <v>0</v>
-      </c>
-      <c r="C54" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Ryan",'Game Log Season 3'!$D$3:$D$1000,A54,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D54" s="49" t="n">
+      <c r="A54" s="47" t="s">
+        <v>70</v>
+      </c>
+      <c r="B54" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A54)</f>
+        <v>2</v>
+      </c>
+      <c r="C54" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A54,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D54" s="48" t="n">
         <f aca="false">IFERROR(C54/B54,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="47" t="s">
-        <v>70</v>
-      </c>
-      <c r="B55" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A55)</f>
-        <v>2</v>
-      </c>
-      <c r="C55" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A55,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D55" s="48" t="n">
+      <c r="A55" s="49" t="s">
+        <v>71</v>
+      </c>
+      <c r="B55" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A55)</f>
+        <v>0</v>
+      </c>
+      <c r="C55" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A55,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D55" s="49" t="n">
         <f aca="false">IFERROR(C55/B55,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="49" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="B56" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A56)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C56" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A56,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -28177,11 +27959,11 @@
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="49" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="B57" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A57)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C57" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A57,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -28194,7 +27976,7 @@
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="49" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B58" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A58)</f>
@@ -28211,11 +27993,11 @@
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="49" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B59" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A59)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C59" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A59,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -28227,42 +28009,42 @@
       </c>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="49" t="s">
-        <v>93</v>
-      </c>
-      <c r="B60" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A60)</f>
-        <v>1</v>
-      </c>
-      <c r="C60" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Kristy",'Game Log Season 3'!$D$3:$D$1000,A60,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D60" s="49" t="n">
+      <c r="A60" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="B60" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A60)</f>
+        <v>1</v>
+      </c>
+      <c r="C60" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A60,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D60" s="48" t="n">
         <f aca="false">IFERROR(C60/B60,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="47" t="s">
-        <v>38</v>
-      </c>
-      <c r="B61" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A61)</f>
-        <v>1</v>
-      </c>
-      <c r="C61" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A61,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D61" s="48" t="n">
+      <c r="A61" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="B61" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A61)</f>
+        <v>0</v>
+      </c>
+      <c r="C61" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A61,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D61" s="49" t="n">
         <f aca="false">IFERROR(C61/B61,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="49" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="B62" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A62)</f>
@@ -28279,7 +28061,7 @@
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="49" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B63" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A63)</f>
@@ -28296,7 +28078,7 @@
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="49" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="B64" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A64)</f>
@@ -28313,11 +28095,11 @@
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B65" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A65)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C65" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A65,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -28329,42 +28111,42 @@
       </c>
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="49" t="s">
-        <v>63</v>
-      </c>
-      <c r="B66" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A66)</f>
-        <v>1</v>
-      </c>
-      <c r="C66" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Joseph",'Game Log Season 3'!$D$3:$D$1000,A66,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D66" s="49" t="n">
+      <c r="A66" s="47" t="s">
+        <v>59</v>
+      </c>
+      <c r="B66" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A66)</f>
+        <v>0</v>
+      </c>
+      <c r="C66" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A66,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D66" s="48" t="n">
         <f aca="false">IFERROR(C66/B66,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="47" t="s">
-        <v>59</v>
-      </c>
-      <c r="B67" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A67)</f>
-        <v>0</v>
-      </c>
-      <c r="C67" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A67,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D67" s="48" t="n">
+      <c r="A67" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="B67" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A67)</f>
+        <v>0</v>
+      </c>
+      <c r="C67" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A67,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D67" s="49" t="n">
         <f aca="false">IFERROR(C67/B67,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="49" t="s">
-        <v>33</v>
+        <v>69</v>
       </c>
       <c r="B68" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A68)</f>
@@ -28381,7 +28163,7 @@
     </row>
     <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="49" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="B69" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A69)</f>
@@ -28397,46 +28179,46 @@
       </c>
     </row>
     <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="49" t="s">
-        <v>84</v>
-      </c>
-      <c r="B70" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A70)</f>
-        <v>0</v>
-      </c>
-      <c r="C70" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Red",'Game Log Season 3'!$D$3:$D$1000,A70,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D70" s="49" t="n">
+      <c r="A70" s="47" t="s">
+        <v>51</v>
+      </c>
+      <c r="B70" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A70)</f>
+        <v>4</v>
+      </c>
+      <c r="C70" s="48" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A70,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D70" s="48" t="n">
         <f aca="false">IFERROR(C70/B70,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="47" t="s">
-        <v>51</v>
-      </c>
-      <c r="B71" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A71)</f>
-        <v>4</v>
-      </c>
-      <c r="C71" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A71,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D71" s="48" t="n">
+      <c r="A71" s="49" t="s">
+        <v>52</v>
+      </c>
+      <c r="B71" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A71)</f>
+        <v>3</v>
+      </c>
+      <c r="C71" s="49" t="n">
+        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A71,'Game Log Season 3'!$F$3:$F$1000,1)</f>
+        <v>0</v>
+      </c>
+      <c r="D71" s="49" t="n">
         <f aca="false">IFERROR(C71/B71,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="49" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B72" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A72)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C72" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A72,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -28449,11 +28231,11 @@
     </row>
     <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="49" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="B73" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A73)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C73" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A73,'Game Log Season 3'!$F$3:$F$1000,1)</f>
@@ -28461,244 +28243,6 @@
       </c>
       <c r="D73" s="49" t="n">
         <f aca="false">IFERROR(C73/B73,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="49" t="s">
-        <v>96</v>
-      </c>
-      <c r="B74" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A74)</f>
-        <v>1</v>
-      </c>
-      <c r="C74" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Michelle",'Game Log Season 3'!$D$3:$D$1000,A74,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D74" s="49" t="n">
-        <f aca="false">IFERROR(C74/B74,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="47" t="s">
-        <v>165</v>
-      </c>
-      <c r="B75" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A75)</f>
-        <v>0</v>
-      </c>
-      <c r="C75" s="48" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,A75,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D75" s="48" t="n">
-        <f aca="false">IFERROR(C75/B75,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="49" t="s">
-        <v>37</v>
-      </c>
-      <c r="B76" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A76)</f>
-        <v>0</v>
-      </c>
-      <c r="C76" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A76,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D76" s="49" t="n">
-        <f aca="false">IFERROR(C76/B76,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="49" t="s">
-        <v>48</v>
-      </c>
-      <c r="B77" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A77)</f>
-        <v>0</v>
-      </c>
-      <c r="C77" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A77,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D77" s="49" t="n">
-        <f aca="false">IFERROR(C77/B77,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="49" t="s">
-        <v>168</v>
-      </c>
-      <c r="B78" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A78)</f>
-        <v>0</v>
-      </c>
-      <c r="C78" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A78,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D78" s="49" t="n">
-        <f aca="false">IFERROR(C78/B78,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="49" t="s">
-        <v>119</v>
-      </c>
-      <c r="B79" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A79)</f>
-        <v>0</v>
-      </c>
-      <c r="C79" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A79,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D79" s="49" t="n">
-        <f aca="false">IFERROR(C79/B79,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="49" t="s">
-        <v>68</v>
-      </c>
-      <c r="B80" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A80)</f>
-        <v>0</v>
-      </c>
-      <c r="C80" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A80,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D80" s="49" t="n">
-        <f aca="false">IFERROR(C80/B80,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="49" t="s">
-        <v>91</v>
-      </c>
-      <c r="B81" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A81)</f>
-        <v>0</v>
-      </c>
-      <c r="C81" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A81,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D81" s="49" t="n">
-        <f aca="false">IFERROR(C81/B81,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="49" t="s">
-        <v>82</v>
-      </c>
-      <c r="B82" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A82)</f>
-        <v>0</v>
-      </c>
-      <c r="C82" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A82,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D82" s="49" t="n">
-        <f aca="false">IFERROR(C82/B82,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="49" t="s">
-        <v>121</v>
-      </c>
-      <c r="B83" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A83)</f>
-        <v>0</v>
-      </c>
-      <c r="C83" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A83,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D83" s="49" t="n">
-        <f aca="false">IFERROR(C83/B83,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="49" t="s">
-        <v>175</v>
-      </c>
-      <c r="B84" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A84)</f>
-        <v>0</v>
-      </c>
-      <c r="C84" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A84,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D84" s="49" t="n">
-        <f aca="false">IFERROR(C84/B84,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="49" t="s">
-        <v>123</v>
-      </c>
-      <c r="B85" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A85)</f>
-        <v>0</v>
-      </c>
-      <c r="C85" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A85,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D85" s="49" t="n">
-        <f aca="false">IFERROR(C85/B85,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="49" t="s">
-        <v>156</v>
-      </c>
-      <c r="B86" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A86)</f>
-        <v>0</v>
-      </c>
-      <c r="C86" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A86,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D86" s="49" t="n">
-        <f aca="false">IFERROR(C86/B86,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="49" t="s">
-        <v>88</v>
-      </c>
-      <c r="B87" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A87)</f>
-        <v>0</v>
-      </c>
-      <c r="C87" s="49" t="n">
-        <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Hiccup_The_Hero",'Game Log Season 3'!$D$3:$D$1000,A87,'Game Log Season 3'!$F$3:$F$1000,1)</f>
-        <v>0</v>
-      </c>
-      <c r="D87" s="49" t="n">
-        <f aca="false">IFERROR(C87/B87,0)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Edit three deck entries: Leonardo rename/reprice, Katara and Sokka power/bracket updates
Add scripts/edit_deck.py for in-place deck row edits (rename, reprice,
set bracket note). Leonardo, the Balance -> Leonardo, the Balance/
Michelangelo, the Heart (power 2.6); Katara, the Fearless -> power 2.0,
Bracket 2; Sokka, Tenacious Tactician -> power 3.0, Bracket 3.
</commit_message>
<xml_diff>
--- a/deck-strength.xlsx
+++ b/deck-strength.xlsx
@@ -25943,9 +25943,13 @@
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Becca")*('Game Log Season 3'!$D$3:$D$1000=A7)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D7)</f>
         <v>3.9</v>
       </c>
-      <c r="C7" s="46"/>
+      <c r="C7" s="46" t="inlineStr">
+        <is>
+          <t>*Bracket 2</t>
+        </is>
+      </c>
       <c r="D7" s="49" t="n">
-        <v>3.9</v>
+        <v>2</v>
       </c>
       <c r="E7" s="47" t="s">
         <v>107</v>
@@ -26165,9 +26169,13 @@
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Manny")*('Game Log Season 3'!$D$3:$D$1000=A21)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D21)</f>
         <v>4.1</v>
       </c>
-      <c r="C21" s="46"/>
+      <c r="C21" s="46" t="inlineStr">
+        <is>
+          <t>*Bracket 3</t>
+        </is>
+      </c>
       <c r="D21" s="49" t="n">
-        <v>4.1</v>
+        <v>3</v>
       </c>
       <c r="E21" s="47" t="s">
         <v>124</v>
@@ -26443,8 +26451,10 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="49" t="s">
-        <v>144</v>
+      <c r="A39" s="49" t="inlineStr">
+        <is>
+          <t>Leonardo, the Balance/Michelangelo, the Heart</t>
+        </is>
       </c>
       <c r="B39" s="49" t="n">
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Mateo")*('Game Log Season 3'!$D$3:$D$1000=A39)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D39)</f>
@@ -26452,7 +26462,7 @@
       </c>
       <c r="C39" s="46"/>
       <c r="D39" s="49" t="n">
-        <v>3.4</v>
+        <v>2.6</v>
       </c>
       <c r="E39" s="47" t="s">
         <v>145</v>
@@ -27623,8 +27633,10 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="49" t="s">
-        <v>144</v>
+      <c r="A39" s="49" t="inlineStr">
+        <is>
+          <t>Leonardo, the Balance/Michelangelo, the Heart</t>
+        </is>
       </c>
       <c r="B39" s="49" t="n">
         <f aca="false">COUNTIFS('Game Log Season 3'!$C$3:$C$1000,"Mateo",'Game Log Season 3'!$D$3:$D$1000,A39)</f>

</xml_diff>

<commit_message>
Set bracket note on Ryan's Fire Lord Zuko to Bracket 4
Bracket is a free-text note (column C) independent of the power/
strength formula, so this doesn't change the deck's computed power.
</commit_message>
<xml_diff>
--- a/deck-strength.xlsx
+++ b/deck-strength.xlsx
@@ -26544,7 +26544,11 @@
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A45)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D45)</f>
         <v>3.77816666666667</v>
       </c>
-      <c r="C45" s="46"/>
+      <c r="C45" s="46" t="inlineStr">
+        <is>
+          <t>*Bracket 4</t>
+        </is>
+      </c>
       <c r="D45" s="49" t="n">
         <v>3.8</v>
       </c>

</xml_diff>

<commit_message>
Revert bracket note on Ryan's Fire Lord Zuko
Confirmed bracket doesn't affect calculated power; reverting the note
back to its prior empty state per request.
</commit_message>
<xml_diff>
--- a/deck-strength.xlsx
+++ b/deck-strength.xlsx
@@ -26547,9 +26547,7 @@
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Ryan")*('Game Log Season 3'!$D$3:$D$1000=A45)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D45)</f>
         <v>3.77816666666667</v>
       </c>
-      <c r="C45" s="46" t="s">
-        <v>150</v>
-      </c>
+      <c r="C45" s="46"/>
       <c r="D45" s="49" t="n">
         <v>3.8</v>
       </c>

</xml_diff>

<commit_message>
Update Katara, the Fearless to Bracket 3, raising power to ~3.9
Bracket feeds directly into Game Calculated Deck Strength
(X = weighted_score + bracket, no normalization), so bumping Game 15's
logged bracket from 2 to 3 shifts the calculated power from 2.899 to
~3.899 -- the power change requested is a direct consequence of the
bracket change, not a separate edit. Updated both the Game Log's own
bracket column (Game 15, row 56) and Current Deck Strength's bracket
note to match.
</commit_message>
<xml_diff>
--- a/deck-strength.xlsx
+++ b/deck-strength.xlsx
@@ -25833,7 +25833,7 @@
         <v>0</v>
       </c>
       <c r="W56" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X56" s="15" t="n">
         <f aca="false">((O56*0.3)+(Q56*0.175)+(R56*0.175)+(U56*0.175)+((1-V56)*0.175))+W56</f>
@@ -26735,8 +26735,10 @@
         <f aca="false">IFERROR(LOOKUP(2,1/(('Game Log Season 3'!$C$3:$C$1000="Becca")*('Game Log Season 3'!$D$3:$D$1000=A7)*('Game Log Season 3'!$X$3:$X$1000&lt;&gt;"")),'Game Log Season 3'!$X$3:$X$1000), D7)</f>
         <v>2.89916666666667</v>
       </c>
-      <c r="C7" s="45" t="s">
-        <v>109</v>
+      <c r="C7" s="45" t="inlineStr">
+        <is>
+          <t>*Bracket 3</t>
+        </is>
       </c>
       <c r="D7" s="48" t="n">
         <v>2</v>

</xml_diff>